<commit_message>
Update latest output (run 587)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,42 +470,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46278.22916666666</v>
+        <v>46278.1875</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46278.72916666666</v>
+        <v>46278.75</v>
       </c>
       <c r="C2" t="n">
-        <v>12</v>
+        <v>13.5</v>
       </c>
       <c r="D2" t="n">
-        <v>45.36</v>
+        <v>51.02999999999999</v>
       </c>
       <c r="E2" t="n">
-        <v>91.34072999999998</v>
+        <v>328.918356</v>
       </c>
       <c r="F2" t="n">
-        <v>2.013684523809523</v>
+        <v>6.445588007054675</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46278.77083333334</v>
+        <v>46278.89583333334</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46278.9375</v>
+        <v>46279.14583333334</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D3" t="n">
-        <v>15.12</v>
+        <v>22.68</v>
       </c>
       <c r="E3" t="n">
-        <v>590.5495927500001</v>
+        <v>792.7506697499998</v>
       </c>
       <c r="F3" t="n">
-        <v>39.05751274801588</v>
+        <v>34.95373323412698</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46279.3125</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46279.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>32.13</v>
+      </c>
+      <c r="E4" t="n">
+        <v>45.00618525</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.400752731092437</v>
       </c>
     </row>
   </sheetData>
@@ -519,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,14 +571,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46278.02083333334</v>
+        <v>46278</v>
       </c>
       <c r="B2" t="n">
-        <v>83.98999999999999</v>
+        <v>75.9601</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
@@ -572,14 +592,14 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46278.04166666666</v>
+        <v>46278.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>79.65407</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
@@ -593,14 +613,14 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46278.0625</v>
+        <v>46278.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>80.25073999999999</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
@@ -614,14 +634,14 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46278.08333333334</v>
+        <v>46278.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>71.40000000000001</v>
+        <v>80.24146</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
@@ -635,14 +655,14 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46278.10416666666</v>
+        <v>46278.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>80.34601000000001</v>
+        <v>79.78327</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
@@ -656,14 +676,14 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46278.125</v>
+        <v>46278.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>80.36269</v>
+        <v>79.80694</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
@@ -677,14 +697,14 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46278.14583333334</v>
+        <v>46278.125</v>
       </c>
       <c r="B8" t="n">
-        <v>79.33799</v>
+        <v>79.81386999999999</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
@@ -698,14 +718,14 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46278.16666666666</v>
+        <v>46278.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>75.96007</v>
+        <v>79.30059</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -719,14 +739,14 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46278.1875</v>
+        <v>46278.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>75.96007</v>
+        <v>78.79389999999999</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
@@ -740,14 +760,14 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46278.20833333334</v>
+        <v>46278.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>75.96007</v>
+        <v>79.27057000000001</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -755,20 +775,20 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46278.22916666666</v>
+        <v>46278.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>70.06726999999999</v>
+        <v>79.23627</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
@@ -782,14 +802,14 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46278.25</v>
+        <v>46278.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>67.84366</v>
+        <v>75.96007</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
@@ -803,14 +823,14 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46278.27083333334</v>
+        <v>46278.25</v>
       </c>
       <c r="B14" t="n">
-        <v>67.01438</v>
+        <v>68.26627999999999</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
@@ -824,14 +844,14 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46278.29166666666</v>
+        <v>46278.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>4e-05</v>
+        <v>66.58056000000001</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
@@ -845,14 +865,14 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46278.3125</v>
+        <v>46278.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>-4.00838</v>
+        <v>4e-05</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
@@ -866,14 +886,14 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46278.33333333334</v>
+        <v>46278.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>-6.5</v>
+        <v>-4</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
@@ -887,14 +907,14 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46278.35416666666</v>
+        <v>46278.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>-7.84826</v>
+        <v>-6.10928</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -908,14 +928,14 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46278.375</v>
+        <v>46278.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>-9.32</v>
+        <v>-7.97188</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -929,14 +949,14 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46278.39583333334</v>
+        <v>46278.375</v>
       </c>
       <c r="B20" t="n">
-        <v>-8.855409999999999</v>
+        <v>-9.39762</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -950,14 +970,14 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46278.41666666666</v>
+        <v>46278.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>-9.89791</v>
+        <v>-9.00601</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -971,14 +991,14 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46278.4375</v>
+        <v>46278.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-9.32</v>
+        <v>-10.02464</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -992,14 +1012,14 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46278.45833333334</v>
+        <v>46278.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-9.580080000000001</v>
+        <v>-10.5</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1013,14 +1033,14 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46278.47916666666</v>
+        <v>46278.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-8.50357</v>
+        <v>-14.27101</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1034,14 +1054,14 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46278.5</v>
+        <v>46278.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-9.516830000000001</v>
+        <v>-10.5</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1055,14 +1075,14 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46278.52083333334</v>
+        <v>46278.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-12.88107</v>
+        <v>-9.47307</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1076,14 +1096,14 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46278.54166666666</v>
+        <v>46278.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-23.5</v>
+        <v>-18.51</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1097,14 +1117,14 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46278.5625</v>
+        <v>46278.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-18.51</v>
+        <v>-13</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1118,14 +1138,14 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46278.58333333334</v>
+        <v>46278.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-13.79881</v>
+        <v>-13</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1139,14 +1159,14 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46278.60416666666</v>
+        <v>46278.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-9.818989999999999</v>
+        <v>-13.22659</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1160,14 +1180,14 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46278.625</v>
+        <v>46278.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-8.969659999999999</v>
+        <v>-9.192640000000001</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1181,14 +1201,14 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46278.64583333334</v>
+        <v>46278.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-7.67665</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1202,14 +1222,14 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46278.66666666666</v>
+        <v>46278.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>-3.3275</v>
+        <v>-7.16264</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1223,14 +1243,14 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46278.6875</v>
+        <v>46278.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>13.20028</v>
+        <v>-4.53692</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1244,14 +1264,14 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46278.70833333334</v>
+        <v>46278.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>57.39029</v>
+        <v>13.20028</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1265,14 +1285,14 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46278.72916666666</v>
+        <v>46278.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>80.51408000000001</v>
+        <v>57.39029</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1280,20 +1300,20 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46278.75</v>
+        <v>46278.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>82.25605</v>
+        <v>75.9601</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1301,20 +1321,20 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46278.77083333334</v>
+        <v>46278.75</v>
       </c>
       <c r="B38" t="n">
-        <v>71.40000000000001</v>
+        <v>79.66528</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1322,20 +1342,20 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46278.79166666666</v>
+        <v>46278.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>71.40000000000001</v>
+        <v>82.64327</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1343,20 +1363,20 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46278.8125</v>
+        <v>46278.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>78.67683</v>
+        <v>76.34065</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1364,20 +1384,20 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46278.83333333334</v>
+        <v>46278.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>80.36554</v>
+        <v>80.21342</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1385,20 +1405,20 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46278.85416666666</v>
+        <v>46278.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>79.05289</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -1406,20 +1426,20 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46278.875</v>
+        <v>46278.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>75.9601</v>
+        <v>83.68952</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
@@ -1427,20 +1447,20 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46278.89583333334</v>
+        <v>46278.875</v>
       </c>
       <c r="B44" t="n">
-        <v>72.79474999999999</v>
+        <v>81.58286</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D44" s="3" t="n">
@@ -1448,20 +1468,20 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46278.91666666666</v>
+        <v>46278.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>76.04178</v>
+        <v>77.60453</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D45" s="3" t="n">
@@ -1475,14 +1495,14 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46278.9375</v>
+        <v>46278.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>78.41924</v>
+        <v>71.61559</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D46" s="3" t="n">
@@ -1490,13 +1510,13 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46278.95833333334</v>
+        <v>46278.9375</v>
       </c>
       <c r="B47" t="n">
         <v>75.9601</v>
@@ -1511,26 +1531,1055 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
+        <v>46278.95833333334</v>
+      </c>
+      <c r="B48" t="n">
+        <v>66.52</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
         <v>46278.97916666666</v>
       </c>
-      <c r="B48" t="n">
-        <v>71.44861</v>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>forecast</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="n">
-        <v>46278</v>
-      </c>
-      <c r="E48" t="inlineStr">
+      <c r="B49" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B50" t="n">
+        <v>65.46812</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46279.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46279.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46279.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>64.95</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46279.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>64.95</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46279.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>64.95</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46279.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>64.55927</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46279.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>64.95</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46279.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>65.36306</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46279.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>78.83566</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46279.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>79.05168</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46279.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>66.52</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46279.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46279.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46279.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>71.38</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46279.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>42.79977</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46279.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46279.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46279.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46279.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46279.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46279.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-6.33</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46279.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46279.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46279.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>9.64106</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46279.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>9.820550000000001</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46279.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>10.1498</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46279.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-6.70372</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46279.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>0.63007</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46279.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-9.32</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46279.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>-9.01998</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46279.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>-8.887409999999999</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46279.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>-7.07898</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46279.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>9.85308</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46279.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>75.15013</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46279.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>87.16236000000001</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46279.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>97.96795</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46279.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46279.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46279.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46279.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>94.73505</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46279.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46279.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46279.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>84.02566</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46279.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46279.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46279.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46279.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>77.21008999999999</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 662)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>353.9966430000001</v>
+        <v>377.6530875000001</v>
       </c>
       <c r="F2" t="n">
-        <v>8.51362777777778</v>
+        <v>9.082565836940841</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46280.20833333334</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46280.66666666666</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>131.26513725</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3.156929707792207</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -853,7 +873,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
@@ -870,11 +890,11 @@
         <v>46279.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>32.43984</v>
+        <v>28.01</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -895,7 +915,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -912,11 +932,11 @@
         <v>46279.375</v>
       </c>
       <c r="B20" t="n">
-        <v>11.86408</v>
+        <v>5e-05</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -933,11 +953,11 @@
         <v>46279.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>-6.5</v>
+        <v>2.12</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +974,11 @@
         <v>46279.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-7.40377</v>
+        <v>2.12</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +995,11 @@
         <v>46279.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-6.5</v>
+        <v>2.12</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46279.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-6.94385</v>
+        <v>-6.33</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46279.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-3.61458</v>
+        <v>-4.37354</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46279.5</v>
       </c>
       <c r="B26" t="n">
-        <v>0</v>
+        <v>-7.18059</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46279.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>0.63007</v>
+        <v>-6.5</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46279.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>9.78703</v>
+        <v>11.5</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1121,11 @@
         <v>46279.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-8.85327</v>
+        <v>0.63007</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46279.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-8.59679</v>
+        <v>8.75872</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1163,11 @@
         <v>46279.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-9.20458</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46279.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-8.612579999999999</v>
+        <v>-9.10793</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1205,11 @@
         <v>46279.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>-8.45914</v>
+        <v>-8.8413</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1226,11 @@
         <v>46279.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>-6.64715</v>
+        <v>-7.07855</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1247,11 @@
         <v>46279.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>10.42317</v>
+        <v>9.851839999999999</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1268,11 @@
         <v>46279.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>75.9601</v>
+        <v>74.82621</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1289,11 @@
         <v>46279.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>83.98999999999999</v>
+        <v>82.78774</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1310,11 @@
         <v>46279.75</v>
       </c>
       <c r="B38" t="n">
-        <v>96.02845000000001</v>
+        <v>97.28787</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,7 +1331,7 @@
         <v>46279.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>91.27021000000001</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1332,7 +1352,7 @@
         <v>46279.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>90.59363</v>
+        <v>83.02303000000001</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1353,7 +1373,7 @@
         <v>46279.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>94.80435</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1374,7 +1394,7 @@
         <v>46279.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>93.26376999999999</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1415,7 @@
         <v>46279.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>89.84389</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1436,7 @@
         <v>46279.875</v>
       </c>
       <c r="B44" t="n">
-        <v>84.48653</v>
+        <v>79.33472999999999</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46279.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>91.92803000000001</v>
+        <v>81.17221000000001</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46279.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>83.98999999999999</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46279.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>83.98999999999999</v>
+        <v>71.38</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1520,7 @@
         <v>46279.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>83.98999999999999</v>
+        <v>77.02012999999999</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,7 +1541,7 @@
         <v>46279.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>83.98999999999999</v>
+        <v>65.5</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46279</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B50" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46280.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>65.67729</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46280.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>65.51000000000001</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46280.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>66.73651</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46280.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>66.78704</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46280.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>66.39022</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46280.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>64.95</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46280.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>64.95</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46280.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>64.95</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46280.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>65.51000000000001</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46280.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>69.91</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46280.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>66.52</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46280.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>65.51000000000001</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46280.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>75.9601</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46280.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>57.39007</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46280.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>0.0107</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46280.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>-0.9174</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46280.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>-5.61161</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46280.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>-7.64944</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46280.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>-8.48827</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46280.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>-8.950710000000001</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46280.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-8.762219999999999</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46280.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46280.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>-12.98734</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46280.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>-12.81486</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46280.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>-9.167339999999999</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46280.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46280.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-23.5</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46280.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-23.5</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46280.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-26.61479</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46280.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>-18.51</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46280.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>-12.19598</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46280.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>-6.87393</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46280.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>-3.7991</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46280.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>51.83245</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46280.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46280.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>69.63330000000001</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46280.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>77.76276</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46280.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>86.74499</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46280.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>85.77661999999999</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46280.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>77.06949</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46280.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>76.32823</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46280.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>80.5784</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46280.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>74.6568</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46280.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>75.9601</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46280.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46280.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>75.82084999999999</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46280.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>70.1652</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 588)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,62 +470,82 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46278.1875</v>
+        <v>46279</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46278.75</v>
+        <v>46279.1875</v>
       </c>
       <c r="C2" t="n">
-        <v>13.5</v>
+        <v>4.5</v>
       </c>
       <c r="D2" t="n">
-        <v>51.02999999999999</v>
+        <v>17.01</v>
       </c>
       <c r="E2" t="n">
-        <v>328.918356</v>
+        <v>566.704203</v>
       </c>
       <c r="F2" t="n">
-        <v>6.445588007054675</v>
+        <v>33.31594373897708</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46278.89583333334</v>
+        <v>46279.20833333334</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46279.14583333334</v>
+        <v>46279.66666666666</v>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D3" t="n">
-        <v>22.68</v>
+        <v>41.58</v>
       </c>
       <c r="E3" t="n">
-        <v>792.7506697499998</v>
+        <v>377.6530875000001</v>
       </c>
       <c r="F3" t="n">
-        <v>34.95373323412698</v>
+        <v>9.082565836940841</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46279.3125</v>
+        <v>46279.97916666666</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>46279.66666666666</v>
+        <v>46280.14583333334</v>
       </c>
       <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="E4" t="n">
+        <v>542.3622067499999</v>
+      </c>
+      <c r="F4" t="n">
+        <v>35.87051631944444</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46280.3125</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46280.66666666666</v>
+      </c>
+      <c r="C5" t="n">
         <v>8.5</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D5" t="n">
         <v>32.13</v>
       </c>
-      <c r="E4" t="n">
-        <v>45.00618525</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1.400752731092437</v>
+      <c r="E5" t="n">
+        <v>-147.2346915</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-4.582467833800188</v>
       </c>
     </row>
   </sheetData>
@@ -571,10 +591,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="B2" t="n">
-        <v>75.9601</v>
+        <v>65.44708</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -582,20 +602,20 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46278.02083333334</v>
+        <v>46279.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>71.40000000000001</v>
+        <v>66.79613999999999</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -603,20 +623,20 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46278.04166666666</v>
+        <v>46279.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>83.98999999999999</v>
+        <v>65.5</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -624,20 +644,20 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46278.0625</v>
+        <v>46279.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>80.24146</v>
+        <v>64.95</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -645,20 +665,20 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46278.08333333334</v>
+        <v>46279.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>79.78327</v>
+        <v>64.95</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -666,20 +686,20 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46278.10416666666</v>
+        <v>46279.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>79.80694</v>
+        <v>63.59102</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -687,20 +707,20 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46278.125</v>
+        <v>46279.125</v>
       </c>
       <c r="B8" t="n">
-        <v>79.81386999999999</v>
+        <v>58.53084</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -708,20 +728,20 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46278.14583333334</v>
+        <v>46279.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>79.30059</v>
+        <v>64.95</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -729,20 +749,20 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46278.16666666666</v>
+        <v>46279.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>78.79389999999999</v>
+        <v>66.52</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -750,20 +770,20 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46278.1875</v>
+        <v>46279.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>79.27057000000001</v>
+        <v>75.96007</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -771,20 +791,20 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46278.20833333334</v>
+        <v>46279.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>79.23627</v>
+        <v>64.95</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -792,7 +812,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -802,10 +822,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46278.22916666666</v>
+        <v>46279.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>75.96007</v>
+        <v>64.95</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -813,7 +833,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -823,10 +843,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46278.25</v>
+        <v>46279.25</v>
       </c>
       <c r="B14" t="n">
-        <v>68.26627999999999</v>
+        <v>64.89</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -834,7 +854,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -844,10 +864,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46278.27083333334</v>
+        <v>46279.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>66.58056000000001</v>
+        <v>71.95125</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -855,7 +875,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -865,10 +885,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46278.29166666666</v>
+        <v>46279.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>4e-05</v>
+        <v>71.38</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -876,7 +896,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -886,10 +906,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46278.3125</v>
+        <v>46279.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>-4</v>
+        <v>42.79977</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -897,7 +917,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -907,10 +927,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46278.33333333334</v>
+        <v>46279.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>-6.10928</v>
+        <v>28.01</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,7 +938,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -928,10 +948,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46278.35416666666</v>
+        <v>46279.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>-7.97188</v>
+        <v>2.12</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -939,7 +959,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -949,10 +969,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46278.375</v>
+        <v>46279.375</v>
       </c>
       <c r="B20" t="n">
-        <v>-9.39762</v>
+        <v>5e-05</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -960,7 +980,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -970,10 +990,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46278.39583333334</v>
+        <v>46279.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>-9.00601</v>
+        <v>2.12</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -981,7 +1001,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -991,10 +1011,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46278.41666666666</v>
+        <v>46279.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-10.02464</v>
+        <v>2.12</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1002,7 +1022,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1012,10 +1032,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46278.4375</v>
+        <v>46279.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-10.5</v>
+        <v>2.12</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1023,7 +1043,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1033,10 +1053,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46278.45833333334</v>
+        <v>46279.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-14.27101</v>
+        <v>-6.33</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1044,7 +1064,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1054,10 +1074,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46278.47916666666</v>
+        <v>46279.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-10.5</v>
+        <v>-4.37354</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1065,7 +1085,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1075,10 +1095,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46278.5</v>
+        <v>46279.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-9.47307</v>
+        <v>-7.18059</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1086,7 +1106,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1096,10 +1116,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46278.52083333334</v>
+        <v>46279.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-18.51</v>
+        <v>-6.5</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1107,7 +1127,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1117,10 +1137,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46278.54166666666</v>
+        <v>46279.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-13</v>
+        <v>11.5</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1128,7 +1148,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1138,10 +1158,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46278.5625</v>
+        <v>46279.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-13</v>
+        <v>0.63007</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1149,7 +1169,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1159,10 +1179,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46278.58333333334</v>
+        <v>46279.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-13.22659</v>
+        <v>8.75872</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1170,7 +1190,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1180,10 +1200,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46278.60416666666</v>
+        <v>46279.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-9.192640000000001</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1191,7 +1211,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1201,10 +1221,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46278.625</v>
+        <v>46279.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-8.630000000000001</v>
+        <v>-9.10793</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1212,7 +1232,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1222,10 +1242,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46278.64583333334</v>
+        <v>46279.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>-7.16264</v>
+        <v>-8.8413</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1233,7 +1253,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1243,10 +1263,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46278.66666666666</v>
+        <v>46279.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>-4.53692</v>
+        <v>-7.07855</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1254,20 +1274,20 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46278.6875</v>
+        <v>46279.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>13.20028</v>
+        <v>9.851839999999999</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1275,20 +1295,20 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46278.70833333334</v>
+        <v>46279.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>57.39029</v>
+        <v>74.82621</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1296,20 +1316,20 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46278.72916666666</v>
+        <v>46279.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>75.9601</v>
+        <v>82.78774</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1317,20 +1337,20 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46278.75</v>
+        <v>46279.75</v>
       </c>
       <c r="B38" t="n">
-        <v>79.66528</v>
+        <v>97.28787</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1338,7 +1358,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1348,10 +1368,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46278.77083333334</v>
+        <v>46279.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>82.64327</v>
+        <v>99.64353</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1359,7 +1379,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1369,10 +1389,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46278.79166666666</v>
+        <v>46279.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>76.34065</v>
+        <v>99.92856999999999</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1380,7 +1400,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1390,10 +1410,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46278.8125</v>
+        <v>46279.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>80.21342</v>
+        <v>93.91200000000001</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1401,7 +1421,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1411,10 +1431,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46278.83333333334</v>
+        <v>46279.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>83.98999999999999</v>
+        <v>94.40582999999999</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1422,7 +1442,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1432,10 +1452,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46278.85416666666</v>
+        <v>46279.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>83.68952</v>
+        <v>93.49764</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1443,7 +1463,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1453,10 +1473,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46278.875</v>
+        <v>46279.875</v>
       </c>
       <c r="B44" t="n">
-        <v>81.58286</v>
+        <v>85.03485000000001</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1464,7 +1484,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1474,10 +1494,10 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46278.89583333334</v>
+        <v>46279.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>77.60453</v>
+        <v>84.02096</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1485,20 +1505,20 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46278.91666666666</v>
+        <v>46279.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>71.61559</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1506,62 +1526,62 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46278.9375</v>
+        <v>46279.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>75.9601</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46278.95833333334</v>
+        <v>46279.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>66.52</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46278.97916666666</v>
+        <v>46279.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>65.5</v>
+        <v>71.38</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1569,7 +1589,7 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1579,10 +1599,10 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="B50" t="n">
-        <v>65.46812</v>
+        <v>69.7102</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1590,7 +1610,7 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1600,10 +1620,10 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46279.02083333334</v>
+        <v>46280.02083333334</v>
       </c>
       <c r="B51" t="n">
-        <v>65.5</v>
+        <v>75.9601</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1611,7 +1631,7 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1621,10 +1641,10 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46279.04166666666</v>
+        <v>46280.04166666666</v>
       </c>
       <c r="B52" t="n">
-        <v>65.5</v>
+        <v>67.71827999999999</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1632,7 +1652,7 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1642,10 +1662,10 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46279.0625</v>
+        <v>46280.0625</v>
       </c>
       <c r="B53" t="n">
-        <v>64.95</v>
+        <v>66.57662999999999</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1653,7 +1673,7 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1663,10 +1683,10 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46279.08333333334</v>
+        <v>46280.08333333334</v>
       </c>
       <c r="B54" t="n">
-        <v>64.95</v>
+        <v>68.28270999999999</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1674,7 +1694,7 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1684,10 +1704,10 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46279.10416666666</v>
+        <v>46280.10416666666</v>
       </c>
       <c r="B55" t="n">
-        <v>64.95</v>
+        <v>68.31310999999999</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1695,7 +1715,7 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1705,10 +1725,10 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46279.125</v>
+        <v>46280.125</v>
       </c>
       <c r="B56" t="n">
-        <v>64.55927</v>
+        <v>68.3279</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1716,7 +1736,7 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1726,10 +1746,10 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46279.14583333334</v>
+        <v>46280.14583333334</v>
       </c>
       <c r="B57" t="n">
-        <v>64.95</v>
+        <v>64.89</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1737,7 +1757,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1747,10 +1767,10 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46279.16666666666</v>
+        <v>46280.16666666666</v>
       </c>
       <c r="B58" t="n">
-        <v>65.36306</v>
+        <v>75.96007</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1758,7 +1778,7 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1768,10 +1788,10 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46279.1875</v>
+        <v>46280.1875</v>
       </c>
       <c r="B59" t="n">
-        <v>78.83566</v>
+        <v>75.96007</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1779,7 +1799,7 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1789,10 +1809,10 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46279.20833333334</v>
+        <v>46280.20833333334</v>
       </c>
       <c r="B60" t="n">
-        <v>79.05168</v>
+        <v>82.90672000000001</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1800,7 +1820,7 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1810,10 +1830,10 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46279.22916666666</v>
+        <v>46280.22916666666</v>
       </c>
       <c r="B61" t="n">
-        <v>66.52</v>
+        <v>75.96007</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1821,7 +1841,7 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1831,10 +1851,10 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46279.25</v>
+        <v>46280.25</v>
       </c>
       <c r="B62" t="n">
-        <v>71.40000000000001</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1842,7 +1862,7 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1852,10 +1872,10 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46279.27083333334</v>
+        <v>46280.27083333334</v>
       </c>
       <c r="B63" t="n">
-        <v>71.40000000000001</v>
+        <v>80.52894999999999</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1863,7 +1883,7 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1873,10 +1893,10 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46279.29166666666</v>
+        <v>46280.29166666666</v>
       </c>
       <c r="B64" t="n">
-        <v>71.38</v>
+        <v>64.38779</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1884,7 +1904,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1894,10 +1914,10 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46279.3125</v>
+        <v>46280.3125</v>
       </c>
       <c r="B65" t="n">
-        <v>42.79977</v>
+        <v>7.44655</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1905,7 +1925,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1915,10 +1935,10 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46279.33333333334</v>
+        <v>46280.33333333334</v>
       </c>
       <c r="B66" t="n">
-        <v>11.4</v>
+        <v>0</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1926,7 +1946,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1936,10 +1956,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46279.35416666666</v>
+        <v>46280.35416666666</v>
       </c>
       <c r="B67" t="n">
-        <v>2.12</v>
+        <v>-5.1785</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1947,7 +1967,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1957,10 +1977,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46279.375</v>
+        <v>46280.375</v>
       </c>
       <c r="B68" t="n">
-        <v>2.12</v>
+        <v>-6.82818</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1968,7 +1988,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1978,10 +1998,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46279.39583333334</v>
+        <v>46280.39583333334</v>
       </c>
       <c r="B69" t="n">
-        <v>2.12</v>
+        <v>-8.39645</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1989,7 +2009,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1999,10 +2019,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46279.41666666666</v>
+        <v>46280.41666666666</v>
       </c>
       <c r="B70" t="n">
-        <v>5e-05</v>
+        <v>-8.883559999999999</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -2010,7 +2030,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2020,10 +2040,10 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46279.4375</v>
+        <v>46280.4375</v>
       </c>
       <c r="B71" t="n">
-        <v>-6.33</v>
+        <v>-8.922700000000001</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2031,7 +2051,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2041,10 +2061,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46279.45833333334</v>
+        <v>46280.45833333334</v>
       </c>
       <c r="B72" t="n">
-        <v>-6.5</v>
+        <v>-8.74572</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2052,7 +2072,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2062,10 +2082,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46279.47916666666</v>
+        <v>46280.47916666666</v>
       </c>
       <c r="B73" t="n">
-        <v>2.12</v>
+        <v>-8.81972</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2073,7 +2093,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2083,10 +2103,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46279.5</v>
+        <v>46280.5</v>
       </c>
       <c r="B74" t="n">
-        <v>9.64106</v>
+        <v>-10.5</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2094,7 +2114,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2104,10 +2124,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46279.52083333334</v>
+        <v>46280.52083333334</v>
       </c>
       <c r="B75" t="n">
-        <v>9.820550000000001</v>
+        <v>-8.75784</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2115,7 +2135,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2125,10 +2145,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46279.54166666666</v>
+        <v>46280.54166666666</v>
       </c>
       <c r="B76" t="n">
-        <v>10.1498</v>
+        <v>-10.09551</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2136,7 +2156,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2146,10 +2166,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46279.5625</v>
+        <v>46280.5625</v>
       </c>
       <c r="B77" t="n">
-        <v>-6.70372</v>
+        <v>-12.79051</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2157,7 +2177,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2167,10 +2187,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46279.58333333334</v>
+        <v>46280.58333333334</v>
       </c>
       <c r="B78" t="n">
-        <v>0.63007</v>
+        <v>-13.0178</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2178,7 +2198,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2188,10 +2208,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46279.60416666666</v>
+        <v>46280.60416666666</v>
       </c>
       <c r="B79" t="n">
-        <v>-9.32</v>
+        <v>-18.51</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2199,7 +2219,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2209,10 +2229,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46279.625</v>
+        <v>46280.625</v>
       </c>
       <c r="B80" t="n">
-        <v>-9.01998</v>
+        <v>-18.51</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2220,7 +2240,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2230,10 +2250,10 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46279.64583333334</v>
+        <v>46280.64583333334</v>
       </c>
       <c r="B81" t="n">
-        <v>-8.887409999999999</v>
+        <v>-10.5</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2241,7 +2261,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2251,10 +2271,10 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46279.66666666666</v>
+        <v>46280.66666666666</v>
       </c>
       <c r="B82" t="n">
-        <v>-7.07898</v>
+        <v>-6.5</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2262,7 +2282,7 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2272,10 +2292,10 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46279.6875</v>
+        <v>46280.6875</v>
       </c>
       <c r="B83" t="n">
-        <v>9.85308</v>
+        <v>-1.82925</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2283,7 +2303,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2293,10 +2313,10 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46279.70833333334</v>
+        <v>46280.70833333334</v>
       </c>
       <c r="B84" t="n">
-        <v>75.15013</v>
+        <v>51.80481</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2304,7 +2324,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2314,10 +2334,10 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46279.72916666666</v>
+        <v>46280.72916666666</v>
       </c>
       <c r="B85" t="n">
-        <v>87.16236000000001</v>
+        <v>69.91</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2325,7 +2345,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2335,10 +2355,10 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>46279.75</v>
+        <v>46280.75</v>
       </c>
       <c r="B86" t="n">
-        <v>97.96795</v>
+        <v>72.48299</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2346,7 +2366,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2356,10 +2376,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>46279.77083333334</v>
+        <v>46280.77083333334</v>
       </c>
       <c r="B87" t="n">
-        <v>96.98999999999999</v>
+        <v>72.43409</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2367,7 +2387,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2377,10 +2397,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>46279.79166666666</v>
+        <v>46280.79166666666</v>
       </c>
       <c r="B88" t="n">
-        <v>95.2</v>
+        <v>73.33</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2388,7 +2408,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2398,10 +2418,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>46279.8125</v>
+        <v>46280.8125</v>
       </c>
       <c r="B89" t="n">
-        <v>95.2</v>
+        <v>72.79982</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2409,7 +2429,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2419,10 +2439,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>46279.83333333334</v>
+        <v>46280.83333333334</v>
       </c>
       <c r="B90" t="n">
-        <v>94.73505</v>
+        <v>77.49128</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2430,7 +2450,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2440,10 +2460,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>46279.85416666666</v>
+        <v>46280.85416666666</v>
       </c>
       <c r="B91" t="n">
-        <v>83.98999999999999</v>
+        <v>77.26082</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2451,7 +2471,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2461,10 +2481,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46279.875</v>
+        <v>46280.875</v>
       </c>
       <c r="B92" t="n">
-        <v>82.90000000000001</v>
+        <v>73.85874</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2472,7 +2492,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2482,10 +2502,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>46279.89583333334</v>
+        <v>46280.89583333334</v>
       </c>
       <c r="B93" t="n">
-        <v>84.02566</v>
+        <v>77.03176999999999</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2493,7 +2513,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2503,10 +2523,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>46279.91666666666</v>
+        <v>46280.91666666666</v>
       </c>
       <c r="B94" t="n">
-        <v>83.98999999999999</v>
+        <v>76.71131</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2514,7 +2534,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2524,10 +2544,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>46279.9375</v>
+        <v>46280.9375</v>
       </c>
       <c r="B95" t="n">
-        <v>83.98999999999999</v>
+        <v>82.67967</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2535,7 +2555,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2545,10 +2565,10 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>46279.95833333334</v>
+        <v>46280.95833333334</v>
       </c>
       <c r="B96" t="n">
-        <v>83.98999999999999</v>
+        <v>69.91</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2556,7 +2576,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2566,10 +2586,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>46279.97916666666</v>
+        <v>46280.97916666666</v>
       </c>
       <c r="B97" t="n">
-        <v>77.21008999999999</v>
+        <v>82.24023</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2577,7 +2597,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 664)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>194.0665154999999</v>
+        <v>202.16588925</v>
       </c>
       <c r="F2" t="n">
-        <v>4.667304365079363</v>
+        <v>4.862094498556999</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46281.20833333334</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46281.66666666666</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>235.5391057500001</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5.66472115800866</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -891,11 +911,11 @@
         <v>46280.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>11.5</v>
+        <v>-6.33</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -912,11 +932,11 @@
         <v>46280.375</v>
       </c>
       <c r="B20" t="n">
-        <v>-4.13816</v>
+        <v>-6.82843</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -933,11 +953,11 @@
         <v>46280.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>-8.345750000000001</v>
+        <v>-8.504849999999999</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +974,11 @@
         <v>46280.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-8.52899</v>
+        <v>-8.848280000000001</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +995,11 @@
         <v>46280.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-8.88449</v>
+        <v>-8.980130000000001</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46280.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-8.95208</v>
+        <v>-9.32</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46280.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-10.5</v>
+        <v>-10.34</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46280.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-10.5</v>
+        <v>-10.01</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46280.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-10.5</v>
+        <v>-12.80227</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46280.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-10.5</v>
+        <v>-12.55846</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1105,7 +1125,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46280.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-23.5</v>
+        <v>-18.51</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1163,11 @@
         <v>46280.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-23.5</v>
+        <v>-18.51</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46280.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-23.5</v>
+        <v>-13</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1205,11 @@
         <v>46280.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>-23.5</v>
+        <v>-10.5</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1226,11 @@
         <v>46280.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>-7.71305</v>
+        <v>-6.5</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1247,11 @@
         <v>46280.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>-5.01</v>
+        <v>-1.84121</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1268,11 @@
         <v>46280.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>42.25</v>
+        <v>52.14336</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1273,7 +1293,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1310,11 @@
         <v>46280.75</v>
       </c>
       <c r="B38" t="n">
-        <v>82.32514</v>
+        <v>72.48368000000001</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,7 +1331,7 @@
         <v>46280.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>77.16593</v>
+        <v>75.08619</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1332,7 +1352,7 @@
         <v>46280.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>77.03879000000001</v>
+        <v>77.78194999999999</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1353,7 +1373,7 @@
         <v>46280.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>83.98999999999999</v>
+        <v>73.33</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1374,7 +1394,7 @@
         <v>46280.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>83.9901</v>
+        <v>75.6208</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1415,7 @@
         <v>46280.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>83.9901</v>
+        <v>75.17106</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1436,7 @@
         <v>46280.875</v>
       </c>
       <c r="B44" t="n">
-        <v>84.35881999999999</v>
+        <v>75.24702000000001</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46280.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>84.07955</v>
+        <v>68.38254999999999</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46280.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>93.51473</v>
+        <v>75.9601</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46280.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>90.47311000000001</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1520,7 @@
         <v>46280.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>96.98999999999999</v>
+        <v>81.03371</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,7 +1541,7 @@
         <v>46280.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>82.76542999999999</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46280</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B50" t="n">
+        <v>80.07357</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46281.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>75.9601</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46281.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>75.9601</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46281.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>75.96012</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46281.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>74.35288</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46281.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>74.38934</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46281.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>75.96007</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46281.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>81.63789</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46281.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>80.04313999999999</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46281.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>69.47857999999999</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46281.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>69.58535000000001</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46281.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>69.90052</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46281.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46281.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>69.91</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46281.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>73.31112</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46281.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>24.98998</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46281.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>-5.01</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46281.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>-6.33</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46281.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>-6.33</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46281.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>-6.61283</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46281.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>-6.33</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46281.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-6.97498</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46281.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-6.90648</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46281.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>-6.51</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46281.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>-7.48707</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46281.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>-8.29946</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46281.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>-6.51</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46281.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-8.82442</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46281.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-12.84777</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46281.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-18.5098</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46281.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>-12.03559</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46281.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46281.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>-6.84391</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46281.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>-3.76207</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46281.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>50.77094</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46281.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>93.14024000000001</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46281.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>123.43048</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46281.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>241.9455</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46281.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>281.32373</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46281.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>177.98929</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46281.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>170.7211</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46281.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>142.9</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46281.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>189.41031</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46281.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>142.9</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46281.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>125.29596</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46281.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>134.86</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46281.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>118.67</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46281.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>118.67</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 589)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -470,10 +470,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46279.1875</v>
+        <v>46280.1875</v>
       </c>
       <c r="C2" t="n">
         <v>4.5</v>
@@ -482,38 +482,38 @@
         <v>17.01</v>
       </c>
       <c r="E2" t="n">
-        <v>566.704203</v>
+        <v>623.1506092499999</v>
       </c>
       <c r="F2" t="n">
-        <v>33.31594373897708</v>
+        <v>36.63436856261023</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46279.20833333334</v>
+        <v>46280.29166666666</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46279.66666666666</v>
+        <v>46280.66666666666</v>
       </c>
       <c r="C3" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>41.58</v>
+        <v>34.02</v>
       </c>
       <c r="E3" t="n">
-        <v>377.6530875000001</v>
+        <v>-98.68511250000002</v>
       </c>
       <c r="F3" t="n">
-        <v>9.082565836940841</v>
+        <v>-2.900796957671958</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46279.97916666666</v>
+        <v>46280.89583333334</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>46280.14583333334</v>
+        <v>46281.0625</v>
       </c>
       <c r="C4" t="n">
         <v>4</v>
@@ -522,30 +522,30 @@
         <v>15.12</v>
       </c>
       <c r="E4" t="n">
-        <v>542.3622067499999</v>
+        <v>557.6791350000001</v>
       </c>
       <c r="F4" t="n">
-        <v>35.87051631944444</v>
+        <v>36.88354067460318</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46280.3125</v>
+        <v>46281.22916666666</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>46280.66666666666</v>
+        <v>46281.66666666666</v>
       </c>
       <c r="C5" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="D5" t="n">
-        <v>32.13</v>
+        <v>39.69</v>
       </c>
       <c r="E5" t="n">
-        <v>-147.2346915</v>
+        <v>191.3662237500001</v>
       </c>
       <c r="F5" t="n">
-        <v>-4.582467833800188</v>
+        <v>4.821522392290253</v>
       </c>
     </row>
   </sheetData>
@@ -591,10 +591,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="B2" t="n">
-        <v>65.44708</v>
+        <v>69.2433</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -602,7 +602,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -612,10 +612,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46279.02083333334</v>
+        <v>46280.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>66.79613999999999</v>
+        <v>68.46629</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -633,10 +633,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46279.04166666666</v>
+        <v>46280.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>65.5</v>
+        <v>69.02540999999999</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -644,7 +644,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -654,10 +654,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46279.0625</v>
+        <v>46280.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>64.95</v>
+        <v>74.61357</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -675,10 +675,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46279.08333333334</v>
+        <v>46280.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>64.95</v>
+        <v>75.96012</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -696,10 +696,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46279.10416666666</v>
+        <v>46280.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>63.59102</v>
+        <v>75.96007</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -717,10 +717,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46279.125</v>
+        <v>46280.125</v>
       </c>
       <c r="B8" t="n">
-        <v>58.53084</v>
+        <v>75.96007</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -738,7 +738,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46279.14583333334</v>
+        <v>46280.14583333334</v>
       </c>
       <c r="B9" t="n">
         <v>64.95</v>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -759,10 +759,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46279.16666666666</v>
+        <v>46280.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>66.52</v>
+        <v>64.95</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -780,10 +780,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46279.1875</v>
+        <v>46280.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>75.96007</v>
+        <v>76.17485000000001</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -801,10 +801,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46279.20833333334</v>
+        <v>46280.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>64.95</v>
+        <v>82.38552</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -812,20 +812,20 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46279.22916666666</v>
+        <v>46280.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>64.95</v>
+        <v>73.50393</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -833,20 +833,20 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46279.25</v>
+        <v>46280.25</v>
       </c>
       <c r="B14" t="n">
-        <v>64.89</v>
+        <v>73.36023</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -854,20 +854,20 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46279.27083333334</v>
+        <v>46280.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>71.95125</v>
+        <v>79.31545</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -875,20 +875,20 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46279.29166666666</v>
+        <v>46280.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>71.38</v>
+        <v>64.89</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -906,10 +906,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46279.3125</v>
+        <v>46280.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>42.79977</v>
+        <v>7.44692</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -917,7 +917,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -927,10 +927,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46279.33333333334</v>
+        <v>46280.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>28.01</v>
+        <v>0</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -948,10 +948,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46279.35416666666</v>
+        <v>46280.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>2.12</v>
+        <v>-6.33</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -959,7 +959,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -969,10 +969,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46279.375</v>
+        <v>46280.375</v>
       </c>
       <c r="B20" t="n">
-        <v>5e-05</v>
+        <v>-6.82843</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -980,7 +980,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -990,10 +990,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46279.39583333334</v>
+        <v>46280.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>2.12</v>
+        <v>-8.504849999999999</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1011,10 +1011,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46279.41666666666</v>
+        <v>46280.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>2.12</v>
+        <v>-8.848280000000001</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1032,10 +1032,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46279.4375</v>
+        <v>46280.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>2.12</v>
+        <v>-8.980130000000001</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1053,10 +1053,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46279.45833333334</v>
+        <v>46280.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-6.33</v>
+        <v>-9.32</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1074,10 +1074,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46279.47916666666</v>
+        <v>46280.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-4.37354</v>
+        <v>-10.34</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1095,10 +1095,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46279.5</v>
+        <v>46280.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-7.18059</v>
+        <v>-10.01</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1106,7 +1106,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1116,10 +1116,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46279.52083333334</v>
+        <v>46280.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-6.5</v>
+        <v>-12.80227</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1137,10 +1137,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46279.54166666666</v>
+        <v>46280.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>11.5</v>
+        <v>-12.55846</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1158,10 +1158,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46279.5625</v>
+        <v>46280.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>0.63007</v>
+        <v>-18.51</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1179,10 +1179,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46279.58333333334</v>
+        <v>46280.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>8.75872</v>
+        <v>-18.51</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1200,10 +1200,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46279.60416666666</v>
+        <v>46280.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-8.630000000000001</v>
+        <v>-18.51</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1211,7 +1211,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1221,10 +1221,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46279.625</v>
+        <v>46280.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-9.10793</v>
+        <v>-13</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1232,7 +1232,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1242,10 +1242,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46279.64583333334</v>
+        <v>46280.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>-8.8413</v>
+        <v>-10.5</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1253,7 +1253,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1263,10 +1263,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46279.66666666666</v>
+        <v>46280.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>-7.07855</v>
+        <v>-6.5</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1284,10 +1284,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46279.6875</v>
+        <v>46280.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>9.851839999999999</v>
+        <v>-1.84121</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1295,7 +1295,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1305,10 +1305,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46279.70833333334</v>
+        <v>46280.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>74.82621</v>
+        <v>52.14336</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1316,7 +1316,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1326,10 +1326,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46279.72916666666</v>
+        <v>46280.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>82.78774</v>
+        <v>69.91</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46279.75</v>
+        <v>46280.75</v>
       </c>
       <c r="B38" t="n">
-        <v>97.28787</v>
+        <v>72.48368000000001</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1368,10 +1368,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46279.77083333334</v>
+        <v>46280.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>99.64353</v>
+        <v>66.52</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1389,10 +1389,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46279.79166666666</v>
+        <v>46280.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>99.92856999999999</v>
+        <v>73.37508</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1400,7 +1400,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1410,10 +1410,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46279.8125</v>
+        <v>46280.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>93.91200000000001</v>
+        <v>73.10159</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1421,7 +1421,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1431,10 +1431,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46279.83333333334</v>
+        <v>46280.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>94.40582999999999</v>
+        <v>73.33</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1442,7 +1442,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1452,10 +1452,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46279.85416666666</v>
+        <v>46280.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>93.49764</v>
+        <v>72.76372000000001</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1463,7 +1463,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1473,10 +1473,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46279.875</v>
+        <v>46280.875</v>
       </c>
       <c r="B44" t="n">
-        <v>85.03485000000001</v>
+        <v>73.27328</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1484,7 +1484,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1494,10 +1494,10 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46279.89583333334</v>
+        <v>46280.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>84.02096</v>
+        <v>71.45058</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1505,20 +1505,20 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46279.91666666666</v>
+        <v>46280.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>83.98999999999999</v>
+        <v>76.62685</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1526,62 +1526,62 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46279.9375</v>
+        <v>46280.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>83.98999999999999</v>
+        <v>75.9601</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>forecast</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46279.95833333334</v>
+        <v>46280.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>83.98999999999999</v>
+        <v>69.91</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>forecast</t>
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46279.97916666666</v>
+        <v>46280.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>71.38</v>
+        <v>69.91</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1589,7 +1589,7 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1599,10 +1599,10 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B50" t="n">
-        <v>69.7102</v>
+        <v>65.5</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1610,7 +1610,7 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1620,10 +1620,10 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46280.02083333334</v>
+        <v>46281.02083333334</v>
       </c>
       <c r="B51" t="n">
-        <v>75.9601</v>
+        <v>69.91</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1641,10 +1641,10 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46280.04166666666</v>
+        <v>46281.04166666666</v>
       </c>
       <c r="B52" t="n">
-        <v>67.71827999999999</v>
+        <v>72.71107000000001</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1652,7 +1652,7 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1662,10 +1662,10 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46280.0625</v>
+        <v>46281.0625</v>
       </c>
       <c r="B53" t="n">
-        <v>66.57662999999999</v>
+        <v>75.96012</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1673,20 +1673,20 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46280.08333333334</v>
+        <v>46281.08333333334</v>
       </c>
       <c r="B54" t="n">
-        <v>68.28270999999999</v>
+        <v>74.73574000000001</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1694,20 +1694,20 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46280.10416666666</v>
+        <v>46281.10416666666</v>
       </c>
       <c r="B55" t="n">
-        <v>68.31310999999999</v>
+        <v>75.96007</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1715,20 +1715,20 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46280.125</v>
+        <v>46281.125</v>
       </c>
       <c r="B56" t="n">
-        <v>68.3279</v>
+        <v>73.37101</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1736,20 +1736,20 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46280.14583333334</v>
+        <v>46281.14583333334</v>
       </c>
       <c r="B57" t="n">
-        <v>64.89</v>
+        <v>72.43522</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1767,10 +1767,10 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46280.16666666666</v>
+        <v>46281.16666666666</v>
       </c>
       <c r="B58" t="n">
-        <v>75.96007</v>
+        <v>71.95572</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1778,7 +1778,7 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1788,10 +1788,10 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46280.1875</v>
+        <v>46281.1875</v>
       </c>
       <c r="B59" t="n">
-        <v>75.96007</v>
+        <v>72.35821</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1809,10 +1809,10 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46280.20833333334</v>
+        <v>46281.20833333334</v>
       </c>
       <c r="B60" t="n">
-        <v>82.90672000000001</v>
+        <v>70.87689</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1820,7 +1820,7 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1830,10 +1830,10 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46280.22916666666</v>
+        <v>46281.22916666666</v>
       </c>
       <c r="B61" t="n">
-        <v>75.96007</v>
+        <v>69.91</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1841,17 +1841,17 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46280.25</v>
+        <v>46281.25</v>
       </c>
       <c r="B62" t="n">
         <v>69.90000000000001</v>
@@ -1862,20 +1862,20 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46280.27083333334</v>
+        <v>46281.27083333334</v>
       </c>
       <c r="B63" t="n">
-        <v>80.52894999999999</v>
+        <v>72.40473</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1883,20 +1883,20 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46280.29166666666</v>
+        <v>46281.29166666666</v>
       </c>
       <c r="B64" t="n">
-        <v>64.38779</v>
+        <v>82.54409</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1904,20 +1904,20 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46280.3125</v>
+        <v>46281.3125</v>
       </c>
       <c r="B65" t="n">
-        <v>7.44655</v>
+        <v>17.02562</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1935,10 +1935,10 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46280.33333333334</v>
+        <v>46281.33333333334</v>
       </c>
       <c r="B66" t="n">
-        <v>0</v>
+        <v>-3.74718</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1946,7 +1946,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1956,10 +1956,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46280.35416666666</v>
+        <v>46281.35416666666</v>
       </c>
       <c r="B67" t="n">
-        <v>-5.1785</v>
+        <v>-6.33</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1967,7 +1967,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1977,10 +1977,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46280.375</v>
+        <v>46281.375</v>
       </c>
       <c r="B68" t="n">
-        <v>-6.82818</v>
+        <v>-6.5414</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1988,7 +1988,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1998,10 +1998,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46280.39583333334</v>
+        <v>46281.39583333334</v>
       </c>
       <c r="B69" t="n">
-        <v>-8.39645</v>
+        <v>-4.13098</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -2009,7 +2009,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2019,10 +2019,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46280.41666666666</v>
+        <v>46281.41666666666</v>
       </c>
       <c r="B70" t="n">
-        <v>-8.883559999999999</v>
+        <v>-6.93394</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -2030,7 +2030,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2040,10 +2040,10 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46280.4375</v>
+        <v>46281.4375</v>
       </c>
       <c r="B71" t="n">
-        <v>-8.922700000000001</v>
+        <v>-6.89232</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2051,7 +2051,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2061,10 +2061,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46280.45833333334</v>
+        <v>46281.45833333334</v>
       </c>
       <c r="B72" t="n">
-        <v>-8.74572</v>
+        <v>-6.33</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2072,7 +2072,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2082,10 +2082,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46280.47916666666</v>
+        <v>46281.47916666666</v>
       </c>
       <c r="B73" t="n">
-        <v>-8.81972</v>
+        <v>-6.51</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2093,7 +2093,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2103,10 +2103,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46280.5</v>
+        <v>46281.5</v>
       </c>
       <c r="B74" t="n">
-        <v>-10.5</v>
+        <v>-7.48013</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2114,7 +2114,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2124,10 +2124,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46280.52083333334</v>
+        <v>46281.52083333334</v>
       </c>
       <c r="B75" t="n">
-        <v>-8.75784</v>
+        <v>-7.70687</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2145,10 +2145,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46280.54166666666</v>
+        <v>46281.54166666666</v>
       </c>
       <c r="B76" t="n">
-        <v>-10.09551</v>
+        <v>-6.52656</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2156,7 +2156,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2166,10 +2166,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46280.5625</v>
+        <v>46281.5625</v>
       </c>
       <c r="B77" t="n">
-        <v>-12.79051</v>
+        <v>-8.459519999999999</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2187,10 +2187,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46280.58333333334</v>
+        <v>46281.58333333334</v>
       </c>
       <c r="B78" t="n">
-        <v>-13.0178</v>
+        <v>-8.782489999999999</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2208,10 +2208,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46280.60416666666</v>
+        <v>46281.60416666666</v>
       </c>
       <c r="B79" t="n">
-        <v>-18.51</v>
+        <v>-10.5</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2229,10 +2229,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46280.625</v>
+        <v>46281.625</v>
       </c>
       <c r="B80" t="n">
-        <v>-18.51</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2240,7 +2240,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2250,10 +2250,10 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46280.64583333334</v>
+        <v>46281.64583333334</v>
       </c>
       <c r="B81" t="n">
-        <v>-10.5</v>
+        <v>-10.01</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2261,7 +2261,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2271,7 +2271,7 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46280.66666666666</v>
+        <v>46281.66666666666</v>
       </c>
       <c r="B82" t="n">
         <v>-6.5</v>
@@ -2282,7 +2282,7 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2292,10 +2292,10 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46280.6875</v>
+        <v>46281.6875</v>
       </c>
       <c r="B83" t="n">
-        <v>-1.82925</v>
+        <v>-2.75782</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2303,7 +2303,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2313,10 +2313,10 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46280.70833333334</v>
+        <v>46281.70833333334</v>
       </c>
       <c r="B84" t="n">
-        <v>51.80481</v>
+        <v>51.01773</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2324,7 +2324,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2334,10 +2334,10 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46280.72916666666</v>
+        <v>46281.72916666666</v>
       </c>
       <c r="B85" t="n">
-        <v>69.91</v>
+        <v>98.45703</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2345,7 +2345,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2355,10 +2355,10 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>46280.75</v>
+        <v>46281.75</v>
       </c>
       <c r="B86" t="n">
-        <v>72.48299</v>
+        <v>151.39483</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2366,7 +2366,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2376,10 +2376,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>46280.77083333334</v>
+        <v>46281.77083333334</v>
       </c>
       <c r="B87" t="n">
-        <v>72.43409</v>
+        <v>153.51418</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2397,10 +2397,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>46280.79166666666</v>
+        <v>46281.79166666666</v>
       </c>
       <c r="B88" t="n">
-        <v>73.33</v>
+        <v>160.80685</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2418,10 +2418,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>46280.8125</v>
+        <v>46281.8125</v>
       </c>
       <c r="B89" t="n">
-        <v>72.79982</v>
+        <v>169.02042</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2429,7 +2429,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2439,10 +2439,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>46280.83333333334</v>
+        <v>46281.83333333334</v>
       </c>
       <c r="B90" t="n">
-        <v>77.49128</v>
+        <v>239.9624</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2450,7 +2450,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>46280.85416666666</v>
+        <v>46281.85416666666</v>
       </c>
       <c r="B91" t="n">
-        <v>77.26082</v>
+        <v>276.68247</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2471,7 +2471,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2481,10 +2481,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46280.875</v>
+        <v>46281.875</v>
       </c>
       <c r="B92" t="n">
-        <v>73.85874</v>
+        <v>223.34624</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2492,7 +2492,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2502,10 +2502,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>46280.89583333334</v>
+        <v>46281.89583333334</v>
       </c>
       <c r="B93" t="n">
-        <v>77.03176999999999</v>
+        <v>153.32629</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2523,10 +2523,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>46280.91666666666</v>
+        <v>46281.91666666666</v>
       </c>
       <c r="B94" t="n">
-        <v>76.71131</v>
+        <v>148.33485</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2534,7 +2534,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2544,10 +2544,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>46280.9375</v>
+        <v>46281.9375</v>
       </c>
       <c r="B95" t="n">
-        <v>82.67967</v>
+        <v>134.86</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2565,10 +2565,10 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>46280.95833333334</v>
+        <v>46281.95833333334</v>
       </c>
       <c r="B96" t="n">
-        <v>69.91</v>
+        <v>123.18227</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2586,10 +2586,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>46280.97916666666</v>
+        <v>46281.97916666666</v>
       </c>
       <c r="B97" t="n">
-        <v>82.24023</v>
+        <v>121.48346</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2597,7 +2597,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 666)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,22 +470,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46281.20833333334</v>
+        <v>46281.25</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46281.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>41.58</v>
+        <v>37.8</v>
       </c>
       <c r="E2" t="n">
-        <v>298.0451565</v>
+        <v>124.8992842499999</v>
       </c>
       <c r="F2" t="n">
-        <v>7.167993181818181</v>
+        <v>3.304213869047617</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46281.95833333334</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46282.125</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="E3" t="n">
+        <v>704.430519</v>
+      </c>
+      <c r="F3" t="n">
+        <v>46.58932003968254</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46282.33333333334</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46282.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D4" t="n">
+        <v>30.24</v>
+      </c>
+      <c r="E4" t="n">
+        <v>83.00119425000001</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.744748487103175</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -756,7 +796,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -777,7 +817,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -870,11 +910,11 @@
         <v>46281.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>23.95</v>
+        <v>-4.39116</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -891,11 +931,11 @@
         <v>46281.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>-5.04</v>
+        <v>-6.33</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -912,11 +952,11 @@
         <v>46281.375</v>
       </c>
       <c r="B20" t="n">
-        <v>-6.09956</v>
+        <v>-6.72728</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -933,11 +973,11 @@
         <v>46281.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>-6.33</v>
+        <v>-6.9535</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +994,11 @@
         <v>46281.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-5.9371</v>
+        <v>-7.01005</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +1015,11 @@
         <v>46281.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-6.57484</v>
+        <v>-7.01257</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1036,11 @@
         <v>46281.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-6.57227</v>
+        <v>-7.20848</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1057,11 @@
         <v>46281.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-5.17</v>
+        <v>-7.46184</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1078,11 @@
         <v>46281.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-6.60916</v>
+        <v>-7.21175</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1099,11 @@
         <v>46281.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-6.56563</v>
+        <v>-8.298299999999999</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1120,11 @@
         <v>46281.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-7.61084</v>
+        <v>-6.58479</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1141,11 @@
         <v>46281.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-8.397819999999999</v>
+        <v>-7.6084</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1162,11 @@
         <v>46281.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-9.794499999999999</v>
+        <v>-8.838570000000001</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1183,11 @@
         <v>46281.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-10.5</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1204,11 @@
         <v>46281.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-9.360900000000001</v>
+        <v>-8.01</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1189,7 +1229,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1246,11 @@
         <v>46281.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>-6.51</v>
+        <v>-6.5</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1267,11 @@
         <v>46281.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>-2.77545</v>
+        <v>-2.75771</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1288,11 @@
         <v>46281.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>50.02351</v>
+        <v>51.01579</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1309,11 @@
         <v>46281.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>95.2</v>
+        <v>98.76300999999999</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1330,11 @@
         <v>46281.75</v>
       </c>
       <c r="B38" t="n">
-        <v>121.14258</v>
+        <v>165.52747</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,7 +1351,7 @@
         <v>46281.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>129.68024</v>
+        <v>113.90254</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1332,7 +1372,7 @@
         <v>46281.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>150.35755</v>
+        <v>129.65</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1353,7 +1393,7 @@
         <v>46281.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>180.28266</v>
+        <v>124.85607</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1374,7 +1414,7 @@
         <v>46281.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>125.80114</v>
+        <v>126.58971</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1435,7 @@
         <v>46281.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>122.88132</v>
+        <v>107.2407</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1456,7 @@
         <v>46281.875</v>
       </c>
       <c r="B44" t="n">
-        <v>121.1</v>
+        <v>113.5</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1477,7 @@
         <v>46281.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>142.9</v>
+        <v>118.67</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1498,7 @@
         <v>46281.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>141.38522</v>
+        <v>108.74273</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1519,7 @@
         <v>46281.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>110.17723</v>
+        <v>102.36619</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1540,7 @@
         <v>46281.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>118.67</v>
+        <v>94.35503</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1512,7 +1552,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1561,7 @@
         <v>46281.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>113.16114</v>
+        <v>96.99005</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1572,1014 @@
         <v>46281</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B50" t="n">
+        <v>96.07209</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46282.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>95.53822</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46282.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>88.39573</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46282.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46282.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46282.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>83.16172</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46282.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>82.60715</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46282.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>82.88999</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46282.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>82.86681</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46282.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46282.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46282.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46282.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>100.84306</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46282.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>118.05819</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46282.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>113.32799</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46282.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>57.38977</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46282.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46282.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46282.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46282.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>10.49835</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46282.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>-5.68434</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46282.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-3.4069</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46282.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>0.009939999999999999</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46282.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>-5.50213</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46282.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>2.34864</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46282.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>-2.79385</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46282.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>-4.86936</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46282.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-5.68434</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46282.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-4.88896</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46282.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-8.495229999999999</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46282.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>-7.70431</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46282.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>-7.11808</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46282.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>-6.43985</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46282.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>0.01085</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46282.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>62.02739</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46282.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46282.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>129.38</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46282.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>288.61933</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46282.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46282.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>297.99</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46282.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>297.99</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46282.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>222.1925</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46282.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>204.37586</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46282.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>151.37012</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46282.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>143.25371</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46282.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>123.74307</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46282.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>113.10557</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46282.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>113.38985</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 590)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,82 +470,42 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46280.1875</v>
+        <v>46281.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>4.5</v>
+        <v>16</v>
       </c>
       <c r="D2" t="n">
-        <v>17.01</v>
+        <v>60.48</v>
       </c>
       <c r="E2" t="n">
-        <v>623.1506092499999</v>
+        <v>983.51907225</v>
       </c>
       <c r="F2" t="n">
-        <v>36.63436856261023</v>
+        <v>16.26188942212302</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46280.29166666666</v>
+        <v>46282.16666666666</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46280.66666666666</v>
+        <v>46282.66666666666</v>
       </c>
       <c r="C3" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D3" t="n">
-        <v>34.02</v>
+        <v>45.36</v>
       </c>
       <c r="E3" t="n">
-        <v>-98.68511250000002</v>
+        <v>744.6677354999999</v>
       </c>
       <c r="F3" t="n">
-        <v>-2.900796957671958</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>46280.89583333334</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>46281.0625</v>
-      </c>
-      <c r="C4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D4" t="n">
-        <v>15.12</v>
-      </c>
-      <c r="E4" t="n">
-        <v>557.6791350000001</v>
-      </c>
-      <c r="F4" t="n">
-        <v>36.88354067460318</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>46281.22916666666</v>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>46281.66666666666</v>
-      </c>
-      <c r="C5" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="D5" t="n">
-        <v>39.69</v>
-      </c>
-      <c r="E5" t="n">
-        <v>191.3662237500001</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4.821522392290253</v>
+        <v>16.41683720238095</v>
       </c>
     </row>
   </sheetData>
@@ -591,10 +551,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B2" t="n">
-        <v>69.2433</v>
+        <v>69.91</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -602,7 +562,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -612,10 +572,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46280.02083333334</v>
+        <v>46281.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>68.46629</v>
+        <v>75.9601</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -623,7 +583,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -633,10 +593,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46280.04166666666</v>
+        <v>46281.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>69.02540999999999</v>
+        <v>74.58717</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -644,7 +604,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -654,10 +614,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46280.0625</v>
+        <v>46281.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>74.61357</v>
+        <v>76.60890000000001</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -665,7 +625,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -675,10 +635,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46280.08333333334</v>
+        <v>46281.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>75.96012</v>
+        <v>69.91</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -686,7 +646,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -696,10 +656,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46280.10416666666</v>
+        <v>46281.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>75.96007</v>
+        <v>79.93566</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -707,7 +667,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -717,10 +677,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46280.125</v>
+        <v>46281.125</v>
       </c>
       <c r="B8" t="n">
-        <v>75.96007</v>
+        <v>74.30526</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -728,7 +688,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -738,10 +698,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46280.14583333334</v>
+        <v>46281.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>64.95</v>
+        <v>71.96028</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -749,7 +709,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -759,10 +719,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46280.16666666666</v>
+        <v>46281.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>64.95</v>
+        <v>71.02630000000001</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -770,7 +730,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -780,10 +740,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46280.1875</v>
+        <v>46281.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>76.17485000000001</v>
+        <v>70.51057</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -791,20 +751,20 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46280.20833333334</v>
+        <v>46281.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>82.38552</v>
+        <v>69.96137</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -812,20 +772,20 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46280.22916666666</v>
+        <v>46281.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>73.50393</v>
+        <v>75.96007</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -833,20 +793,20 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46280.25</v>
+        <v>46281.25</v>
       </c>
       <c r="B14" t="n">
-        <v>73.36023</v>
+        <v>75.9601</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -854,20 +814,20 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46280.27083333334</v>
+        <v>46281.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>79.31545</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -875,20 +835,20 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46280.29166666666</v>
+        <v>46281.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>64.89</v>
+        <v>83.9901</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -896,7 +856,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -906,10 +866,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46280.3125</v>
+        <v>46281.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>7.44692</v>
+        <v>17.02832</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -917,7 +877,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -927,10 +887,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46280.33333333334</v>
+        <v>46281.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>-4.39116</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -938,7 +898,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -948,7 +908,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46280.35416666666</v>
+        <v>46281.35416666666</v>
       </c>
       <c r="B19" t="n">
         <v>-6.33</v>
@@ -959,7 +919,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -969,10 +929,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46280.375</v>
+        <v>46281.375</v>
       </c>
       <c r="B20" t="n">
-        <v>-6.82843</v>
+        <v>-6.72728</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -980,7 +940,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -990,10 +950,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46280.39583333334</v>
+        <v>46281.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>-8.504849999999999</v>
+        <v>-6.9535</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1001,7 +961,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1011,10 +971,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46280.41666666666</v>
+        <v>46281.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-8.848280000000001</v>
+        <v>-7.01005</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1022,7 +982,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1032,10 +992,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46280.4375</v>
+        <v>46281.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-8.980130000000001</v>
+        <v>-7.01257</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1043,7 +1003,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1053,10 +1013,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46280.45833333334</v>
+        <v>46281.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-9.32</v>
+        <v>-7.20848</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1064,7 +1024,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1074,10 +1034,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46280.47916666666</v>
+        <v>46281.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-10.34</v>
+        <v>-7.46184</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1085,7 +1045,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1095,10 +1055,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46280.5</v>
+        <v>46281.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-10.01</v>
+        <v>-7.21175</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1106,7 +1066,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1116,10 +1076,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46280.52083333334</v>
+        <v>46281.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-12.80227</v>
+        <v>-8.298299999999999</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1127,7 +1087,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1137,10 +1097,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46280.54166666666</v>
+        <v>46281.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-12.55846</v>
+        <v>-6.58479</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1148,7 +1108,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1158,10 +1118,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46280.5625</v>
+        <v>46281.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-18.51</v>
+        <v>-7.6084</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1169,7 +1129,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1179,10 +1139,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46280.58333333334</v>
+        <v>46281.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-18.51</v>
+        <v>-8.838570000000001</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1190,7 +1150,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1200,10 +1160,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46280.60416666666</v>
+        <v>46281.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-18.51</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1211,7 +1171,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1221,10 +1181,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46280.625</v>
+        <v>46281.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-13</v>
+        <v>-8.01</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1232,7 +1192,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1242,7 +1202,7 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46280.64583333334</v>
+        <v>46281.64583333334</v>
       </c>
       <c r="B33" t="n">
         <v>-10.5</v>
@@ -1253,7 +1213,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1263,7 +1223,7 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46280.66666666666</v>
+        <v>46281.66666666666</v>
       </c>
       <c r="B34" t="n">
         <v>-6.5</v>
@@ -1274,7 +1234,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1284,10 +1244,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46280.6875</v>
+        <v>46281.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>-1.84121</v>
+        <v>-2.75771</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1295,7 +1255,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1305,10 +1265,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46280.70833333334</v>
+        <v>46281.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>52.14336</v>
+        <v>51.01579</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1316,7 +1276,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1326,10 +1286,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46280.72916666666</v>
+        <v>46281.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>69.91</v>
+        <v>98.76300999999999</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1337,7 +1297,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1347,10 +1307,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46280.75</v>
+        <v>46281.75</v>
       </c>
       <c r="B38" t="n">
-        <v>72.48368000000001</v>
+        <v>165.52747</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1358,7 +1318,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1368,10 +1328,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46280.77083333334</v>
+        <v>46281.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>66.52</v>
+        <v>160.08285</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1379,7 +1339,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1389,10 +1349,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46280.79166666666</v>
+        <v>46281.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>73.37508</v>
+        <v>172.21889</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1400,7 +1360,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1410,10 +1370,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46280.8125</v>
+        <v>46281.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>73.10159</v>
+        <v>164.7379</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1421,7 +1381,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1431,10 +1391,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46280.83333333334</v>
+        <v>46281.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>73.33</v>
+        <v>464.84209</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1442,7 +1402,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1452,10 +1412,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46280.85416666666</v>
+        <v>46281.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>72.76372000000001</v>
+        <v>255.34244</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1463,7 +1423,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1473,10 +1433,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46280.875</v>
+        <v>46281.875</v>
       </c>
       <c r="B44" t="n">
-        <v>73.27328</v>
+        <v>221.59578</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1484,7 +1444,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1494,10 +1454,10 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46280.89583333334</v>
+        <v>46281.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>71.45058</v>
+        <v>147.11843</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1505,20 +1465,20 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46280.91666666666</v>
+        <v>46281.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>76.62685</v>
+        <v>222.71327</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1526,20 +1486,20 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46280.9375</v>
+        <v>46281.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>75.9601</v>
+        <v>118.67</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1547,20 +1507,20 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46280.95833333334</v>
+        <v>46281.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>69.91</v>
+        <v>101.48761</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1568,20 +1528,20 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46280.97916666666</v>
+        <v>46281.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>69.91</v>
+        <v>98.2206</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1589,20 +1549,20 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B50" t="n">
-        <v>65.5</v>
+        <v>96.74621999999999</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1610,20 +1570,20 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46281.02083333334</v>
+        <v>46282.02083333334</v>
       </c>
       <c r="B51" t="n">
-        <v>69.91</v>
+        <v>94.32701</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1631,20 +1591,20 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46281.04166666666</v>
+        <v>46282.04166666666</v>
       </c>
       <c r="B52" t="n">
-        <v>72.71107000000001</v>
+        <v>87.80963</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1652,20 +1612,20 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46281.0625</v>
+        <v>46282.0625</v>
       </c>
       <c r="B53" t="n">
-        <v>75.96012</v>
+        <v>90.08280999999999</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1673,7 +1633,7 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1683,10 +1643,10 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46281.08333333334</v>
+        <v>46282.08333333334</v>
       </c>
       <c r="B54" t="n">
-        <v>74.73574000000001</v>
+        <v>89.08074999999999</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1694,7 +1654,7 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1704,10 +1664,10 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46281.10416666666</v>
+        <v>46282.10416666666</v>
       </c>
       <c r="B55" t="n">
-        <v>75.96007</v>
+        <v>85.74454</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1715,7 +1675,7 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1725,10 +1685,10 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46281.125</v>
+        <v>46282.125</v>
       </c>
       <c r="B56" t="n">
-        <v>73.37101</v>
+        <v>81.78581</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1736,7 +1696,7 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1746,10 +1706,10 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46281.14583333334</v>
+        <v>46282.14583333334</v>
       </c>
       <c r="B57" t="n">
-        <v>72.43522</v>
+        <v>85.44902</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1757,7 +1717,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1767,10 +1727,10 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46281.16666666666</v>
+        <v>46282.16666666666</v>
       </c>
       <c r="B58" t="n">
-        <v>71.95572</v>
+        <v>82.27869</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1778,20 +1738,20 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46281.1875</v>
+        <v>46282.1875</v>
       </c>
       <c r="B59" t="n">
-        <v>72.35821</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1799,20 +1759,20 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46281.20833333334</v>
+        <v>46282.20833333334</v>
       </c>
       <c r="B60" t="n">
-        <v>70.87689</v>
+        <v>92.08955</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1820,20 +1780,20 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46281.22916666666</v>
+        <v>46282.22916666666</v>
       </c>
       <c r="B61" t="n">
-        <v>69.91</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1841,7 +1801,7 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1851,10 +1811,10 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46281.25</v>
+        <v>46282.25</v>
       </c>
       <c r="B62" t="n">
-        <v>69.90000000000001</v>
+        <v>93.24739</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1862,7 +1822,7 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1872,10 +1832,10 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46281.27083333334</v>
+        <v>46282.27083333334</v>
       </c>
       <c r="B63" t="n">
-        <v>72.40473</v>
+        <v>98.64118000000001</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1883,7 +1843,7 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1893,10 +1853,10 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46281.29166666666</v>
+        <v>46282.29166666666</v>
       </c>
       <c r="B64" t="n">
-        <v>82.54409</v>
+        <v>86.83065999999999</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1904,7 +1864,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1914,10 +1874,10 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46281.3125</v>
+        <v>46282.3125</v>
       </c>
       <c r="B65" t="n">
-        <v>17.02562</v>
+        <v>57.38977</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1925,7 +1885,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1935,10 +1895,10 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46281.33333333334</v>
+        <v>46282.33333333334</v>
       </c>
       <c r="B66" t="n">
-        <v>-3.74718</v>
+        <v>42.94</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1946,7 +1906,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1956,10 +1916,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46281.35416666666</v>
+        <v>46282.35416666666</v>
       </c>
       <c r="B67" t="n">
-        <v>-6.33</v>
+        <v>42.8001</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1967,7 +1927,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1977,10 +1937,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46281.375</v>
+        <v>46282.375</v>
       </c>
       <c r="B68" t="n">
-        <v>-6.5414</v>
+        <v>42.54</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1988,7 +1948,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1998,10 +1958,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46281.39583333334</v>
+        <v>46282.39583333334</v>
       </c>
       <c r="B69" t="n">
-        <v>-4.13098</v>
+        <v>2.12</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -2009,7 +1969,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2019,10 +1979,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46281.41666666666</v>
+        <v>46282.41666666666</v>
       </c>
       <c r="B70" t="n">
-        <v>-6.93394</v>
+        <v>2.12</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -2030,7 +1990,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2040,10 +2000,10 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46281.4375</v>
+        <v>46282.4375</v>
       </c>
       <c r="B71" t="n">
-        <v>-6.89232</v>
+        <v>2.12</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2051,7 +2011,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2061,10 +2021,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46281.45833333334</v>
+        <v>46282.45833333334</v>
       </c>
       <c r="B72" t="n">
-        <v>-6.33</v>
+        <v>2.12</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2072,7 +2032,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2082,10 +2042,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46281.47916666666</v>
+        <v>46282.47916666666</v>
       </c>
       <c r="B73" t="n">
-        <v>-6.51</v>
+        <v>-6.5</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2093,7 +2053,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2103,10 +2063,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46281.5</v>
+        <v>46282.5</v>
       </c>
       <c r="B74" t="n">
-        <v>-7.48013</v>
+        <v>2.12</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2114,7 +2074,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2124,10 +2084,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46281.52083333334</v>
+        <v>46282.52083333334</v>
       </c>
       <c r="B75" t="n">
-        <v>-7.70687</v>
+        <v>2.12</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2135,7 +2095,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2145,10 +2105,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46281.54166666666</v>
+        <v>46282.54166666666</v>
       </c>
       <c r="B76" t="n">
-        <v>-6.52656</v>
+        <v>-8.415179999999999</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2156,7 +2116,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2166,10 +2126,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46281.5625</v>
+        <v>46282.5625</v>
       </c>
       <c r="B77" t="n">
-        <v>-8.459519999999999</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2177,7 +2137,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2187,10 +2147,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46281.58333333334</v>
+        <v>46282.58333333334</v>
       </c>
       <c r="B78" t="n">
-        <v>-8.782489999999999</v>
+        <v>-8.72222</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2198,7 +2158,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2208,10 +2168,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46281.60416666666</v>
+        <v>46282.60416666666</v>
       </c>
       <c r="B79" t="n">
-        <v>-10.5</v>
+        <v>-9.15035</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2219,7 +2179,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2229,10 +2189,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46281.625</v>
+        <v>46282.625</v>
       </c>
       <c r="B80" t="n">
-        <v>-8.630000000000001</v>
+        <v>-7.24729</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2240,7 +2200,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2250,10 +2210,10 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46281.64583333334</v>
+        <v>46282.64583333334</v>
       </c>
       <c r="B81" t="n">
-        <v>-10.01</v>
+        <v>-7.03052</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2261,7 +2221,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2271,10 +2231,10 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46281.66666666666</v>
+        <v>46282.66666666666</v>
       </c>
       <c r="B82" t="n">
-        <v>-6.5</v>
+        <v>-6.31457</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2282,7 +2242,7 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2292,10 +2252,10 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46281.6875</v>
+        <v>46282.6875</v>
       </c>
       <c r="B83" t="n">
-        <v>-2.75782</v>
+        <v>0.01063</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2303,7 +2263,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2313,10 +2273,10 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46281.70833333334</v>
+        <v>46282.70833333334</v>
       </c>
       <c r="B84" t="n">
-        <v>51.01773</v>
+        <v>61.18634</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2324,7 +2284,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2334,10 +2294,10 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46281.72916666666</v>
+        <v>46282.72916666666</v>
       </c>
       <c r="B85" t="n">
-        <v>98.45703</v>
+        <v>90.93531</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2345,7 +2305,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2355,10 +2315,10 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>46281.75</v>
+        <v>46282.75</v>
       </c>
       <c r="B86" t="n">
-        <v>151.39483</v>
+        <v>133.82812</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2366,7 +2326,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2376,10 +2336,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>46281.77083333334</v>
+        <v>46282.77083333334</v>
       </c>
       <c r="B87" t="n">
-        <v>153.51418</v>
+        <v>124.65701</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2387,7 +2347,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2397,10 +2357,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>46281.79166666666</v>
+        <v>46282.79166666666</v>
       </c>
       <c r="B88" t="n">
-        <v>160.80685</v>
+        <v>128.2673</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2408,7 +2368,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2418,10 +2378,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>46281.8125</v>
+        <v>46282.8125</v>
       </c>
       <c r="B89" t="n">
-        <v>169.02042</v>
+        <v>129.65</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2429,7 +2389,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2439,10 +2399,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>46281.83333333334</v>
+        <v>46282.83333333334</v>
       </c>
       <c r="B90" t="n">
-        <v>239.9624</v>
+        <v>129.65</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2450,7 +2410,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2460,10 +2420,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>46281.85416666666</v>
+        <v>46282.85416666666</v>
       </c>
       <c r="B91" t="n">
-        <v>276.68247</v>
+        <v>129.65</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2471,7 +2431,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2481,10 +2441,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46281.875</v>
+        <v>46282.875</v>
       </c>
       <c r="B92" t="n">
-        <v>223.34624</v>
+        <v>129.65</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2492,7 +2452,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2502,10 +2462,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>46281.89583333334</v>
+        <v>46282.89583333334</v>
       </c>
       <c r="B93" t="n">
-        <v>153.32629</v>
+        <v>129.38</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2513,7 +2473,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2523,10 +2483,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>46281.91666666666</v>
+        <v>46282.91666666666</v>
       </c>
       <c r="B94" t="n">
-        <v>148.33485</v>
+        <v>122.19838</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2534,7 +2494,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2544,10 +2504,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>46281.9375</v>
+        <v>46282.9375</v>
       </c>
       <c r="B95" t="n">
-        <v>134.86</v>
+        <v>115.44164</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2555,7 +2515,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2565,10 +2525,10 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>46281.95833333334</v>
+        <v>46282.95833333334</v>
       </c>
       <c r="B96" t="n">
-        <v>123.18227</v>
+        <v>106.8635</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2576,7 +2536,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2586,10 +2546,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>46281.97916666666</v>
+        <v>46282.97916666666</v>
       </c>
       <c r="B97" t="n">
-        <v>121.48346</v>
+        <v>107.13971</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2597,7 +2557,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 668)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>513.1791210000001</v>
+        <v>584.3739817500001</v>
       </c>
       <c r="F2" t="n">
-        <v>12.3419702020202</v>
+        <v>14.05420831529582</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46283.20833333334</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46283.66666666666</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>473.03368125</v>
+      </c>
+      <c r="F3" t="n">
+        <v>11.37647141053391</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -870,11 +890,11 @@
         <v>46282.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>42.94</v>
+        <v>42.79988</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -891,11 +911,11 @@
         <v>46282.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>42.94</v>
+        <v>42.8001</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -912,11 +932,11 @@
         <v>46282.375</v>
       </c>
       <c r="B20" t="n">
-        <v>2.12</v>
+        <v>34.94352</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -933,11 +953,11 @@
         <v>46282.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>-5.05</v>
+        <v>2.12</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +974,11 @@
         <v>46282.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>2.12</v>
+        <v>12.62239</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +995,11 @@
         <v>46282.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-5.04</v>
+        <v>9.809290000000001</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46282.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-8.72498</v>
+        <v>0.69548</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46282.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-9.049709999999999</v>
+        <v>-5.68434</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46282.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-6.20952</v>
+        <v>-6.5</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46282.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-5.68434</v>
+        <v>0.01015</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46282.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-6.5</v>
+        <v>-8.35943</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1121,11 @@
         <v>46282.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-8.630000000000001</v>
+        <v>-8.5139</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46282.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>1.80673</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1147,7 +1167,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46282.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-8.099460000000001</v>
+        <v>-6.5</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1205,11 @@
         <v>46282.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>-8.403079999999999</v>
+        <v>-8.057130000000001</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1226,11 @@
         <v>46282.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>-6.51</v>
+        <v>-6.07163</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1247,11 @@
         <v>46282.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>3e-05</v>
+        <v>0.0107</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1268,11 @@
         <v>46282.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>55.3485</v>
+        <v>63.20151</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1289,11 @@
         <v>46282.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>92.12625</v>
+        <v>91.38206</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1294,7 +1314,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,7 +1331,7 @@
         <v>46282.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>129.65</v>
+        <v>107.02339</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1332,7 +1352,7 @@
         <v>46282.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>129.65</v>
+        <v>121.1</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1353,7 +1373,7 @@
         <v>46282.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>125.44079</v>
+        <v>121.1</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1374,7 +1394,7 @@
         <v>46282.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>121.1</v>
+        <v>122.65173</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1415,7 @@
         <v>46282.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>111.98</v>
+        <v>119.79941</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1436,7 @@
         <v>46282.875</v>
       </c>
       <c r="B44" t="n">
-        <v>115.26987</v>
+        <v>122.24935</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46282.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>119.95299</v>
+        <v>125.84529</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46282.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>113.05013</v>
+        <v>153.50079</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46282.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>108.1927</v>
+        <v>129.35525</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1520,7 @@
         <v>46282.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>100.11443</v>
+        <v>126.08259</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,7 +1541,7 @@
         <v>46282.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>98.86336</v>
+        <v>125.79233</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46282</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B50" t="n">
+        <v>112.60831</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46283.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>114.48912</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46283.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>124.08728</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46283.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>119</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46283.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>108.22787</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46283.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>96.74655</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46283.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>94.70135999999999</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46283.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>97.63005</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46283.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46283.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>92.42628000000001</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46283.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>91.4812</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46283.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>90</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46283.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46283.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>138.34487</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46283.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>103.14299</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46283.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>63.1348</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46283.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>9.638030000000001</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46283.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>0.00946</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46283.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>-5.68434</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46283.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>-7.54245</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46283.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>-8.462009999999999</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46283.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-8.72369</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46283.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-8.829090000000001</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46283.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>-8.9978</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46283.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>-8.211819999999999</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46283.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>-8.31598</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46283.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>-8.812620000000001</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46283.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-9.02744</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46283.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-9.32</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46283.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-9.21889</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46283.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>-8.55247</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46283.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46283.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>-5.46242</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46283.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46283.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46283.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46283.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>88.86011000000001</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46283.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>178.70177</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46283.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>120.24363</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46283.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>192.38456</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46283.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>119.01</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46283.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>123.24924</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46283.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>212.72281</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46283.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>196.41648</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46283.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>191.93145</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46283.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>187.54629</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46283.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>119.01</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46283.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>107.37568</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 591)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,10 +470,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46281.66666666666</v>
+        <v>46282.66666666666</v>
       </c>
       <c r="C2" t="n">
         <v>16</v>
@@ -482,30 +482,50 @@
         <v>60.48</v>
       </c>
       <c r="E2" t="n">
-        <v>983.51907225</v>
+        <v>1462.04131125</v>
       </c>
       <c r="F2" t="n">
-        <v>16.26188942212302</v>
+        <v>24.1739634796627</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46282.16666666666</v>
+        <v>46283.10416666666</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46282.66666666666</v>
+        <v>46283.27083333334</v>
       </c>
       <c r="C3" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>45.36</v>
+        <v>15.12</v>
       </c>
       <c r="E3" t="n">
-        <v>744.6677354999999</v>
+        <v>724.7977619999999</v>
       </c>
       <c r="F3" t="n">
-        <v>16.41683720238095</v>
+        <v>47.93635992063492</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46283.33333333334</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46283.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D4" t="n">
+        <v>30.24</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-116.2775835</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-3.84515818452381</v>
       </c>
     </row>
   </sheetData>
@@ -551,10 +571,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B2" t="n">
-        <v>69.91</v>
+        <v>96.90548</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -562,7 +582,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -572,10 +592,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46281.02083333334</v>
+        <v>46282.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>75.9601</v>
+        <v>95.09088</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -583,7 +603,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -593,10 +613,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46281.04166666666</v>
+        <v>46282.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>74.58717</v>
+        <v>93.9953</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -604,7 +624,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -614,10 +634,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46281.0625</v>
+        <v>46282.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>76.60890000000001</v>
+        <v>90.88932</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -625,7 +645,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -635,10 +655,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46281.08333333334</v>
+        <v>46282.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>69.91</v>
+        <v>89.03032</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -646,7 +666,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -656,10 +676,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46281.10416666666</v>
+        <v>46282.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>79.93566</v>
+        <v>88.88</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -667,7 +687,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -677,10 +697,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46281.125</v>
+        <v>46282.125</v>
       </c>
       <c r="B8" t="n">
-        <v>74.30526</v>
+        <v>88.54156</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -688,7 +708,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -698,10 +718,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46281.14583333334</v>
+        <v>46282.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>71.96028</v>
+        <v>88.88</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -709,7 +729,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -719,10 +739,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46281.16666666666</v>
+        <v>46282.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>71.02630000000001</v>
+        <v>83.96876</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -730,7 +750,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -740,10 +760,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46281.1875</v>
+        <v>46282.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>70.51057</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -751,7 +771,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -761,10 +781,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46281.20833333334</v>
+        <v>46282.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>69.96137</v>
+        <v>92.07459</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -772,7 +792,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -782,10 +802,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46281.22916666666</v>
+        <v>46282.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>75.96007</v>
+        <v>86.81858</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -793,7 +813,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -803,10 +823,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46281.25</v>
+        <v>46282.25</v>
       </c>
       <c r="B14" t="n">
-        <v>75.9601</v>
+        <v>93.24209</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -814,7 +834,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -824,10 +844,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46281.27083333334</v>
+        <v>46282.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>69.90000000000001</v>
+        <v>98.63189</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -835,7 +855,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -845,10 +865,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46281.29166666666</v>
+        <v>46282.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>83.9901</v>
+        <v>86.27500000000001</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -856,7 +876,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -866,10 +886,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46281.3125</v>
+        <v>46282.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>17.02832</v>
+        <v>57.38977</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -877,7 +897,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -887,10 +907,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46281.33333333334</v>
+        <v>46282.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>-4.39116</v>
+        <v>42.79988</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -898,7 +918,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -908,10 +928,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46281.35416666666</v>
+        <v>46282.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>-6.33</v>
+        <v>42.8001</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -919,7 +939,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -929,10 +949,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46281.375</v>
+        <v>46282.375</v>
       </c>
       <c r="B20" t="n">
-        <v>-6.72728</v>
+        <v>34.94352</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -940,7 +960,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -950,10 +970,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46281.39583333334</v>
+        <v>46282.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>-6.9535</v>
+        <v>2.12</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -961,7 +981,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -971,10 +991,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46281.41666666666</v>
+        <v>46282.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-7.01005</v>
+        <v>12.62239</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -982,7 +1002,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -992,10 +1012,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46281.4375</v>
+        <v>46282.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-7.01257</v>
+        <v>9.809290000000001</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1003,7 +1023,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1013,10 +1033,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46281.45833333334</v>
+        <v>46282.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-7.20848</v>
+        <v>0.69548</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1024,7 +1044,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1034,10 +1054,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46281.47916666666</v>
+        <v>46282.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-7.46184</v>
+        <v>-5.68434</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1045,7 +1065,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1055,10 +1075,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46281.5</v>
+        <v>46282.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-7.21175</v>
+        <v>-6.5</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1066,7 +1086,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1076,10 +1096,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46281.52083333334</v>
+        <v>46282.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-8.298299999999999</v>
+        <v>0.01015</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1087,7 +1107,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1097,10 +1117,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46281.54166666666</v>
+        <v>46282.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-6.58479</v>
+        <v>-8.35943</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1108,7 +1128,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1118,10 +1138,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46281.5625</v>
+        <v>46282.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-7.6084</v>
+        <v>-8.5139</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1129,7 +1149,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1139,10 +1159,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46281.58333333334</v>
+        <v>46282.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-8.838570000000001</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1150,7 +1170,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1160,7 +1180,7 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46281.60416666666</v>
+        <v>46282.60416666666</v>
       </c>
       <c r="B31" t="n">
         <v>-8.630000000000001</v>
@@ -1171,7 +1191,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1181,10 +1201,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46281.625</v>
+        <v>46282.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-8.01</v>
+        <v>-6.5</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1192,7 +1212,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1202,10 +1222,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46281.64583333334</v>
+        <v>46282.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>-10.5</v>
+        <v>-8.057130000000001</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1213,7 +1233,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1223,10 +1243,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46281.66666666666</v>
+        <v>46282.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>-6.5</v>
+        <v>-6.07163</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1234,7 +1254,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1244,10 +1264,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46281.6875</v>
+        <v>46282.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>-2.75771</v>
+        <v>0.0107</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1255,7 +1275,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1265,10 +1285,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46281.70833333334</v>
+        <v>46282.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>51.01579</v>
+        <v>63.20151</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1276,7 +1296,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1286,10 +1306,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46281.72916666666</v>
+        <v>46282.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>98.76300999999999</v>
+        <v>91.38206</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1297,7 +1317,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1307,10 +1327,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46281.75</v>
+        <v>46282.75</v>
       </c>
       <c r="B38" t="n">
-        <v>165.52747</v>
+        <v>129.38</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1318,7 +1338,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1328,10 +1348,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46281.77083333334</v>
+        <v>46282.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>160.08285</v>
+        <v>129.65</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1339,7 +1359,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1349,10 +1369,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46281.79166666666</v>
+        <v>46282.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>172.21889</v>
+        <v>127.04177</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1360,7 +1380,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1370,10 +1390,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46281.8125</v>
+        <v>46282.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>164.7379</v>
+        <v>129.65</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1381,7 +1401,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1391,10 +1411,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46281.83333333334</v>
+        <v>46282.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>464.84209</v>
+        <v>129.65</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1402,7 +1422,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1412,10 +1432,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46281.85416666666</v>
+        <v>46282.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>255.34244</v>
+        <v>129.65</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1423,7 +1443,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1433,10 +1453,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46281.875</v>
+        <v>46282.875</v>
       </c>
       <c r="B44" t="n">
-        <v>221.59578</v>
+        <v>129.65</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1444,7 +1464,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1454,10 +1474,10 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46281.89583333334</v>
+        <v>46282.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>147.11843</v>
+        <v>121.05581</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1465,7 +1485,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1475,10 +1495,10 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46281.91666666666</v>
+        <v>46282.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>222.71327</v>
+        <v>122.08005</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1486,7 +1506,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1496,10 +1516,10 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46281.9375</v>
+        <v>46282.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>118.67</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1507,7 +1527,7 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1517,10 +1537,10 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46281.95833333334</v>
+        <v>46282.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>101.48761</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1528,7 +1548,7 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1538,10 +1558,10 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46281.97916666666</v>
+        <v>46282.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>98.2206</v>
+        <v>129.38</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1549,7 +1569,7 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1559,10 +1579,10 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B50" t="n">
-        <v>96.74621999999999</v>
+        <v>102.55423</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1570,7 +1590,7 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1580,10 +1600,10 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46282.02083333334</v>
+        <v>46283.02083333334</v>
       </c>
       <c r="B51" t="n">
-        <v>94.32701</v>
+        <v>110.6441</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1591,7 +1611,7 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1601,10 +1621,10 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46282.04166666666</v>
+        <v>46283.04166666666</v>
       </c>
       <c r="B52" t="n">
-        <v>87.80963</v>
+        <v>111.5911</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1612,7 +1632,7 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1622,10 +1642,10 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46282.0625</v>
+        <v>46283.0625</v>
       </c>
       <c r="B53" t="n">
-        <v>90.08280999999999</v>
+        <v>107.17216</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1633,7 +1653,7 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1643,10 +1663,10 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46282.08333333334</v>
+        <v>46283.08333333334</v>
       </c>
       <c r="B54" t="n">
-        <v>89.08074999999999</v>
+        <v>105.51807</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1654,7 +1674,7 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1664,10 +1684,10 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46282.10416666666</v>
+        <v>46283.10416666666</v>
       </c>
       <c r="B55" t="n">
-        <v>85.74454</v>
+        <v>98.52148</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1675,20 +1695,20 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46282.125</v>
+        <v>46283.125</v>
       </c>
       <c r="B56" t="n">
-        <v>81.78581</v>
+        <v>97.63005</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1696,20 +1716,20 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46282.14583333334</v>
+        <v>46283.14583333334</v>
       </c>
       <c r="B57" t="n">
-        <v>85.44902</v>
+        <v>90</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1717,20 +1737,20 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46282.16666666666</v>
+        <v>46283.16666666666</v>
       </c>
       <c r="B58" t="n">
-        <v>82.27869</v>
+        <v>88.88</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1738,7 +1758,7 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1748,10 +1768,10 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46282.1875</v>
+        <v>46283.1875</v>
       </c>
       <c r="B59" t="n">
-        <v>83.98999999999999</v>
+        <v>94.13703</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1759,7 +1779,7 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1769,10 +1789,10 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46282.20833333334</v>
+        <v>46283.20833333334</v>
       </c>
       <c r="B60" t="n">
-        <v>92.08955</v>
+        <v>94.00376</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1780,7 +1800,7 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1790,10 +1810,10 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46282.22916666666</v>
+        <v>46283.22916666666</v>
       </c>
       <c r="B61" t="n">
-        <v>83.98999999999999</v>
+        <v>90</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1801,7 +1821,7 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1811,10 +1831,10 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46282.25</v>
+        <v>46283.25</v>
       </c>
       <c r="B62" t="n">
-        <v>93.24739</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1822,7 +1842,7 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1832,10 +1852,10 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46282.27083333334</v>
+        <v>46283.27083333334</v>
       </c>
       <c r="B63" t="n">
-        <v>98.64118000000001</v>
+        <v>130.81226</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1843,20 +1863,20 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46282.29166666666</v>
+        <v>46283.29166666666</v>
       </c>
       <c r="B64" t="n">
-        <v>86.83065999999999</v>
+        <v>103.75127</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1864,20 +1884,20 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46282.3125</v>
+        <v>46283.3125</v>
       </c>
       <c r="B65" t="n">
-        <v>57.38977</v>
+        <v>64.81689</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1885,20 +1905,20 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46282.33333333334</v>
+        <v>46283.33333333334</v>
       </c>
       <c r="B66" t="n">
-        <v>42.94</v>
+        <v>0.00859</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1906,7 +1926,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1916,10 +1936,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46282.35416666666</v>
+        <v>46283.35416666666</v>
       </c>
       <c r="B67" t="n">
-        <v>42.8001</v>
+        <v>0.00916</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1927,7 +1947,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1937,10 +1957,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46282.375</v>
+        <v>46283.375</v>
       </c>
       <c r="B68" t="n">
-        <v>42.54</v>
+        <v>-6.52885</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1948,7 +1968,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1958,10 +1978,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46282.39583333334</v>
+        <v>46283.39583333334</v>
       </c>
       <c r="B69" t="n">
-        <v>2.12</v>
+        <v>-7.98974</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1969,7 +1989,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1979,10 +1999,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46282.41666666666</v>
+        <v>46283.41666666666</v>
       </c>
       <c r="B70" t="n">
-        <v>2.12</v>
+        <v>-8.842879999999999</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -1990,7 +2010,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2000,10 +2020,10 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46282.4375</v>
+        <v>46283.4375</v>
       </c>
       <c r="B71" t="n">
-        <v>2.12</v>
+        <v>-9.230460000000001</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2011,7 +2031,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2021,10 +2041,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46282.45833333334</v>
+        <v>46283.45833333334</v>
       </c>
       <c r="B72" t="n">
-        <v>2.12</v>
+        <v>-8.99091</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2032,7 +2052,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2042,10 +2062,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46282.47916666666</v>
+        <v>46283.47916666666</v>
       </c>
       <c r="B73" t="n">
-        <v>-6.5</v>
+        <v>-8.488580000000001</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2053,7 +2073,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2063,10 +2083,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46282.5</v>
+        <v>46283.5</v>
       </c>
       <c r="B74" t="n">
-        <v>2.12</v>
+        <v>-8.3123</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2074,7 +2094,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2084,10 +2104,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46282.52083333334</v>
+        <v>46283.52083333334</v>
       </c>
       <c r="B75" t="n">
-        <v>2.12</v>
+        <v>-8.971</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2095,7 +2115,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2105,10 +2125,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46282.54166666666</v>
+        <v>46283.54166666666</v>
       </c>
       <c r="B76" t="n">
-        <v>-8.415179999999999</v>
+        <v>-10</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2116,7 +2136,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2126,10 +2146,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46282.5625</v>
+        <v>46283.5625</v>
       </c>
       <c r="B77" t="n">
-        <v>-8.630000000000001</v>
+        <v>-10.5</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2137,7 +2157,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2147,10 +2167,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46282.58333333334</v>
+        <v>46283.58333333334</v>
       </c>
       <c r="B78" t="n">
-        <v>-8.72222</v>
+        <v>-9.242089999999999</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2158,7 +2178,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2168,10 +2188,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46282.60416666666</v>
+        <v>46283.60416666666</v>
       </c>
       <c r="B79" t="n">
-        <v>-9.15035</v>
+        <v>-10.5</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2179,7 +2199,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2189,10 +2209,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46282.625</v>
+        <v>46283.625</v>
       </c>
       <c r="B80" t="n">
-        <v>-7.24729</v>
+        <v>-6.51</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2200,7 +2220,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2210,10 +2230,10 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46282.64583333334</v>
+        <v>46283.64583333334</v>
       </c>
       <c r="B81" t="n">
-        <v>-7.03052</v>
+        <v>-5.17</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2221,7 +2241,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2231,10 +2251,10 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46282.66666666666</v>
+        <v>46283.66666666666</v>
       </c>
       <c r="B82" t="n">
-        <v>-6.31457</v>
+        <v>-5.63951</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2242,7 +2262,7 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2252,10 +2272,10 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46282.6875</v>
+        <v>46283.6875</v>
       </c>
       <c r="B83" t="n">
-        <v>0.01063</v>
+        <v>11.5</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2263,7 +2283,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2273,10 +2293,10 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46282.70833333334</v>
+        <v>46283.70833333334</v>
       </c>
       <c r="B84" t="n">
-        <v>61.18634</v>
+        <v>65.38905</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2284,7 +2304,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2294,10 +2314,10 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46282.72916666666</v>
+        <v>46283.72916666666</v>
       </c>
       <c r="B85" t="n">
-        <v>90.93531</v>
+        <v>80.21098000000001</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2305,7 +2325,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2315,10 +2335,10 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>46282.75</v>
+        <v>46283.75</v>
       </c>
       <c r="B86" t="n">
-        <v>133.82812</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2326,7 +2346,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2336,10 +2356,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>46282.77083333334</v>
+        <v>46283.77083333334</v>
       </c>
       <c r="B87" t="n">
-        <v>124.65701</v>
+        <v>90.86496</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2347,7 +2367,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2357,10 +2377,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>46282.79166666666</v>
+        <v>46283.79166666666</v>
       </c>
       <c r="B88" t="n">
-        <v>128.2673</v>
+        <v>90</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2368,7 +2388,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2378,10 +2398,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>46282.8125</v>
+        <v>46283.8125</v>
       </c>
       <c r="B89" t="n">
-        <v>129.65</v>
+        <v>90</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2389,7 +2409,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2399,10 +2419,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>46282.83333333334</v>
+        <v>46283.83333333334</v>
       </c>
       <c r="B90" t="n">
-        <v>129.65</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2410,7 +2430,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2420,10 +2440,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>46282.85416666666</v>
+        <v>46283.85416666666</v>
       </c>
       <c r="B91" t="n">
-        <v>129.65</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2431,7 +2451,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2441,10 +2461,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46282.875</v>
+        <v>46283.875</v>
       </c>
       <c r="B92" t="n">
-        <v>129.65</v>
+        <v>101.67956</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2452,7 +2472,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2462,10 +2482,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>46282.89583333334</v>
+        <v>46283.89583333334</v>
       </c>
       <c r="B93" t="n">
-        <v>129.38</v>
+        <v>95.2</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2473,7 +2493,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2483,10 +2503,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>46282.91666666666</v>
+        <v>46283.91666666666</v>
       </c>
       <c r="B94" t="n">
-        <v>122.19838</v>
+        <v>95.48381999999999</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2494,7 +2514,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2504,10 +2524,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>46282.9375</v>
+        <v>46283.9375</v>
       </c>
       <c r="B95" t="n">
-        <v>115.44164</v>
+        <v>115.36236</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2515,7 +2535,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2525,10 +2545,10 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>46282.95833333334</v>
+        <v>46283.95833333334</v>
       </c>
       <c r="B96" t="n">
-        <v>106.8635</v>
+        <v>112.5769</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2536,7 +2556,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2546,10 +2566,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>46282.97916666666</v>
+        <v>46283.97916666666</v>
       </c>
       <c r="B97" t="n">
-        <v>107.13971</v>
+        <v>107.98126</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2557,7 +2577,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 670)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>462.6162547499998</v>
+        <v>438.7619925</v>
       </c>
       <c r="F2" t="n">
-        <v>11.12593205266955</v>
+        <v>10.55223647186147</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46284.29166666666</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46284.75</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-313.743378</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-7.545535786435787</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -870,11 +890,11 @@
         <v>46283.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>9.84177</v>
+        <v>0.00859</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -891,11 +911,11 @@
         <v>46283.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>10.3857</v>
+        <v>0.0094</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -912,11 +932,11 @@
         <v>46283.375</v>
       </c>
       <c r="B20" t="n">
-        <v>-5.68434</v>
+        <v>-6.65207</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -933,11 +953,11 @@
         <v>46283.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>-7.75218</v>
+        <v>-7.9281</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +974,11 @@
         <v>46283.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-8.37627</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +995,11 @@
         <v>46283.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-10.43257</v>
+        <v>-9.182180000000001</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46283.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-9.353020000000001</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46283.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-9.11041</v>
+        <v>-8.707660000000001</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46283.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-9.04646</v>
+        <v>-8.32752</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46283.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-8.984730000000001</v>
+        <v>-8.970700000000001</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46283.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-10.34</v>
+        <v>-8.64104</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1105,7 +1125,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46283.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-9.088380000000001</v>
+        <v>-9.21904</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1163,11 @@
         <v>46283.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-13</v>
+        <v>-10.5</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46283.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-8.01</v>
+        <v>-8.61251</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1205,11 @@
         <v>46283.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>2.12</v>
+        <v>-7.31397</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1226,11 @@
         <v>46283.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>-4.49628</v>
+        <v>-5.68434</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1231,7 +1251,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1268,11 @@
         <v>46283.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>68.69448</v>
+        <v>65.38909</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1289,11 @@
         <v>46283.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>75.9601</v>
+        <v>80.20885</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,7 +1310,7 @@
         <v>46283.75</v>
       </c>
       <c r="B38" t="n">
-        <v>88.86011000000001</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1311,7 +1331,7 @@
         <v>46283.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>90</v>
+        <v>87.37794</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1332,7 +1352,7 @@
         <v>46283.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>90</v>
+        <v>88.86011000000001</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1353,7 +1373,7 @@
         <v>46283.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>89.20347</v>
+        <v>85.23862</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1374,7 +1394,7 @@
         <v>46283.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>95.57767</v>
+        <v>84.05946</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1415,7 @@
         <v>46283.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>96.98999999999999</v>
+        <v>91.27021000000001</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1436,7 @@
         <v>46283.875</v>
       </c>
       <c r="B44" t="n">
-        <v>90.20999999999999</v>
+        <v>95.2</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46283.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>85.89</v>
+        <v>101.01937</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46283.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>90.20999999999999</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46283.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>204.7258</v>
+        <v>95.2</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1520,7 @@
         <v>46283.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>115.6222</v>
+        <v>95.2</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,7 +1541,7 @@
         <v>46283.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>107.28419</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46283</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B50" t="n">
+        <v>90.20999999999999</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46284.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>90.20999999999999</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46284.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>97.65003</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46284.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46284.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46284.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>84.6388</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46284.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46284.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46284.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>82.31174</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46284.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>75.96007</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46284.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>77.91104</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46284.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46284.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46284.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>72.86112</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46284.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46284.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>-8.34075</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46284.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>-10.45</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46284.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>-14.10806</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46284.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>-14.73618</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46284.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>-18.51</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46284.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>-31.98</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46284.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-29.59882</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46284.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-32.05</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46284.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>-30.21395</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46284.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>-23.5</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46284.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>-23.5</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46284.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>-38.87498</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46284.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-39.43</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46284.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-41.536</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46284.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-42</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46284.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>-32.26767</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46284.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>-27.86299</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46284.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46284.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>-6.80585</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46284.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>42.03717</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46284.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46284.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>106.38945</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46284.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>116.15263</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46284.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>116.8763</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46284.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>110.36734</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46284.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>106.00079</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46284.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>111.3632</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46284.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46284.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>98.72714000000001</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46284.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>96.21351</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46284.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>93.70184999999999</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46284.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>92.59086000000001</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46284.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>91.41459999999999</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 592)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,62 +470,82 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46282</v>
+        <v>46283.10416666666</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46282.66666666666</v>
+        <v>46283.27083333334</v>
       </c>
       <c r="C2" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>60.48</v>
+        <v>15.12</v>
       </c>
       <c r="E2" t="n">
-        <v>1462.04131125</v>
+        <v>733.8681869999999</v>
       </c>
       <c r="F2" t="n">
-        <v>24.1739634796627</v>
+        <v>48.53625575396825</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46283.10416666666</v>
+        <v>46283.3125</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46283.27083333334</v>
+        <v>46283.66666666666</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>8.5</v>
       </c>
       <c r="D3" t="n">
-        <v>15.12</v>
+        <v>32.13</v>
       </c>
       <c r="E3" t="n">
-        <v>724.7977619999999</v>
+        <v>-55.42556175000001</v>
       </c>
       <c r="F3" t="n">
-        <v>47.93635992063492</v>
+        <v>-1.725040826330533</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46283.33333333334</v>
+        <v>46283.85416666666</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>46283.66666666666</v>
+        <v>46284.02083333334</v>
       </c>
       <c r="C4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D4" t="n">
-        <v>30.24</v>
+        <v>15.12</v>
       </c>
       <c r="E4" t="n">
-        <v>-116.2775835</v>
+        <v>701.4837765</v>
       </c>
       <c r="F4" t="n">
-        <v>-3.84515818452381</v>
+        <v>46.39442966269841</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46284.27083333334</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46284.75</v>
+      </c>
+      <c r="C5" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>43.47</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-85.85296199999999</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-1.974993374741201</v>
       </c>
     </row>
   </sheetData>
@@ -571,10 +591,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B2" t="n">
-        <v>96.90548</v>
+        <v>104.35911</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -582,20 +602,20 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46282.02083333334</v>
+        <v>46283.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>95.09088</v>
+        <v>99.98721999999999</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -603,20 +623,20 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46282.04166666666</v>
+        <v>46283.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>93.9953</v>
+        <v>108.06864</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -624,20 +644,20 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46282.0625</v>
+        <v>46283.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>90.88932</v>
+        <v>108.99166</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -645,20 +665,20 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46282.08333333334</v>
+        <v>46283.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>89.03032</v>
+        <v>97.83360999999999</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -666,20 +686,20 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46282.10416666666</v>
+        <v>46283.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>88.88</v>
+        <v>99.13146</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -687,7 +707,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -697,10 +717,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46282.125</v>
+        <v>46283.125</v>
       </c>
       <c r="B8" t="n">
-        <v>88.54156</v>
+        <v>97.63005</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -708,7 +728,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -718,10 +738,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46282.14583333334</v>
+        <v>46283.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>88.88</v>
+        <v>92.23253</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -729,7 +749,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -739,10 +759,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46282.16666666666</v>
+        <v>46283.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>83.96876</v>
+        <v>88.88</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -750,7 +770,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -760,10 +780,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46282.1875</v>
+        <v>46283.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>83.98999999999999</v>
+        <v>94.13094</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -771,7 +791,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -781,10 +801,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46282.20833333334</v>
+        <v>46283.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>92.07459</v>
+        <v>93.99876999999999</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -792,7 +812,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -802,10 +822,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46282.22916666666</v>
+        <v>46283.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>86.81858</v>
+        <v>90</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -813,7 +833,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -823,10 +843,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46282.25</v>
+        <v>46283.25</v>
       </c>
       <c r="B14" t="n">
-        <v>93.24209</v>
+        <v>96.68156999999999</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -834,7 +854,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -844,10 +864,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46282.27083333334</v>
+        <v>46283.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>98.63189</v>
+        <v>122.81974</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -855,20 +875,20 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46282.29166666666</v>
+        <v>46283.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>86.27500000000001</v>
+        <v>103.35895</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -876,20 +896,20 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46282.3125</v>
+        <v>46283.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>57.38977</v>
+        <v>64.95007</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -897,7 +917,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -907,10 +927,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46282.33333333334</v>
+        <v>46283.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>42.79988</v>
+        <v>0.00859</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,7 +938,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -928,10 +948,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46282.35416666666</v>
+        <v>46283.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>42.8001</v>
+        <v>0.0094</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -939,7 +959,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -949,10 +969,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46282.375</v>
+        <v>46283.375</v>
       </c>
       <c r="B20" t="n">
-        <v>34.94352</v>
+        <v>-6.65207</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -960,7 +980,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -970,10 +990,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46282.39583333334</v>
+        <v>46283.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>2.12</v>
+        <v>-7.9281</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -981,7 +1001,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -991,10 +1011,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46282.41666666666</v>
+        <v>46283.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>12.62239</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1002,7 +1022,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1012,10 +1032,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46282.4375</v>
+        <v>46283.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>9.809290000000001</v>
+        <v>-9.182180000000001</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1023,7 +1043,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1033,10 +1053,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46282.45833333334</v>
+        <v>46283.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>0.69548</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1044,7 +1064,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1054,10 +1074,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46282.47916666666</v>
+        <v>46283.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-5.68434</v>
+        <v>-8.707660000000001</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1065,7 +1085,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1075,10 +1095,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46282.5</v>
+        <v>46283.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-6.5</v>
+        <v>-8.32752</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1086,7 +1106,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1096,10 +1116,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46282.52083333334</v>
+        <v>46283.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>0.01015</v>
+        <v>-8.970700000000001</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1107,7 +1127,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1117,10 +1137,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46282.54166666666</v>
+        <v>46283.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-8.35943</v>
+        <v>-8.64104</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1128,7 +1148,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1138,10 +1158,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46282.5625</v>
+        <v>46283.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-8.5139</v>
+        <v>-10.5</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1149,7 +1169,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1159,10 +1179,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46282.58333333334</v>
+        <v>46283.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-8.630000000000001</v>
+        <v>-9.21904</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1170,7 +1190,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1180,10 +1200,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46282.60416666666</v>
+        <v>46283.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-8.630000000000001</v>
+        <v>-10.5</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1191,7 +1211,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1201,10 +1221,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46282.625</v>
+        <v>46283.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-6.5</v>
+        <v>-8.61251</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1212,7 +1232,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1222,10 +1242,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46282.64583333334</v>
+        <v>46283.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>-8.057130000000001</v>
+        <v>-7.31397</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1233,7 +1253,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1243,10 +1263,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46282.66666666666</v>
+        <v>46283.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>-6.07163</v>
+        <v>-5.68434</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1254,7 +1274,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1264,10 +1284,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46282.6875</v>
+        <v>46283.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>0.0107</v>
+        <v>11.5</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1275,7 +1295,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1285,10 +1305,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46282.70833333334</v>
+        <v>46283.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>63.20151</v>
+        <v>65.38909</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1296,7 +1316,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1306,10 +1326,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46282.72916666666</v>
+        <v>46283.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>91.38206</v>
+        <v>80.20885</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1317,7 +1337,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1327,10 +1347,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46282.75</v>
+        <v>46283.75</v>
       </c>
       <c r="B38" t="n">
-        <v>129.38</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1338,7 +1358,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1348,10 +1368,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46282.77083333334</v>
+        <v>46283.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>129.65</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1359,7 +1379,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1369,10 +1389,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46282.79166666666</v>
+        <v>46283.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>127.04177</v>
+        <v>90</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1380,7 +1400,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1390,10 +1410,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46282.8125</v>
+        <v>46283.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>129.65</v>
+        <v>90</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1401,7 +1421,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1411,10 +1431,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46282.83333333334</v>
+        <v>46283.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>129.65</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1422,7 +1442,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1432,10 +1452,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46282.85416666666</v>
+        <v>46283.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>129.65</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1443,20 +1463,20 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46282.875</v>
+        <v>46283.875</v>
       </c>
       <c r="B44" t="n">
-        <v>129.65</v>
+        <v>106.91918</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1464,20 +1484,20 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46282.89583333334</v>
+        <v>46283.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>121.05581</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1485,41 +1505,41 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46282.91666666666</v>
+        <v>46283.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>122.08005</v>
+        <v>85.53967</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>forecast</t>
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46282.9375</v>
+        <v>46283.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>90.20999999999999</v>
+        <v>84.20708999999999</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1527,20 +1547,20 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46282.95833333334</v>
+        <v>46283.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>90.20999999999999</v>
+        <v>85.50554</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1548,20 +1568,20 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46282.97916666666</v>
+        <v>46283.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>129.38</v>
+        <v>86.10906</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1569,20 +1589,20 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B50" t="n">
-        <v>102.55423</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1590,20 +1610,20 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46283.02083333334</v>
+        <v>46284.02083333334</v>
       </c>
       <c r="B51" t="n">
-        <v>110.6441</v>
+        <v>105.00806</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1611,7 +1631,7 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1621,10 +1641,10 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46283.04166666666</v>
+        <v>46284.04166666666</v>
       </c>
       <c r="B52" t="n">
-        <v>111.5911</v>
+        <v>97.65000000000001</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1632,7 +1652,7 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1642,10 +1662,10 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46283.0625</v>
+        <v>46284.0625</v>
       </c>
       <c r="B53" t="n">
-        <v>107.17216</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1653,7 +1673,7 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1663,10 +1683,10 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46283.08333333334</v>
+        <v>46284.08333333334</v>
       </c>
       <c r="B54" t="n">
-        <v>105.51807</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1674,7 +1694,7 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1684,10 +1704,10 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46283.10416666666</v>
+        <v>46284.10416666666</v>
       </c>
       <c r="B55" t="n">
-        <v>98.52148</v>
+        <v>84.02557</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1695,20 +1715,20 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46283.125</v>
+        <v>46284.125</v>
       </c>
       <c r="B56" t="n">
-        <v>97.63005</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1716,20 +1736,20 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46283.14583333334</v>
+        <v>46284.14583333334</v>
       </c>
       <c r="B57" t="n">
-        <v>90</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1737,20 +1757,20 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46283.16666666666</v>
+        <v>46284.16666666666</v>
       </c>
       <c r="B58" t="n">
-        <v>88.88</v>
+        <v>82.98161</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1758,20 +1778,20 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46283.1875</v>
+        <v>46284.1875</v>
       </c>
       <c r="B59" t="n">
-        <v>94.13703</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1779,20 +1799,20 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46283.20833333334</v>
+        <v>46284.20833333334</v>
       </c>
       <c r="B60" t="n">
-        <v>94.00376</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1800,20 +1820,20 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46283.22916666666</v>
+        <v>46284.22916666666</v>
       </c>
       <c r="B61" t="n">
-        <v>90</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1821,20 +1841,20 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46283.25</v>
+        <v>46284.25</v>
       </c>
       <c r="B62" t="n">
-        <v>90.20999999999999</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1842,20 +1862,20 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46283.27083333334</v>
+        <v>46284.27083333334</v>
       </c>
       <c r="B63" t="n">
-        <v>130.81226</v>
+        <v>75.9601</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1863,20 +1883,20 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46283.29166666666</v>
+        <v>46284.29166666666</v>
       </c>
       <c r="B64" t="n">
-        <v>103.75127</v>
+        <v>42.80002</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1884,20 +1904,20 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46283.3125</v>
+        <v>46284.3125</v>
       </c>
       <c r="B65" t="n">
-        <v>64.81689</v>
+        <v>-6.51</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1905,20 +1925,20 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46283.33333333334</v>
+        <v>46284.33333333334</v>
       </c>
       <c r="B66" t="n">
-        <v>0.00859</v>
+        <v>-7.86155</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1926,7 +1946,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1936,10 +1956,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46283.35416666666</v>
+        <v>46284.35416666666</v>
       </c>
       <c r="B67" t="n">
-        <v>0.00916</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1947,7 +1967,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1957,10 +1977,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46283.375</v>
+        <v>46284.375</v>
       </c>
       <c r="B68" t="n">
-        <v>-6.52885</v>
+        <v>-10.45</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1968,7 +1988,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1978,10 +1998,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46283.39583333334</v>
+        <v>46284.39583333334</v>
       </c>
       <c r="B69" t="n">
-        <v>-7.98974</v>
+        <v>-10.5</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1989,7 +2009,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1999,10 +2019,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46283.41666666666</v>
+        <v>46284.41666666666</v>
       </c>
       <c r="B70" t="n">
-        <v>-8.842879999999999</v>
+        <v>-18.51</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -2010,7 +2030,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2020,10 +2040,10 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46283.4375</v>
+        <v>46284.4375</v>
       </c>
       <c r="B71" t="n">
-        <v>-9.230460000000001</v>
+        <v>-20.67</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2031,7 +2051,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2041,10 +2061,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46283.45833333334</v>
+        <v>46284.45833333334</v>
       </c>
       <c r="B72" t="n">
-        <v>-8.99091</v>
+        <v>-20.67</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2052,7 +2072,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2062,10 +2082,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46283.47916666666</v>
+        <v>46284.47916666666</v>
       </c>
       <c r="B73" t="n">
-        <v>-8.488580000000001</v>
+        <v>-18.51</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2073,7 +2093,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2083,10 +2103,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46283.5</v>
+        <v>46284.5</v>
       </c>
       <c r="B74" t="n">
-        <v>-8.3123</v>
+        <v>-14.26856</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2094,7 +2114,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2104,10 +2124,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46283.52083333334</v>
+        <v>46284.52083333334</v>
       </c>
       <c r="B75" t="n">
-        <v>-8.971</v>
+        <v>-18.51</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2115,7 +2135,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2125,10 +2145,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46283.54166666666</v>
+        <v>46284.54166666666</v>
       </c>
       <c r="B76" t="n">
-        <v>-10</v>
+        <v>-23.5</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2136,7 +2156,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2146,10 +2166,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46283.5625</v>
+        <v>46284.5625</v>
       </c>
       <c r="B77" t="n">
-        <v>-10.5</v>
+        <v>-28.32508</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2157,7 +2177,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2167,10 +2187,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46283.58333333334</v>
+        <v>46284.58333333334</v>
       </c>
       <c r="B78" t="n">
-        <v>-9.242089999999999</v>
+        <v>-32.05</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2178,7 +2198,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2188,10 +2208,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46283.60416666666</v>
+        <v>46284.60416666666</v>
       </c>
       <c r="B79" t="n">
-        <v>-10.5</v>
+        <v>-32.05</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2199,7 +2219,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2209,10 +2229,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46283.625</v>
+        <v>46284.625</v>
       </c>
       <c r="B80" t="n">
-        <v>-6.51</v>
+        <v>-26.65912</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2220,7 +2240,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2230,10 +2250,10 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46283.64583333334</v>
+        <v>46284.64583333334</v>
       </c>
       <c r="B81" t="n">
-        <v>-5.17</v>
+        <v>-18.51</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2241,7 +2261,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2251,10 +2271,10 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46283.66666666666</v>
+        <v>46284.66666666666</v>
       </c>
       <c r="B82" t="n">
-        <v>-5.63951</v>
+        <v>-7.52214</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2262,20 +2282,20 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46283.6875</v>
+        <v>46284.6875</v>
       </c>
       <c r="B83" t="n">
-        <v>11.5</v>
+        <v>-5.38422</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2283,20 +2303,20 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46283.70833333334</v>
+        <v>46284.70833333334</v>
       </c>
       <c r="B84" t="n">
-        <v>65.38905</v>
+        <v>52.37623</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2304,20 +2324,20 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46283.72916666666</v>
+        <v>46284.72916666666</v>
       </c>
       <c r="B85" t="n">
-        <v>80.21098000000001</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2325,20 +2345,20 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>46283.75</v>
+        <v>46284.75</v>
       </c>
       <c r="B86" t="n">
-        <v>90.20999999999999</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2346,7 +2366,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2356,10 +2376,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>46283.77083333334</v>
+        <v>46284.77083333334</v>
       </c>
       <c r="B87" t="n">
-        <v>90.86496</v>
+        <v>85.20646000000001</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2367,7 +2387,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2377,10 +2397,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>46283.79166666666</v>
+        <v>46284.79166666666</v>
       </c>
       <c r="B88" t="n">
-        <v>90</v>
+        <v>99.01000000000001</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2388,7 +2408,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2398,10 +2418,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>46283.8125</v>
+        <v>46284.8125</v>
       </c>
       <c r="B89" t="n">
-        <v>90</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2409,7 +2429,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2419,10 +2439,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>46283.83333333334</v>
+        <v>46284.83333333334</v>
       </c>
       <c r="B90" t="n">
-        <v>96.98999999999999</v>
+        <v>90</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2430,7 +2450,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2440,10 +2460,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>46283.85416666666</v>
+        <v>46284.85416666666</v>
       </c>
       <c r="B91" t="n">
-        <v>96.98999999999999</v>
+        <v>90</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2451,7 +2471,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2461,10 +2481,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46283.875</v>
+        <v>46284.875</v>
       </c>
       <c r="B92" t="n">
-        <v>101.67956</v>
+        <v>89</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2472,7 +2492,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2482,10 +2502,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>46283.89583333334</v>
+        <v>46284.89583333334</v>
       </c>
       <c r="B93" t="n">
-        <v>95.2</v>
+        <v>97.23515</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2493,7 +2513,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2503,10 +2523,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>46283.91666666666</v>
+        <v>46284.91666666666</v>
       </c>
       <c r="B94" t="n">
-        <v>95.48381999999999</v>
+        <v>90</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2514,7 +2534,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2524,10 +2544,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>46283.9375</v>
+        <v>46284.9375</v>
       </c>
       <c r="B95" t="n">
-        <v>115.36236</v>
+        <v>90</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2535,7 +2555,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2545,10 +2565,10 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>46283.95833333334</v>
+        <v>46284.95833333334</v>
       </c>
       <c r="B96" t="n">
-        <v>112.5769</v>
+        <v>93.11920000000001</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2556,7 +2576,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2566,10 +2586,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>46283.97916666666</v>
+        <v>46284.97916666666</v>
       </c>
       <c r="B97" t="n">
-        <v>107.98126</v>
+        <v>91.49603</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2577,7 +2597,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 672)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>-100.25493075</v>
+        <v>-128.55255075</v>
       </c>
       <c r="F2" t="n">
-        <v>-2.411133495670995</v>
+        <v>-3.091691937229437</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46285.27083333334</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46285.72916666666</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-194.400804</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-4.675344011544012</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -849,11 +869,11 @@
         <v>46284.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>-3.52698</v>
+        <v>-6.5996</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
@@ -870,11 +890,11 @@
         <v>46284.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>-6.5</v>
+        <v>-8.222759999999999</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -891,11 +911,11 @@
         <v>46284.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>-7.60137</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -916,7 +936,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -937,7 +957,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -958,7 +978,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -979,7 +999,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46284.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-25.93252</v>
+        <v>-20.67</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46284.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-13.62309</v>
+        <v>-18.51</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46284.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-13.79019</v>
+        <v>-13.99696</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46284.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-13.52265</v>
+        <v>-18.51</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46284.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-18.51</v>
+        <v>-13.71567</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1121,11 @@
         <v>46284.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-13.44172</v>
+        <v>-27.01739</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46284.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-23.5</v>
+        <v>-28.36077</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1163,11 @@
         <v>46284.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-31.98</v>
+        <v>-32.05</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46284.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-23.5</v>
+        <v>-26.14787</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1189,7 +1209,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1226,11 @@
         <v>46284.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>-7.08971</v>
+        <v>-7.56967</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1247,11 @@
         <v>46284.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>-3.84272</v>
+        <v>-5.38346</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1252,7 +1272,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1273,7 +1293,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,7 +1310,7 @@
         <v>46284.75</v>
       </c>
       <c r="B38" t="n">
-        <v>82.90000000000001</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1311,7 +1331,7 @@
         <v>46284.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>77.6435</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1332,7 +1352,7 @@
         <v>46284.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>85.29822</v>
+        <v>77.50557000000001</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1353,7 +1373,7 @@
         <v>46284.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>85.32284</v>
+        <v>80.9922</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1374,7 +1394,7 @@
         <v>46284.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>85.49151999999999</v>
+        <v>80.48269999999999</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1415,7 @@
         <v>46284.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>86.32835</v>
+        <v>75.95001999999999</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1436,7 @@
         <v>46284.875</v>
       </c>
       <c r="B44" t="n">
-        <v>85.07485</v>
+        <v>75.94</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46284.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>92.49014</v>
+        <v>75.94</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46284.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>90</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46284.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>88.74948999999999</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1520,7 @@
         <v>46284.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>90</v>
+        <v>88.86</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,7 +1541,7 @@
         <v>46284.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>90</v>
+        <v>89.82409</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46284</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B50" t="n">
+        <v>88.06882</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46285.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>84.79000000000001</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46285.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>73.26275</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46285.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46285.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>79.14097</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46285.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>77.35319</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46285.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>76.88495</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46285.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>75.95</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46285.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>75.92700000000001</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46285.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>75.41942</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46285.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>74.90673</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46285.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>75.96007</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46285.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>75.9601</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46285.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>63.73</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46285.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>3e-05</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46285.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>-8.93938</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46285.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>-10.45</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46285.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>-10.45</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46285.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>-10.45</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46285.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>-18.5098</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46285.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>-18.51</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46285.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-20.67</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46285.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-24.47881</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46285.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>-18.51</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46285.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>-12.87947</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46285.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>-20.67</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46285.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>-18.51</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46285.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-31.98</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46285.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-31.98</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46285.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-27.00561</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46285.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>-18.51</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46285.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>-8.60571</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46285.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>-7.28853</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46285.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>-4.45924</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46285.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>59.74108</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46285.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46285.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>119.07284</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46285.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>193.78277</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46285.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>176.94788</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46285.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>220.63235</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46285.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>216.91948</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46285.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46285.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46285.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>109.37821</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46285.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>210.0001</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46285.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>114.22215</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46285.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46285.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>87.11994</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 594)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,42 +470,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46284.0625</v>
+        <v>46284.22916666666</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46284.22916666666</v>
+        <v>46284.77083333334</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="D2" t="n">
-        <v>15.12</v>
+        <v>49.14</v>
       </c>
       <c r="E2" t="n">
-        <v>653.58728175</v>
+        <v>188.8219807500001</v>
       </c>
       <c r="F2" t="n">
-        <v>43.2266720734127</v>
+        <v>3.842531150793652</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46284.27083333334</v>
+        <v>46284.875</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46284.77083333334</v>
+        <v>46285.04166666666</v>
       </c>
       <c r="C3" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>45.36</v>
+        <v>15.12</v>
       </c>
       <c r="E3" t="n">
-        <v>45.83390175000001</v>
+        <v>634.9066132500001</v>
       </c>
       <c r="F3" t="n">
-        <v>1.010447569444445</v>
+        <v>41.991178125</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46285.27083333334</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46285.72916666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>11</v>
+      </c>
+      <c r="D4" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-154.1609745</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-3.707575144300144</v>
       </c>
     </row>
   </sheetData>
@@ -519,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -617,11 +637,11 @@
         <v>46284.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>83.98999999999999</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
@@ -629,7 +649,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -638,11 +658,11 @@
         <v>46284.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>83.44104</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
@@ -650,7 +670,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -663,7 +683,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
@@ -671,7 +691,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -684,7 +704,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
@@ -692,7 +712,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -705,7 +725,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -713,7 +733,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -722,11 +742,11 @@
         <v>46284.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>82.96489</v>
+        <v>82.96753</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
@@ -734,7 +754,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -743,11 +763,11 @@
         <v>46284.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>83.98999999999999</v>
+        <v>83.26596000000001</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -755,7 +775,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -764,11 +784,11 @@
         <v>46284.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>83.98999999999999</v>
+        <v>83.95513</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
@@ -776,7 +796,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -785,11 +805,11 @@
         <v>46284.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>83.98999999999999</v>
+        <v>83.87582</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
@@ -797,7 +817,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -806,11 +826,11 @@
         <v>46284.25</v>
       </c>
       <c r="B14" t="n">
-        <v>83.98999999999999</v>
+        <v>82.78652</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
@@ -818,7 +838,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -827,11 +847,11 @@
         <v>46284.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>75.9601</v>
+        <v>75.95</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
@@ -848,11 +868,11 @@
         <v>46284.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>53.06637</v>
+        <v>52.72531</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
@@ -869,11 +889,11 @@
         <v>46284.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>-6.59924</v>
+        <v>-6.5996</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
@@ -890,11 +910,11 @@
         <v>46284.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>-8.195349999999999</v>
+        <v>-8.222759999999999</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -911,11 +931,11 @@
         <v>46284.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>-7.85115</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -936,7 +956,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -957,7 +977,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -974,11 +994,11 @@
         <v>46284.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-13.94563</v>
+        <v>-18.51</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -995,11 +1015,11 @@
         <v>46284.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-13.80155</v>
+        <v>-18.51</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1016,11 +1036,11 @@
         <v>46284.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-18.51</v>
+        <v>-20.67</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1041,7 +1061,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1058,11 +1078,11 @@
         <v>46284.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-13.64388</v>
+        <v>-13.99696</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1079,11 +1099,11 @@
         <v>46284.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-18.5098</v>
+        <v>-18.51</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1100,11 +1120,11 @@
         <v>46284.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-18.5098</v>
+        <v>-13.71567</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1121,11 +1141,11 @@
         <v>46284.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-18.51</v>
+        <v>-27.01739</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1142,11 +1162,11 @@
         <v>46284.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-23.5</v>
+        <v>-28.36077</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1163,11 +1183,11 @@
         <v>46284.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-31.98</v>
+        <v>-32.05</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1184,11 +1204,11 @@
         <v>46284.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-26.82818</v>
+        <v>-26.14787</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1205,11 +1225,11 @@
         <v>46284.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>-13</v>
+        <v>-18.51</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1226,11 +1246,11 @@
         <v>46284.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>-7.1906</v>
+        <v>-7.56967</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1247,11 +1267,11 @@
         <v>46284.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>-5.38438</v>
+        <v>-5.38346</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1268,11 +1288,11 @@
         <v>46284.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>52.47849</v>
+        <v>57.39007</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1293,7 +1313,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1310,11 +1330,11 @@
         <v>46284.75</v>
       </c>
       <c r="B38" t="n">
-        <v>81.02373</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1335,7 +1355,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1352,11 +1372,11 @@
         <v>46284.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>95.88609</v>
+        <v>99.01000000000001</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1377,7 +1397,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1394,11 +1414,11 @@
         <v>46284.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>85.63066000000001</v>
+        <v>89</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -1415,11 +1435,11 @@
         <v>46284.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>86.32682</v>
+        <v>86.31001000000001</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
@@ -1436,11 +1456,11 @@
         <v>46284.875</v>
       </c>
       <c r="B44" t="n">
-        <v>88.67072</v>
+        <v>85.05902</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D44" s="3" t="n">
@@ -1448,7 +1468,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1457,11 +1477,11 @@
         <v>46284.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>89.26503</v>
+        <v>88.86</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D45" s="3" t="n">
@@ -1469,7 +1489,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1498,7 @@
         <v>46284.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>90</v>
+        <v>84.17119</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1490,7 +1510,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1531,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1540,7 @@
         <v>46284.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>92.06316</v>
+        <v>83.25357</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1532,7 +1552,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1561,7 @@
         <v>46284.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>90</v>
+        <v>75.9601</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1552,6 +1572,1014 @@
         <v>46284</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B50" t="n">
+        <v>73.98239</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46285.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46285.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>75.95</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46285.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>72.43929</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46285.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46285.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46285.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>76.33591</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46285.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>75.95</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46285.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>75.8647</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46285.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>75.35809999999999</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46285.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>75.95003</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46285.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>75.96007</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46285.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>75.9601</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46285.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>63.27248</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46285.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>0</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46285.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>-8.464880000000001</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46285.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>-8.50142</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46285.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>-10.45</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46285.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>-10.45</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46285.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>-12.92849</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46285.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>-18.51</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46285.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-18.51</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46285.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-25.42245</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46285.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>-13.13004</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46285.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>-12.43893</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46285.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>-12.45474</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46285.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>-18.51</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46285.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-20.67</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46285.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-27.27176</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46285.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-26.98405</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46285.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>-18.51</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46285.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>-9.32</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46285.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>-6.54882</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46285.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>-2.67244</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46285.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>60.36172</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46285.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>73.40833000000001</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46285.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46285.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46285.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>104.5967</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46285.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>96.37272</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46285.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>94.06099</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46285.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>99.01000000000001</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46285.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46285.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>93.72411</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46285.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>97.59650999999999</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46285.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46285.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46285.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>86.49375000000001</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 674)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>-119.349633</v>
+        <v>-193.30670775</v>
       </c>
       <c r="F2" t="n">
-        <v>-2.870361544011545</v>
+        <v>-4.649030970418471</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46286.20833333334</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46286.66666666666</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>922.7536402499998</v>
+      </c>
+      <c r="F3" t="n">
+        <v>22.19224724025974</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -849,11 +869,11 @@
         <v>46285.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>0.00049</v>
+        <v>-8.40917</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
@@ -870,11 +890,11 @@
         <v>46285.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>-6.51</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -891,11 +911,11 @@
         <v>46285.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>-7.98509</v>
+        <v>-10.45</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -912,11 +932,11 @@
         <v>46285.375</v>
       </c>
       <c r="B20" t="n">
-        <v>-10.5</v>
+        <v>-10.45605</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -933,11 +953,11 @@
         <v>46285.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>-12.37601</v>
+        <v>-13.40244</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +974,11 @@
         <v>46285.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-20.67</v>
+        <v>-18.51</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -979,7 +999,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46285.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-20.67</v>
+        <v>-24.77803</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46285.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-18.48</v>
+        <v>-20.67</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46285.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-18.48</v>
+        <v>-18.51</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46285.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-12.37883</v>
+        <v>-18.51</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46285.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-18.51</v>
+        <v>-23.5</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1121,11 @@
         <v>46285.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-25.80591</v>
+        <v>-31.45321</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46285.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-27.26637</v>
+        <v>-31.98</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1163,11 @@
         <v>46285.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-23.5</v>
+        <v>-20.67</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46285.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-18.51</v>
+        <v>-23.5</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1205,11 @@
         <v>46285.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>-10.34</v>
+        <v>-12.18097</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1226,11 @@
         <v>46285.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>-5.7546</v>
+        <v>-6.78199</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1247,11 @@
         <v>46285.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>23.6082</v>
+        <v>-0.72396</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1268,11 @@
         <v>46285.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>67.22528</v>
+        <v>60.35957</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1289,11 @@
         <v>46285.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>77.83329000000001</v>
+        <v>79.95317</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1294,7 +1314,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,7 +1331,7 @@
         <v>46285.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>94.20929</v>
+        <v>111.47814</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1332,7 +1352,7 @@
         <v>46285.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>99.28644</v>
+        <v>111.98</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1353,7 +1373,7 @@
         <v>46285.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>91.75359</v>
+        <v>97.5568</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1374,7 +1394,7 @@
         <v>46285.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>96.98999999999999</v>
+        <v>96.51594</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1415,7 @@
         <v>46285.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>96.98999999999999</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1436,7 @@
         <v>46285.875</v>
       </c>
       <c r="B44" t="n">
-        <v>94.26227</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46285.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>100.4427</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46285.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>119</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46285.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>104.23713</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1520,7 @@
         <v>46285.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>96.98999999999999</v>
+        <v>94.45914</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,7 +1541,7 @@
         <v>46285.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>85.91652000000001</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46285</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B50" t="n">
+        <v>83.87978</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46286.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>83.34857</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46286.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46286.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46286.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>75.95001999999999</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46286.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>71.63506</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46286.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>71.18539</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46286.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>70.27211</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46286.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>69.80465</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46286.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>75.95001999999999</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46286.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>82.42552999999999</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46286.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>87.64866000000001</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46286.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>86.95738</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46286.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>90</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46286.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>58.68034</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46286.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46286.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46286.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46286.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>52.21</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46286.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46286.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46286.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46286.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46286.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>29.73016</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46286.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>28.99639</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46286.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46286.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>27.43411</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46286.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>45.92903</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46286.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>29</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46286.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>54.04777</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46286.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46286.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>53.19462</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46286.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>49.40252</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46286.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>66.27257</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46286.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46286.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>109.30632</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46286.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>933.03482</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46286.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>20250.21096</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46286.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>23199.96</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46286.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>21255.68357</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46286.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>20643.42802</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46286.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>20820.21488</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46286.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>997.09978</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46286.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>294.42721</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46286.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>165.87432</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46286.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>239.9</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46286.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>118.01176</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46286.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 596)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,42 +470,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46285.0625</v>
+        <v>46285.04166666666</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46285.22916666666</v>
+        <v>46285.25</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" t="n">
-        <v>15.12</v>
+        <v>18.9</v>
       </c>
       <c r="E2" t="n">
-        <v>635.976978</v>
+        <v>756.00570825</v>
       </c>
       <c r="F2" t="n">
-        <v>42.06196944444445</v>
+        <v>40.00030202380952</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46285.25</v>
+        <v>46285.27083333334</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46285.75</v>
+        <v>46285.72916666666</v>
       </c>
       <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-193.30670775</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-4.649030970418471</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46286.16666666666</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46286.66666666666</v>
+      </c>
+      <c r="C4" t="n">
         <v>12</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D4" t="n">
         <v>45.36</v>
       </c>
-      <c r="E3" t="n">
-        <v>-28.83659999999999</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-0.635727513227513</v>
+      <c r="E4" t="n">
+        <v>1187.45958825</v>
+      </c>
+      <c r="F4" t="n">
+        <v>26.17856235119048</v>
       </c>
     </row>
   </sheetData>
@@ -519,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,14 +571,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46285.04166666666</v>
+        <v>46285</v>
       </c>
       <c r="B2" t="n">
-        <v>84.79000000000001</v>
+        <v>86.43449</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
@@ -572,14 +592,14 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46285.0625</v>
+        <v>46285.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>73.74236000000001</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
@@ -587,20 +607,20 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46285.08333333334</v>
+        <v>46285.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>83.98999999999999</v>
+        <v>75.95</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
@@ -614,14 +634,14 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46285.10416666666</v>
+        <v>46285.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>83.98999999999999</v>
+        <v>75.96012</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
@@ -635,14 +655,14 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46285.125</v>
+        <v>46285.08333333334</v>
       </c>
       <c r="B6" t="n">
         <v>83.98999999999999</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
@@ -656,14 +676,14 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46285.14583333334</v>
+        <v>46285.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>82.63164999999999</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
@@ -677,14 +697,14 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46285.16666666666</v>
+        <v>46285.125</v>
       </c>
       <c r="B8" t="n">
-        <v>75.96007</v>
+        <v>76.32367000000001</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
@@ -698,14 +718,14 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46285.1875</v>
+        <v>46285.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>83.98999999999999</v>
+        <v>75.95</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -719,14 +739,14 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46285.20833333334</v>
+        <v>46285.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>83.98999999999999</v>
+        <v>75.36655</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
@@ -740,14 +760,14 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46285.22916666666</v>
+        <v>46285.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>83.85923</v>
+        <v>75.95003</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -755,20 +775,20 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46285.25</v>
+        <v>46285.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>76.48175999999999</v>
+        <v>75.95003</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
@@ -782,14 +802,14 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46285.27083333334</v>
+        <v>46285.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>63.25212</v>
+        <v>75.96007</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
@@ -803,14 +823,14 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46285.29166666666</v>
+        <v>46285.25</v>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>75.9601</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
@@ -818,20 +838,20 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46285.3125</v>
+        <v>46285.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>-8.268050000000001</v>
+        <v>63.00306</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
@@ -845,14 +865,14 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46285.33333333334</v>
+        <v>46285.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>-8.01</v>
+        <v>-0.0001</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
@@ -866,14 +886,14 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46285.35416666666</v>
+        <v>46285.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>-10.45</v>
+        <v>-8.40917</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
@@ -887,14 +907,14 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46285.375</v>
+        <v>46285.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>-10.45</v>
+        <v>-8.630000000000001</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -908,14 +928,14 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46285.39583333334</v>
+        <v>46285.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>-13.06173</v>
+        <v>-10.45</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -929,14 +949,14 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46285.41666666666</v>
+        <v>46285.375</v>
       </c>
       <c r="B20" t="n">
-        <v>-23.5</v>
+        <v>-10.45605</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -950,14 +970,14 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46285.4375</v>
+        <v>46285.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>-20.67</v>
+        <v>-13.40244</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -971,14 +991,14 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46285.45833333334</v>
+        <v>46285.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-20.67</v>
+        <v>-18.51</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -992,14 +1012,14 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46285.47916666666</v>
+        <v>46285.4375</v>
       </c>
       <c r="B23" t="n">
         <v>-18.51</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1013,14 +1033,14 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46285.5</v>
+        <v>46285.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-12.46135</v>
+        <v>-24.77803</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1034,14 +1054,14 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46285.52083333334</v>
+        <v>46285.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-18.51</v>
+        <v>-20.67</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1055,14 +1075,14 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46285.54166666666</v>
+        <v>46285.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-20.67</v>
+        <v>-18.51</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1076,14 +1096,14 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46285.5625</v>
+        <v>46285.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-25.64146</v>
+        <v>-18.51</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1097,14 +1117,14 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46285.58333333334</v>
+        <v>46285.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-31.98</v>
+        <v>-23.5</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1118,14 +1138,14 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46285.60416666666</v>
+        <v>46285.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-30.93851</v>
+        <v>-31.45321</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1139,14 +1159,14 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46285.625</v>
+        <v>46285.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-18.51</v>
+        <v>-31.98</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1160,14 +1180,14 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46285.64583333334</v>
+        <v>46285.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-8.28457</v>
+        <v>-20.67</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1181,14 +1201,14 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46285.66666666666</v>
+        <v>46285.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-6.51</v>
+        <v>-23.5</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1202,14 +1222,14 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46285.6875</v>
+        <v>46285.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>-2.67231</v>
+        <v>-12.18097</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1223,14 +1243,14 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46285.70833333334</v>
+        <v>46285.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>60.3581</v>
+        <v>-6.78199</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1244,14 +1264,14 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46285.72916666666</v>
+        <v>46285.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>80.09999999999999</v>
+        <v>-0.72396</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1265,14 +1285,14 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46285.75</v>
+        <v>46285.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>88.86011000000001</v>
+        <v>60.35957</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1280,20 +1300,20 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46285.77083333334</v>
+        <v>46285.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>90.61456</v>
+        <v>79.95317</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1307,14 +1327,14 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46285.79166666666</v>
+        <v>46285.75</v>
       </c>
       <c r="B38" t="n">
-        <v>102.985</v>
+        <v>88.86011000000001</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1328,14 +1348,14 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46285.8125</v>
+        <v>46285.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>96.90506000000001</v>
+        <v>89.37313</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1349,14 +1369,14 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46285.83333333334</v>
+        <v>46285.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>87.91777</v>
+        <v>111.26179</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1370,14 +1390,14 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46285.85416666666</v>
+        <v>46285.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>84.79000000000001</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1391,14 +1411,14 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46285.875</v>
+        <v>46285.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>100.65376</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -1412,14 +1432,14 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46285.89583333334</v>
+        <v>46285.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>98.51983</v>
+        <v>99.01000000000001</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
@@ -1433,14 +1453,14 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46285.91666666666</v>
+        <v>46285.875</v>
       </c>
       <c r="B44" t="n">
-        <v>115.19655</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D44" s="3" t="n">
@@ -1454,14 +1474,14 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46285.9375</v>
+        <v>46285.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>106.54337</v>
+        <v>93.11112</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D45" s="3" t="n">
@@ -1475,10 +1495,10 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46285.95833333334</v>
+        <v>46285.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>96.98999999999999</v>
+        <v>142.9</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1496,20 +1516,1070 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
+        <v>46285.9375</v>
+      </c>
+      <c r="B47" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46285.95833333334</v>
+      </c>
+      <c r="B48" t="n">
+        <v>96.89567</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
         <v>46285.97916666666</v>
       </c>
-      <c r="B47" t="n">
-        <v>85.89619999999999</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>forecast</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="n">
-        <v>46285</v>
-      </c>
-      <c r="E47" t="inlineStr">
+      <c r="B49" t="n">
+        <v>84.79000000000001</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B50" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46286.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>81.76554</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46286.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>82.84747</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46286.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>82.30788</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46286.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>83.61612</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46286.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>81.31466</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46286.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>75.95001999999999</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46286.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>75.95001999999999</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46286.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>75.95001999999999</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46286.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>75.96007</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46286.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>81.82988</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46286.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46286.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>85.68185</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46286.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>95.14924999999999</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46286.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>60.97017</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46286.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46286.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46286.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>28.54462</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46286.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>52.21</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46286.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46286.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46286.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>41.88</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46286.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>41.88</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46286.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>59.36972</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46286.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>34.52087</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46286.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46286.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>29</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46286.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>29.10896</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46286.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>29</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46286.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46286.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>53.39373</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46286.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>55.14813</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46286.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>50.32169</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46286.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>75.11443</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46286.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46286.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>101.15054</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46286.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>2024.69369</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46286.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>20506.17073</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46286.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>20199.99003</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46286.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>9684.55637</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46286.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>956.35391</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46286.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>941.27979</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46286.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>516.15317</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46286.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>286.493</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46286.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>122.17293</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46286.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>189.46135</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46286.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>119</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46286.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>103.24672</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 676)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>641.006184</v>
+        <v>877.4101439999999</v>
       </c>
       <c r="F2" t="n">
-        <v>15.41621414141414</v>
+        <v>21.10173506493506</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46287.20833333334</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46287.66666666666</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1228.3279515</v>
+      </c>
+      <c r="F3" t="n">
+        <v>29.54131677489178</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -849,11 +869,11 @@
         <v>46286.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>52.9</v>
+        <v>28.88316</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
@@ -870,11 +890,11 @@
         <v>46286.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>45.86746</v>
+        <v>52.21</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -891,11 +911,11 @@
         <v>46286.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>42.7999</v>
+        <v>10.64282</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -912,11 +932,11 @@
         <v>46286.375</v>
       </c>
       <c r="B20" t="n">
-        <v>42.94</v>
+        <v>7.6648</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -933,11 +953,11 @@
         <v>46286.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>1.00075</v>
+        <v>2.12</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +974,11 @@
         <v>46286.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>0.98476</v>
+        <v>11.5</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +995,11 @@
         <v>46286.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>0.9611</v>
+        <v>23.14512</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46286.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>0.01061</v>
+        <v>22.24446</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46286.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>0.01074</v>
+        <v>41.32391</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46286.5</v>
       </c>
       <c r="B26" t="n">
-        <v>0</v>
+        <v>52.21</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46286.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-3.64772</v>
+        <v>31.77163</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46286.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-3.97186</v>
+        <v>29</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1121,11 @@
         <v>46286.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-3.31359</v>
+        <v>29</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46286.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-5.38293</v>
+        <v>14.57416</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1163,11 @@
         <v>46286.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>0.01111</v>
+        <v>42.94</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46286.625</v>
       </c>
       <c r="B32" t="n">
-        <v>42.54</v>
+        <v>53.41132</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1205,11 @@
         <v>46286.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>51.60935</v>
+        <v>55.1439</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1226,11 @@
         <v>46286.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>49.99469</v>
+        <v>50.31708</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1247,11 @@
         <v>46286.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>80.3216</v>
+        <v>75.10842</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1268,11 @@
         <v>46286.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>85.1455</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1289,11 @@
         <v>46286.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>111.98</v>
+        <v>99.96858</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1310,11 @@
         <v>46286.75</v>
       </c>
       <c r="B38" t="n">
-        <v>287.41682</v>
+        <v>932.72699</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,7 +1331,7 @@
         <v>46286.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>413.89145</v>
+        <v>171.43987</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1332,7 +1352,7 @@
         <v>46286.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>239.56411</v>
+        <v>242.95302</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1353,7 +1373,7 @@
         <v>46286.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>277.65762</v>
+        <v>182.84932</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1374,7 +1394,7 @@
         <v>46286.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>426.8976</v>
+        <v>142.9</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1415,7 @@
         <v>46286.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>272.50339</v>
+        <v>203.11508</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1436,7 @@
         <v>46286.875</v>
       </c>
       <c r="B44" t="n">
-        <v>129.65</v>
+        <v>163.64</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46286.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>111.98</v>
+        <v>497.27596</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46286.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>100.12785</v>
+        <v>243.51273</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46286.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>162.84711</v>
+        <v>123.74868</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1520,7 @@
         <v>46286.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>119</v>
+        <v>128.96079</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,7 +1541,7 @@
         <v>46286.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>99.18042</v>
+        <v>113.62646</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46286</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B50" t="n">
+        <v>119</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46287.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>136.00279</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46287.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>114.42552</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46287.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>92.18526</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46287.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>87.44719000000001</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46287.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46287.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46287.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46287.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46287.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>94.93574</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46287.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>96.97275</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46287.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>102.99</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46287.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>112.48542</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46287.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>119.01</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46287.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>97.63005</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46287.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>58.93212</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46287.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>42.8001</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46287.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46287.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46287.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>24.99023</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46287.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46287.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>42.8001</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46287.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>42.8001</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46287.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>42.8001</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46287.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46287.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>24.99064</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46287.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>24.99028</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46287.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46287.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46287.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46287.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>40.77897</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46287.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>39.77268</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46287.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>38.18024</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46287.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>57.39012</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46287.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>90.20999999999999</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46287.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>103.22076</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46287.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>122.92373</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46287.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>191.31596</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46287.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>196.37555</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46287.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>146.54976</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46287.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>142.9</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46287.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>138</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46287.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>132.55</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46287.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>124.90002</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46287.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>117.80302</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46287.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>117.03351</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46287.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>96.93517</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46287.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>98.76058</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 598)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,62 +470,42 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46286.04166666666</v>
+        <v>46286</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46286.20833333334</v>
+        <v>46286.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D2" t="n">
-        <v>15.12</v>
+        <v>60.48</v>
       </c>
       <c r="E2" t="n">
-        <v>650.7678157500001</v>
+        <v>1685.5022145</v>
       </c>
       <c r="F2" t="n">
-        <v>43.04019945436509</v>
+        <v>27.86875354662699</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46286.3125</v>
+        <v>46287.16666666666</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46286.64583333334</v>
+        <v>46287.66666666666</v>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D3" t="n">
-        <v>30.24</v>
+        <v>45.36</v>
       </c>
       <c r="E3" t="n">
-        <v>539.9118074999999</v>
+        <v>1377.40986825</v>
       </c>
       <c r="F3" t="n">
-        <v>17.85422643849206</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>46286.83333333334</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>46287</v>
-      </c>
-      <c r="C4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D4" t="n">
-        <v>15.12</v>
-      </c>
-      <c r="E4" t="n">
-        <v>3088.18271775</v>
-      </c>
-      <c r="F4" t="n">
-        <v>204.2448887400794</v>
+        <v>30.36617875330687</v>
       </c>
     </row>
   </sheetData>
@@ -539,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -571,14 +551,14 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46286.04166666666</v>
+        <v>46286</v>
       </c>
       <c r="B2" t="n">
-        <v>83.98999999999999</v>
+        <v>84.56471000000001</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
@@ -592,14 +572,14 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46286.0625</v>
+        <v>46286.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>83.46975999999999</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
@@ -613,14 +593,14 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46286.08333333334</v>
+        <v>46286.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>82.45486</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
@@ -634,14 +614,14 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46286.10416666666</v>
+        <v>46286.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>81.42594</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
@@ -655,14 +635,14 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46286.125</v>
+        <v>46286.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>79.17354</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
@@ -676,14 +656,14 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46286.14583333334</v>
+        <v>46286.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>75.96007</v>
+        <v>83.09568</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
@@ -697,14 +677,14 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46286.16666666666</v>
+        <v>46286.125</v>
       </c>
       <c r="B8" t="n">
-        <v>96.98999999999999</v>
+        <v>81.50857000000001</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
@@ -718,14 +698,14 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46286.1875</v>
+        <v>46286.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>83.98999999999999</v>
+        <v>79.74406999999999</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -739,14 +719,14 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46286.20833333334</v>
+        <v>46286.16666666666</v>
       </c>
       <c r="B10" t="n">
         <v>83.98999999999999</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
@@ -754,20 +734,20 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46286.22916666666</v>
+        <v>46286.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>95.90349000000001</v>
+        <v>79.94935</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -775,20 +755,20 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46286.25</v>
+        <v>46286.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>96.98999999999999</v>
+        <v>81.29104</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
@@ -796,20 +776,20 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46286.27083333334</v>
+        <v>46286.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>95.1091</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
@@ -817,20 +797,20 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46286.29166666666</v>
+        <v>46286.25</v>
       </c>
       <c r="B14" t="n">
-        <v>61.02</v>
+        <v>85.76063000000001</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
@@ -838,20 +818,20 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46286.3125</v>
+        <v>46286.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>52.21</v>
+        <v>90</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
@@ -865,14 +845,14 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46286.33333333334</v>
+        <v>46286.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>11.5</v>
+        <v>51.08089</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
@@ -886,14 +866,14 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46286.35416666666</v>
+        <v>46286.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>16.23416</v>
+        <v>28.88316</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
@@ -907,14 +887,14 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46286.375</v>
+        <v>46286.33333333334</v>
       </c>
       <c r="B18" t="n">
         <v>52.21</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -928,14 +908,14 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46286.39583333334</v>
+        <v>46286.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>42.8</v>
+        <v>10.64282</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -949,14 +929,14 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46286.41666666666</v>
+        <v>46286.375</v>
       </c>
       <c r="B20" t="n">
-        <v>23.14435</v>
+        <v>7.6648</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -970,14 +950,14 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46286.4375</v>
+        <v>46286.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>23.94957</v>
+        <v>2.12</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -991,14 +971,14 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46286.45833333334</v>
+        <v>46286.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>20.30948</v>
+        <v>11.5</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -1012,14 +992,14 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46286.47916666666</v>
+        <v>46286.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>42.74894</v>
+        <v>23.14512</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1033,14 +1013,14 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46286.5</v>
+        <v>46286.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>36.16533</v>
+        <v>22.24446</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1054,14 +1034,14 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46286.52083333334</v>
+        <v>46286.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>11.5</v>
+        <v>41.32391</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1075,14 +1055,14 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46286.54166666666</v>
+        <v>46286.5</v>
       </c>
       <c r="B26" t="n">
-        <v>29</v>
+        <v>52.21</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1096,14 +1076,14 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46286.5625</v>
+        <v>46286.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>40.69459</v>
+        <v>31.77163</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1117,14 +1097,14 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46286.58333333334</v>
+        <v>46286.54166666666</v>
       </c>
       <c r="B28" t="n">
         <v>29</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1138,14 +1118,14 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46286.60416666666</v>
+        <v>46286.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>64.95</v>
+        <v>29</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1159,14 +1139,14 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46286.625</v>
+        <v>46286.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>57.33928</v>
+        <v>14.57416</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1180,14 +1160,14 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46286.64583333334</v>
+        <v>46286.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>55.1458</v>
+        <v>42.94</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1195,20 +1175,20 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46286.66666666666</v>
+        <v>46286.625</v>
       </c>
       <c r="B32" t="n">
-        <v>49.99734</v>
+        <v>53.41132</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1216,20 +1196,20 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46286.6875</v>
+        <v>46286.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>64.89</v>
+        <v>55.1439</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1237,20 +1217,20 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46286.70833333334</v>
+        <v>46286.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>90.17044</v>
+        <v>50.31708</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1264,14 +1244,14 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46286.72916666666</v>
+        <v>46286.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>105.92906</v>
+        <v>75.10842</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1285,14 +1265,14 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46286.75</v>
+        <v>46286.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>944.86794</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1306,14 +1286,14 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46286.77083333334</v>
+        <v>46286.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>1004.3776</v>
+        <v>99.96858</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1327,14 +1307,14 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46286.79166666666</v>
+        <v>46286.75</v>
       </c>
       <c r="B38" t="n">
-        <v>20199.99003</v>
+        <v>932.72699</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1348,14 +1328,14 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46286.8125</v>
+        <v>46286.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>963.6446099999999</v>
+        <v>20373.7864</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1369,14 +1349,14 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46286.83333333334</v>
+        <v>46286.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>931.83253</v>
+        <v>20263.70201</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1384,20 +1364,20 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46286.85416666666</v>
+        <v>46286.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>989.56316</v>
+        <v>480.2463</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1405,20 +1385,20 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46286.875</v>
+        <v>46286.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>495.44701</v>
+        <v>494.13317</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -1426,20 +1406,20 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46286.89583333334</v>
+        <v>46286.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>277.21306</v>
+        <v>989.63057</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
@@ -1447,20 +1427,20 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46286.91666666666</v>
+        <v>46286.875</v>
       </c>
       <c r="B44" t="n">
-        <v>122.50579</v>
+        <v>512.80454</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D44" s="3" t="n">
@@ -1468,20 +1448,20 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46286.9375</v>
+        <v>46286.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>129.66292</v>
+        <v>213.39429</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D45" s="3" t="n">
@@ -1489,20 +1469,20 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46286.95833333334</v>
+        <v>46286.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>119.2444</v>
+        <v>120.49362</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D46" s="3" t="n">
@@ -1510,28 +1490,1078 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
+        <v>46286.9375</v>
+      </c>
+      <c r="B47" t="n">
+        <v>164.99097</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>historical</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46286.95833333334</v>
+      </c>
+      <c r="B48" t="n">
+        <v>119.25421</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>historical</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
         <v>46286.97916666666</v>
       </c>
-      <c r="B47" t="n">
-        <v>101.89802</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>forecast</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="n">
-        <v>46286</v>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>ON</t>
+      <c r="B49" t="n">
+        <v>91.62027</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B50" t="n">
+        <v>90.20999999999999</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46287.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>117.60899</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46287.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>110.58695</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46287.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46287.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>99.01000000000001</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46287.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>99.01000000000001</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46287.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46287.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>90.70661</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46287.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>78.13097</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46287.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>92.53837</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46287.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>95.70035</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46287.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>90.20999999999999</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46287.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>93.37031</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46287.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>98.30658</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46287.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46287.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>57.39007</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46287.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>42.8001</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46287.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>46.76851</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46287.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46287.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>42.80005</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46287.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46287.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46287.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46287.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46287.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46287.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>24.99001</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46287.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>24.99028</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46287.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>33.62732</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46287.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46287.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>27.35533</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46287.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>27.03148</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46287.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>30.50834</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46287.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>36.4635</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46287.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>64.89</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46287.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>94.51672000000001</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46287.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>118.67</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46287.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>119.75405</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46287.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>121.1</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46287.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>121.1</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46287.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>122.15</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46287.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>126.5219</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46287.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>122.15</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46287.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>119</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46287.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>115.40909</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46287.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>112.22809</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46287.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>105.69209</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46287.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>99.01000000000001</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46287.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update latest output (run 678)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,50 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>1221.77516175</v>
+        <v>1223.43174525</v>
       </c>
       <c r="F2" t="n">
-        <v>29.38372202380951</v>
+        <v>29.42356289682539</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46288.04166666666</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46288.20833333334</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="E3" t="n">
+        <v>706.855227</v>
+      </c>
+      <c r="F3" t="n">
+        <v>46.74968432539683</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46288.3125</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46288.60416666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>7</v>
+      </c>
+      <c r="D4" t="n">
+        <v>26.46</v>
+      </c>
+      <c r="E4" t="n">
+        <v>691.3246079999999</v>
+      </c>
+      <c r="F4" t="n">
+        <v>26.12715827664399</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -895,7 +935,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -912,11 +952,11 @@
         <v>46287.375</v>
       </c>
       <c r="B20" t="n">
-        <v>42.54006</v>
+        <v>42.8001</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -933,11 +973,11 @@
         <v>46287.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>42.94</v>
+        <v>42.8001</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +994,11 @@
         <v>46287.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>42.8001</v>
+        <v>42.54</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +1015,11 @@
         <v>46287.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>42.45</v>
+        <v>42.94</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1000,7 +1040,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1021,7 +1061,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1042,7 +1082,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1099,11 @@
         <v>46287.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>24.94</v>
+        <v>24.9399</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1084,7 +1124,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1105,7 +1145,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1162,11 @@
         <v>46287.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>28.80424</v>
+        <v>24.99001</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1183,11 @@
         <v>46287.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>38.72835</v>
+        <v>24.94</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1204,11 @@
         <v>46287.625</v>
       </c>
       <c r="B32" t="n">
-        <v>24.99028</v>
+        <v>34.88763</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1225,11 @@
         <v>46287.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>24.99028</v>
+        <v>34.04463</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1246,11 @@
         <v>46287.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>36.8271</v>
+        <v>36.22451</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1267,11 @@
         <v>46287.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>57.39007</v>
+        <v>64.89</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1288,11 @@
         <v>46287.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>86.31334</v>
+        <v>93.80363</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1309,11 @@
         <v>46287.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>112.53463</v>
+        <v>119.26503</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1330,11 @@
         <v>46287.75</v>
       </c>
       <c r="B38" t="n">
-        <v>113.5</v>
+        <v>112.98</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,7 +1351,7 @@
         <v>46287.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>119</v>
+        <v>112.98</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1332,7 +1372,7 @@
         <v>46287.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>113.94</v>
+        <v>114.44758</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1353,7 +1393,7 @@
         <v>46287.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>119.02</v>
+        <v>117.21324</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1374,7 +1414,7 @@
         <v>46287.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>113.94</v>
+        <v>112.98</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1435,7 @@
         <v>46287.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>122.15</v>
+        <v>119</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1456,7 @@
         <v>46287.875</v>
       </c>
       <c r="B44" t="n">
-        <v>122.15</v>
+        <v>112.98</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1477,7 @@
         <v>46287.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>110.88658</v>
+        <v>113.5</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1498,7 @@
         <v>46287.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>108.36579</v>
+        <v>112.98</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1519,7 @@
         <v>46287.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>98.87715</v>
+        <v>112.98</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1540,7 @@
         <v>46287.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>91.60925</v>
+        <v>94.60368</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,7 +1561,7 @@
         <v>46287.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>92.98258</v>
+        <v>109.1395</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1572,1014 @@
         <v>46287</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B50" t="n">
+        <v>115.86941</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46288.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>96.21796000000001</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46288.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>94.11264</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46288.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>90.97315</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46288.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>90.55</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46288.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>89.95395000000001</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46288.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>90.55</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46288.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>90.55</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46288.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>90.55</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46288.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>87.73998</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46288.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>94.70072999999999</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46288.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>93.32841000000001</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46288.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>117.48099</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46288.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>119.33845</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46288.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>105.86</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46288.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>59.5678</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46288.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>48.99</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46288.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46288.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>24.98988</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46288.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46288.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>53.75441</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46288.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46288.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>58.90381</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46288.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>57.60561</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46288.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>57.60941</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46288.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>36.91948</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46288.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>24.99028</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46288.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>42.8002</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46288.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>61.02</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46288.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46288.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46288.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>42.8001</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46288.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46288.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>64.89</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46288.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>80.09999999999999</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46288.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>102.44534</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46288.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>175.27716</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46288.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>293.0003</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46288.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>268.15399</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46288.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46288.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>298.54</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46288.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>206.81004</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46288.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>138</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46288.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>132.55</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46288.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>119.96963</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46288.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>119</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46288.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>112.08144</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46288.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>118.67</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 599)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,42 +470,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46286</v>
+        <v>46287.04166666666</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46286.66666666666</v>
+        <v>46287.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D2" t="n">
-        <v>60.48</v>
+        <v>56.7</v>
       </c>
       <c r="E2" t="n">
-        <v>1685.5022145</v>
+        <v>1965.702687</v>
       </c>
       <c r="F2" t="n">
-        <v>27.86875354662699</v>
+        <v>34.66847772486773</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46287.16666666666</v>
+        <v>46287.95833333334</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46287.66666666666</v>
+        <v>46288.14583333334</v>
       </c>
       <c r="C3" t="n">
-        <v>12</v>
+        <v>4.5</v>
       </c>
       <c r="D3" t="n">
-        <v>45.36</v>
+        <v>17.01</v>
       </c>
       <c r="E3" t="n">
-        <v>1377.40986825</v>
+        <v>789.0634830000001</v>
       </c>
       <c r="F3" t="n">
-        <v>30.36617875330687</v>
+        <v>46.3882118165785</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46288.3125</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46288.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>32.13</v>
+      </c>
+      <c r="E4" t="n">
+        <v>810.0719932500001</v>
+      </c>
+      <c r="F4" t="n">
+        <v>25.21232471988796</v>
       </c>
     </row>
   </sheetData>
@@ -551,10 +571,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="B2" t="n">
-        <v>84.56471000000001</v>
+        <v>119.01</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -562,20 +582,20 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46286.02083333334</v>
+        <v>46287.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>83.98999999999999</v>
+        <v>117.64099</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -583,20 +603,20 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46286.04166666666</v>
+        <v>46287.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>83.98999999999999</v>
+        <v>100.04672</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -604,7 +624,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -614,10 +634,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46286.0625</v>
+        <v>46287.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>83.98999999999999</v>
+        <v>97.63005</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -625,7 +645,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -635,10 +655,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46286.08333333334</v>
+        <v>46287.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>83.98999999999999</v>
+        <v>99.01000000000001</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -646,7 +666,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -656,10 +676,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46286.10416666666</v>
+        <v>46287.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>83.09568</v>
+        <v>97.63005</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -667,7 +687,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -677,10 +697,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46286.125</v>
+        <v>46287.125</v>
       </c>
       <c r="B8" t="n">
-        <v>81.50857000000001</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -688,7 +708,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -698,10 +718,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46286.14583333334</v>
+        <v>46287.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>79.74406999999999</v>
+        <v>94.17734</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -709,7 +729,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -719,7 +739,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46286.16666666666</v>
+        <v>46287.16666666666</v>
       </c>
       <c r="B10" t="n">
         <v>83.98999999999999</v>
@@ -730,7 +750,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -740,10 +760,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46286.1875</v>
+        <v>46287.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>79.94935</v>
+        <v>91.82937</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -751,7 +771,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -761,10 +781,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46286.20833333334</v>
+        <v>46287.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>81.29104</v>
+        <v>91.13996</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -772,7 +792,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -782,10 +802,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46286.22916666666</v>
+        <v>46287.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>83.98999999999999</v>
+        <v>90.33924</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -793,7 +813,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -803,10 +823,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46286.25</v>
+        <v>46287.25</v>
       </c>
       <c r="B14" t="n">
-        <v>85.76063000000001</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -814,7 +834,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -824,10 +844,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46286.27083333334</v>
+        <v>46287.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>90</v>
+        <v>97.63005</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -835,7 +855,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -845,10 +865,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46286.29166666666</v>
+        <v>46287.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>51.08089</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -856,7 +876,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -866,10 +886,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46286.3125</v>
+        <v>46287.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>28.88316</v>
+        <v>57.39007</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -877,7 +897,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -887,10 +907,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46286.33333333334</v>
+        <v>46287.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>52.21</v>
+        <v>42.8001</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -898,7 +918,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -908,10 +928,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46286.35416666666</v>
+        <v>46287.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>10.64282</v>
+        <v>52.9</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -919,7 +939,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -929,10 +949,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46286.375</v>
+        <v>46287.375</v>
       </c>
       <c r="B20" t="n">
-        <v>7.6648</v>
+        <v>42.8001</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -940,7 +960,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -950,10 +970,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46286.39583333334</v>
+        <v>46287.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>2.12</v>
+        <v>42.8001</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -961,7 +981,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -971,10 +991,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46286.41666666666</v>
+        <v>46287.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>11.5</v>
+        <v>42.54</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -982,7 +1002,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -992,10 +1012,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46286.4375</v>
+        <v>46287.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>23.14512</v>
+        <v>42.94</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1003,7 +1023,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1013,10 +1033,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46286.45833333334</v>
+        <v>46287.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>22.24446</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1024,7 +1044,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1034,10 +1054,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46286.47916666666</v>
+        <v>46287.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>41.32391</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1045,7 +1065,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1055,10 +1075,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46286.5</v>
+        <v>46287.5</v>
       </c>
       <c r="B26" t="n">
-        <v>52.21</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1066,7 +1086,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1076,10 +1096,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46286.52083333334</v>
+        <v>46287.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>31.77163</v>
+        <v>24.9399</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1087,7 +1107,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1097,10 +1117,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46286.54166666666</v>
+        <v>46287.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>29</v>
+        <v>52.21</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1108,7 +1128,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1118,10 +1138,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46286.5625</v>
+        <v>46287.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>29</v>
+        <v>52.21</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1129,7 +1149,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1139,10 +1159,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46286.58333333334</v>
+        <v>46287.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>14.57416</v>
+        <v>24.99001</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1150,7 +1170,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1160,10 +1180,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46286.60416666666</v>
+        <v>46287.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>42.94</v>
+        <v>24.94</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1171,7 +1191,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1181,10 +1201,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46286.625</v>
+        <v>46287.625</v>
       </c>
       <c r="B32" t="n">
-        <v>53.41132</v>
+        <v>34.88763</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1192,7 +1212,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1202,10 +1222,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46286.64583333334</v>
+        <v>46287.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>55.1439</v>
+        <v>34.04463</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1213,7 +1233,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1223,10 +1243,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46286.66666666666</v>
+        <v>46287.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>50.31708</v>
+        <v>36.22451</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1234,7 +1254,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1244,10 +1264,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46286.6875</v>
+        <v>46287.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>75.10842</v>
+        <v>64.89</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1255,7 +1275,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1265,10 +1285,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46286.70833333334</v>
+        <v>46287.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>83.98999999999999</v>
+        <v>93.80363</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1276,7 +1296,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1286,10 +1306,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46286.72916666666</v>
+        <v>46287.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>99.96858</v>
+        <v>119.26503</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1297,7 +1317,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1307,10 +1327,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46286.75</v>
+        <v>46287.75</v>
       </c>
       <c r="B38" t="n">
-        <v>932.72699</v>
+        <v>121.1</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1318,7 +1338,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1328,10 +1348,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46286.77083333334</v>
+        <v>46287.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>20373.7864</v>
+        <v>118.67</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1339,7 +1359,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1349,10 +1369,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46286.79166666666</v>
+        <v>46287.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>20263.70201</v>
+        <v>118.16262</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1360,7 +1380,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1370,10 +1390,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46286.8125</v>
+        <v>46287.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>480.2463</v>
+        <v>123.84237</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1381,7 +1401,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1391,10 +1411,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46286.83333333334</v>
+        <v>46287.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>494.13317</v>
+        <v>126.01537</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1402,7 +1422,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1412,10 +1432,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46286.85416666666</v>
+        <v>46287.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>989.63057</v>
+        <v>125.06157</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1423,7 +1443,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1433,10 +1453,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46286.875</v>
+        <v>46287.875</v>
       </c>
       <c r="B44" t="n">
-        <v>512.80454</v>
+        <v>119</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1444,7 +1464,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1454,10 +1474,10 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46286.89583333334</v>
+        <v>46287.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>213.39429</v>
+        <v>113.14689</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1465,7 +1485,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1475,10 +1495,10 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46286.91666666666</v>
+        <v>46287.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>120.49362</v>
+        <v>105.39817</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1486,7 +1506,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1496,18 +1516,18 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46286.9375</v>
+        <v>46287.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>164.99097</v>
+        <v>109.54189</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>forecast</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1517,31 +1537,31 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46286.95833333334</v>
+        <v>46287.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>119.25421</v>
+        <v>94.55646</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>forecast</t>
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46286.97916666666</v>
+        <v>46287.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>91.62027</v>
+        <v>90.77976</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1549,20 +1569,20 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B50" t="n">
-        <v>90.20999999999999</v>
+        <v>94.37232</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1570,20 +1590,20 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46287.02083333334</v>
+        <v>46288.02083333334</v>
       </c>
       <c r="B51" t="n">
-        <v>117.60899</v>
+        <v>96.0993</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1591,20 +1611,20 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46287.04166666666</v>
+        <v>46288.04166666666</v>
       </c>
       <c r="B52" t="n">
-        <v>110.58695</v>
+        <v>90</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1612,20 +1632,20 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46287.0625</v>
+        <v>46288.0625</v>
       </c>
       <c r="B53" t="n">
-        <v>96.98999999999999</v>
+        <v>88.97776</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1633,20 +1653,20 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46287.08333333334</v>
+        <v>46288.08333333334</v>
       </c>
       <c r="B54" t="n">
-        <v>99.01000000000001</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1654,20 +1674,20 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46287.10416666666</v>
+        <v>46288.10416666666</v>
       </c>
       <c r="B55" t="n">
-        <v>99.01000000000001</v>
+        <v>84.25865</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1675,20 +1695,20 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46287.125</v>
+        <v>46288.125</v>
       </c>
       <c r="B56" t="n">
-        <v>96.98999999999999</v>
+        <v>85.46163</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1696,20 +1716,20 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46287.14583333334</v>
+        <v>46288.14583333334</v>
       </c>
       <c r="B57" t="n">
-        <v>90.70661</v>
+        <v>85.97253000000001</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1717,7 +1737,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1727,10 +1747,10 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46287.16666666666</v>
+        <v>46288.16666666666</v>
       </c>
       <c r="B58" t="n">
-        <v>78.13097</v>
+        <v>88.85151999999999</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1738,20 +1758,20 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46287.1875</v>
+        <v>46288.1875</v>
       </c>
       <c r="B59" t="n">
-        <v>92.53837</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1759,20 +1779,20 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46287.20833333334</v>
+        <v>46288.20833333334</v>
       </c>
       <c r="B60" t="n">
-        <v>95.70035</v>
+        <v>92.81086999999999</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1780,20 +1800,20 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46287.22916666666</v>
+        <v>46288.22916666666</v>
       </c>
       <c r="B61" t="n">
-        <v>90.20999999999999</v>
+        <v>94.86404</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1801,20 +1821,20 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46287.25</v>
+        <v>46288.25</v>
       </c>
       <c r="B62" t="n">
-        <v>93.37031</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1822,20 +1842,20 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46287.27083333334</v>
+        <v>46288.27083333334</v>
       </c>
       <c r="B63" t="n">
-        <v>98.30658</v>
+        <v>114.13865</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1843,20 +1863,20 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46287.29166666666</v>
+        <v>46288.29166666666</v>
       </c>
       <c r="B64" t="n">
-        <v>96.98999999999999</v>
+        <v>102.22245</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1864,20 +1884,20 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46287.3125</v>
+        <v>46288.3125</v>
       </c>
       <c r="B65" t="n">
-        <v>57.39007</v>
+        <v>59.56589</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1885,7 +1905,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1895,10 +1915,10 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46287.33333333334</v>
+        <v>46288.33333333334</v>
       </c>
       <c r="B66" t="n">
-        <v>42.8001</v>
+        <v>68.02</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1906,7 +1926,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1916,10 +1936,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46287.35416666666</v>
+        <v>46288.35416666666</v>
       </c>
       <c r="B67" t="n">
-        <v>46.76851</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1927,7 +1947,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1937,10 +1957,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46287.375</v>
+        <v>46288.375</v>
       </c>
       <c r="B68" t="n">
-        <v>52.9</v>
+        <v>53.97352</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1948,7 +1968,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1958,10 +1978,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46287.39583333334</v>
+        <v>46288.39583333334</v>
       </c>
       <c r="B69" t="n">
-        <v>42.80005</v>
+        <v>59.30543</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1969,7 +1989,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1979,10 +1999,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46287.41666666666</v>
+        <v>46288.41666666666</v>
       </c>
       <c r="B70" t="n">
-        <v>42.54</v>
+        <v>46.45</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -1990,7 +2010,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2000,10 +2020,10 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46287.4375</v>
+        <v>46288.4375</v>
       </c>
       <c r="B71" t="n">
-        <v>42.94</v>
+        <v>54.48116</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2011,7 +2031,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2021,10 +2041,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46287.45833333334</v>
+        <v>46288.45833333334</v>
       </c>
       <c r="B72" t="n">
-        <v>76.09999999999999</v>
+        <v>54.03275</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2032,7 +2052,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2042,10 +2062,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46287.47916666666</v>
+        <v>46288.47916666666</v>
       </c>
       <c r="B73" t="n">
-        <v>76.09999999999999</v>
+        <v>58.91508</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2053,7 +2073,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2063,10 +2083,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46287.5</v>
+        <v>46288.5</v>
       </c>
       <c r="B74" t="n">
-        <v>76.09999999999999</v>
+        <v>61.02</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2074,7 +2094,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2084,10 +2104,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46287.52083333334</v>
+        <v>46288.52083333334</v>
       </c>
       <c r="B75" t="n">
-        <v>24.99001</v>
+        <v>24.98996</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2095,7 +2115,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2105,10 +2125,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46287.54166666666</v>
+        <v>46288.54166666666</v>
       </c>
       <c r="B76" t="n">
-        <v>24.99028</v>
+        <v>24.98998</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2116,7 +2136,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2126,10 +2146,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46287.5625</v>
+        <v>46288.5625</v>
       </c>
       <c r="B77" t="n">
-        <v>33.62732</v>
+        <v>24.99028</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2137,7 +2157,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2147,10 +2167,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46287.58333333334</v>
+        <v>46288.58333333334</v>
       </c>
       <c r="B78" t="n">
-        <v>42.54</v>
+        <v>24.99028</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2158,7 +2178,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2168,10 +2188,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46287.60416666666</v>
+        <v>46288.60416666666</v>
       </c>
       <c r="B79" t="n">
-        <v>27.35533</v>
+        <v>40.82082</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2179,7 +2199,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2189,10 +2209,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46287.625</v>
+        <v>46288.625</v>
       </c>
       <c r="B80" t="n">
-        <v>27.03148</v>
+        <v>55.39782</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2200,7 +2220,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2210,10 +2230,10 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46287.64583333334</v>
+        <v>46288.64583333334</v>
       </c>
       <c r="B81" t="n">
-        <v>30.50834</v>
+        <v>42.8001</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2221,7 +2241,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2231,10 +2251,10 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46287.66666666666</v>
+        <v>46288.66666666666</v>
       </c>
       <c r="B82" t="n">
-        <v>36.4635</v>
+        <v>42.54</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2242,7 +2262,7 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2252,10 +2272,10 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46287.6875</v>
+        <v>46288.6875</v>
       </c>
       <c r="B83" t="n">
-        <v>64.89</v>
+        <v>75.9601</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2263,7 +2283,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2273,10 +2293,10 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46287.70833333334</v>
+        <v>46288.70833333334</v>
       </c>
       <c r="B84" t="n">
-        <v>94.51672000000001</v>
+        <v>83.58322</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2284,7 +2304,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2294,10 +2314,10 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46287.72916666666</v>
+        <v>46288.72916666666</v>
       </c>
       <c r="B85" t="n">
-        <v>118.67</v>
+        <v>96.27352999999999</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2305,7 +2325,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2315,10 +2335,10 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>46287.75</v>
+        <v>46288.75</v>
       </c>
       <c r="B86" t="n">
-        <v>119.75405</v>
+        <v>119</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2326,7 +2346,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2336,10 +2356,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>46287.77083333334</v>
+        <v>46288.77083333334</v>
       </c>
       <c r="B87" t="n">
-        <v>121.1</v>
+        <v>169.5</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2347,7 +2367,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2357,10 +2377,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>46287.79166666666</v>
+        <v>46288.79166666666</v>
       </c>
       <c r="B88" t="n">
-        <v>121.1</v>
+        <v>128.53172</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2368,7 +2388,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2378,10 +2398,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>46287.8125</v>
+        <v>46288.8125</v>
       </c>
       <c r="B89" t="n">
-        <v>122.15</v>
+        <v>138</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2389,7 +2409,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2399,10 +2419,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>46287.83333333334</v>
+        <v>46288.83333333334</v>
       </c>
       <c r="B90" t="n">
-        <v>126.5219</v>
+        <v>237.21615</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2410,7 +2430,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2420,10 +2440,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>46287.85416666666</v>
+        <v>46288.85416666666</v>
       </c>
       <c r="B91" t="n">
-        <v>122.15</v>
+        <v>195.3306</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2431,7 +2451,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2441,10 +2461,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46287.875</v>
+        <v>46288.875</v>
       </c>
       <c r="B92" t="n">
-        <v>119</v>
+        <v>126.03078</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2452,7 +2472,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2462,10 +2482,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>46287.89583333334</v>
+        <v>46288.89583333334</v>
       </c>
       <c r="B93" t="n">
-        <v>115.40909</v>
+        <v>132.55</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2473,7 +2493,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2483,10 +2503,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>46287.91666666666</v>
+        <v>46288.91666666666</v>
       </c>
       <c r="B94" t="n">
-        <v>112.22809</v>
+        <v>119</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2494,7 +2514,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2504,10 +2524,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>46287.9375</v>
+        <v>46288.9375</v>
       </c>
       <c r="B95" t="n">
-        <v>105.69209</v>
+        <v>112.83579</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2515,7 +2535,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2525,10 +2545,10 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>46287.95833333334</v>
+        <v>46288.95833333334</v>
       </c>
       <c r="B96" t="n">
-        <v>99.01000000000001</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2536,7 +2556,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2546,10 +2566,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>46287.97916666666</v>
+        <v>46288.97916666666</v>
       </c>
       <c r="B97" t="n">
-        <v>96.98999999999999</v>
+        <v>118.67</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2557,7 +2577,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 680)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -470,42 +470,42 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46288.0625</v>
+        <v>46288.20833333334</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46288.22916666666</v>
+        <v>46288.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D2" t="n">
-        <v>15.12</v>
+        <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>710.623836</v>
+        <v>1358.8042845</v>
       </c>
       <c r="F2" t="n">
-        <v>46.99893095238095</v>
+        <v>32.67927572150073</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46288.375</v>
+        <v>46289.20833333334</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46288.66666666666</v>
+        <v>46289.66666666666</v>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D3" t="n">
-        <v>26.46</v>
+        <v>41.58</v>
       </c>
       <c r="E3" t="n">
-        <v>793.4548440000001</v>
+        <v>1014.76497525</v>
       </c>
       <c r="F3" t="n">
-        <v>29.98695555555556</v>
+        <v>24.40512205988457</v>
       </c>
     </row>
   </sheetData>
@@ -519,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -629,7 +629,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -713,7 +713,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -734,7 +734,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -890,11 +890,11 @@
         <v>46288.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>89.84075</v>
+        <v>46.45</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -902,7 +902,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -911,11 +911,11 @@
         <v>46288.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>84.79000000000001</v>
+        <v>46.45</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -923,7 +923,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -932,11 +932,11 @@
         <v>46288.375</v>
       </c>
       <c r="B20" t="n">
-        <v>61.02</v>
+        <v>46.45</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -953,11 +953,11 @@
         <v>46288.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>40.60566</v>
+        <v>53.74529</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -974,11 +974,11 @@
         <v>46288.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>76.09999999999999</v>
+        <v>57.26658</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -995,11 +995,11 @@
         <v>46288.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>76.09999999999999</v>
+        <v>54.27301</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1016,11 +1016,11 @@
         <v>46288.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>65.98999999999999</v>
+        <v>58.51351</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1037,11 +1037,11 @@
         <v>46288.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>76.09999999999999</v>
+        <v>57.06375</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1058,11 +1058,11 @@
         <v>46288.5</v>
       </c>
       <c r="B26" t="n">
-        <v>76.15000000000001</v>
+        <v>65.98999999999999</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1079,11 +1079,11 @@
         <v>46288.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>57.00854</v>
+        <v>52.21</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1100,11 +1100,11 @@
         <v>46288.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>42.8001</v>
+        <v>52.21</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1121,11 +1121,11 @@
         <v>46288.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>42.8001</v>
+        <v>53.25197</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1142,11 +1142,11 @@
         <v>46288.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>55.79388</v>
+        <v>42.8001</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1163,11 +1163,11 @@
         <v>46288.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>48.19187</v>
+        <v>42.8001</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1205,11 +1205,11 @@
         <v>46288.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>52.33959</v>
+        <v>31.1521</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1226,11 +1226,11 @@
         <v>46288.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>65.98999999999999</v>
+        <v>42.54035</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1247,11 +1247,11 @@
         <v>46288.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>83.98999999999999</v>
+        <v>75.46811</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1268,11 +1268,11 @@
         <v>46288.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>96.11775</v>
+        <v>86.63203</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1289,11 +1289,11 @@
         <v>46288.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>118.67</v>
+        <v>101.8087</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1310,11 +1310,11 @@
         <v>46288.75</v>
       </c>
       <c r="B38" t="n">
-        <v>129.9292</v>
+        <v>142.9</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1331,7 +1331,7 @@
         <v>46288.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>136.91367</v>
+        <v>122.15</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1352,7 +1352,7 @@
         <v>46288.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>169.5</v>
+        <v>125.43001</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
         <v>46288.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>325.5672</v>
+        <v>131.47583</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
         <v>46288.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>260.54578</v>
+        <v>132.55</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1415,7 +1415,7 @@
         <v>46288.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>132.55</v>
+        <v>123.32414</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1436,7 +1436,7 @@
         <v>46288.875</v>
       </c>
       <c r="B44" t="n">
-        <v>124.28557</v>
+        <v>131.58042</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1457,7 +1457,7 @@
         <v>46288.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>212.52137</v>
+        <v>122.15</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1478,7 +1478,7 @@
         <v>46288.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>218.1353</v>
+        <v>119</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
         <v>46288.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>118.67</v>
+        <v>114.95</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1520,7 +1520,7 @@
         <v>46288.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>97.63005</v>
+        <v>106.32954</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1541,7 +1541,7 @@
         <v>46288.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>106.36483</v>
+        <v>119</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1552,6 +1552,1014 @@
         <v>46288</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B50" t="n">
+        <v>110.60748</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46289.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>119</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46289.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>119.22687</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46289.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>119</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46289.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46289.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>97.26810999999999</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46289.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>98.50716</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46289.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>93.03565999999999</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46289.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>90</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46289.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46289.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46289.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>89.18832999999999</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46289.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>89.62293</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46289.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>90.69824</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46289.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>69.18917999999999</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46289.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>46.45</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46289.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>42.8001</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46289.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>39.38617</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46289.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>43.86204</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46289.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46289.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>24.37921</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46289.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>24.99028</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46289.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>39.72748</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46289.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>42.8001</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46289.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>24.99028</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46289.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>24.98999</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46289.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>24.99059</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46289.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46289.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>41.58129</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46289.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>28.77873</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46289.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>39.2682</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46289.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>38.33145</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46289.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46289.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>84.79000000000001</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46289.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>90.20999999999999</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46289.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>121.1</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46289.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>132.11418</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46289.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46289.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46289.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>297.99</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46289.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46289.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>263.66748</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46289.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>179.77796</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46289.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>140.85903</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46289.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>121.01</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46289.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>121.01</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46289.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>113.19181</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46289.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>107.6583</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 600)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,62 +470,42 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46287.04166666666</v>
+        <v>46288</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46287.66666666666</v>
+        <v>46288.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D2" t="n">
-        <v>56.7</v>
+        <v>60.48</v>
       </c>
       <c r="E2" t="n">
-        <v>1965.702687</v>
+        <v>2301.004592249999</v>
       </c>
       <c r="F2" t="n">
-        <v>34.66847772486773</v>
+        <v>38.04571085069443</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46287.95833333334</v>
+        <v>46289.16666666666</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46288.14583333334</v>
+        <v>46289.66666666666</v>
       </c>
       <c r="C3" t="n">
-        <v>4.5</v>
+        <v>12</v>
       </c>
       <c r="D3" t="n">
-        <v>17.01</v>
+        <v>45.36</v>
       </c>
       <c r="E3" t="n">
-        <v>789.0634830000001</v>
+        <v>1323.6406755</v>
       </c>
       <c r="F3" t="n">
-        <v>46.3882118165785</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>46288.3125</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>46288.66666666666</v>
-      </c>
-      <c r="C4" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="D4" t="n">
-        <v>32.13</v>
-      </c>
-      <c r="E4" t="n">
-        <v>810.0719932500001</v>
-      </c>
-      <c r="F4" t="n">
-        <v>25.21232471988796</v>
+        <v>29.18079090608466</v>
       </c>
     </row>
   </sheetData>
@@ -571,10 +551,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="B2" t="n">
-        <v>119.01</v>
+        <v>116.66394</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -582,20 +562,20 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46287.02083333334</v>
+        <v>46288.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>117.64099</v>
+        <v>119</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -603,20 +583,20 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46287.04166666666</v>
+        <v>46288.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>100.04672</v>
+        <v>95.84378</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -624,7 +604,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -634,10 +614,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46287.0625</v>
+        <v>46288.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>97.63005</v>
+        <v>95.34954999999999</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -645,7 +625,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -655,10 +635,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46287.08333333334</v>
+        <v>46288.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>99.01000000000001</v>
+        <v>91.05071</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -666,7 +646,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -676,10 +656,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46287.10416666666</v>
+        <v>46288.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>97.63005</v>
+        <v>88.18908</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -687,7 +667,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -697,10 +677,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46287.125</v>
+        <v>46288.125</v>
       </c>
       <c r="B8" t="n">
-        <v>96.98999999999999</v>
+        <v>90.26223</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -708,7 +688,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -718,10 +698,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46287.14583333334</v>
+        <v>46288.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>94.17734</v>
+        <v>90</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -729,7 +709,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -739,10 +719,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46287.16666666666</v>
+        <v>46288.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>83.98999999999999</v>
+        <v>90</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -750,7 +730,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -760,10 +740,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46287.1875</v>
+        <v>46288.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>91.82937</v>
+        <v>90</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -771,7 +751,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -781,10 +761,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46287.20833333334</v>
+        <v>46288.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>91.13996</v>
+        <v>93.99339000000001</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -792,7 +772,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -802,10 +782,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46287.22916666666</v>
+        <v>46288.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>90.33924</v>
+        <v>103.75652</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -813,7 +793,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -823,10 +803,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46287.25</v>
+        <v>46288.25</v>
       </c>
       <c r="B14" t="n">
-        <v>90.20999999999999</v>
+        <v>110.91931</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -834,7 +814,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -844,10 +824,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46287.27083333334</v>
+        <v>46288.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>97.63005</v>
+        <v>116.47844</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -855,7 +835,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -865,10 +845,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46287.29166666666</v>
+        <v>46288.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>84.79000000000001</v>
+        <v>107.09515</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -876,7 +856,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -886,10 +866,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46287.3125</v>
+        <v>46288.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>57.39007</v>
+        <v>57.9761</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -897,7 +877,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -907,10 +887,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46287.33333333334</v>
+        <v>46288.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>42.8001</v>
+        <v>46.45</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,7 +898,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -928,10 +908,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46287.35416666666</v>
+        <v>46288.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>52.9</v>
+        <v>46.45</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -939,7 +919,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -949,10 +929,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46287.375</v>
+        <v>46288.375</v>
       </c>
       <c r="B20" t="n">
-        <v>42.8001</v>
+        <v>46.45</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -960,7 +940,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -970,10 +950,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46287.39583333334</v>
+        <v>46288.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>42.8001</v>
+        <v>53.74529</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -981,7 +961,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -991,10 +971,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46287.41666666666</v>
+        <v>46288.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>42.54</v>
+        <v>57.26658</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1002,7 +982,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1012,10 +992,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46287.4375</v>
+        <v>46288.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>42.94</v>
+        <v>54.27301</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1023,7 +1003,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1033,10 +1013,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46287.45833333334</v>
+        <v>46288.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>76.09999999999999</v>
+        <v>58.51351</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1044,7 +1024,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1054,10 +1034,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46287.47916666666</v>
+        <v>46288.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>76.09999999999999</v>
+        <v>57.06375</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1065,7 +1045,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1075,10 +1055,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46287.5</v>
+        <v>46288.5</v>
       </c>
       <c r="B26" t="n">
-        <v>76.09999999999999</v>
+        <v>65.98999999999999</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1086,7 +1066,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1096,10 +1076,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46287.52083333334</v>
+        <v>46288.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>24.9399</v>
+        <v>52.21</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1107,7 +1087,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1117,7 +1097,7 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46287.54166666666</v>
+        <v>46288.54166666666</v>
       </c>
       <c r="B28" t="n">
         <v>52.21</v>
@@ -1128,7 +1108,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1138,10 +1118,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46287.5625</v>
+        <v>46288.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>52.21</v>
+        <v>53.25197</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1149,7 +1129,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1159,10 +1139,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46287.58333333334</v>
+        <v>46288.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>24.99001</v>
+        <v>42.8001</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1170,7 +1150,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1180,10 +1160,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46287.60416666666</v>
+        <v>46288.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>24.94</v>
+        <v>42.8001</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1191,7 +1171,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1201,10 +1181,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46287.625</v>
+        <v>46288.625</v>
       </c>
       <c r="B32" t="n">
-        <v>34.88763</v>
+        <v>42.8001</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1212,7 +1192,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1222,10 +1202,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46287.64583333334</v>
+        <v>46288.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>34.04463</v>
+        <v>31.1521</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1233,7 +1213,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1243,10 +1223,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46287.66666666666</v>
+        <v>46288.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>36.22451</v>
+        <v>42.54035</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1254,7 +1234,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1264,10 +1244,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46287.6875</v>
+        <v>46288.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>64.89</v>
+        <v>75.46811</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1275,7 +1255,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1285,10 +1265,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46287.70833333334</v>
+        <v>46288.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>93.80363</v>
+        <v>86.63203</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1296,7 +1276,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1306,10 +1286,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46287.72916666666</v>
+        <v>46288.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>119.26503</v>
+        <v>101.8087</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1317,7 +1297,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1327,10 +1307,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46287.75</v>
+        <v>46288.75</v>
       </c>
       <c r="B38" t="n">
-        <v>121.1</v>
+        <v>142.9</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1338,7 +1318,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1348,10 +1328,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46287.77083333334</v>
+        <v>46288.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>118.67</v>
+        <v>279.08519</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1359,7 +1339,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1369,10 +1349,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46287.79166666666</v>
+        <v>46288.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>118.16262</v>
+        <v>169.5</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1380,7 +1360,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1390,10 +1370,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46287.8125</v>
+        <v>46288.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>123.84237</v>
+        <v>126.07284</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1401,7 +1381,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1411,10 +1391,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46287.83333333334</v>
+        <v>46288.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>126.01537</v>
+        <v>161.45096</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1422,7 +1402,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1432,10 +1412,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46287.85416666666</v>
+        <v>46288.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>125.06157</v>
+        <v>192.11469</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1443,7 +1423,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1453,10 +1433,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46287.875</v>
+        <v>46288.875</v>
       </c>
       <c r="B44" t="n">
-        <v>119</v>
+        <v>195.51288</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1464,7 +1444,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1474,10 +1454,10 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46287.89583333334</v>
+        <v>46288.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>113.14689</v>
+        <v>142.9</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1485,7 +1465,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1495,10 +1475,10 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46287.91666666666</v>
+        <v>46288.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>105.39817</v>
+        <v>128.74605</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1506,7 +1486,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1516,10 +1496,10 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46287.9375</v>
+        <v>46288.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>109.54189</v>
+        <v>118.73356</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1527,7 +1507,7 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1537,10 +1517,10 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46287.95833333334</v>
+        <v>46288.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>94.55646</v>
+        <v>119.01</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1548,20 +1528,20 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46287.97916666666</v>
+        <v>46288.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>90.77976</v>
+        <v>119.01</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1569,20 +1549,20 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B50" t="n">
-        <v>94.37232</v>
+        <v>107.2743</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1590,20 +1570,20 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46288.02083333334</v>
+        <v>46289.02083333334</v>
       </c>
       <c r="B51" t="n">
-        <v>96.0993</v>
+        <v>119.01</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1611,20 +1591,20 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46288.04166666666</v>
+        <v>46289.04166666666</v>
       </c>
       <c r="B52" t="n">
-        <v>90</v>
+        <v>98.11595</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1632,20 +1612,20 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46288.0625</v>
+        <v>46289.0625</v>
       </c>
       <c r="B53" t="n">
-        <v>88.97776</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1653,20 +1633,20 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46288.08333333334</v>
+        <v>46289.08333333334</v>
       </c>
       <c r="B54" t="n">
-        <v>84.79000000000001</v>
+        <v>96.01725</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1674,20 +1654,20 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46288.10416666666</v>
+        <v>46289.10416666666</v>
       </c>
       <c r="B55" t="n">
-        <v>84.25865</v>
+        <v>97.63005</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1695,20 +1675,20 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46288.125</v>
+        <v>46289.125</v>
       </c>
       <c r="B56" t="n">
-        <v>85.46163</v>
+        <v>90</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1716,20 +1696,20 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46288.14583333334</v>
+        <v>46289.14583333334</v>
       </c>
       <c r="B57" t="n">
-        <v>85.97253000000001</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1737,7 +1717,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1747,10 +1727,10 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46288.16666666666</v>
+        <v>46289.16666666666</v>
       </c>
       <c r="B58" t="n">
-        <v>88.85151999999999</v>
+        <v>81.35774000000001</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1758,20 +1738,20 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46288.1875</v>
+        <v>46289.1875</v>
       </c>
       <c r="B59" t="n">
-        <v>84.79000000000001</v>
+        <v>76.12672000000001</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1779,20 +1759,20 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46288.20833333334</v>
+        <v>46289.20833333334</v>
       </c>
       <c r="B60" t="n">
-        <v>92.81086999999999</v>
+        <v>77.52597</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1800,20 +1780,20 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46288.22916666666</v>
+        <v>46289.22916666666</v>
       </c>
       <c r="B61" t="n">
-        <v>94.86404</v>
+        <v>86.12323000000001</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1821,20 +1801,20 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46288.25</v>
+        <v>46289.25</v>
       </c>
       <c r="B62" t="n">
-        <v>96.98999999999999</v>
+        <v>86.61931</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1842,20 +1822,20 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46288.27083333334</v>
+        <v>46289.27083333334</v>
       </c>
       <c r="B63" t="n">
-        <v>114.13865</v>
+        <v>93.36319</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1863,20 +1843,20 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46288.29166666666</v>
+        <v>46289.29166666666</v>
       </c>
       <c r="B64" t="n">
-        <v>102.22245</v>
+        <v>61.68887</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1884,20 +1864,20 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46288.3125</v>
+        <v>46289.3125</v>
       </c>
       <c r="B65" t="n">
-        <v>59.56589</v>
+        <v>49.46337</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1905,7 +1885,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1915,10 +1895,10 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46288.33333333334</v>
+        <v>46289.33333333334</v>
       </c>
       <c r="B66" t="n">
-        <v>68.02</v>
+        <v>48.41254</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1926,7 +1906,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1936,10 +1916,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46288.35416666666</v>
+        <v>46289.35416666666</v>
       </c>
       <c r="B67" t="n">
-        <v>76.09999999999999</v>
+        <v>42.80005</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1947,7 +1927,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1957,10 +1937,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46288.375</v>
+        <v>46289.375</v>
       </c>
       <c r="B68" t="n">
-        <v>53.97352</v>
+        <v>52.21</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1968,7 +1948,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1978,10 +1958,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46288.39583333334</v>
+        <v>46289.39583333334</v>
       </c>
       <c r="B69" t="n">
-        <v>59.30543</v>
+        <v>46.45</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1989,7 +1969,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1999,10 +1979,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46288.41666666666</v>
+        <v>46289.41666666666</v>
       </c>
       <c r="B70" t="n">
-        <v>46.45</v>
+        <v>52.21</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -2010,7 +1990,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2020,10 +2000,10 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46288.4375</v>
+        <v>46289.4375</v>
       </c>
       <c r="B71" t="n">
-        <v>54.48116</v>
+        <v>42.54</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2031,7 +2011,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2041,10 +2021,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46288.45833333334</v>
+        <v>46289.45833333334</v>
       </c>
       <c r="B72" t="n">
-        <v>54.03275</v>
+        <v>42.94</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2052,7 +2032,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2062,10 +2042,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46288.47916666666</v>
+        <v>46289.47916666666</v>
       </c>
       <c r="B73" t="n">
-        <v>58.91508</v>
+        <v>42.79992</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2073,7 +2053,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2083,10 +2063,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46288.5</v>
+        <v>46289.5</v>
       </c>
       <c r="B74" t="n">
-        <v>61.02</v>
+        <v>48.61426</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2094,7 +2074,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2104,10 +2084,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46288.52083333334</v>
+        <v>46289.52083333334</v>
       </c>
       <c r="B75" t="n">
-        <v>24.98996</v>
+        <v>54.51345</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2115,7 +2095,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2125,10 +2105,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46288.54166666666</v>
+        <v>46289.54166666666</v>
       </c>
       <c r="B76" t="n">
-        <v>24.98998</v>
+        <v>52.23725</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2136,7 +2116,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2146,10 +2126,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46288.5625</v>
+        <v>46289.5625</v>
       </c>
       <c r="B77" t="n">
-        <v>24.99028</v>
+        <v>52.17102</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2157,7 +2137,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2167,10 +2147,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46288.58333333334</v>
+        <v>46289.58333333334</v>
       </c>
       <c r="B78" t="n">
-        <v>24.99028</v>
+        <v>41.18843</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2178,7 +2158,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2188,10 +2168,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46288.60416666666</v>
+        <v>46289.60416666666</v>
       </c>
       <c r="B79" t="n">
-        <v>40.82082</v>
+        <v>40.88476</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2199,7 +2179,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2209,10 +2189,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46288.625</v>
+        <v>46289.625</v>
       </c>
       <c r="B80" t="n">
-        <v>55.39782</v>
+        <v>42.54</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2220,7 +2200,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2230,7 +2210,7 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46288.64583333334</v>
+        <v>46289.64583333334</v>
       </c>
       <c r="B81" t="n">
         <v>42.8001</v>
@@ -2241,7 +2221,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2251,7 +2231,7 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46288.66666666666</v>
+        <v>46289.66666666666</v>
       </c>
       <c r="B82" t="n">
         <v>42.54</v>
@@ -2262,7 +2242,7 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2272,10 +2252,10 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46288.6875</v>
+        <v>46289.6875</v>
       </c>
       <c r="B83" t="n">
-        <v>75.9601</v>
+        <v>55.13763</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2283,7 +2263,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2293,10 +2273,10 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46288.70833333334</v>
+        <v>46289.70833333334</v>
       </c>
       <c r="B84" t="n">
-        <v>83.58322</v>
+        <v>86.45837</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2304,7 +2284,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2314,10 +2294,10 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46288.72916666666</v>
+        <v>46289.72916666666</v>
       </c>
       <c r="B85" t="n">
-        <v>96.27352999999999</v>
+        <v>114.54</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2325,7 +2305,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2335,10 +2315,10 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>46288.75</v>
+        <v>46289.75</v>
       </c>
       <c r="B86" t="n">
-        <v>119</v>
+        <v>125.86605</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2346,7 +2326,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2356,10 +2336,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>46288.77083333334</v>
+        <v>46289.77083333334</v>
       </c>
       <c r="B87" t="n">
-        <v>169.5</v>
+        <v>142.70401</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2367,7 +2347,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2377,10 +2357,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>46288.79166666666</v>
+        <v>46289.79166666666</v>
       </c>
       <c r="B88" t="n">
-        <v>128.53172</v>
+        <v>144.66048</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2388,7 +2368,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2398,10 +2378,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>46288.8125</v>
+        <v>46289.8125</v>
       </c>
       <c r="B89" t="n">
-        <v>138</v>
+        <v>167.5</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2409,7 +2389,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2419,10 +2399,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>46288.83333333334</v>
+        <v>46289.83333333334</v>
       </c>
       <c r="B90" t="n">
-        <v>237.21615</v>
+        <v>136.21627</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2430,7 +2410,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2440,10 +2420,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>46288.85416666666</v>
+        <v>46289.85416666666</v>
       </c>
       <c r="B91" t="n">
-        <v>195.3306</v>
+        <v>128.44849</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2451,7 +2431,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2461,10 +2441,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46288.875</v>
+        <v>46289.875</v>
       </c>
       <c r="B92" t="n">
-        <v>126.03078</v>
+        <v>125.98584</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2472,7 +2452,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2482,10 +2462,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>46288.89583333334</v>
+        <v>46289.89583333334</v>
       </c>
       <c r="B93" t="n">
-        <v>132.55</v>
+        <v>119.01</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2493,7 +2473,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2503,10 +2483,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>46288.91666666666</v>
+        <v>46289.91666666666</v>
       </c>
       <c r="B94" t="n">
-        <v>119</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2514,7 +2494,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2524,10 +2504,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>46288.9375</v>
+        <v>46289.9375</v>
       </c>
       <c r="B95" t="n">
-        <v>112.83579</v>
+        <v>114.65206</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2535,7 +2515,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2545,7 +2525,7 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>46288.95833333334</v>
+        <v>46289.95833333334</v>
       </c>
       <c r="B96" t="n">
         <v>96.98999999999999</v>
@@ -2556,7 +2536,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2566,10 +2546,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>46288.97916666666</v>
+        <v>46289.97916666666</v>
       </c>
       <c r="B97" t="n">
-        <v>118.67</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2577,7 +2557,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 682)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>945.7283842499999</v>
+        <v>1142.46669225</v>
       </c>
       <c r="F2" t="n">
-        <v>22.74479038600288</v>
+        <v>27.47635142496393</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46290.20833333334</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46290.66666666666</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>774.9811679999999</v>
+      </c>
+      <c r="F3" t="n">
+        <v>18.63831572871573</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -874,7 +894,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -891,11 +911,11 @@
         <v>46289.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>64.53413999999999</v>
+        <v>57.39007</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -912,11 +932,11 @@
         <v>46289.375</v>
       </c>
       <c r="B20" t="n">
-        <v>52.33952</v>
+        <v>51.49746</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -937,7 +957,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +974,11 @@
         <v>46289.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>28.65451</v>
+        <v>42.94</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +995,11 @@
         <v>46289.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>24.86321</v>
+        <v>42.8001</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46289.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>16.46759</v>
+        <v>42.94</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46289.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>25.21079</v>
+        <v>42.8001</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46289.5</v>
       </c>
       <c r="B26" t="n">
-        <v>31.70724</v>
+        <v>42.8001</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46289.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>42.94</v>
+        <v>42.8001</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46289.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>42.8001</v>
+        <v>42.94</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1121,11 @@
         <v>46289.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>25.8107</v>
+        <v>42.8001</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46289.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>2.29932</v>
+        <v>41.78018</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1163,11 @@
         <v>46289.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-3.91594</v>
+        <v>41.14329</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46289.625</v>
       </c>
       <c r="B32" t="n">
-        <v>23.12981</v>
+        <v>42.54</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1205,11 @@
         <v>46289.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>41.08763</v>
+        <v>42.54</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1210,7 +1230,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1247,11 @@
         <v>46289.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>81.64815</v>
+        <v>75.9601</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1268,11 @@
         <v>46289.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>87.71040000000001</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1289,11 @@
         <v>46289.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>108.39304</v>
+        <v>114.54</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1310,11 @@
         <v>46289.75</v>
       </c>
       <c r="B38" t="n">
-        <v>121.1</v>
+        <v>121.01</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,7 +1331,7 @@
         <v>46289.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>135.66112</v>
+        <v>126.80467</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1332,7 +1352,7 @@
         <v>46289.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>125.67343</v>
+        <v>147.1272</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1353,7 +1373,7 @@
         <v>46289.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>121.1</v>
+        <v>137.46051</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1374,7 +1394,7 @@
         <v>46289.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>121.01</v>
+        <v>132.53123</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1415,7 @@
         <v>46289.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>128.41278</v>
+        <v>126.62945</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1436,7 @@
         <v>46289.875</v>
       </c>
       <c r="B44" t="n">
-        <v>121.01</v>
+        <v>121.01002</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46289.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>119.01</v>
+        <v>191.82266</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46289.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>97.48025</v>
+        <v>133.45451</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46289.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>115.22974</v>
+        <v>111.43101</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1520,7 @@
         <v>46289.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>117.29697</v>
+        <v>107.71993</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,7 +1541,7 @@
         <v>46289.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>116.5487</v>
+        <v>98.77572000000001</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46289</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B50" t="n">
+        <v>97.29233000000001</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46290.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>97.17661</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46290.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>93.70126</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46290.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>92.60213</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46290.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46290.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>92.73527</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46290.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46290.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>84.79000000000001</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46290.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>84.79000000000001</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46290.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>96.65284</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46290.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>97.63005</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46290.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>96.04164</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46290.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>97.71729999999999</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46290.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>97.63005</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46290.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>82.69542</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46290.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>64.95</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46290.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>35.0115</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46290.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>15.30906</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46290.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>10.33883</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46290.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>8.73021</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46290.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46290.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46290.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>0.01114</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46290.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>0.01127</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46290.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>9.611050000000001</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46290.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>9.16081</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46290.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>0.01553</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46290.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>0.00932</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46290.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>9.668850000000001</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46290.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>24.99025</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46290.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>42.5402</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46290.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46290.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>42.45</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46290.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>57.64302</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46290.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>80.03727000000001</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46290.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>101.64679</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46290.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>183.29517</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46290.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46290.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46290.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>249.78154</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46290.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>239.96026</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46290.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>226.10574</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46290.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>279.15323</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46290.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>177.97751</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46290.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>173.97094</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46290.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>130.29945</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46290.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>120.80654</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46290.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>121.83916</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 601)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,42 +470,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46288</v>
+        <v>46289.0625</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46288.66666666666</v>
+        <v>46289.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>16</v>
+        <v>14.5</v>
       </c>
       <c r="D2" t="n">
-        <v>60.48</v>
+        <v>54.81</v>
       </c>
       <c r="E2" t="n">
-        <v>2301.004592249999</v>
+        <v>1757.0848425</v>
       </c>
       <c r="F2" t="n">
-        <v>38.04571085069443</v>
+        <v>32.05774206349207</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46289.16666666666</v>
+        <v>46289.9375</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46289.66666666666</v>
+        <v>46290.125</v>
       </c>
       <c r="C3" t="n">
-        <v>12</v>
+        <v>4.5</v>
       </c>
       <c r="D3" t="n">
-        <v>45.36</v>
+        <v>17.01</v>
       </c>
       <c r="E3" t="n">
-        <v>1323.6406755</v>
+        <v>837.436587</v>
       </c>
       <c r="F3" t="n">
-        <v>29.18079090608466</v>
+        <v>49.23201569664904</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46290.29166666666</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46290.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D4" t="n">
+        <v>34.02</v>
+      </c>
+      <c r="E4" t="n">
+        <v>408.1783485</v>
+      </c>
+      <c r="F4" t="n">
+        <v>11.99818778659612</v>
       </c>
     </row>
   </sheetData>
@@ -551,10 +571,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B2" t="n">
-        <v>116.66394</v>
+        <v>119.01</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -562,20 +582,20 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46288.02083333334</v>
+        <v>46289.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>119</v>
+        <v>119.01</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -583,20 +603,20 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46288.04166666666</v>
+        <v>46289.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>95.84378</v>
+        <v>115.73055</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -604,20 +624,20 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46288.0625</v>
+        <v>46289.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>95.34954999999999</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -625,7 +645,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -635,10 +655,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46288.08333333334</v>
+        <v>46289.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>91.05071</v>
+        <v>96.57861</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -646,7 +666,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -656,10 +676,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46288.10416666666</v>
+        <v>46289.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>88.18908</v>
+        <v>97.63005</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -667,7 +687,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -677,10 +697,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46288.125</v>
+        <v>46289.125</v>
       </c>
       <c r="B8" t="n">
-        <v>90.26223</v>
+        <v>90</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -688,7 +708,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -698,10 +718,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46288.14583333334</v>
+        <v>46289.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>90</v>
+        <v>88.88</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -709,7 +729,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -719,10 +739,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46288.16666666666</v>
+        <v>46289.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>90</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -730,7 +750,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -740,10 +760,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46288.1875</v>
+        <v>46289.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>90</v>
+        <v>76.30893</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -751,7 +771,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -761,10 +781,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46288.20833333334</v>
+        <v>46289.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>93.99339000000001</v>
+        <v>77.51611</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -772,7 +792,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -782,10 +802,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46288.22916666666</v>
+        <v>46289.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>103.75652</v>
+        <v>87.11633999999999</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -793,7 +813,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -803,10 +823,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46288.25</v>
+        <v>46289.25</v>
       </c>
       <c r="B14" t="n">
-        <v>110.91931</v>
+        <v>87.16424000000001</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -814,7 +834,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -824,10 +844,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46288.27083333334</v>
+        <v>46289.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>116.47844</v>
+        <v>95.33</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -835,7 +855,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -845,10 +865,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46288.29166666666</v>
+        <v>46289.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>107.09515</v>
+        <v>51.62299</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -856,7 +876,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -866,10 +886,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46288.3125</v>
+        <v>46289.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>57.9761</v>
+        <v>49.45946</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -877,7 +897,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -887,10 +907,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46288.33333333334</v>
+        <v>46289.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>46.45</v>
+        <v>57.39007</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -898,7 +918,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -908,10 +928,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46288.35416666666</v>
+        <v>46289.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>46.45</v>
+        <v>57.39007</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -919,7 +939,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -929,10 +949,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46288.375</v>
+        <v>46289.375</v>
       </c>
       <c r="B20" t="n">
-        <v>46.45</v>
+        <v>51.49746</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -940,7 +960,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -950,10 +970,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46288.39583333334</v>
+        <v>46289.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>53.74529</v>
+        <v>46.45</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -961,7 +981,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -971,10 +991,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46288.41666666666</v>
+        <v>46289.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>57.26658</v>
+        <v>42.94</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -982,7 +1002,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -992,10 +1012,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46288.4375</v>
+        <v>46289.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>54.27301</v>
+        <v>42.8001</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1003,7 +1023,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1013,10 +1033,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46288.45833333334</v>
+        <v>46289.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>58.51351</v>
+        <v>42.94</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1024,7 +1044,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1034,10 +1054,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46288.47916666666</v>
+        <v>46289.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>57.06375</v>
+        <v>42.8001</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1045,7 +1065,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1055,10 +1075,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46288.5</v>
+        <v>46289.5</v>
       </c>
       <c r="B26" t="n">
-        <v>65.98999999999999</v>
+        <v>42.8001</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1066,7 +1086,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1076,10 +1096,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46288.52083333334</v>
+        <v>46289.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>52.21</v>
+        <v>42.8001</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1087,7 +1107,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1097,10 +1117,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46288.54166666666</v>
+        <v>46289.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>52.21</v>
+        <v>42.94</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1108,7 +1128,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1118,10 +1138,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46288.5625</v>
+        <v>46289.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>53.25197</v>
+        <v>42.8001</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1129,7 +1149,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1139,10 +1159,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46288.58333333334</v>
+        <v>46289.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>42.8001</v>
+        <v>41.78018</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1150,7 +1170,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1160,10 +1180,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46288.60416666666</v>
+        <v>46289.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>42.8001</v>
+        <v>41.14329</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1171,7 +1191,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1181,10 +1201,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46288.625</v>
+        <v>46289.625</v>
       </c>
       <c r="B32" t="n">
-        <v>42.8001</v>
+        <v>42.54</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1192,7 +1212,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1202,10 +1222,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46288.64583333334</v>
+        <v>46289.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>31.1521</v>
+        <v>42.54</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1213,7 +1233,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1223,10 +1243,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46288.66666666666</v>
+        <v>46289.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>42.54035</v>
+        <v>42.54</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1234,7 +1254,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1244,10 +1264,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46288.6875</v>
+        <v>46289.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>75.46811</v>
+        <v>75.9601</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1255,7 +1275,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1265,10 +1285,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46288.70833333334</v>
+        <v>46289.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>86.63203</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1276,7 +1296,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1286,10 +1306,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46288.72916666666</v>
+        <v>46289.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>101.8087</v>
+        <v>114.54</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1297,7 +1317,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1307,10 +1327,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46288.75</v>
+        <v>46289.75</v>
       </c>
       <c r="B38" t="n">
-        <v>142.9</v>
+        <v>128.3889</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1318,7 +1338,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1328,10 +1348,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46288.77083333334</v>
+        <v>46289.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>279.08519</v>
+        <v>135.93959</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1339,7 +1359,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1349,10 +1369,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46288.79166666666</v>
+        <v>46289.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>169.5</v>
+        <v>162.99728</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1360,7 +1380,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1370,10 +1390,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46288.8125</v>
+        <v>46289.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>126.07284</v>
+        <v>148.27538</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1381,7 +1401,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1391,10 +1411,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46288.83333333334</v>
+        <v>46289.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>161.45096</v>
+        <v>137.33935</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1402,7 +1422,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1412,10 +1432,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46288.85416666666</v>
+        <v>46289.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>192.11469</v>
+        <v>129.65</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1423,7 +1443,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1433,10 +1453,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46288.875</v>
+        <v>46289.875</v>
       </c>
       <c r="B44" t="n">
-        <v>195.51288</v>
+        <v>121.01</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1444,7 +1464,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1454,10 +1474,10 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46288.89583333334</v>
+        <v>46289.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>142.9</v>
+        <v>119.01</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1465,7 +1485,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1475,10 +1495,10 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46288.91666666666</v>
+        <v>46289.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>128.74605</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1486,7 +1506,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1496,10 +1516,10 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46288.9375</v>
+        <v>46289.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>118.73356</v>
+        <v>110.98</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1507,20 +1527,20 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46288.95833333334</v>
+        <v>46289.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>119.01</v>
+        <v>110.98</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1528,20 +1548,20 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46288.97916666666</v>
+        <v>46289.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>119.01</v>
+        <v>99.76040999999999</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1549,20 +1569,20 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B50" t="n">
-        <v>107.2743</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1570,20 +1590,20 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46289.02083333334</v>
+        <v>46290.02083333334</v>
       </c>
       <c r="B51" t="n">
-        <v>119.01</v>
+        <v>94.31704999999999</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1591,20 +1611,20 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46289.04166666666</v>
+        <v>46290.04166666666</v>
       </c>
       <c r="B52" t="n">
-        <v>98.11595</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1612,20 +1632,20 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46289.0625</v>
+        <v>46290.0625</v>
       </c>
       <c r="B53" t="n">
-        <v>96.98999999999999</v>
+        <v>88.93362</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1633,20 +1653,20 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46289.08333333334</v>
+        <v>46290.08333333334</v>
       </c>
       <c r="B54" t="n">
-        <v>96.01725</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1654,20 +1674,20 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46289.10416666666</v>
+        <v>46290.10416666666</v>
       </c>
       <c r="B55" t="n">
-        <v>97.63005</v>
+        <v>88.16824</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1675,20 +1695,20 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46289.125</v>
+        <v>46290.125</v>
       </c>
       <c r="B56" t="n">
-        <v>90</v>
+        <v>88.88</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1696,7 +1716,7 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1706,10 +1726,10 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46289.14583333334</v>
+        <v>46290.14583333334</v>
       </c>
       <c r="B57" t="n">
-        <v>83.98999999999999</v>
+        <v>88.88</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1717,7 +1737,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1727,10 +1747,10 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46289.16666666666</v>
+        <v>46290.16666666666</v>
       </c>
       <c r="B58" t="n">
-        <v>81.35774000000001</v>
+        <v>88.41632</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1738,20 +1758,20 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46289.1875</v>
+        <v>46290.1875</v>
       </c>
       <c r="B59" t="n">
-        <v>76.12672000000001</v>
+        <v>97.63005</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1759,20 +1779,20 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46289.20833333334</v>
+        <v>46290.20833333334</v>
       </c>
       <c r="B60" t="n">
-        <v>77.52597</v>
+        <v>97.63005</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1780,20 +1800,20 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46289.22916666666</v>
+        <v>46290.22916666666</v>
       </c>
       <c r="B61" t="n">
-        <v>86.12323000000001</v>
+        <v>96.87844</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1801,20 +1821,20 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46289.25</v>
+        <v>46290.25</v>
       </c>
       <c r="B62" t="n">
-        <v>86.61931</v>
+        <v>97.37456</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1822,20 +1842,20 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46289.27083333334</v>
+        <v>46290.27083333334</v>
       </c>
       <c r="B63" t="n">
-        <v>93.36319</v>
+        <v>97.31990999999999</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1843,20 +1863,20 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46289.29166666666</v>
+        <v>46290.29166666666</v>
       </c>
       <c r="B64" t="n">
-        <v>61.68887</v>
+        <v>82.08586</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1864,7 +1884,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1874,10 +1894,10 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46289.3125</v>
+        <v>46290.3125</v>
       </c>
       <c r="B65" t="n">
-        <v>49.46337</v>
+        <v>64.95</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1885,7 +1905,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1895,10 +1915,10 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46289.33333333334</v>
+        <v>46290.33333333334</v>
       </c>
       <c r="B66" t="n">
-        <v>48.41254</v>
+        <v>42.08</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1906,7 +1926,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1916,10 +1936,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46289.35416666666</v>
+        <v>46290.35416666666</v>
       </c>
       <c r="B67" t="n">
-        <v>42.80005</v>
+        <v>24.98984</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1927,7 +1947,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1937,10 +1957,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46289.375</v>
+        <v>46290.375</v>
       </c>
       <c r="B68" t="n">
-        <v>52.21</v>
+        <v>9.64687</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1948,7 +1968,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1958,10 +1978,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46289.39583333334</v>
+        <v>46290.39583333334</v>
       </c>
       <c r="B69" t="n">
-        <v>46.45</v>
+        <v>0.01093</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1969,7 +1989,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1979,10 +1999,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46289.41666666666</v>
+        <v>46290.41666666666</v>
       </c>
       <c r="B70" t="n">
-        <v>52.21</v>
+        <v>0.0003</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -1990,7 +2010,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2000,10 +2020,10 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46289.4375</v>
+        <v>46290.4375</v>
       </c>
       <c r="B71" t="n">
-        <v>42.54</v>
+        <v>7.57418</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2011,7 +2031,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2021,10 +2041,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46289.45833333334</v>
+        <v>46290.45833333334</v>
       </c>
       <c r="B72" t="n">
-        <v>42.94</v>
+        <v>12.27254</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2032,7 +2052,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2042,10 +2062,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46289.47916666666</v>
+        <v>46290.47916666666</v>
       </c>
       <c r="B73" t="n">
-        <v>42.79992</v>
+        <v>42.94</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2053,7 +2073,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2063,10 +2083,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46289.5</v>
+        <v>46290.5</v>
       </c>
       <c r="B74" t="n">
-        <v>48.61426</v>
+        <v>42.8</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2074,7 +2094,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2084,10 +2104,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46289.52083333334</v>
+        <v>46290.52083333334</v>
       </c>
       <c r="B75" t="n">
-        <v>54.51345</v>
+        <v>25.1</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2095,7 +2115,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2105,10 +2125,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46289.54166666666</v>
+        <v>46290.54166666666</v>
       </c>
       <c r="B76" t="n">
-        <v>52.23725</v>
+        <v>2e-05</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2116,7 +2136,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2126,10 +2146,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46289.5625</v>
+        <v>46290.5625</v>
       </c>
       <c r="B77" t="n">
-        <v>52.17102</v>
+        <v>4.76513</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2137,7 +2157,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2147,10 +2167,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46289.58333333334</v>
+        <v>46290.58333333334</v>
       </c>
       <c r="B78" t="n">
-        <v>41.18843</v>
+        <v>9.438789999999999</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2158,7 +2178,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2168,10 +2188,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46289.60416666666</v>
+        <v>46290.60416666666</v>
       </c>
       <c r="B79" t="n">
-        <v>40.88476</v>
+        <v>0.01</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2179,7 +2199,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2189,10 +2209,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46289.625</v>
+        <v>46290.625</v>
       </c>
       <c r="B80" t="n">
-        <v>42.54</v>
+        <v>24.99</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2200,7 +2220,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2210,10 +2230,10 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46289.64583333334</v>
+        <v>46290.64583333334</v>
       </c>
       <c r="B81" t="n">
-        <v>42.8001</v>
+        <v>24.99</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2221,7 +2241,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2231,10 +2251,10 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46289.66666666666</v>
+        <v>46290.66666666666</v>
       </c>
       <c r="B82" t="n">
-        <v>42.54</v>
+        <v>26.75263</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2242,7 +2262,7 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2252,10 +2272,10 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46289.6875</v>
+        <v>46290.6875</v>
       </c>
       <c r="B83" t="n">
-        <v>55.13763</v>
+        <v>55.955</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2263,7 +2283,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2273,10 +2293,10 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46289.70833333334</v>
+        <v>46290.70833333334</v>
       </c>
       <c r="B84" t="n">
-        <v>86.45837</v>
+        <v>80.2428</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2284,7 +2304,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2294,10 +2314,10 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46289.72916666666</v>
+        <v>46290.72916666666</v>
       </c>
       <c r="B85" t="n">
-        <v>114.54</v>
+        <v>99.21146</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2305,7 +2325,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2315,10 +2335,10 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>46289.75</v>
+        <v>46290.75</v>
       </c>
       <c r="B86" t="n">
-        <v>125.86605</v>
+        <v>121.40389</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2326,7 +2346,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2336,10 +2356,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>46289.77083333334</v>
+        <v>46290.77083333334</v>
       </c>
       <c r="B87" t="n">
-        <v>142.70401</v>
+        <v>124.83318</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2347,7 +2367,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2357,10 +2377,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>46289.79166666666</v>
+        <v>46290.79166666666</v>
       </c>
       <c r="B88" t="n">
-        <v>144.66048</v>
+        <v>134.71319</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2368,7 +2388,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2378,10 +2398,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>46289.8125</v>
+        <v>46290.8125</v>
       </c>
       <c r="B89" t="n">
-        <v>167.5</v>
+        <v>132.3809</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2389,7 +2409,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2399,10 +2419,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>46289.83333333334</v>
+        <v>46290.83333333334</v>
       </c>
       <c r="B90" t="n">
-        <v>136.21627</v>
+        <v>154.20422</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2410,7 +2430,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2420,10 +2440,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>46289.85416666666</v>
+        <v>46290.85416666666</v>
       </c>
       <c r="B91" t="n">
-        <v>128.44849</v>
+        <v>148.54429</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2431,7 +2451,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2441,10 +2461,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46289.875</v>
+        <v>46290.875</v>
       </c>
       <c r="B92" t="n">
-        <v>125.98584</v>
+        <v>154.37021</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2452,7 +2472,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2462,10 +2482,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>46289.89583333334</v>
+        <v>46290.89583333334</v>
       </c>
       <c r="B93" t="n">
-        <v>119.01</v>
+        <v>116.90411</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2473,7 +2493,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2483,10 +2503,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>46289.91666666666</v>
+        <v>46290.91666666666</v>
       </c>
       <c r="B94" t="n">
-        <v>96.98999999999999</v>
+        <v>129.65</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2494,7 +2514,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2504,10 +2524,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>46289.9375</v>
+        <v>46290.9375</v>
       </c>
       <c r="B95" t="n">
-        <v>114.65206</v>
+        <v>130.99994</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2515,7 +2535,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2525,10 +2545,10 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>46289.95833333334</v>
+        <v>46290.95833333334</v>
       </c>
       <c r="B96" t="n">
-        <v>96.98999999999999</v>
+        <v>120.70416</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2536,7 +2556,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2546,10 +2566,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>46289.97916666666</v>
+        <v>46290.97916666666</v>
       </c>
       <c r="B97" t="n">
-        <v>96.98999999999999</v>
+        <v>122.30466</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2557,7 +2577,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 684)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>1076.246496</v>
+        <v>792.4369634999996</v>
       </c>
       <c r="F2" t="n">
-        <v>25.88375411255411</v>
+        <v>19.05812803030302</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46291.27083333334</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46291.72916666666</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>190.83387375</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.589559253246753</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -870,11 +890,11 @@
         <v>46290.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>57.39003</v>
+        <v>35.22344</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -891,11 +911,11 @@
         <v>46290.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>43.55663</v>
+        <v>28.82675</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -912,11 +932,11 @@
         <v>46290.375</v>
       </c>
       <c r="B20" t="n">
-        <v>24.98988</v>
+        <v>27.72294</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -933,11 +953,11 @@
         <v>46290.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>0.79818</v>
+        <v>24.99</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +974,11 @@
         <v>46290.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>42.94</v>
+        <v>19.55703</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +995,11 @@
         <v>46290.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>0.01135</v>
+        <v>7.62205</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46290.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>42.08</v>
+        <v>9.032690000000001</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46290.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>24.99</v>
+        <v>0</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46290.5</v>
       </c>
       <c r="B26" t="n">
-        <v>52.21</v>
+        <v>0.05189</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46290.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>51.66844</v>
+        <v>10.12993</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46290.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>42.08</v>
+        <v>0.02296</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1121,11 @@
         <v>46290.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>9.2585</v>
+        <v>9.26285</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46290.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>43.11622</v>
+        <v>24.99</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1163,11 @@
         <v>46290.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>42.8</v>
+        <v>24.99</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46290.625</v>
       </c>
       <c r="B32" t="n">
-        <v>42.8</v>
+        <v>24.99</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1205,11 @@
         <v>46290.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>42.8</v>
+        <v>24.99</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1226,11 @@
         <v>46290.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>43.78834</v>
+        <v>26.57993</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1247,11 @@
         <v>46290.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>81.38357000000001</v>
+        <v>57.32074</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1268,11 @@
         <v>46290.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>85.1133</v>
+        <v>80.11099</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1289,11 @@
         <v>46290.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>103.21513</v>
+        <v>100.39281</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1310,11 @@
         <v>46290.75</v>
       </c>
       <c r="B38" t="n">
-        <v>118.92945</v>
+        <v>125.53176</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,7 +1331,7 @@
         <v>46290.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>126.74784</v>
+        <v>93.01000000000001</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1332,7 +1352,7 @@
         <v>46290.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>126.25544</v>
+        <v>101.67455</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1353,7 +1373,7 @@
         <v>46290.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>126.20632</v>
+        <v>97.86469</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1374,7 +1394,7 @@
         <v>46290.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>124.04274</v>
+        <v>96.59514</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1415,7 @@
         <v>46290.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>128.39285</v>
+        <v>95.67353</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1436,7 @@
         <v>46290.875</v>
       </c>
       <c r="B44" t="n">
-        <v>128.5147</v>
+        <v>101.44843</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46290.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>119.92221</v>
+        <v>94.6022</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46290.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>117.0873</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46290.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>118.86297</v>
+        <v>90.24948999999999</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1520,7 @@
         <v>46290.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>110.98</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,7 +1541,7 @@
         <v>46290.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>122.48478</v>
+        <v>99.10978</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46290</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B50" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46291.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46291.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46291.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>88.66996</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46291.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>88.52603000000001</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46291.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46291.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46291.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46291.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>81.77992</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46291.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46291.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46291.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46291.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46291.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>74.74754</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46291.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46291.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>4e-05</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46291.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>3e-05</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46291.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>0</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46291.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>-3.42456</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46291.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>-5.25579</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46291.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>-5.6722</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46291.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-6.53231</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46291.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-7.37712</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46291.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>-4.49525</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46291.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>-4.51247</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46291.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>-3.46115</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46291.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>-6.36048</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46291.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-6.76007</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46291.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-3.45989</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46291.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-4.35881</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46291.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>-5.16907</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46291.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>-5.41037</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46291.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>24.99028</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46291.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>47.49814</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46291.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>78.20056</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46291.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46291.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>86.60538</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46291.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>110.98</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46291.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>110.96504</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46291.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>110.98</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46291.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>88.84</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46291.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>88.84</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46291.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>88.84</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46291.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>88.84</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46291.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>88.84</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46291.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46291.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46291.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 602)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,62 +470,42 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46289.0625</v>
+        <v>46290</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46289.66666666666</v>
+        <v>46290.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>14.5</v>
+        <v>16</v>
       </c>
       <c r="D2" t="n">
-        <v>54.81</v>
+        <v>60.48</v>
       </c>
       <c r="E2" t="n">
-        <v>1757.0848425</v>
+        <v>1699.46982075</v>
       </c>
       <c r="F2" t="n">
-        <v>32.05774206349207</v>
+        <v>28.0996994171627</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46289.9375</v>
+        <v>46291.25</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46290.125</v>
+        <v>46291.75</v>
       </c>
       <c r="C3" t="n">
-        <v>4.5</v>
+        <v>12</v>
       </c>
       <c r="D3" t="n">
-        <v>17.01</v>
+        <v>45.36</v>
       </c>
       <c r="E3" t="n">
-        <v>837.436587</v>
+        <v>349.0669065</v>
       </c>
       <c r="F3" t="n">
-        <v>49.23201569664904</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>46290.29166666666</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>46290.66666666666</v>
-      </c>
-      <c r="C4" t="n">
-        <v>9</v>
-      </c>
-      <c r="D4" t="n">
-        <v>34.02</v>
-      </c>
-      <c r="E4" t="n">
-        <v>408.1783485</v>
-      </c>
-      <c r="F4" t="n">
-        <v>11.99818778659612</v>
+        <v>7.695478538359787</v>
       </c>
     </row>
   </sheetData>
@@ -571,10 +551,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B2" t="n">
-        <v>119.01</v>
+        <v>110.98</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -582,20 +562,20 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46289.02083333334</v>
+        <v>46290.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>119.01</v>
+        <v>98.11246</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -603,20 +583,20 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46289.04166666666</v>
+        <v>46290.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>115.73055</v>
+        <v>90</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -624,20 +604,20 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46289.0625</v>
+        <v>46290.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>96.98999999999999</v>
+        <v>88.93985000000001</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -645,7 +625,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -655,10 +635,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46289.08333333334</v>
+        <v>46290.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>96.57861</v>
+        <v>88.88</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -666,7 +646,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -676,10 +656,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46289.10416666666</v>
+        <v>46290.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>97.63005</v>
+        <v>88.88</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -687,7 +667,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -697,10 +677,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46289.125</v>
+        <v>46290.125</v>
       </c>
       <c r="B8" t="n">
-        <v>90</v>
+        <v>88.95610000000001</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -708,7 +688,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -718,10 +698,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46289.14583333334</v>
+        <v>46290.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>88.88</v>
+        <v>89.03165</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -729,7 +709,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -739,10 +719,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46289.16666666666</v>
+        <v>46290.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>83.98999999999999</v>
+        <v>88.88</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -750,7 +730,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -760,10 +740,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46289.1875</v>
+        <v>46290.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>76.30893</v>
+        <v>97.63005</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -771,7 +751,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -781,10 +761,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46289.20833333334</v>
+        <v>46290.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>77.51611</v>
+        <v>97.63005</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -792,7 +772,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -802,10 +782,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46289.22916666666</v>
+        <v>46290.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>87.11633999999999</v>
+        <v>96.86727</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -813,7 +793,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -823,10 +803,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46289.25</v>
+        <v>46290.25</v>
       </c>
       <c r="B14" t="n">
-        <v>87.16424000000001</v>
+        <v>97.36445999999999</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -834,7 +814,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -844,10 +824,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46289.27083333334</v>
+        <v>46290.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>95.33</v>
+        <v>96.69481</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -855,7 +835,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -865,10 +845,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46289.29166666666</v>
+        <v>46290.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>51.62299</v>
+        <v>82.68539</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -876,7 +856,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -886,10 +866,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46289.3125</v>
+        <v>46290.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>49.45946</v>
+        <v>69.11135</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -897,7 +877,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -907,10 +887,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46289.33333333334</v>
+        <v>46290.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>57.39007</v>
+        <v>35.22344</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -918,7 +898,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -928,10 +908,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46289.35416666666</v>
+        <v>46290.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>57.39007</v>
+        <v>28.82675</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -939,7 +919,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -949,10 +929,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46289.375</v>
+        <v>46290.375</v>
       </c>
       <c r="B20" t="n">
-        <v>51.49746</v>
+        <v>27.72294</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -960,7 +940,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -970,10 +950,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46289.39583333334</v>
+        <v>46290.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>46.45</v>
+        <v>24.99</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -981,7 +961,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -991,10 +971,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46289.41666666666</v>
+        <v>46290.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>42.94</v>
+        <v>19.55703</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1002,7 +982,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1012,10 +992,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46289.4375</v>
+        <v>46290.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>42.8001</v>
+        <v>7.62205</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1023,7 +1003,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1033,10 +1013,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46289.45833333334</v>
+        <v>46290.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>42.94</v>
+        <v>9.032690000000001</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1044,7 +1024,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1054,10 +1034,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46289.47916666666</v>
+        <v>46290.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>42.8001</v>
+        <v>0</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1065,7 +1045,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1075,10 +1055,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46289.5</v>
+        <v>46290.5</v>
       </c>
       <c r="B26" t="n">
-        <v>42.8001</v>
+        <v>0.05189</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1086,7 +1066,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1096,10 +1076,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46289.52083333334</v>
+        <v>46290.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>42.8001</v>
+        <v>10.12993</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1107,7 +1087,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1117,10 +1097,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46289.54166666666</v>
+        <v>46290.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>42.94</v>
+        <v>0.02296</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1128,7 +1108,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1138,10 +1118,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46289.5625</v>
+        <v>46290.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>42.8001</v>
+        <v>9.26285</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1149,7 +1129,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1159,10 +1139,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46289.58333333334</v>
+        <v>46290.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>41.78018</v>
+        <v>24.99</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1170,7 +1150,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1180,10 +1160,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46289.60416666666</v>
+        <v>46290.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>41.14329</v>
+        <v>24.99</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1191,7 +1171,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1201,10 +1181,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46289.625</v>
+        <v>46290.625</v>
       </c>
       <c r="B32" t="n">
-        <v>42.54</v>
+        <v>24.99</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1212,7 +1192,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1222,10 +1202,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46289.64583333334</v>
+        <v>46290.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>42.54</v>
+        <v>24.99</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1233,7 +1213,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1243,10 +1223,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46289.66666666666</v>
+        <v>46290.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>42.54</v>
+        <v>26.57993</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1254,7 +1234,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1264,10 +1244,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46289.6875</v>
+        <v>46290.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>75.9601</v>
+        <v>57.32074</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1275,7 +1255,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1285,10 +1265,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46289.70833333334</v>
+        <v>46290.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>84.79000000000001</v>
+        <v>80.11099</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1296,7 +1276,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1306,10 +1286,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46289.72916666666</v>
+        <v>46290.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>114.54</v>
+        <v>100.39281</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1317,7 +1297,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1327,10 +1307,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46289.75</v>
+        <v>46290.75</v>
       </c>
       <c r="B38" t="n">
-        <v>128.3889</v>
+        <v>125.53176</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1338,7 +1318,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1348,10 +1328,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46289.77083333334</v>
+        <v>46290.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>135.93959</v>
+        <v>125.96583</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1359,7 +1339,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1369,10 +1349,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46289.79166666666</v>
+        <v>46290.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>162.99728</v>
+        <v>144.67161</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1380,7 +1360,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1390,10 +1370,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46289.8125</v>
+        <v>46290.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>148.27538</v>
+        <v>171.80608</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1401,7 +1381,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1411,10 +1391,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46289.83333333334</v>
+        <v>46290.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>137.33935</v>
+        <v>141.80387</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1422,7 +1402,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1432,10 +1412,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46289.85416666666</v>
+        <v>46290.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>129.65</v>
+        <v>140.80199</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1443,7 +1423,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1453,10 +1433,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46289.875</v>
+        <v>46290.875</v>
       </c>
       <c r="B44" t="n">
-        <v>121.01</v>
+        <v>115.35266</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1464,7 +1444,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1474,10 +1454,10 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46289.89583333334</v>
+        <v>46290.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>119.01</v>
+        <v>116.89871</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1485,7 +1465,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1495,10 +1475,10 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46289.91666666666</v>
+        <v>46290.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>96.98999999999999</v>
+        <v>172.6106</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1506,7 +1486,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1516,10 +1496,10 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46289.9375</v>
+        <v>46290.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>110.98</v>
+        <v>95.42327</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1527,20 +1507,20 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46289.95833333334</v>
+        <v>46290.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>110.98</v>
+        <v>94.84641999999999</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1548,20 +1528,20 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46289.97916666666</v>
+        <v>46290.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>99.76040999999999</v>
+        <v>84.78010999999999</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1569,20 +1549,20 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B50" t="n">
-        <v>96.98999999999999</v>
+        <v>85.37081999999999</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1590,20 +1570,20 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46290.02083333334</v>
+        <v>46291.02083333334</v>
       </c>
       <c r="B51" t="n">
-        <v>94.31704999999999</v>
+        <v>91.92282</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1611,20 +1591,20 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46290.04166666666</v>
+        <v>46291.04166666666</v>
       </c>
       <c r="B52" t="n">
-        <v>84.79000000000001</v>
+        <v>90.03279000000001</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1632,20 +1612,20 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46290.0625</v>
+        <v>46291.0625</v>
       </c>
       <c r="B53" t="n">
-        <v>88.93362</v>
+        <v>87.0455</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1653,20 +1633,20 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46290.08333333334</v>
+        <v>46291.08333333334</v>
       </c>
       <c r="B54" t="n">
-        <v>83.98999999999999</v>
+        <v>88.88</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1674,20 +1654,20 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46290.10416666666</v>
+        <v>46291.10416666666</v>
       </c>
       <c r="B55" t="n">
-        <v>88.16824</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1695,20 +1675,20 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46290.125</v>
+        <v>46291.125</v>
       </c>
       <c r="B56" t="n">
-        <v>88.88</v>
+        <v>85.187</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1716,7 +1696,7 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1726,10 +1706,10 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46290.14583333334</v>
+        <v>46291.14583333334</v>
       </c>
       <c r="B57" t="n">
-        <v>88.88</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1737,7 +1717,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1747,10 +1727,10 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46290.16666666666</v>
+        <v>46291.16666666666</v>
       </c>
       <c r="B58" t="n">
-        <v>88.41632</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1758,7 +1738,7 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1768,10 +1748,10 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46290.1875</v>
+        <v>46291.1875</v>
       </c>
       <c r="B59" t="n">
-        <v>97.63005</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1779,7 +1759,7 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1789,10 +1769,10 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46290.20833333334</v>
+        <v>46291.20833333334</v>
       </c>
       <c r="B60" t="n">
-        <v>97.63005</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1800,7 +1780,7 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1810,10 +1790,10 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46290.22916666666</v>
+        <v>46291.22916666666</v>
       </c>
       <c r="B61" t="n">
-        <v>96.87844</v>
+        <v>86.74215</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1821,7 +1801,7 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1831,10 +1811,10 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46290.25</v>
+        <v>46291.25</v>
       </c>
       <c r="B62" t="n">
-        <v>97.37456</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1842,20 +1822,20 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46290.27083333334</v>
+        <v>46291.27083333334</v>
       </c>
       <c r="B63" t="n">
-        <v>97.31990999999999</v>
+        <v>75.95028000000001</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1863,20 +1843,20 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46290.29166666666</v>
+        <v>46291.29166666666</v>
       </c>
       <c r="B64" t="n">
-        <v>82.08586</v>
+        <v>42.54</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1884,7 +1864,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1894,10 +1874,10 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46290.3125</v>
+        <v>46291.3125</v>
       </c>
       <c r="B65" t="n">
-        <v>64.95</v>
+        <v>4e-05</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1905,7 +1885,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1915,10 +1895,10 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46290.33333333334</v>
+        <v>46291.33333333334</v>
       </c>
       <c r="B66" t="n">
-        <v>42.08</v>
+        <v>3e-05</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1926,7 +1906,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1936,10 +1916,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46290.35416666666</v>
+        <v>46291.35416666666</v>
       </c>
       <c r="B67" t="n">
-        <v>24.98984</v>
+        <v>-2.91428</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1947,7 +1927,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1957,10 +1937,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46290.375</v>
+        <v>46291.375</v>
       </c>
       <c r="B68" t="n">
-        <v>9.64687</v>
+        <v>0.03157</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1968,7 +1948,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1978,10 +1958,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46290.39583333334</v>
+        <v>46291.39583333334</v>
       </c>
       <c r="B69" t="n">
-        <v>0.01093</v>
+        <v>2e-05</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1989,7 +1969,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1999,10 +1979,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46290.41666666666</v>
+        <v>46291.41666666666</v>
       </c>
       <c r="B70" t="n">
-        <v>0.0003</v>
+        <v>-3.13729</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -2010,7 +1990,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2020,10 +2000,10 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46290.4375</v>
+        <v>46291.4375</v>
       </c>
       <c r="B71" t="n">
-        <v>7.57418</v>
+        <v>-6.24403</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2031,7 +2011,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2041,10 +2021,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46290.45833333334</v>
+        <v>46291.45833333334</v>
       </c>
       <c r="B72" t="n">
-        <v>12.27254</v>
+        <v>-6.17363</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2052,7 +2032,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2062,10 +2042,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46290.47916666666</v>
+        <v>46291.47916666666</v>
       </c>
       <c r="B73" t="n">
-        <v>42.94</v>
+        <v>-6.25197</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2073,7 +2053,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2083,10 +2063,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46290.5</v>
+        <v>46291.5</v>
       </c>
       <c r="B74" t="n">
-        <v>42.8</v>
+        <v>-5.50874</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2094,7 +2074,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2104,10 +2084,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46290.52083333334</v>
+        <v>46291.52083333334</v>
       </c>
       <c r="B75" t="n">
-        <v>25.1</v>
+        <v>-6.51</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2115,7 +2095,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2125,10 +2105,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46290.54166666666</v>
+        <v>46291.54166666666</v>
       </c>
       <c r="B76" t="n">
-        <v>2e-05</v>
+        <v>-6.80768</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2136,7 +2116,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2146,10 +2126,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46290.5625</v>
+        <v>46291.5625</v>
       </c>
       <c r="B77" t="n">
-        <v>4.76513</v>
+        <v>-6.19048</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2157,7 +2137,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2167,10 +2147,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46290.58333333334</v>
+        <v>46291.58333333334</v>
       </c>
       <c r="B78" t="n">
-        <v>9.438789999999999</v>
+        <v>-6.51</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2178,7 +2158,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2188,10 +2168,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46290.60416666666</v>
+        <v>46291.60416666666</v>
       </c>
       <c r="B79" t="n">
-        <v>0.01</v>
+        <v>-6.07227</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2199,7 +2179,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2209,10 +2189,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46290.625</v>
+        <v>46291.625</v>
       </c>
       <c r="B80" t="n">
-        <v>24.99</v>
+        <v>-5.68434</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2220,7 +2200,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2230,10 +2210,10 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46290.64583333334</v>
+        <v>46291.64583333334</v>
       </c>
       <c r="B81" t="n">
-        <v>24.99</v>
+        <v>-5.52205</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2241,7 +2221,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2251,10 +2231,10 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46290.66666666666</v>
+        <v>46291.66666666666</v>
       </c>
       <c r="B82" t="n">
-        <v>26.75263</v>
+        <v>7.96956</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2262,20 +2242,20 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46290.6875</v>
+        <v>46291.6875</v>
       </c>
       <c r="B83" t="n">
-        <v>55.955</v>
+        <v>55.22206</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2283,20 +2263,20 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46290.70833333334</v>
+        <v>46291.70833333334</v>
       </c>
       <c r="B84" t="n">
-        <v>80.2428</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2304,20 +2284,20 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46290.72916666666</v>
+        <v>46291.72916666666</v>
       </c>
       <c r="B85" t="n">
-        <v>99.21146</v>
+        <v>85.74054</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2325,20 +2305,20 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>46290.75</v>
+        <v>46291.75</v>
       </c>
       <c r="B86" t="n">
-        <v>121.40389</v>
+        <v>109.64095</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2346,7 +2326,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2356,10 +2336,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>46290.77083333334</v>
+        <v>46291.77083333334</v>
       </c>
       <c r="B87" t="n">
-        <v>124.83318</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2367,7 +2347,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2377,10 +2357,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>46290.79166666666</v>
+        <v>46291.79166666666</v>
       </c>
       <c r="B88" t="n">
-        <v>134.71319</v>
+        <v>90.01000000000001</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2388,7 +2368,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2398,10 +2378,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>46290.8125</v>
+        <v>46291.8125</v>
       </c>
       <c r="B89" t="n">
-        <v>132.3809</v>
+        <v>96.99005</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2409,7 +2389,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2419,10 +2399,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>46290.83333333334</v>
+        <v>46291.83333333334</v>
       </c>
       <c r="B90" t="n">
-        <v>154.20422</v>
+        <v>88.84</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2430,7 +2410,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2440,10 +2420,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>46290.85416666666</v>
+        <v>46291.85416666666</v>
       </c>
       <c r="B91" t="n">
-        <v>148.54429</v>
+        <v>85.07687</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2451,7 +2431,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2461,10 +2441,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46290.875</v>
+        <v>46291.875</v>
       </c>
       <c r="B92" t="n">
-        <v>154.37021</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2472,7 +2452,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2482,10 +2462,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>46290.89583333334</v>
+        <v>46291.89583333334</v>
       </c>
       <c r="B93" t="n">
-        <v>116.90411</v>
+        <v>88.84</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2493,7 +2473,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2503,10 +2483,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>46290.91666666666</v>
+        <v>46291.91666666666</v>
       </c>
       <c r="B94" t="n">
-        <v>129.65</v>
+        <v>88.84</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2514,7 +2494,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2524,10 +2504,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>46290.9375</v>
+        <v>46291.9375</v>
       </c>
       <c r="B95" t="n">
-        <v>130.99994</v>
+        <v>87.53769</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2535,7 +2515,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2545,10 +2525,10 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>46290.95833333334</v>
+        <v>46291.95833333334</v>
       </c>
       <c r="B96" t="n">
-        <v>120.70416</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2556,7 +2536,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2566,10 +2546,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>46290.97916666666</v>
+        <v>46291.97916666666</v>
       </c>
       <c r="B97" t="n">
-        <v>122.30466</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2577,7 +2557,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 686)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>250.2749535</v>
+        <v>197.0537985</v>
       </c>
       <c r="F2" t="n">
-        <v>6.019118650793652</v>
+        <v>4.739148593073593</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46292.29166666666</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46292.75</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>880.87707825</v>
+      </c>
+      <c r="F3" t="n">
+        <v>21.18511491702742</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -870,11 +890,11 @@
         <v>46291.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>25.1</v>
+        <v>-1.26985</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -891,11 +911,11 @@
         <v>46291.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>9.60561</v>
+        <v>-4.6421</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -912,11 +932,11 @@
         <v>46291.375</v>
       </c>
       <c r="B20" t="n">
-        <v>3e-05</v>
+        <v>-5.25879</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -933,11 +953,11 @@
         <v>46291.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>3e-05</v>
+        <v>-0.72396</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +974,11 @@
         <v>46291.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-5.01</v>
+        <v>-3.13724</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +995,11 @@
         <v>46291.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-5.01</v>
+        <v>-1.32866</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46291.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-5.84303</v>
+        <v>-2.96986</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46291.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-6.51</v>
+        <v>-7.48</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46291.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-3.87579</v>
+        <v>-4.48552</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46291.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>0.91</v>
+        <v>-4.14405</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46291.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>0.00983</v>
+        <v>-4.63482</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1121,11 @@
         <v>46291.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>-3.54064</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46291.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>0.009339999999999999</v>
+        <v>0.009639999999999999</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1163,11 @@
         <v>46291.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>0.91</v>
+        <v>-6.08598</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46291.625</v>
       </c>
       <c r="B32" t="n">
-        <v>2.39385</v>
+        <v>-4.49196</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1205,11 @@
         <v>46291.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>-0.40883</v>
+        <v>-5.82547</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1226,11 @@
         <v>46291.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>-3.57558</v>
+        <v>7.96906</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1247,11 @@
         <v>46291.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>49.0622</v>
+        <v>55.22206</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1252,7 +1272,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1289,11 @@
         <v>46291.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>82.45231</v>
+        <v>85.7353</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1310,11 @@
         <v>46291.75</v>
       </c>
       <c r="B38" t="n">
-        <v>89.34569999999999</v>
+        <v>109.97954</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,7 +1331,7 @@
         <v>46291.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>88.86011000000001</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1332,7 +1352,7 @@
         <v>46291.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>88.86011000000001</v>
+        <v>96.37687</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1353,7 +1373,7 @@
         <v>46291.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>89.98305999999999</v>
+        <v>88.86011000000001</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1416,7 +1436,7 @@
         <v>46291.875</v>
       </c>
       <c r="B44" t="n">
-        <v>88.84</v>
+        <v>86.18835</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46291.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>83.98999999999999</v>
+        <v>86.19718</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46291.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>88.84</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46291.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>88.10212</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46291</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B50" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46292.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46292.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>73.96719</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46292.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>76.70283000000001</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46292.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46292.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>77.80079000000001</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46292.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>76.15000000000001</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46292.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>75.96007</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46292.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>75.95028000000001</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46292.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>75.95005</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46292.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>75.95005</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46292.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>75.96007</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46292.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>75.95005</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46292.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>75.68655</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46292.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46292.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>26.05</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46292.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46292.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46292.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>25.35245</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46292.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>26.05</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46292.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>26.05</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46292.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46292.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46292.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46292.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46292.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46292.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46292.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>46.45</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46292.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46292.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46292.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>46.45</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46292.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46292.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46292.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>39.37055</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46292.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>54.65067</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46292.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46292.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>68.72131</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46292.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>89.98218</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46292.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>93.88516</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46292.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>95.20981</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46292.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>95.81755</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46292.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>90</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46292.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>88.84</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46292.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>86.75029000000001</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46292.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46292.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>75.95005</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46292.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>65.51000000000001</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46292.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>65.51000000000001</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 603)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,42 +470,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46290</v>
+        <v>46291.20833333334</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46290.66666666666</v>
+        <v>46291.72916666666</v>
       </c>
       <c r="C2" t="n">
-        <v>16</v>
+        <v>12.5</v>
       </c>
       <c r="D2" t="n">
-        <v>60.48</v>
+        <v>47.25</v>
       </c>
       <c r="E2" t="n">
-        <v>1699.46982075</v>
+        <v>447.5431154999999</v>
       </c>
       <c r="F2" t="n">
-        <v>28.0996994171627</v>
+        <v>9.471811968253967</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46291.25</v>
+        <v>46291.85416666666</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46291.75</v>
+        <v>46292.02083333334</v>
       </c>
       <c r="C3" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>45.36</v>
+        <v>15.12</v>
       </c>
       <c r="E3" t="n">
-        <v>349.0669065</v>
+        <v>628.482972</v>
       </c>
       <c r="F3" t="n">
-        <v>7.695478538359787</v>
+        <v>41.56633412698413</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46292.27083333334</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46292.75</v>
+      </c>
+      <c r="C4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>43.47</v>
+      </c>
+      <c r="E4" t="n">
+        <v>997.25686125</v>
+      </c>
+      <c r="F4" t="n">
+        <v>22.94126664941339</v>
       </c>
     </row>
   </sheetData>
@@ -551,10 +571,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="B2" t="n">
-        <v>110.98</v>
+        <v>86.83904</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -562,20 +582,20 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46290.02083333334</v>
+        <v>46291.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>98.11246</v>
+        <v>96.90159</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -583,20 +603,20 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46290.04166666666</v>
+        <v>46291.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>90</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -604,20 +624,20 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46290.0625</v>
+        <v>46291.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>88.93985000000001</v>
+        <v>90</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -625,17 +645,17 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46290.08333333334</v>
+        <v>46291.08333333334</v>
       </c>
       <c r="B6" t="n">
         <v>88.88</v>
@@ -646,20 +666,20 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46290.10416666666</v>
+        <v>46291.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>88.88</v>
+        <v>87.23359000000001</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -667,20 +687,20 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46290.125</v>
+        <v>46291.125</v>
       </c>
       <c r="B8" t="n">
-        <v>88.95610000000001</v>
+        <v>87.9945</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -688,20 +708,20 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46290.14583333334</v>
+        <v>46291.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>89.03165</v>
+        <v>87.21228000000001</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -709,20 +729,20 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46290.16666666666</v>
+        <v>46291.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>88.88</v>
+        <v>86.19396</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -730,20 +750,20 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46290.1875</v>
+        <v>46291.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>97.63005</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -751,20 +771,20 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46290.20833333334</v>
+        <v>46291.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>97.63005</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -772,7 +792,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -782,10 +802,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46290.22916666666</v>
+        <v>46291.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>96.86727</v>
+        <v>88.13212</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -793,7 +813,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -803,10 +823,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46290.25</v>
+        <v>46291.25</v>
       </c>
       <c r="B14" t="n">
-        <v>97.36445999999999</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -814,7 +834,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -824,10 +844,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46290.27083333334</v>
+        <v>46291.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>96.69481</v>
+        <v>76.02454</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -835,7 +855,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -845,10 +865,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46290.29166666666</v>
+        <v>46291.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>82.68539</v>
+        <v>42.80002</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -856,7 +876,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -866,10 +886,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46290.3125</v>
+        <v>46291.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>69.11135</v>
+        <v>4e-05</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -877,7 +897,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -887,10 +907,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46290.33333333334</v>
+        <v>46291.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>35.22344</v>
+        <v>-1.26985</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -898,7 +918,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -908,10 +928,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46290.35416666666</v>
+        <v>46291.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>28.82675</v>
+        <v>-4.6421</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -919,7 +939,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -929,10 +949,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46290.375</v>
+        <v>46291.375</v>
       </c>
       <c r="B20" t="n">
-        <v>27.72294</v>
+        <v>-5.25879</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -940,7 +960,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -950,10 +970,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46290.39583333334</v>
+        <v>46291.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>24.99</v>
+        <v>-0.72396</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -961,7 +981,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -971,10 +991,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46290.41666666666</v>
+        <v>46291.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>19.55703</v>
+        <v>-3.13724</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -982,7 +1002,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -992,10 +1012,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46290.4375</v>
+        <v>46291.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>7.62205</v>
+        <v>-1.32866</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1003,7 +1023,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1013,10 +1033,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46290.45833333334</v>
+        <v>46291.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>9.032690000000001</v>
+        <v>-2.96986</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1024,7 +1044,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1034,10 +1054,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46290.47916666666</v>
+        <v>46291.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>0</v>
+        <v>-7.48</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1045,7 +1065,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1055,10 +1075,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46290.5</v>
+        <v>46291.5</v>
       </c>
       <c r="B26" t="n">
-        <v>0.05189</v>
+        <v>-4.48552</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1066,7 +1086,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1076,10 +1096,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46290.52083333334</v>
+        <v>46291.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>10.12993</v>
+        <v>-4.14405</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1087,7 +1107,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1097,10 +1117,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46290.54166666666</v>
+        <v>46291.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>0.02296</v>
+        <v>-4.63482</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1108,7 +1128,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1118,10 +1138,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46290.5625</v>
+        <v>46291.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>9.26285</v>
+        <v>-3.54064</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1129,7 +1149,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1139,10 +1159,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46290.58333333334</v>
+        <v>46291.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>24.99</v>
+        <v>0.009639999999999999</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1150,7 +1170,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1160,10 +1180,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46290.60416666666</v>
+        <v>46291.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>24.99</v>
+        <v>-6.08598</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1171,7 +1191,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1181,10 +1201,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46290.625</v>
+        <v>46291.625</v>
       </c>
       <c r="B32" t="n">
-        <v>24.99</v>
+        <v>-4.49196</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1192,7 +1212,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1202,10 +1222,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46290.64583333334</v>
+        <v>46291.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>24.99</v>
+        <v>-5.82547</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1213,7 +1233,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1223,10 +1243,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46290.66666666666</v>
+        <v>46291.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>26.57993</v>
+        <v>7.96906</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1234,20 +1254,20 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46290.6875</v>
+        <v>46291.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>57.32074</v>
+        <v>55.22206</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1255,20 +1275,20 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46290.70833333334</v>
+        <v>46291.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>80.11099</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1276,20 +1296,20 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46290.72916666666</v>
+        <v>46291.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>100.39281</v>
+        <v>85.7353</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1297,7 +1317,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1307,10 +1327,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46290.75</v>
+        <v>46291.75</v>
       </c>
       <c r="B38" t="n">
-        <v>125.53176</v>
+        <v>109.97954</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1318,7 +1338,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1328,10 +1348,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46290.77083333334</v>
+        <v>46291.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>125.96583</v>
+        <v>106.85</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1339,7 +1359,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1349,10 +1369,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46290.79166666666</v>
+        <v>46291.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>144.67161</v>
+        <v>110.63868</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1360,7 +1380,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1370,10 +1390,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46290.8125</v>
+        <v>46291.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>171.80608</v>
+        <v>90.01000000000001</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1381,7 +1401,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1391,10 +1411,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46290.83333333334</v>
+        <v>46291.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>141.80387</v>
+        <v>88.84</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1402,7 +1422,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1412,10 +1432,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46290.85416666666</v>
+        <v>46291.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>140.80199</v>
+        <v>88.84</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1423,20 +1443,20 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46290.875</v>
+        <v>46291.875</v>
       </c>
       <c r="B44" t="n">
-        <v>115.35266</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1444,20 +1464,20 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46290.89583333334</v>
+        <v>46291.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>116.89871</v>
+        <v>81.41273</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1465,41 +1485,41 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46290.91666666666</v>
+        <v>46291.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>172.6106</v>
+        <v>86.88</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>forecast</t>
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46290.9375</v>
+        <v>46291.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>95.42327</v>
+        <v>75.9503</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1507,20 +1527,20 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46290.95833333334</v>
+        <v>46291.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>94.84641999999999</v>
+        <v>75.63461</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1528,20 +1548,20 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46290.97916666666</v>
+        <v>46291.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>84.78010999999999</v>
+        <v>75.94</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1549,20 +1569,20 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="B50" t="n">
-        <v>85.37081999999999</v>
+        <v>75.95028000000001</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1570,20 +1590,20 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46291.02083333334</v>
+        <v>46292.02083333334</v>
       </c>
       <c r="B51" t="n">
-        <v>91.92282</v>
+        <v>88.84</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1591,7 +1611,7 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1601,10 +1621,10 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46291.04166666666</v>
+        <v>46292.04166666666</v>
       </c>
       <c r="B52" t="n">
-        <v>90.03279000000001</v>
+        <v>88.84</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1612,7 +1632,7 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1622,10 +1642,10 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46291.0625</v>
+        <v>46292.0625</v>
       </c>
       <c r="B53" t="n">
-        <v>87.0455</v>
+        <v>72.43926999999999</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1633,7 +1653,7 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1643,10 +1663,10 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46291.08333333334</v>
+        <v>46292.08333333334</v>
       </c>
       <c r="B54" t="n">
-        <v>88.88</v>
+        <v>76.20227</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1654,7 +1674,7 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1664,10 +1684,10 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46291.10416666666</v>
+        <v>46292.10416666666</v>
       </c>
       <c r="B55" t="n">
-        <v>84.79000000000001</v>
+        <v>75.27775</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1675,7 +1695,7 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1685,10 +1705,10 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46291.125</v>
+        <v>46292.125</v>
       </c>
       <c r="B56" t="n">
-        <v>85.187</v>
+        <v>73.87103999999999</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1696,7 +1716,7 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1706,10 +1726,10 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46291.14583333334</v>
+        <v>46292.14583333334</v>
       </c>
       <c r="B57" t="n">
-        <v>84.79000000000001</v>
+        <v>74.82613000000001</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1717,7 +1737,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1727,10 +1747,10 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46291.16666666666</v>
+        <v>46292.16666666666</v>
       </c>
       <c r="B58" t="n">
-        <v>84.79000000000001</v>
+        <v>73.87437</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1738,7 +1758,7 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1748,10 +1768,10 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46291.1875</v>
+        <v>46292.1875</v>
       </c>
       <c r="B59" t="n">
-        <v>84.79000000000001</v>
+        <v>75.96007</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1759,7 +1779,7 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1769,10 +1789,10 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46291.20833333334</v>
+        <v>46292.20833333334</v>
       </c>
       <c r="B60" t="n">
-        <v>83.98999999999999</v>
+        <v>75.96007</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1780,7 +1800,7 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1790,10 +1810,10 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46291.22916666666</v>
+        <v>46292.22916666666</v>
       </c>
       <c r="B61" t="n">
-        <v>86.74215</v>
+        <v>78.94398</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1801,7 +1821,7 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1811,10 +1831,10 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46291.25</v>
+        <v>46292.25</v>
       </c>
       <c r="B62" t="n">
-        <v>83.98999999999999</v>
+        <v>75.9601</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1822,20 +1842,20 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46291.27083333334</v>
+        <v>46292.27083333334</v>
       </c>
       <c r="B63" t="n">
-        <v>75.95028000000001</v>
+        <v>75.24312999999999</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1843,7 +1863,7 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1853,10 +1873,10 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46291.29166666666</v>
+        <v>46292.29166666666</v>
       </c>
       <c r="B64" t="n">
-        <v>42.54</v>
+        <v>57.95275</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1864,7 +1884,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1874,10 +1894,10 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46291.3125</v>
+        <v>46292.3125</v>
       </c>
       <c r="B65" t="n">
-        <v>4e-05</v>
+        <v>52.21</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1885,7 +1905,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1895,10 +1915,10 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46291.33333333334</v>
+        <v>46292.33333333334</v>
       </c>
       <c r="B66" t="n">
-        <v>3e-05</v>
+        <v>26.05</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1906,7 +1926,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1916,10 +1936,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46291.35416666666</v>
+        <v>46292.35416666666</v>
       </c>
       <c r="B67" t="n">
-        <v>-2.91428</v>
+        <v>46.45</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1927,7 +1947,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1937,10 +1957,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46291.375</v>
+        <v>46292.375</v>
       </c>
       <c r="B68" t="n">
-        <v>0.03157</v>
+        <v>28.95</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1948,7 +1968,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1958,10 +1978,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46291.39583333334</v>
+        <v>46292.39583333334</v>
       </c>
       <c r="B69" t="n">
-        <v>2e-05</v>
+        <v>26.05</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1969,7 +1989,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1979,10 +1999,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46291.41666666666</v>
+        <v>46292.41666666666</v>
       </c>
       <c r="B70" t="n">
-        <v>-3.13729</v>
+        <v>26.05</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -1990,7 +2010,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2000,10 +2020,10 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46291.4375</v>
+        <v>46292.4375</v>
       </c>
       <c r="B71" t="n">
-        <v>-6.24403</v>
+        <v>42.54</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2011,7 +2031,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2021,10 +2041,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46291.45833333334</v>
+        <v>46292.45833333334</v>
       </c>
       <c r="B72" t="n">
-        <v>-6.17363</v>
+        <v>42.54</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2032,7 +2052,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2042,10 +2062,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46291.47916666666</v>
+        <v>46292.47916666666</v>
       </c>
       <c r="B73" t="n">
-        <v>-6.25197</v>
+        <v>42.54</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2053,7 +2073,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2063,10 +2083,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46291.5</v>
+        <v>46292.5</v>
       </c>
       <c r="B74" t="n">
-        <v>-5.50874</v>
+        <v>42.54</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2074,7 +2094,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2084,10 +2104,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46291.52083333334</v>
+        <v>46292.52083333334</v>
       </c>
       <c r="B75" t="n">
-        <v>-6.51</v>
+        <v>42.54</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2095,7 +2115,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2105,10 +2125,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46291.54166666666</v>
+        <v>46292.54166666666</v>
       </c>
       <c r="B76" t="n">
-        <v>-6.80768</v>
+        <v>42.54</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2116,7 +2136,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2126,10 +2146,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46291.5625</v>
+        <v>46292.5625</v>
       </c>
       <c r="B77" t="n">
-        <v>-6.19048</v>
+        <v>42.54</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2137,7 +2157,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2147,10 +2167,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46291.58333333334</v>
+        <v>46292.58333333334</v>
       </c>
       <c r="B78" t="n">
-        <v>-6.51</v>
+        <v>46.45</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2158,7 +2178,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2168,10 +2188,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46291.60416666666</v>
+        <v>46292.60416666666</v>
       </c>
       <c r="B79" t="n">
-        <v>-6.07227</v>
+        <v>42.08</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2179,7 +2199,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2189,10 +2209,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46291.625</v>
+        <v>46292.625</v>
       </c>
       <c r="B80" t="n">
-        <v>-5.68434</v>
+        <v>42.54</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2200,7 +2220,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2210,10 +2230,10 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46291.64583333334</v>
+        <v>46292.64583333334</v>
       </c>
       <c r="B81" t="n">
-        <v>-5.52205</v>
+        <v>42.54</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2221,7 +2241,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2231,10 +2251,10 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46291.66666666666</v>
+        <v>46292.66666666666</v>
       </c>
       <c r="B82" t="n">
-        <v>7.96956</v>
+        <v>42.54</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2242,7 +2262,7 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2252,10 +2272,10 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46291.6875</v>
+        <v>46292.6875</v>
       </c>
       <c r="B83" t="n">
-        <v>55.22206</v>
+        <v>38.86844</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2263,7 +2283,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2273,10 +2293,10 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46291.70833333334</v>
+        <v>46292.70833333334</v>
       </c>
       <c r="B84" t="n">
-        <v>80.09999999999999</v>
+        <v>64.95014</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2284,7 +2304,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2294,10 +2314,10 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46291.72916666666</v>
+        <v>46292.72916666666</v>
       </c>
       <c r="B85" t="n">
-        <v>85.74054</v>
+        <v>66.12309</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2305,7 +2325,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2315,10 +2335,10 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>46291.75</v>
+        <v>46292.75</v>
       </c>
       <c r="B86" t="n">
-        <v>109.64095</v>
+        <v>80.76272</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2326,7 +2346,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2336,10 +2356,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>46291.77083333334</v>
+        <v>46292.77083333334</v>
       </c>
       <c r="B87" t="n">
-        <v>96.98999999999999</v>
+        <v>82.39077</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2347,7 +2367,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2357,10 +2377,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>46291.79166666666</v>
+        <v>46292.79166666666</v>
       </c>
       <c r="B88" t="n">
-        <v>90.01000000000001</v>
+        <v>93.16784</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2368,7 +2388,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2378,10 +2398,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>46291.8125</v>
+        <v>46292.8125</v>
       </c>
       <c r="B89" t="n">
-        <v>96.99005</v>
+        <v>90</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2389,7 +2409,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2399,10 +2419,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>46291.83333333334</v>
+        <v>46292.83333333334</v>
       </c>
       <c r="B90" t="n">
-        <v>88.84</v>
+        <v>86.0836</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2410,7 +2430,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2420,10 +2440,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>46291.85416666666</v>
+        <v>46292.85416666666</v>
       </c>
       <c r="B91" t="n">
-        <v>85.07687</v>
+        <v>78.24862</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2431,7 +2451,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2441,10 +2461,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46291.875</v>
+        <v>46292.875</v>
       </c>
       <c r="B92" t="n">
-        <v>83.98999999999999</v>
+        <v>75.9601</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2452,7 +2472,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2462,10 +2482,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>46291.89583333334</v>
+        <v>46292.89583333334</v>
       </c>
       <c r="B93" t="n">
-        <v>88.84</v>
+        <v>70.70860999999999</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2473,7 +2493,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2483,10 +2503,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>46291.91666666666</v>
+        <v>46292.91666666666</v>
       </c>
       <c r="B94" t="n">
-        <v>88.84</v>
+        <v>84.0985</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2494,7 +2514,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2504,10 +2524,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>46291.9375</v>
+        <v>46292.9375</v>
       </c>
       <c r="B95" t="n">
-        <v>87.53769</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2515,7 +2535,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2525,10 +2545,10 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>46291.95833333334</v>
+        <v>46292.95833333334</v>
       </c>
       <c r="B96" t="n">
-        <v>83.98999999999999</v>
+        <v>65.51000000000001</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2536,7 +2556,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2546,10 +2566,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>46291.97916666666</v>
+        <v>46292.97916666666</v>
       </c>
       <c r="B97" t="n">
-        <v>83.98999999999999</v>
+        <v>65.73559</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2557,7 +2577,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46291</v>
+        <v>46292</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 688)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,22 +470,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46292.29166666666</v>
+        <v>46292.3125</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46292.75</v>
+        <v>46292.70833333334</v>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>9.5</v>
       </c>
       <c r="D2" t="n">
-        <v>41.58</v>
+        <v>35.91</v>
       </c>
       <c r="E2" t="n">
-        <v>944.2931257500001</v>
+        <v>747.3635519999998</v>
       </c>
       <c r="F2" t="n">
-        <v>22.71027238455989</v>
+        <v>20.81212898913951</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46292.9375</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46293.10416666666</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="E3" t="n">
+        <v>514.4181705</v>
+      </c>
+      <c r="F3" t="n">
+        <v>34.02236577380953</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46293.3125</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46293.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>32.13</v>
+      </c>
+      <c r="E4" t="n">
+        <v>833.821326</v>
+      </c>
+      <c r="F4" t="n">
+        <v>25.95148851540617</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -840,7 +880,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -870,11 +910,11 @@
         <v>46292.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>47.14741</v>
+        <v>46.45</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -891,11 +931,11 @@
         <v>46292.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>-5.04</v>
+        <v>26.05</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -912,11 +952,11 @@
         <v>46292.375</v>
       </c>
       <c r="B20" t="n">
-        <v>-5.02565</v>
+        <v>42.54</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -933,11 +973,11 @@
         <v>46292.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>38.29057</v>
+        <v>46.45</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +994,11 @@
         <v>46292.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>46.45</v>
+        <v>26.05</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +1015,11 @@
         <v>46292.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>46.45</v>
+        <v>42.54</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1036,11 @@
         <v>46292.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>46.45</v>
+        <v>42.54</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1057,11 @@
         <v>46292.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>46.45</v>
+        <v>42.54</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1078,11 @@
         <v>46292.5</v>
       </c>
       <c r="B26" t="n">
-        <v>46.45</v>
+        <v>42.54</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1099,11 @@
         <v>46292.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>46.45</v>
+        <v>42.54</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1120,11 @@
         <v>46292.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>46.45</v>
+        <v>42.54</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1141,11 @@
         <v>46292.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>61.02</v>
+        <v>46.45</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1162,11 @@
         <v>46292.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>61.02</v>
+        <v>42.54</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1183,11 @@
         <v>46292.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>52.21</v>
+        <v>42.54</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1204,11 @@
         <v>46292.625</v>
       </c>
       <c r="B32" t="n">
-        <v>46.45</v>
+        <v>42.54</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1225,11 @@
         <v>46292.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>46.45</v>
+        <v>42.54</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1210,7 +1250,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1267,11 @@
         <v>46292.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>42.8</v>
+        <v>38.54672</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1288,11 @@
         <v>46292.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>64.95014</v>
+        <v>65.2</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1260,7 +1300,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -1269,11 +1309,11 @@
         <v>46292.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>66.55381</v>
+        <v>66.54884</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1281,7 +1321,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -1290,11 +1330,11 @@
         <v>46292.75</v>
       </c>
       <c r="B38" t="n">
-        <v>75.95007</v>
+        <v>80.75978000000001</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,11 +1351,11 @@
         <v>46292.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>75.9601</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1332,7 +1372,7 @@
         <v>46292.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>79.80914</v>
+        <v>86.14483</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1353,7 +1393,7 @@
         <v>46292.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>83.98999999999999</v>
+        <v>88.84</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1374,7 +1414,7 @@
         <v>46292.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>77.62909999999999</v>
+        <v>89.20401</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1435,7 @@
         <v>46292.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>75.9601</v>
+        <v>82.01671</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1456,7 @@
         <v>46292.875</v>
       </c>
       <c r="B44" t="n">
-        <v>83.98999999999999</v>
+        <v>79.48554</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1477,7 @@
         <v>46292.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>83.98999999999999</v>
+        <v>75.94</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1498,7 @@
         <v>46292.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>75.9601</v>
+        <v>69.94314</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1519,7 @@
         <v>46292.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>81.43228000000001</v>
+        <v>65.69015</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1491,7 +1531,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1540,7 @@
         <v>46292.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>65.95191</v>
+        <v>64.95</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1512,7 +1552,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1521,17 +1561,1025 @@
         <v>46292.97916666666</v>
       </c>
       <c r="B49" t="n">
+        <v>64.95</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B50" t="n">
+        <v>64.95</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46293.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>66.13674</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46293.04166666666</v>
+      </c>
+      <c r="B52" t="n">
         <v>65.51000000000001</v>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>forecast</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="n">
-        <v>46292</v>
-      </c>
-      <c r="E49" t="inlineStr">
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46293.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46293.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>69.43149</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46293.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>70.33107</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46293.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>69.02651</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46293.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>69.00096000000001</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46293.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>68.98083</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46293.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>68.0398</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46293.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>68.10778000000001</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46293.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>74.34886</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46293.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>75.92310999999999</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46293.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>77.59356</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46293.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>75.95005</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46293.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46293.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>46.45</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46293.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46293.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46293.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>45.86551</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46293.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>52.83102</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46293.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>46.80524</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46293.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>46.40225</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46293.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>53.15</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46293.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>53.15</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46293.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>49.85314</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46293.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>53.15</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46293.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>44.55926</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46293.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>51.44266</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46293.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46293.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>48.36506</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46293.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>48.20722</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46293.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>52.5862</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46293.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>44.52853</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46293.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46293.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>83.34</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46293.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>91.14085</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46293.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>94.70672999999999</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46293.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>131.18438</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46293.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>110.98</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46293.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>110.44234</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46293.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>98.73353</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46293.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>92.87206</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46293.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>91.73354999999999</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46293.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>88.84</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46293.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>78.18237000000001</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46293.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>73.54428</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46293.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 605)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,42 +470,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46292</v>
+        <v>46292.10416666666</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46292.1875</v>
+        <v>46292.75</v>
       </c>
       <c r="C2" t="n">
-        <v>4.5</v>
+        <v>15.5</v>
       </c>
       <c r="D2" t="n">
-        <v>17.01</v>
+        <v>58.59</v>
       </c>
       <c r="E2" t="n">
-        <v>691.04284275</v>
+        <v>1599.49827375</v>
       </c>
       <c r="F2" t="n">
-        <v>40.62568152557319</v>
+        <v>27.29985106246799</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46292.27083333334</v>
+        <v>46292.97916666666</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46292.75</v>
+        <v>46293.14583333334</v>
       </c>
       <c r="C3" t="n">
-        <v>11.5</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>43.47</v>
+        <v>15.12</v>
       </c>
       <c r="E3" t="n">
-        <v>988.6375590000001</v>
+        <v>581.0676105</v>
       </c>
       <c r="F3" t="n">
-        <v>22.74298502415459</v>
+        <v>38.43039751984127</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46293.3125</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46293.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>32.13</v>
+      </c>
+      <c r="E4" t="n">
+        <v>745.12437675</v>
+      </c>
+      <c r="F4" t="n">
+        <v>23.19092364612512</v>
       </c>
     </row>
   </sheetData>
@@ -519,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -566,7 +586,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -587,7 +607,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -608,7 +628,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -617,11 +637,11 @@
         <v>46292.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>89.53852999999999</v>
+        <v>88.84</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
@@ -629,7 +649,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -642,7 +662,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
@@ -650,7 +670,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -659,11 +679,11 @@
         <v>46292.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>74.76784000000001</v>
+        <v>74.7782</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
@@ -680,11 +700,11 @@
         <v>46292.125</v>
       </c>
       <c r="B8" t="n">
-        <v>73.83288</v>
+        <v>73.85004000000001</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
@@ -701,11 +721,11 @@
         <v>46292.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>75.95028000000001</v>
+        <v>74.80813999999999</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -722,11 +742,11 @@
         <v>46292.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>73.84206</v>
+        <v>73.85768</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
@@ -743,11 +763,11 @@
         <v>46292.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>83.98999999999999</v>
+        <v>76.15000000000001</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -755,7 +775,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -764,11 +784,11 @@
         <v>46292.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>83.98999999999999</v>
+        <v>79.45639</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
@@ -776,7 +796,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -785,11 +805,11 @@
         <v>46292.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>83.98999999999999</v>
+        <v>80.41743</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
@@ -797,7 +817,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -806,11 +826,11 @@
         <v>46292.25</v>
       </c>
       <c r="B14" t="n">
-        <v>83.98999999999999</v>
+        <v>75.95019000000001</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
@@ -818,7 +838,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -827,11 +847,11 @@
         <v>46292.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>75.95005</v>
+        <v>75.02793</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
@@ -848,11 +868,11 @@
         <v>46292.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>64.95</v>
+        <v>57.93949</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
@@ -873,7 +893,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
@@ -890,11 +910,11 @@
         <v>46292.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>2.54286</v>
+        <v>46.45</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -911,11 +931,11 @@
         <v>46292.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>0.52135</v>
+        <v>26.05</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -932,11 +952,11 @@
         <v>46292.375</v>
       </c>
       <c r="B20" t="n">
-        <v>39.21532</v>
+        <v>42.54</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -953,11 +973,11 @@
         <v>46292.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>52.21</v>
+        <v>46.45</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -974,11 +994,11 @@
         <v>46292.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>46.45</v>
+        <v>26.05</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -999,7 +1019,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1016,11 +1036,11 @@
         <v>46292.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>46.45</v>
+        <v>42.54</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1037,11 +1057,11 @@
         <v>46292.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>46.45</v>
+        <v>42.54</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1062,7 +1082,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1083,7 +1103,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1104,7 +1124,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1121,11 +1141,11 @@
         <v>46292.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>52.21</v>
+        <v>46.45</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1146,7 +1166,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1163,11 +1183,11 @@
         <v>46292.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>42.53983</v>
+        <v>42.54</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1184,11 +1204,11 @@
         <v>46292.625</v>
       </c>
       <c r="B32" t="n">
-        <v>46.45</v>
+        <v>42.54</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1209,7 +1229,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1230,7 +1250,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1247,11 +1267,11 @@
         <v>46292.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>41.16734</v>
+        <v>38.54672</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1268,11 +1288,11 @@
         <v>46292.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>64.89</v>
+        <v>65.2</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1289,11 +1309,11 @@
         <v>46292.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>68.16049</v>
+        <v>66.54884</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1310,11 +1330,11 @@
         <v>46292.75</v>
       </c>
       <c r="B38" t="n">
-        <v>83.04161000000001</v>
+        <v>80.75978000000001</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1331,11 +1351,11 @@
         <v>46292.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>88.84</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1352,11 +1372,11 @@
         <v>46292.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>85.68922999999999</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1373,11 +1393,11 @@
         <v>46292.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>90</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1394,11 +1414,11 @@
         <v>46292.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>84.24524</v>
+        <v>87.18109</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -1415,11 +1435,11 @@
         <v>46292.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>81.52546</v>
+        <v>88.84</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
@@ -1440,7 +1460,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D44" s="3" t="n">
@@ -1457,11 +1477,11 @@
         <v>46292.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>88.84</v>
+        <v>75.9601</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D45" s="3" t="n">
@@ -1478,11 +1498,11 @@
         <v>46292.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>83.98999999999999</v>
+        <v>78.41002</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D46" s="3" t="n">
@@ -1499,11 +1519,11 @@
         <v>46292.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>83.98999999999999</v>
+        <v>88.84</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
@@ -1520,7 +1540,7 @@
         <v>46292.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>73.429</v>
+        <v>88.84</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1541,7 +1561,7 @@
         <v>46292.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>66.9096</v>
+        <v>76.15000000000001</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1552,6 +1572,1014 @@
         <v>46292</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B50" t="n">
+        <v>76.15000000000001</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46293.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>83.61659</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46293.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46293.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46293.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>75.96012</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46293.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>76.15000000000001</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46293.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>75.96007</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46293.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>75.96007</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46293.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>76.03315000000001</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46293.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>75.96007</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46293.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>76.15000000000001</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46293.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46293.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46293.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46293.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46293.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46293.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>46.11506</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46293.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>46.45</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46293.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>46.45</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46293.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>43.13695</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46293.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>52.21</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46293.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46293.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46293.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>45.54385</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46293.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46293.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46293.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>42.52012</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46293.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46293.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46293.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>37.33789</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46293.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>42.54</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46293.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>49.29626</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46293.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>53.66522</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46293.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>46.06178</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46293.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46293.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>85.37201</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46293.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>98.48381000000001</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46293.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>103.27932</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46293.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>97.48084</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46293.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>100.14722</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46293.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>96.59264</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46293.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46293.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46293.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>94.50303</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46293.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>90.03137</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46293.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46293.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>75.28719</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46293.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>74.11484</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 690)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,42 +470,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46293.04166666666</v>
+        <v>46293.29166666666</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46293.20833333334</v>
+        <v>46293.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>15.12</v>
+        <v>34.02</v>
       </c>
       <c r="E2" t="n">
-        <v>567.8298502499999</v>
+        <v>796.2013117500001</v>
       </c>
       <c r="F2" t="n">
-        <v>37.55488427579365</v>
+        <v>23.4039186287478</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46293.33333333334</v>
+        <v>46293.91666666666</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46293.625</v>
+        <v>46294.10416666666</v>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="D3" t="n">
-        <v>26.46</v>
+        <v>17.01</v>
       </c>
       <c r="E3" t="n">
-        <v>700.85257125</v>
+        <v>620.9846565</v>
       </c>
       <c r="F3" t="n">
-        <v>26.48724759070295</v>
+        <v>36.50703447971782</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46294.3125</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46294.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>32.13</v>
+      </c>
+      <c r="E4" t="n">
+        <v>485.85504825</v>
+      </c>
+      <c r="F4" t="n">
+        <v>15.12153900560224</v>
       </c>
     </row>
   </sheetData>
@@ -519,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -608,7 +628,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -629,7 +649,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -650,7 +670,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -671,7 +691,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -692,7 +712,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -713,7 +733,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -734,7 +754,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -755,7 +775,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -860,7 +880,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -881,7 +901,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -890,11 +910,11 @@
         <v>46293.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>42.8</v>
+        <v>45.87545</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -911,11 +931,11 @@
         <v>46293.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>52.21</v>
+        <v>46.45</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -932,11 +952,11 @@
         <v>46293.375</v>
       </c>
       <c r="B20" t="n">
-        <v>47.04178</v>
+        <v>49.91159</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -953,11 +973,11 @@
         <v>46293.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>46.55033</v>
+        <v>42.8</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -974,11 +994,11 @@
         <v>46293.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>48.77452</v>
+        <v>17.00906</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -995,11 +1015,11 @@
         <v>46293.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>44.88085</v>
+        <v>35.29954</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1016,11 +1036,11 @@
         <v>46293.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>45.79567</v>
+        <v>42.54</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1037,11 +1057,11 @@
         <v>46293.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>57.39</v>
+        <v>52.21</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1058,11 +1078,11 @@
         <v>46293.5</v>
       </c>
       <c r="B26" t="n">
-        <v>61.02</v>
+        <v>37.77207</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1079,11 +1099,11 @@
         <v>46293.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>57.39</v>
+        <v>42.54</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1100,11 +1120,11 @@
         <v>46293.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>57.39</v>
+        <v>42.8</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1121,11 +1141,11 @@
         <v>46293.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>57.39</v>
+        <v>42.54</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1142,11 +1162,11 @@
         <v>46293.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>57.39</v>
+        <v>42.8</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1163,11 +1183,11 @@
         <v>46293.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>42.8</v>
+        <v>42.54</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1184,11 +1204,11 @@
         <v>46293.625</v>
       </c>
       <c r="B32" t="n">
-        <v>57.2429</v>
+        <v>42.54</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1196,7 +1216,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1205,11 +1225,11 @@
         <v>46293.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>57.38709</v>
+        <v>49.60902</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1217,7 +1237,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1226,11 +1246,11 @@
         <v>46293.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>67.96147000000001</v>
+        <v>54.0051</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1247,11 +1267,11 @@
         <v>46293.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>57.39</v>
+        <v>46.06012</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1268,11 +1288,11 @@
         <v>46293.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>63.02818</v>
+        <v>65.2</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1289,11 +1309,11 @@
         <v>46293.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>75.74749</v>
+        <v>84.82559999999999</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1310,11 +1330,11 @@
         <v>46293.75</v>
       </c>
       <c r="B38" t="n">
-        <v>88.84</v>
+        <v>96.73116</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1331,11 +1351,11 @@
         <v>46293.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>93.32584</v>
+        <v>100.88557</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1352,11 +1372,11 @@
         <v>46293.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>92.03167000000001</v>
+        <v>100.1927</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1373,7 +1393,7 @@
         <v>46293.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>88.87676</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1394,7 +1414,7 @@
         <v>46293.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>89.01253</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1415,7 +1435,7 @@
         <v>46293.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>90</v>
+        <v>87.83369999999999</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1436,7 +1456,7 @@
         <v>46293.875</v>
       </c>
       <c r="B44" t="n">
-        <v>88.90625</v>
+        <v>90.66625999999999</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1457,7 +1477,7 @@
         <v>46293.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>88.73833</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1478,7 +1498,7 @@
         <v>46293.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>89.17986000000001</v>
+        <v>77.908</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1490,7 +1510,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1519,7 @@
         <v>46293.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>83.98999999999999</v>
+        <v>75.95005</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1511,7 +1531,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1540,7 @@
         <v>46293.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>74.81005</v>
+        <v>73.34648</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1532,7 +1552,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1561,7 @@
         <v>46293.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>74.96286000000001</v>
+        <v>70.00378000000001</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1552,6 +1572,1014 @@
         <v>46293</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B50" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46294.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>69.47911000000001</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46294.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>67.70974</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46294.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>67.79734999999999</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46294.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>68.72283</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46294.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46294.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46294.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>68.77788</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46294.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>70.03567</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46294.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>69.97408</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46294.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>71.14622</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46294.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>76.15000000000001</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46294.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>80.06397</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46294.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>75.9601</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46294.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>72.3597</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46294.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>60.26964</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46294.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>48.52834</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46294.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>26.45</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46294.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>26.45</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46294.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>42.08</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46294.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>26.45</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46294.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>26.45</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46294.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>28.95</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46294.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>7.586</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46294.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>24.49679</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46294.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>24.36228</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46294.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>24.99018</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46294.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>7.60127</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46294.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>24.36563</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46294.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>24.99018</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46294.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>31.49246</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46294.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>42.8001</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46294.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>42.8001</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46294.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>39.35566</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46294.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>67.0638</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46294.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>79.26689</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46294.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>90.20999999999999</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46294.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>93.81858</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46294.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>90.20999999999999</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46294.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>121.01</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46294.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>119.01</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46294.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>105.17011</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46294.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>110.98</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46294.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46294.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>90</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46294.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>95.77081</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46294.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46294.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 692)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,42 +470,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46294.0625</v>
+        <v>46294.29166666666</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46294.22916666666</v>
+        <v>46294.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>15.12</v>
+        <v>34.02</v>
       </c>
       <c r="E2" t="n">
-        <v>545.1982379999999</v>
+        <v>716.0693865000001</v>
       </c>
       <c r="F2" t="n">
-        <v>36.05808452380952</v>
+        <v>21.04848284832452</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46294.33333333334</v>
+        <v>46294.91666666666</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46294.625</v>
+        <v>46295.08333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>26.46</v>
+        <v>15.12</v>
       </c>
       <c r="E3" t="n">
-        <v>701.5696739999998</v>
+        <v>589.9209712500001</v>
       </c>
       <c r="F3" t="n">
-        <v>26.51434897959183</v>
+        <v>39.01593725198413</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46295.29166666666</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46295.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D4" t="n">
+        <v>34.02</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3.816588749999985</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.1121866181657844</v>
       </c>
     </row>
   </sheetData>
@@ -519,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -629,7 +649,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -650,7 +670,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -671,7 +691,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -692,7 +712,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -713,7 +733,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -734,7 +754,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -755,7 +775,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -776,7 +796,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -860,7 +880,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -881,7 +901,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -974,11 +994,11 @@
         <v>46294.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>65.98999999999999</v>
+        <v>24.99013</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -995,11 +1015,11 @@
         <v>46294.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>68.02</v>
+        <v>24.99018</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1016,11 +1036,11 @@
         <v>46294.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>53.15</v>
+        <v>52.21</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1037,11 +1057,11 @@
         <v>46294.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>57.39007</v>
+        <v>23.99583</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1058,11 +1078,11 @@
         <v>46294.5</v>
       </c>
       <c r="B26" t="n">
-        <v>54.20548</v>
+        <v>32.82505</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1079,11 +1099,11 @@
         <v>46294.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>53.15</v>
+        <v>42.8001</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1100,11 +1120,11 @@
         <v>46294.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>51.55619</v>
+        <v>42.94</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1121,11 +1141,11 @@
         <v>46294.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>46.42946</v>
+        <v>24.99018</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1142,11 +1162,11 @@
         <v>46294.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>46.88</v>
+        <v>24.99018</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1167,7 +1187,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1184,11 +1204,11 @@
         <v>46294.625</v>
       </c>
       <c r="B32" t="n">
-        <v>64.89</v>
+        <v>42.94</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1196,7 +1216,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1205,11 +1225,11 @@
         <v>46294.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>62.95447</v>
+        <v>42.8001</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1217,7 +1237,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1226,11 +1246,11 @@
         <v>46294.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>65.5608</v>
+        <v>42.8001</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1247,11 +1267,11 @@
         <v>46294.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>42.94</v>
+        <v>39.31145</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1268,11 +1288,11 @@
         <v>46294.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>64.87821</v>
+        <v>59.23271</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1289,11 +1309,11 @@
         <v>46294.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>72.51239</v>
+        <v>71.63105</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1310,11 +1330,11 @@
         <v>46294.75</v>
       </c>
       <c r="B38" t="n">
-        <v>88.30537</v>
+        <v>88.86011000000001</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1331,11 +1351,11 @@
         <v>46294.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>90.20999999999999</v>
+        <v>91.76955</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1352,11 +1372,11 @@
         <v>46294.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>119.01</v>
+        <v>98.02097000000001</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1373,7 +1393,7 @@
         <v>46294.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>90.20999999999999</v>
+        <v>88.86011000000001</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1394,7 +1414,7 @@
         <v>46294.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>90</v>
+        <v>83.53569</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1415,7 +1435,7 @@
         <v>46294.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>90.93848</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1436,7 +1456,7 @@
         <v>46294.875</v>
       </c>
       <c r="B44" t="n">
-        <v>90.79783999999999</v>
+        <v>88.84</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1457,7 +1477,7 @@
         <v>46294.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>88.86</v>
+        <v>75.94</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1478,7 +1498,7 @@
         <v>46294.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>83.98999999999999</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1490,7 +1510,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1519,7 @@
         <v>46294.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>83.98999999999999</v>
+        <v>75.9601</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1511,7 +1531,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1540,7 @@
         <v>46294.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>83.98999999999999</v>
+        <v>75.94</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1532,7 +1552,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1552,6 +1572,1014 @@
         <v>46294</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B50" t="n">
+        <v>75.9601</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46295.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>75.9503</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46295.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>72.31044</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46295.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>72.86611000000001</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46295.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>71.7555</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46295.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>71.10296</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46295.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>70.21371000000001</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46295.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>70.20783</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46295.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>71.11296</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46295.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>72.39769</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46295.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>75.96007</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46295.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46295.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>80.23266</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46295.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>75.9601</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46295.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46295.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>24.98991</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46295.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46295.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>0.009849999999999999</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46295.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>0.00937</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46295.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>-1.35253</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46295.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>-1.97281</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46295.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-4.16432</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46295.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-9.297739999999999</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46295.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>-5.50874</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46295.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>-5.50874</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46295.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>-10.34</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46295.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>-10.01</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46295.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-8.630000000000001</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46295.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-5.01296</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46295.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-3.59636</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46295.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>9.49198</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46295.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>11.04754</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46295.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>19.2641</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46295.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>26.9664</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46295.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>80.93308</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46295.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>85.80063</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46295.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>95.86299</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46295.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>99.92975</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46295.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>113.5</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46295.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>136.25953</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46295.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>120.74827</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46295.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>111.49895</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46295.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>120.04999</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46295.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>115.82765</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46295.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>95.81623</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46295.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>118.60976</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46295.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>97.18944999999999</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46295.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 607)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,50 +470,50 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46294.0625</v>
+        <v>46294.02083333334</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46294.22916666666</v>
+        <v>46294.25</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>5.5</v>
       </c>
       <c r="D2" t="n">
-        <v>15.12</v>
+        <v>20.79</v>
       </c>
       <c r="E2" t="n">
-        <v>572.2628535</v>
+        <v>764.85038175</v>
       </c>
       <c r="F2" t="n">
-        <v>37.84807232142857</v>
+        <v>36.78934015151516</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46294.33333333334</v>
+        <v>46294.27083333334</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>46294.66666666666</v>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>9.5</v>
       </c>
       <c r="D3" t="n">
-        <v>30.24</v>
+        <v>35.91</v>
       </c>
       <c r="E3" t="n">
-        <v>655.5222569999999</v>
+        <v>792.4706594999998</v>
       </c>
       <c r="F3" t="n">
-        <v>21.67732331349206</v>
+        <v>22.06824448621553</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46294.83333333334</v>
+        <v>46294.95833333334</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>46295</v>
+        <v>46295.125</v>
       </c>
       <c r="C4" t="n">
         <v>4</v>
@@ -522,10 +522,30 @@
         <v>15.12</v>
       </c>
       <c r="E4" t="n">
-        <v>693.1538932499999</v>
+        <v>597.4123935</v>
       </c>
       <c r="F4" t="n">
-        <v>45.84351145833333</v>
+        <v>39.51140168650794</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46295.29166666666</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46295.66666666666</v>
+      </c>
+      <c r="C5" t="n">
+        <v>9</v>
+      </c>
+      <c r="D5" t="n">
+        <v>34.02</v>
+      </c>
+      <c r="E5" t="n">
+        <v>121.7042385</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3.577432054673722</v>
       </c>
     </row>
   </sheetData>
@@ -539,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -571,10 +591,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46294.02083333334</v>
+        <v>46294</v>
       </c>
       <c r="B2" t="n">
-        <v>75.9601</v>
+        <v>83.57884</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -592,14 +612,14 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46294.04166666666</v>
+        <v>46294.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>72.73699999999999</v>
+        <v>77.54156999999999</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
@@ -607,20 +627,20 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46294.0625</v>
+        <v>46294.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>73.73269000000001</v>
+        <v>71.78261000000001</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
@@ -634,14 +654,14 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46294.08333333334</v>
+        <v>46294.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>74.24498</v>
+        <v>71.66955</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
@@ -655,14 +675,14 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46294.10416666666</v>
+        <v>46294.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>73.80544999999999</v>
+        <v>71.46541000000001</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
@@ -676,14 +696,14 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46294.125</v>
+        <v>46294.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>73.35575</v>
+        <v>71.30043999999999</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
@@ -697,14 +717,14 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46294.14583333334</v>
+        <v>46294.125</v>
       </c>
       <c r="B8" t="n">
-        <v>73.35571</v>
+        <v>65.98999999999999</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
@@ -718,14 +738,14 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46294.16666666666</v>
+        <v>46294.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>75.94</v>
+        <v>65.98999999999999</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -739,14 +759,14 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46294.1875</v>
+        <v>46294.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>70.98609999999999</v>
+        <v>71.77105</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
@@ -760,14 +780,14 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46294.20833333334</v>
+        <v>46294.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>71.51558</v>
+        <v>69.90931</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -781,14 +801,14 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46294.22916666666</v>
+        <v>46294.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>80.92048</v>
+        <v>71.08192</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
@@ -796,20 +816,20 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46294.25</v>
+        <v>46294.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>83.98999999999999</v>
+        <v>75.96007</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
@@ -817,20 +837,20 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46294.27083333334</v>
+        <v>46294.25</v>
       </c>
       <c r="B14" t="n">
         <v>83.98999999999999</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
@@ -844,14 +864,14 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46294.29166666666</v>
+        <v>46294.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>72.14709000000001</v>
+        <v>78.36028</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
@@ -859,20 +879,20 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46294.3125</v>
+        <v>46294.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>63.75633</v>
+        <v>71.34125</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
@@ -880,20 +900,20 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46294.33333333334</v>
+        <v>46294.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>57.39007</v>
+        <v>59.8297</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
@@ -907,14 +927,14 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46294.35416666666</v>
+        <v>46294.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>57.39007</v>
+        <v>48.97744</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -928,14 +948,14 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46294.375</v>
+        <v>46294.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>43.6497</v>
+        <v>52.21</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -949,14 +969,14 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46294.39583333334</v>
+        <v>46294.375</v>
       </c>
       <c r="B20" t="n">
         <v>52.21</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -970,14 +990,14 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46294.41666666666</v>
+        <v>46294.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>46.99</v>
+        <v>26.45</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -991,14 +1011,14 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46294.4375</v>
+        <v>46294.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>45.67264</v>
+        <v>24.99013</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -1012,14 +1032,14 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46294.45833333334</v>
+        <v>46294.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>24.98984</v>
+        <v>24.99018</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1033,14 +1053,14 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46294.47916666666</v>
+        <v>46294.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>26.45</v>
+        <v>52.21</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1054,14 +1074,14 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46294.5</v>
+        <v>46294.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>42.94</v>
+        <v>23.99583</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1075,14 +1095,14 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46294.52083333334</v>
+        <v>46294.5</v>
       </c>
       <c r="B26" t="n">
-        <v>42.94</v>
+        <v>32.82505</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1096,14 +1116,14 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46294.54166666666</v>
+        <v>46294.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>32.46487</v>
+        <v>42.8001</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1117,14 +1137,14 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46294.5625</v>
+        <v>46294.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>24.99018</v>
+        <v>42.94</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1138,14 +1158,14 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46294.58333333334</v>
+        <v>46294.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>42.94</v>
+        <v>24.99018</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1159,14 +1179,14 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46294.60416666666</v>
+        <v>46294.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>44.77108</v>
+        <v>24.99018</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1180,14 +1200,14 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46294.625</v>
+        <v>46294.60416666666</v>
       </c>
       <c r="B31" t="n">
         <v>42.94</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1201,14 +1221,14 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46294.64583333334</v>
+        <v>46294.625</v>
       </c>
       <c r="B32" t="n">
-        <v>43.60207</v>
+        <v>42.94</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1222,14 +1242,14 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46294.66666666666</v>
+        <v>46294.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>49.74071</v>
+        <v>42.8001</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1237,20 +1257,20 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46294.6875</v>
+        <v>46294.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>40.83061</v>
+        <v>42.8001</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1264,14 +1284,14 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46294.70833333334</v>
+        <v>46294.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>65.2</v>
+        <v>39.31145</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1285,14 +1305,14 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46294.72916666666</v>
+        <v>46294.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>70.6011</v>
+        <v>59.23271</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1306,14 +1326,14 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46294.75</v>
+        <v>46294.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>90.20999999999999</v>
+        <v>71.63105</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1327,14 +1347,14 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46294.77083333334</v>
+        <v>46294.75</v>
       </c>
       <c r="B38" t="n">
-        <v>96.98999999999999</v>
+        <v>88.86011000000001</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1348,14 +1368,14 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46294.79166666666</v>
+        <v>46294.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>110.98</v>
+        <v>91.76955</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1369,14 +1389,14 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46294.8125</v>
+        <v>46294.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>96.98999999999999</v>
+        <v>98.02097000000001</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1390,14 +1410,14 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46294.83333333334</v>
+        <v>46294.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>96.98999999999999</v>
+        <v>94.47358</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1405,20 +1425,20 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46294.85416666666</v>
+        <v>46294.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>96.98999999999999</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -1426,20 +1446,20 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46294.875</v>
+        <v>46294.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>92.67283</v>
+        <v>88.86</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
@@ -1447,20 +1467,20 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46294.89583333334</v>
+        <v>46294.875</v>
       </c>
       <c r="B44" t="n">
-        <v>88.86</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D44" s="3" t="n">
@@ -1468,20 +1488,20 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46294.91666666666</v>
+        <v>46294.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>86.62414</v>
+        <v>91.42435999999999</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D45" s="3" t="n">
@@ -1489,20 +1509,20 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46294.9375</v>
+        <v>46294.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>88.84</v>
+        <v>86.63298</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D46" s="3" t="n">
@@ -1510,20 +1530,20 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46294.95833333334</v>
+        <v>46294.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>83.98999999999999</v>
+        <v>88.84</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
@@ -1531,28 +1551,1057 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
+        <v>46294.95833333334</v>
+      </c>
+      <c r="B48" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>historical</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
         <v>46294.97916666666</v>
       </c>
-      <c r="B48" t="n">
+      <c r="B49" t="n">
         <v>75.9601</v>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>forecast</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="n">
-        <v>46294</v>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>ON</t>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B50" t="n">
+        <v>75.9601</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46295.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>75.9601</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46295.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>75.9601</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46295.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46295.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>75.96012</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46295.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>64.95014</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46295.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>57.39007</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46295.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>57.39007</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46295.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>57.39007</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46295.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>71.85695</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46295.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>75.96007</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46295.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>84.7901</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46295.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>90</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46295.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46295.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>33.20768</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46295.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>42.53974</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46295.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>24.99018</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46295.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>0.0105</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46295.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>16.43547</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46295.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>0.00949</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46295.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>0.00966</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46295.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-5.44062</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46295.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-6.80737</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46295.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>-8</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46295.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>-1.26637</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46295.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>0.009180000000000001</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46295.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>2.62489</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46295.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-5.50874</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46295.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-0.66949</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46295.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-2.12239</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46295.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>9.81287</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46295.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>24.99018</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46295.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>24.99018</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46295.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>57.13133</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46295.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>86.37013</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46295.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>88.84</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46295.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>100.69751</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46295.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>113.34715</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46295.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>120.73756</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46295.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>116.75717</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46295.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>107.91205</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46295.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>110.62475</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46295.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>107.20095</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46295.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>96.99575</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46295.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>97.02395</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46295.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>119</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46295.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>100.2663</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46295.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>115.33701</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update latest output (run 694)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>531.2428875000002</v>
+        <v>404.5008630000001</v>
       </c>
       <c r="F2" t="n">
-        <v>12.77640422077923</v>
+        <v>9.728255483405485</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46296.20833333334</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46296.66666666666</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>997.3435289999998</v>
+      </c>
+      <c r="F3" t="n">
+        <v>23.98613585858585</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -912,11 +932,11 @@
         <v>46295.375</v>
       </c>
       <c r="B20" t="n">
-        <v>24.99018</v>
+        <v>0.01033</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -933,11 +953,11 @@
         <v>46295.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>19.23193</v>
+        <v>0.00941</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +974,11 @@
         <v>46295.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-0.56438</v>
+        <v>-0.87817</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +995,11 @@
         <v>46295.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>24.99018</v>
+        <v>-5.50874</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46295.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>23.95</v>
+        <v>-7.19009</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46295.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>23.95</v>
+        <v>-5.79124</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46295.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-6.19048</v>
+        <v>-4.578</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46295.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-9.40428</v>
+        <v>0.00933</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46295.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-8.01</v>
+        <v>-5.17</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1121,11 @@
         <v>46295.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-7.09872</v>
+        <v>-6.51</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46295.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-0.50199</v>
+        <v>-4.23775</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1163,11 @@
         <v>46295.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-0.51153</v>
+        <v>-5.17</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46295.625</v>
       </c>
       <c r="B32" t="n">
-        <v>0.01022</v>
+        <v>9.511749999999999</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1205,11 @@
         <v>46295.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>24.99018</v>
+        <v>15.33266</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1226,11 @@
         <v>46295.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>24.99018</v>
+        <v>15.0623</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1247,11 @@
         <v>46295.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>64.89</v>
+        <v>56.76612</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1268,11 @@
         <v>46295.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>83.84990000000001</v>
+        <v>84.67</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1289,11 @@
         <v>46295.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>85.19166</v>
+        <v>88.84</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1310,11 @@
         <v>46295.75</v>
       </c>
       <c r="B38" t="n">
-        <v>96.49541000000001</v>
+        <v>98.00867</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,11 +1331,11 @@
         <v>46295.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>110.98</v>
+        <v>115.16601</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1332,11 +1352,11 @@
         <v>46295.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>125.45777</v>
+        <v>129.36276</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1353,7 +1373,7 @@
         <v>46295.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>114.76335</v>
+        <v>100.85624</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1374,7 +1394,7 @@
         <v>46295.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>103.96887</v>
+        <v>99.37186</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1415,7 @@
         <v>46295.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>96.98999999999999</v>
+        <v>101.26406</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1436,7 @@
         <v>46295.875</v>
       </c>
       <c r="B44" t="n">
-        <v>96.88139</v>
+        <v>106</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46295.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>94.50664</v>
+        <v>106.01625</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46295.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>90.32294</v>
+        <v>99.90782</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46295.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>103.05399</v>
+        <v>101.98981</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1520,7 @@
         <v>46295.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>100.87926</v>
+        <v>99.79201</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,7 +1541,7 @@
         <v>46295.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>99.81412</v>
+        <v>97.31552000000001</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46295</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B50" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46296.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>99.97613</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46296.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>99.16793</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46296.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>106.52</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46296.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>100.35584</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46296.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>99.41101999999999</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46296.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>100.38585</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46296.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>99.94927</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46296.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>101.03829</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46296.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>106.52</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46296.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>106.52</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46296.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>97.48573</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46296.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>97.63005</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46296.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>118.65</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46296.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>96.34949</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46296.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>64.95014</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46296.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>41.76</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46296.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>52.21</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46296.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46296.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46296.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46296.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-5.17</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46296.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46296.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46296.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46296.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>3.76903</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46296.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>3.24592</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46296.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46296.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>53.15</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46296.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>64.90537</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46296.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>67.18000000000001</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46296.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>65.51071</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46296.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>64.95014</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46296.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>90.20999999999999</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46296.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>121.01</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46296.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>137.63965</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46296.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>351.66943</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46296.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>344.30382</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46296.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>330.65919</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46296.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>368.79279</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46296.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>335.3953</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46296.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>237.85</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46296.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>356.25954</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46296.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>402.40365</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46296.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>389.04607</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46296.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>299.98</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46296.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>205.18582</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46296.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>206.47714</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 608)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,82 +470,42 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46294.02083333334</v>
+        <v>46295</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46294.25</v>
+        <v>46295.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>5.5</v>
+        <v>16</v>
       </c>
       <c r="D2" t="n">
-        <v>20.79</v>
+        <v>60.48</v>
       </c>
       <c r="E2" t="n">
-        <v>764.85038175</v>
+        <v>1088.026758</v>
       </c>
       <c r="F2" t="n">
-        <v>36.78934015151516</v>
+        <v>17.98986041666667</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46294.27083333334</v>
+        <v>46296.16666666666</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46294.66666666666</v>
+        <v>46296.66666666666</v>
       </c>
       <c r="C3" t="n">
-        <v>9.5</v>
+        <v>12</v>
       </c>
       <c r="D3" t="n">
-        <v>35.91</v>
+        <v>45.36</v>
       </c>
       <c r="E3" t="n">
-        <v>792.4706594999998</v>
+        <v>1264.5461205</v>
       </c>
       <c r="F3" t="n">
-        <v>22.06824448621553</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>46294.95833333334</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>46295.125</v>
-      </c>
-      <c r="C4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D4" t="n">
-        <v>15.12</v>
-      </c>
-      <c r="E4" t="n">
-        <v>597.4123935</v>
-      </c>
-      <c r="F4" t="n">
-        <v>39.51140168650794</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>46295.29166666666</v>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>46295.66666666666</v>
-      </c>
-      <c r="C5" t="n">
-        <v>9</v>
-      </c>
-      <c r="D5" t="n">
-        <v>34.02</v>
-      </c>
-      <c r="E5" t="n">
-        <v>121.7042385</v>
-      </c>
-      <c r="F5" t="n">
-        <v>3.577432054673722</v>
+        <v>27.87800089285714</v>
       </c>
     </row>
   </sheetData>
@@ -591,10 +551,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B2" t="n">
-        <v>83.57884</v>
+        <v>75.94</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -602,20 +562,20 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46294.02083333334</v>
+        <v>46295.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>77.54156999999999</v>
+        <v>83.82172</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -623,7 +583,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -633,10 +593,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46294.04166666666</v>
+        <v>46295.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>71.78261000000001</v>
+        <v>75.9601</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -644,7 +604,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -654,10 +614,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46294.0625</v>
+        <v>46295.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>71.66955</v>
+        <v>81.28679</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -665,7 +625,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -675,10 +635,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46294.08333333334</v>
+        <v>46295.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>71.46541000000001</v>
+        <v>75.96012</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -686,7 +646,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -696,10 +656,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46294.10416666666</v>
+        <v>46295.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>71.30043999999999</v>
+        <v>64.95019000000001</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -707,7 +667,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -717,10 +677,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46294.125</v>
+        <v>46295.125</v>
       </c>
       <c r="B8" t="n">
-        <v>65.98999999999999</v>
+        <v>57.39007</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -728,7 +688,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -738,10 +698,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46294.14583333334</v>
+        <v>46295.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>65.98999999999999</v>
+        <v>57.39007</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -749,7 +709,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -759,10 +719,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46294.16666666666</v>
+        <v>46295.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>71.77105</v>
+        <v>57.39007</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -770,7 +730,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -780,10 +740,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46294.1875</v>
+        <v>46295.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>69.90931</v>
+        <v>70.96307</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -791,7 +751,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -801,10 +761,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46294.20833333334</v>
+        <v>46295.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>71.08192</v>
+        <v>75.96007</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -812,7 +772,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -822,10 +782,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46294.22916666666</v>
+        <v>46295.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>75.96007</v>
+        <v>84.7901</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -833,7 +793,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -843,10 +803,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46294.25</v>
+        <v>46295.25</v>
       </c>
       <c r="B14" t="n">
-        <v>83.98999999999999</v>
+        <v>90</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -854,20 +814,20 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46294.27083333334</v>
+        <v>46295.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>78.36028</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -875,7 +835,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -885,10 +845,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46294.29166666666</v>
+        <v>46295.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>71.34125</v>
+        <v>33.21234</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -896,7 +856,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -906,10 +866,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46294.3125</v>
+        <v>46295.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>59.8297</v>
+        <v>42.08</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -917,7 +877,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -927,10 +887,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46294.33333333334</v>
+        <v>46295.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>48.97744</v>
+        <v>24.99018</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -938,7 +898,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -948,10 +908,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46294.35416666666</v>
+        <v>46295.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>52.21</v>
+        <v>0.0105</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -959,7 +919,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -969,10 +929,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46294.375</v>
+        <v>46295.375</v>
       </c>
       <c r="B20" t="n">
-        <v>52.21</v>
+        <v>0.01033</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -980,7 +940,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -990,10 +950,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46294.39583333334</v>
+        <v>46295.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>26.45</v>
+        <v>0.00941</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1001,7 +961,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1011,10 +971,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46294.41666666666</v>
+        <v>46295.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>24.99013</v>
+        <v>-0.87817</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1022,7 +982,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1032,10 +992,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46294.4375</v>
+        <v>46295.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>24.99018</v>
+        <v>-5.50874</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1043,7 +1003,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1053,10 +1013,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46294.45833333334</v>
+        <v>46295.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>52.21</v>
+        <v>-7.19009</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1064,7 +1024,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1074,10 +1034,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46294.47916666666</v>
+        <v>46295.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>23.99583</v>
+        <v>-5.79124</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1085,7 +1045,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1095,10 +1055,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46294.5</v>
+        <v>46295.5</v>
       </c>
       <c r="B26" t="n">
-        <v>32.82505</v>
+        <v>-4.578</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1106,7 +1066,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1116,10 +1076,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46294.52083333334</v>
+        <v>46295.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>42.8001</v>
+        <v>0.00933</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1127,7 +1087,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1137,10 +1097,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46294.54166666666</v>
+        <v>46295.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>42.94</v>
+        <v>-5.17</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1148,7 +1108,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1158,10 +1118,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46294.5625</v>
+        <v>46295.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>24.99018</v>
+        <v>-6.51</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1169,7 +1129,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1179,10 +1139,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46294.58333333334</v>
+        <v>46295.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>24.99018</v>
+        <v>-4.23775</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1190,7 +1150,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1200,10 +1160,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46294.60416666666</v>
+        <v>46295.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>42.94</v>
+        <v>-5.17</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1211,7 +1171,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1221,10 +1181,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46294.625</v>
+        <v>46295.625</v>
       </c>
       <c r="B32" t="n">
-        <v>42.94</v>
+        <v>9.511749999999999</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1232,7 +1192,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1242,10 +1202,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46294.64583333334</v>
+        <v>46295.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>42.8001</v>
+        <v>15.33266</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1253,7 +1213,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1263,10 +1223,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46294.66666666666</v>
+        <v>46295.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>42.8001</v>
+        <v>15.0623</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1274,7 +1234,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1284,10 +1244,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46294.6875</v>
+        <v>46295.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>39.31145</v>
+        <v>56.76612</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1295,7 +1255,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1305,10 +1265,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46294.70833333334</v>
+        <v>46295.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>59.23271</v>
+        <v>84.67</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1316,7 +1276,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1326,10 +1286,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46294.72916666666</v>
+        <v>46295.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>71.63105</v>
+        <v>88.84</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1337,7 +1297,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1347,10 +1307,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46294.75</v>
+        <v>46295.75</v>
       </c>
       <c r="B38" t="n">
-        <v>88.86011000000001</v>
+        <v>98.00867</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1358,7 +1318,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1368,10 +1328,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46294.77083333334</v>
+        <v>46295.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>91.76955</v>
+        <v>115.16601</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1379,7 +1339,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1389,10 +1349,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46294.79166666666</v>
+        <v>46295.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>98.02097000000001</v>
+        <v>129.36276</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1400,7 +1360,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1410,10 +1370,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46294.8125</v>
+        <v>46295.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>94.47358</v>
+        <v>115.79048</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1421,7 +1381,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1431,10 +1391,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46294.83333333334</v>
+        <v>46295.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>90.20999999999999</v>
+        <v>121.21571</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1442,7 +1402,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1452,10 +1412,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46294.85416666666</v>
+        <v>46295.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>88.86</v>
+        <v>114.26124</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1463,7 +1423,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1473,10 +1433,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46294.875</v>
+        <v>46295.875</v>
       </c>
       <c r="B44" t="n">
-        <v>96.98999999999999</v>
+        <v>108.42137</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1484,7 +1444,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1494,10 +1454,10 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46294.89583333334</v>
+        <v>46295.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>91.42435999999999</v>
+        <v>96.99575</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1505,7 +1465,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1515,10 +1475,10 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46294.91666666666</v>
+        <v>46295.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>86.63298</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1526,7 +1486,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1536,10 +1496,10 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46294.9375</v>
+        <v>46295.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>88.84</v>
+        <v>119</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1547,7 +1507,7 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1557,10 +1517,10 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46294.95833333334</v>
+        <v>46295.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>83.98999999999999</v>
+        <v>114.87742</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1568,20 +1528,20 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46294.97916666666</v>
+        <v>46295.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>75.9601</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1589,20 +1549,20 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B50" t="n">
-        <v>75.9601</v>
+        <v>95.43047</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1610,20 +1570,20 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46295.02083333334</v>
+        <v>46296.02083333334</v>
       </c>
       <c r="B51" t="n">
-        <v>75.9601</v>
+        <v>106.52003</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1631,20 +1591,20 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46295.04166666666</v>
+        <v>46296.04166666666</v>
       </c>
       <c r="B52" t="n">
-        <v>75.9601</v>
+        <v>100.03819</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1652,20 +1612,20 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46295.0625</v>
+        <v>46296.0625</v>
       </c>
       <c r="B53" t="n">
-        <v>83.98999999999999</v>
+        <v>98.99784</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1673,20 +1633,20 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46295.08333333334</v>
+        <v>46296.08333333334</v>
       </c>
       <c r="B54" t="n">
-        <v>75.96012</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1694,20 +1654,20 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46295.10416666666</v>
+        <v>46296.10416666666</v>
       </c>
       <c r="B55" t="n">
-        <v>64.95014</v>
+        <v>94.14682999999999</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1715,20 +1675,20 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46295.125</v>
+        <v>46296.125</v>
       </c>
       <c r="B56" t="n">
-        <v>57.39007</v>
+        <v>90.34536</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1736,7 +1696,7 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1746,10 +1706,10 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46295.14583333334</v>
+        <v>46296.14583333334</v>
       </c>
       <c r="B57" t="n">
-        <v>57.39007</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1757,7 +1717,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1767,10 +1727,10 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46295.16666666666</v>
+        <v>46296.16666666666</v>
       </c>
       <c r="B58" t="n">
-        <v>57.39007</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1778,20 +1738,20 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46295.1875</v>
+        <v>46296.1875</v>
       </c>
       <c r="B59" t="n">
-        <v>71.85695</v>
+        <v>88.88</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1799,20 +1759,20 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46295.20833333334</v>
+        <v>46296.20833333334</v>
       </c>
       <c r="B60" t="n">
-        <v>75.96007</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1820,20 +1780,20 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46295.22916666666</v>
+        <v>46296.22916666666</v>
       </c>
       <c r="B61" t="n">
-        <v>84.7901</v>
+        <v>90.20999999999999</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1841,20 +1801,20 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46295.25</v>
+        <v>46296.25</v>
       </c>
       <c r="B62" t="n">
-        <v>90</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1862,20 +1822,20 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46295.27083333334</v>
+        <v>46296.27083333334</v>
       </c>
       <c r="B63" t="n">
-        <v>83.98999999999999</v>
+        <v>100.85704</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1883,20 +1843,20 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46295.29166666666</v>
+        <v>46296.29166666666</v>
       </c>
       <c r="B64" t="n">
-        <v>33.20768</v>
+        <v>89.64077</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1904,7 +1864,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1914,10 +1874,10 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46295.3125</v>
+        <v>46296.3125</v>
       </c>
       <c r="B65" t="n">
-        <v>42.53974</v>
+        <v>68.67</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1925,7 +1885,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1935,10 +1895,10 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46295.33333333334</v>
+        <v>46296.33333333334</v>
       </c>
       <c r="B66" t="n">
-        <v>24.99018</v>
+        <v>44.30883</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1946,7 +1906,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1956,10 +1916,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46295.35416666666</v>
+        <v>46296.35416666666</v>
       </c>
       <c r="B67" t="n">
-        <v>0.0105</v>
+        <v>11.4</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1967,7 +1927,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1977,10 +1937,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46295.375</v>
+        <v>46296.375</v>
       </c>
       <c r="B68" t="n">
-        <v>16.43547</v>
+        <v>11.88</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1988,7 +1948,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1998,10 +1958,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46295.39583333334</v>
+        <v>46296.39583333334</v>
       </c>
       <c r="B69" t="n">
-        <v>0.00949</v>
+        <v>52.21</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -2009,7 +1969,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2019,10 +1979,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46295.41666666666</v>
+        <v>46296.41666666666</v>
       </c>
       <c r="B70" t="n">
-        <v>0.00966</v>
+        <v>52.21</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -2030,7 +1990,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2040,10 +2000,10 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46295.4375</v>
+        <v>46296.4375</v>
       </c>
       <c r="B71" t="n">
-        <v>-5.44062</v>
+        <v>0.99</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2051,7 +2011,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2061,10 +2021,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46295.45833333334</v>
+        <v>46296.45833333334</v>
       </c>
       <c r="B72" t="n">
-        <v>-6.80737</v>
+        <v>1.2</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2072,7 +2032,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2082,10 +2042,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46295.47916666666</v>
+        <v>46296.47916666666</v>
       </c>
       <c r="B73" t="n">
-        <v>-8</v>
+        <v>42.94</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2093,7 +2053,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2103,10 +2063,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46295.5</v>
+        <v>46296.5</v>
       </c>
       <c r="B74" t="n">
-        <v>-1.26637</v>
+        <v>25.11973</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2114,7 +2074,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2124,10 +2084,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46295.52083333334</v>
+        <v>46296.52083333334</v>
       </c>
       <c r="B75" t="n">
-        <v>0.009180000000000001</v>
+        <v>10.25401</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2135,7 +2095,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2145,10 +2105,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46295.54166666666</v>
+        <v>46296.54166666666</v>
       </c>
       <c r="B76" t="n">
-        <v>2.62489</v>
+        <v>42.94</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2156,7 +2116,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2166,10 +2126,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46295.5625</v>
+        <v>46296.5625</v>
       </c>
       <c r="B77" t="n">
-        <v>-5.50874</v>
+        <v>46.99</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2177,7 +2137,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2187,10 +2147,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46295.58333333334</v>
+        <v>46296.58333333334</v>
       </c>
       <c r="B78" t="n">
-        <v>-0.66949</v>
+        <v>53.15</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2198,7 +2158,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2208,10 +2168,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46295.60416666666</v>
+        <v>46296.60416666666</v>
       </c>
       <c r="B79" t="n">
-        <v>-2.12239</v>
+        <v>53.15</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2219,7 +2179,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2229,10 +2189,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46295.625</v>
+        <v>46296.625</v>
       </c>
       <c r="B80" t="n">
-        <v>9.81287</v>
+        <v>64.02</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2240,7 +2200,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2250,10 +2210,10 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46295.64583333334</v>
+        <v>46296.64583333334</v>
       </c>
       <c r="B81" t="n">
-        <v>24.99018</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2261,7 +2221,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2271,10 +2231,10 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46295.66666666666</v>
+        <v>46296.66666666666</v>
       </c>
       <c r="B82" t="n">
-        <v>24.99018</v>
+        <v>75.95028000000001</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2282,7 +2242,7 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2292,10 +2252,10 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46295.6875</v>
+        <v>46296.6875</v>
       </c>
       <c r="B83" t="n">
-        <v>57.13133</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2303,7 +2263,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2313,10 +2273,10 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46295.70833333334</v>
+        <v>46296.70833333334</v>
       </c>
       <c r="B84" t="n">
-        <v>86.37013</v>
+        <v>121.01</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2324,7 +2284,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2334,10 +2294,10 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46295.72916666666</v>
+        <v>46296.72916666666</v>
       </c>
       <c r="B85" t="n">
-        <v>88.84</v>
+        <v>299.98</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2345,7 +2305,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2355,10 +2315,10 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>46295.75</v>
+        <v>46296.75</v>
       </c>
       <c r="B86" t="n">
-        <v>100.69751</v>
+        <v>499.96</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2366,7 +2326,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2376,10 +2336,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>46295.77083333334</v>
+        <v>46296.77083333334</v>
       </c>
       <c r="B87" t="n">
-        <v>113.34715</v>
+        <v>360.68583</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2387,7 +2347,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2397,10 +2357,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>46295.79166666666</v>
+        <v>46296.79166666666</v>
       </c>
       <c r="B88" t="n">
-        <v>120.73756</v>
+        <v>357.88963</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2408,7 +2368,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2418,10 +2378,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>46295.8125</v>
+        <v>46296.8125</v>
       </c>
       <c r="B89" t="n">
-        <v>116.75717</v>
+        <v>318.3497</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2429,7 +2389,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2439,10 +2399,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>46295.83333333334</v>
+        <v>46296.83333333334</v>
       </c>
       <c r="B90" t="n">
-        <v>107.91205</v>
+        <v>352.35971</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2450,7 +2410,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2460,10 +2420,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>46295.85416666666</v>
+        <v>46296.85416666666</v>
       </c>
       <c r="B91" t="n">
-        <v>110.62475</v>
+        <v>352.62794</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2471,7 +2431,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2481,10 +2441,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46295.875</v>
+        <v>46296.875</v>
       </c>
       <c r="B92" t="n">
-        <v>107.20095</v>
+        <v>374.24025</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2492,7 +2452,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2502,10 +2462,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>46295.89583333334</v>
+        <v>46296.89583333334</v>
       </c>
       <c r="B93" t="n">
-        <v>96.99575</v>
+        <v>299.99</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2513,7 +2473,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2523,10 +2483,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>46295.91666666666</v>
+        <v>46296.91666666666</v>
       </c>
       <c r="B94" t="n">
-        <v>97.02395</v>
+        <v>355.25634</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2534,7 +2494,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2544,10 +2504,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>46295.9375</v>
+        <v>46296.9375</v>
       </c>
       <c r="B95" t="n">
-        <v>119</v>
+        <v>299.98</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2555,7 +2515,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2565,10 +2525,10 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>46295.95833333334</v>
+        <v>46296.95833333334</v>
       </c>
       <c r="B96" t="n">
-        <v>100.2663</v>
+        <v>147.42601</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2576,7 +2536,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2586,10 +2546,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>46295.97916666666</v>
+        <v>46296.97916666666</v>
       </c>
       <c r="B97" t="n">
-        <v>115.33701</v>
+        <v>223.15114</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2597,7 +2557,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 696)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>829.1787367499996</v>
+        <v>985.4861639999998</v>
       </c>
       <c r="F2" t="n">
-        <v>19.94176856060605</v>
+        <v>23.70096594516594</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46297.20833333334</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46297.66666666666</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1774.18198425</v>
+      </c>
+      <c r="F3" t="n">
+        <v>42.6691193903319</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -912,11 +932,11 @@
         <v>46296.375</v>
       </c>
       <c r="B20" t="n">
-        <v>28.01</v>
+        <v>11.88</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -933,11 +953,11 @@
         <v>46296.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>28.01</v>
+        <v>51.61406</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -958,7 +978,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -979,7 +999,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46296.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>11.88</v>
+        <v>-5.17</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46296.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>11.88</v>
+        <v>0.99</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46296.5</v>
       </c>
       <c r="B26" t="n">
-        <v>11.88</v>
+        <v>28.8642</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46296.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>0.99</v>
+        <v>11.88</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46296.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-4.68364</v>
+        <v>16.64713</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1121,11 @@
         <v>46296.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>42.08</v>
+        <v>45.05655</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46296.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-4.81546</v>
+        <v>45.62481</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1163,11 @@
         <v>46296.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>46.99</v>
+        <v>61.24946</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46296.625</v>
       </c>
       <c r="B32" t="n">
-        <v>0.99</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1205,11 @@
         <v>46296.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>67.18000000000001</v>
+        <v>64.89</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1226,11 @@
         <v>46296.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>75.96017000000001</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1247,11 @@
         <v>46296.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>90.3616</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1252,7 +1272,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1289,11 @@
         <v>46296.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>139.90384</v>
+        <v>299.99</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1310,11 @@
         <v>46296.75</v>
       </c>
       <c r="B38" t="n">
-        <v>297.99</v>
+        <v>599.60168</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,11 +1331,11 @@
         <v>46296.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>229.69</v>
+        <v>499.41265</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1332,11 +1352,11 @@
         <v>46296.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>299.98</v>
+        <v>499.96</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1353,11 +1373,11 @@
         <v>46296.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>261.12745</v>
+        <v>351.07221</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1374,7 +1394,7 @@
         <v>46296.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>297.99</v>
+        <v>118.65</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1415,7 @@
         <v>46296.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>238.34573</v>
+        <v>119.01</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1436,7 @@
         <v>46296.875</v>
       </c>
       <c r="B44" t="n">
-        <v>130.01</v>
+        <v>118.65</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46296.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>239.06189</v>
+        <v>117.88081</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46296.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>206.2712</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46296.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>138</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1520,7 @@
         <v>46296.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>138</v>
+        <v>115.67446</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,7 +1541,7 @@
         <v>46296.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>203.66065</v>
+        <v>118.12078</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46296</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B50" t="n">
+        <v>116.06316</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46297.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>115.04246</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46297.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>114.8602</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46297.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>118.9189</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46297.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>118.65</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46297.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>119</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46297.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>113.5</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46297.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>119</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46297.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>119.01</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46297.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>99.13245999999999</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46297.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>99.17310999999999</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46297.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>99.06877</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46297.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46297.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>91.27804999999999</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46297.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>81.10374</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46297.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>69.09958</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46297.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46297.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>84.79000000000001</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46297.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>67.18000000000001</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46297.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>76.3</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46297.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>76.3</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46297.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>76.3</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46297.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>75.95014</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46297.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>75.96003</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46297.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>84.79007</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46297.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>75.96003</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46297.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>75.95014</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46297.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>99.01000000000001</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46297.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>75.96003</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46297.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>84.79007</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46297.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46297.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>75.96007</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46297.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>75.95014</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46297.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>75.95014</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46297.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>98.64858</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46297.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>119.01</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46297.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>121.01</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46297.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>118.65</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46297.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>121.01</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46297.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>113.5</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46297.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>132.07773</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46297.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>133.66457</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46297.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46297.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>271.11276</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46297.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>119.01</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46297.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>118.65</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46297.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>100.96721</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46297.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>97.9637</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 609)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -470,10 +470,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46295.66666666666</v>
+        <v>46296.66666666666</v>
       </c>
       <c r="C2" t="n">
         <v>16</v>
@@ -482,18 +482,18 @@
         <v>60.48</v>
       </c>
       <c r="E2" t="n">
-        <v>1088.026758</v>
+        <v>1890.48251925</v>
       </c>
       <c r="F2" t="n">
-        <v>17.98986041666667</v>
+        <v>31.25797816220239</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46296.16666666666</v>
+        <v>46297.16666666666</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46296.66666666666</v>
+        <v>46297.66666666666</v>
       </c>
       <c r="C3" t="n">
         <v>12</v>
@@ -502,10 +502,10 @@
         <v>45.36</v>
       </c>
       <c r="E3" t="n">
-        <v>1264.5461205</v>
+        <v>1818.759111</v>
       </c>
       <c r="F3" t="n">
-        <v>27.87800089285714</v>
+        <v>40.09610033068783</v>
       </c>
     </row>
   </sheetData>
@@ -551,10 +551,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B2" t="n">
-        <v>75.94</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -572,10 +572,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46295.02083333334</v>
+        <v>46296.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>83.82172</v>
+        <v>99.05251</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -593,10 +593,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46295.04166666666</v>
+        <v>46296.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>75.9601</v>
+        <v>97.13883</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -614,10 +614,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46295.0625</v>
+        <v>46296.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>81.28679</v>
+        <v>97.63005</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -635,10 +635,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46295.08333333334</v>
+        <v>46296.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>75.96012</v>
+        <v>88.88</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -656,10 +656,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46295.10416666666</v>
+        <v>46296.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>64.95019000000001</v>
+        <v>88.88</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -677,10 +677,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46295.125</v>
+        <v>46296.125</v>
       </c>
       <c r="B8" t="n">
-        <v>57.39007</v>
+        <v>88.88</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -698,10 +698,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46295.14583333334</v>
+        <v>46296.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>57.39007</v>
+        <v>86.88</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -719,10 +719,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46295.16666666666</v>
+        <v>46296.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>57.39007</v>
+        <v>86.88</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -740,10 +740,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46295.1875</v>
+        <v>46296.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>70.96307</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -761,10 +761,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46295.20833333334</v>
+        <v>46296.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>75.96007</v>
+        <v>95.15612</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -772,7 +772,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -782,10 +782,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46295.22916666666</v>
+        <v>46296.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>84.7901</v>
+        <v>92.5778</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -803,10 +803,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46295.25</v>
+        <v>46296.25</v>
       </c>
       <c r="B14" t="n">
-        <v>90</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -824,10 +824,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46295.27083333334</v>
+        <v>46296.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>83.98999999999999</v>
+        <v>106.25588</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -845,10 +845,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46295.29166666666</v>
+        <v>46296.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>33.21234</v>
+        <v>90.07617999999999</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -866,10 +866,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46295.3125</v>
+        <v>46296.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>42.08</v>
+        <v>64.95014</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -887,10 +887,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46295.33333333334</v>
+        <v>46296.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>24.99018</v>
+        <v>26.07271</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -908,10 +908,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46295.35416666666</v>
+        <v>46296.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>0.0105</v>
+        <v>0.99</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -919,7 +919,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -929,10 +929,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46295.375</v>
+        <v>46296.375</v>
       </c>
       <c r="B20" t="n">
-        <v>0.01033</v>
+        <v>11.88</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -950,10 +950,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46295.39583333334</v>
+        <v>46296.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>0.00941</v>
+        <v>51.61406</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -971,10 +971,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46295.41666666666</v>
+        <v>46296.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-0.87817</v>
+        <v>25.1</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -992,10 +992,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46295.4375</v>
+        <v>46296.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-5.50874</v>
+        <v>11.88</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1013,10 +1013,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46295.45833333334</v>
+        <v>46296.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-7.19009</v>
+        <v>-5.17</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1034,10 +1034,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46295.47916666666</v>
+        <v>46296.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-5.79124</v>
+        <v>0.99</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1055,10 +1055,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46295.5</v>
+        <v>46296.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-4.578</v>
+        <v>28.8642</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1076,10 +1076,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46295.52083333334</v>
+        <v>46296.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>0.00933</v>
+        <v>11.88</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1097,10 +1097,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46295.54166666666</v>
+        <v>46296.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-5.17</v>
+        <v>16.64713</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1118,10 +1118,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46295.5625</v>
+        <v>46296.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-6.51</v>
+        <v>45.05655</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1129,7 +1129,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1139,10 +1139,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46295.58333333334</v>
+        <v>46296.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-4.23775</v>
+        <v>45.62481</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1150,7 +1150,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1160,10 +1160,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46295.60416666666</v>
+        <v>46296.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-5.17</v>
+        <v>61.24946</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1181,10 +1181,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46295.625</v>
+        <v>46296.625</v>
       </c>
       <c r="B32" t="n">
-        <v>9.511749999999999</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1202,10 +1202,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46295.64583333334</v>
+        <v>46296.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>15.33266</v>
+        <v>64.89</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1223,10 +1223,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46295.66666666666</v>
+        <v>46296.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>15.0623</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1244,10 +1244,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46295.6875</v>
+        <v>46296.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>56.76612</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1265,10 +1265,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46295.70833333334</v>
+        <v>46296.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>84.67</v>
+        <v>121.01</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1276,7 +1276,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1286,10 +1286,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46295.72916666666</v>
+        <v>46296.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>88.84</v>
+        <v>299.99</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1297,7 +1297,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1307,10 +1307,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46295.75</v>
+        <v>46296.75</v>
       </c>
       <c r="B38" t="n">
-        <v>98.00867</v>
+        <v>599.60168</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1328,10 +1328,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46295.77083333334</v>
+        <v>46296.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>115.16601</v>
+        <v>499.41265</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1349,10 +1349,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46295.79166666666</v>
+        <v>46296.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>129.36276</v>
+        <v>499.96</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1370,10 +1370,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46295.8125</v>
+        <v>46296.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>115.79048</v>
+        <v>351.07221</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1391,10 +1391,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46295.83333333334</v>
+        <v>46296.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>121.21571</v>
+        <v>299.98</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1402,7 +1402,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1412,10 +1412,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46295.85416666666</v>
+        <v>46296.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>114.26124</v>
+        <v>499.96</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46295.875</v>
+        <v>46296.875</v>
       </c>
       <c r="B44" t="n">
-        <v>108.42137</v>
+        <v>380.26624</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1454,10 +1454,10 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46295.89583333334</v>
+        <v>46296.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>96.99575</v>
+        <v>299.99</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1465,7 +1465,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1475,10 +1475,10 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46295.91666666666</v>
+        <v>46296.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>96.98999999999999</v>
+        <v>348.48031</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1496,10 +1496,10 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46295.9375</v>
+        <v>46296.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>119</v>
+        <v>299</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1507,7 +1507,7 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1517,10 +1517,10 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46295.95833333334</v>
+        <v>46296.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>114.87742</v>
+        <v>161.1737</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1528,7 +1528,7 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1538,18 +1538,18 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46295.97916666666</v>
+        <v>46296.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>96.98999999999999</v>
+        <v>299</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B50" t="n">
-        <v>95.43047</v>
+        <v>115.81316</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1570,7 +1570,7 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1580,10 +1580,10 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46296.02083333334</v>
+        <v>46297.02083333334</v>
       </c>
       <c r="B51" t="n">
-        <v>106.52003</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1591,7 +1591,7 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1601,10 +1601,10 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46296.04166666666</v>
+        <v>46297.04166666666</v>
       </c>
       <c r="B52" t="n">
-        <v>100.03819</v>
+        <v>106.52</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1622,10 +1622,10 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46296.0625</v>
+        <v>46297.0625</v>
       </c>
       <c r="B53" t="n">
-        <v>98.99784</v>
+        <v>95.26188999999999</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1643,10 +1643,10 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46296.08333333334</v>
+        <v>46297.08333333334</v>
       </c>
       <c r="B54" t="n">
-        <v>96.98999999999999</v>
+        <v>93.60917000000001</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1664,10 +1664,10 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46296.10416666666</v>
+        <v>46297.10416666666</v>
       </c>
       <c r="B55" t="n">
-        <v>94.14682999999999</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1685,10 +1685,10 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46296.125</v>
+        <v>46297.125</v>
       </c>
       <c r="B56" t="n">
-        <v>90.34536</v>
+        <v>97.41298999999999</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1706,10 +1706,10 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46296.14583333334</v>
+        <v>46297.14583333334</v>
       </c>
       <c r="B57" t="n">
-        <v>84.79000000000001</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1727,10 +1727,10 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46296.16666666666</v>
+        <v>46297.16666666666</v>
       </c>
       <c r="B58" t="n">
-        <v>84.79000000000001</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1738,7 +1738,7 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1748,10 +1748,10 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46296.1875</v>
+        <v>46297.1875</v>
       </c>
       <c r="B59" t="n">
-        <v>88.88</v>
+        <v>95.31774</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1759,7 +1759,7 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1769,10 +1769,10 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46296.20833333334</v>
+        <v>46297.20833333334</v>
       </c>
       <c r="B60" t="n">
-        <v>96.98999999999999</v>
+        <v>94.00998</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1780,7 +1780,7 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1790,10 +1790,10 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46296.22916666666</v>
+        <v>46297.22916666666</v>
       </c>
       <c r="B61" t="n">
-        <v>90.20999999999999</v>
+        <v>93.00270999999999</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1801,7 +1801,7 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1811,10 +1811,10 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46296.25</v>
+        <v>46297.25</v>
       </c>
       <c r="B62" t="n">
-        <v>96.98999999999999</v>
+        <v>96.19277</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1822,7 +1822,7 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1832,10 +1832,10 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46296.27083333334</v>
+        <v>46297.27083333334</v>
       </c>
       <c r="B63" t="n">
-        <v>100.85704</v>
+        <v>90</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1843,7 +1843,7 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1853,10 +1853,10 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46296.29166666666</v>
+        <v>46297.29166666666</v>
       </c>
       <c r="B64" t="n">
-        <v>89.64077</v>
+        <v>75.95014</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1864,7 +1864,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1874,10 +1874,10 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46296.3125</v>
+        <v>46297.3125</v>
       </c>
       <c r="B65" t="n">
-        <v>68.67</v>
+        <v>67.05934000000001</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1895,10 +1895,10 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46296.33333333334</v>
+        <v>46297.33333333334</v>
       </c>
       <c r="B66" t="n">
-        <v>44.30883</v>
+        <v>75.96017000000001</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1906,7 +1906,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1916,10 +1916,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46296.35416666666</v>
+        <v>46297.35416666666</v>
       </c>
       <c r="B67" t="n">
-        <v>11.4</v>
+        <v>75.95014</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1937,10 +1937,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46296.375</v>
+        <v>46297.375</v>
       </c>
       <c r="B68" t="n">
-        <v>11.88</v>
+        <v>64.02</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1958,10 +1958,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46296.39583333334</v>
+        <v>46297.39583333334</v>
       </c>
       <c r="B69" t="n">
-        <v>52.21</v>
+        <v>76.3</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1979,10 +1979,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46296.41666666666</v>
+        <v>46297.41666666666</v>
       </c>
       <c r="B70" t="n">
-        <v>52.21</v>
+        <v>75.95014</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -1990,7 +1990,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2000,10 +2000,10 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46296.4375</v>
+        <v>46297.4375</v>
       </c>
       <c r="B71" t="n">
-        <v>0.99</v>
+        <v>64.02</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2021,10 +2021,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46296.45833333334</v>
+        <v>46297.45833333334</v>
       </c>
       <c r="B72" t="n">
-        <v>1.2</v>
+        <v>64.02</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2032,7 +2032,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2042,10 +2042,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46296.47916666666</v>
+        <v>46297.47916666666</v>
       </c>
       <c r="B73" t="n">
-        <v>42.94</v>
+        <v>75.95014</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2063,10 +2063,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46296.5</v>
+        <v>46297.5</v>
       </c>
       <c r="B74" t="n">
-        <v>25.11973</v>
+        <v>75.95014</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2074,7 +2074,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2084,10 +2084,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46296.52083333334</v>
+        <v>46297.52083333334</v>
       </c>
       <c r="B75" t="n">
-        <v>10.25401</v>
+        <v>64.02</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2095,7 +2095,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2105,10 +2105,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46296.54166666666</v>
+        <v>46297.54166666666</v>
       </c>
       <c r="B76" t="n">
-        <v>42.94</v>
+        <v>64.95007</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2116,7 +2116,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2126,10 +2126,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46296.5625</v>
+        <v>46297.5625</v>
       </c>
       <c r="B77" t="n">
-        <v>46.99</v>
+        <v>75.96003</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2147,10 +2147,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46296.58333333334</v>
+        <v>46297.58333333334</v>
       </c>
       <c r="B78" t="n">
-        <v>53.15</v>
+        <v>75.95014</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2158,7 +2158,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2168,10 +2168,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46296.60416666666</v>
+        <v>46297.60416666666</v>
       </c>
       <c r="B79" t="n">
-        <v>53.15</v>
+        <v>75.95014</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2179,7 +2179,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2189,10 +2189,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46296.625</v>
+        <v>46297.625</v>
       </c>
       <c r="B80" t="n">
-        <v>64.02</v>
+        <v>75.9601</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2200,7 +2200,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2210,10 +2210,10 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46296.64583333334</v>
+        <v>46297.64583333334</v>
       </c>
       <c r="B81" t="n">
-        <v>67.18000000000001</v>
+        <v>75.96007</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2231,10 +2231,10 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46296.66666666666</v>
+        <v>46297.66666666666</v>
       </c>
       <c r="B82" t="n">
-        <v>75.95028000000001</v>
+        <v>75.95014</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2242,7 +2242,7 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2252,10 +2252,10 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46296.6875</v>
+        <v>46297.6875</v>
       </c>
       <c r="B83" t="n">
-        <v>96.98999999999999</v>
+        <v>75.95014</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2273,10 +2273,10 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46296.70833333334</v>
+        <v>46297.70833333334</v>
       </c>
       <c r="B84" t="n">
-        <v>121.01</v>
+        <v>88.88</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2284,7 +2284,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2294,10 +2294,10 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46296.72916666666</v>
+        <v>46297.72916666666</v>
       </c>
       <c r="B85" t="n">
-        <v>299.98</v>
+        <v>119</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2315,10 +2315,10 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>46296.75</v>
+        <v>46297.75</v>
       </c>
       <c r="B86" t="n">
-        <v>499.96</v>
+        <v>129.65</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2326,7 +2326,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2336,10 +2336,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>46296.77083333334</v>
+        <v>46297.77083333334</v>
       </c>
       <c r="B87" t="n">
-        <v>360.68583</v>
+        <v>121.01</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2347,7 +2347,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2357,10 +2357,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>46296.79166666666</v>
+        <v>46297.79166666666</v>
       </c>
       <c r="B88" t="n">
-        <v>357.88963</v>
+        <v>121.01</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2368,7 +2368,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2378,10 +2378,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>46296.8125</v>
+        <v>46297.8125</v>
       </c>
       <c r="B89" t="n">
-        <v>318.3497</v>
+        <v>124.1558</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2389,7 +2389,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2399,10 +2399,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>46296.83333333334</v>
+        <v>46297.83333333334</v>
       </c>
       <c r="B90" t="n">
-        <v>352.35971</v>
+        <v>129.65</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2410,7 +2410,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2420,10 +2420,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>46296.85416666666</v>
+        <v>46297.85416666666</v>
       </c>
       <c r="B91" t="n">
-        <v>352.62794</v>
+        <v>127.8413</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2431,7 +2431,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2441,10 +2441,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46296.875</v>
+        <v>46297.875</v>
       </c>
       <c r="B92" t="n">
-        <v>374.24025</v>
+        <v>119.01</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2452,7 +2452,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2462,10 +2462,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>46296.89583333334</v>
+        <v>46297.89583333334</v>
       </c>
       <c r="B93" t="n">
-        <v>299.99</v>
+        <v>119.01</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2483,10 +2483,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>46296.91666666666</v>
+        <v>46297.91666666666</v>
       </c>
       <c r="B94" t="n">
-        <v>355.25634</v>
+        <v>119</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2494,7 +2494,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2504,10 +2504,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>46296.9375</v>
+        <v>46297.9375</v>
       </c>
       <c r="B95" t="n">
-        <v>299.98</v>
+        <v>98.14653</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2525,10 +2525,10 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>46296.95833333334</v>
+        <v>46297.95833333334</v>
       </c>
       <c r="B96" t="n">
-        <v>147.42601</v>
+        <v>96.99309</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2536,7 +2536,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2546,10 +2546,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>46296.97916666666</v>
+        <v>46297.97916666666</v>
       </c>
       <c r="B97" t="n">
-        <v>223.15114</v>
+        <v>97.81703</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2557,7 +2557,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 698)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,10 +470,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46297.20833333334</v>
+        <v>46297.16666666666</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46297.66666666666</v>
+        <v>46297.625</v>
       </c>
       <c r="C2" t="n">
         <v>11</v>
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>1623.1855965</v>
+        <v>1673.67143775</v>
       </c>
       <c r="F2" t="n">
-        <v>39.03765263347763</v>
+        <v>40.25183832972584</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46298.27083333334</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46298.72916666666</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1347.03705825</v>
+      </c>
+      <c r="F3" t="n">
+        <v>32.39627364718613</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -714,7 +734,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -735,7 +755,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -912,11 +932,11 @@
         <v>46297.375</v>
       </c>
       <c r="B20" t="n">
-        <v>84.79007</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -937,7 +957,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +974,11 @@
         <v>46297.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>76.3</v>
+        <v>64.95007</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +995,11 @@
         <v>46297.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>75.96003</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46297.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>64.02</v>
+        <v>75.95014</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46297.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>64.02</v>
+        <v>75.95014</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46297.5</v>
       </c>
       <c r="B26" t="n">
-        <v>64.95007</v>
+        <v>75.95014</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46297.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>64.95007</v>
+        <v>64.02</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46297.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>64.02</v>
+        <v>64.95007</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1121,11 @@
         <v>46297.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>64.02</v>
+        <v>64.95007</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46297.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>64.02</v>
+        <v>75.95014</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1163,11 @@
         <v>46297.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>64.95007</v>
+        <v>75.96003</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46297.625</v>
       </c>
       <c r="B32" t="n">
-        <v>73.26000000000001</v>
+        <v>99.01000000000001</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1176,7 +1196,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -1185,11 +1205,11 @@
         <v>46297.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>75.95014</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1197,7 +1217,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -1206,11 +1226,11 @@
         <v>46297.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>64.95007</v>
+        <v>75.95014</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1247,11 @@
         <v>46297.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>64.95007</v>
+        <v>75.95014</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1268,11 @@
         <v>46297.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>82.64259</v>
+        <v>88.88</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1289,11 @@
         <v>46297.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>100.17832</v>
+        <v>119</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1310,11 @@
         <v>46297.75</v>
       </c>
       <c r="B38" t="n">
-        <v>119.01</v>
+        <v>129.65</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,11 +1331,11 @@
         <v>46297.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>119.01</v>
+        <v>129.65</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1332,11 +1352,11 @@
         <v>46297.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>119.01</v>
+        <v>129.65</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1353,7 +1373,7 @@
         <v>46297.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>118.65</v>
+        <v>104.83187</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1374,7 +1394,7 @@
         <v>46297.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>100.60175</v>
+        <v>119</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1415,7 @@
         <v>46297.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>102.08118</v>
+        <v>119.01</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46297.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>124.30907</v>
+        <v>123.33314</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46297.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>119</v>
+        <v>119.01</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46297.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>100.03881</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1520,7 @@
         <v>46297.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>102.2147</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,7 +1541,7 @@
         <v>46297.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>99.6884</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46297</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B50" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46298.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46298.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46298.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46298.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46298.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46298.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>90</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46298.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46298.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>88.82547</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46298.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>87.68183999999999</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46298.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46298.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>88.15746</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46298.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46298.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>80.88647</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46298.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>65.51000000000001</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46298.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46298.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46298.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46298.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46298.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46298.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46298.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46298.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46298.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46298.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>61.02</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46298.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46298.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46298.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>46.99</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46298.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46298.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46298.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46298.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>61.02</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46298.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46298.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46298.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46298.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>95.4966</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46298.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46298.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>102.43569</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46298.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>118.65028</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46298.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>129.65</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46298.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>119.01</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46298.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>119</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46298.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>129.65</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46298.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>128.50057</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46298.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>119.01</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46298.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>119.01</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46298.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>119.01</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46298.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>107.21755</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 610)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -470,10 +470,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46296.66666666666</v>
+        <v>46297.66666666666</v>
       </c>
       <c r="C2" t="n">
         <v>16</v>
@@ -482,18 +482,18 @@
         <v>60.48</v>
       </c>
       <c r="E2" t="n">
-        <v>1890.48251925</v>
+        <v>2613.13440375</v>
       </c>
       <c r="F2" t="n">
-        <v>31.25797816220239</v>
+        <v>43.20658736359127</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46297.16666666666</v>
+        <v>46298.25</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46297.66666666666</v>
+        <v>46298.75</v>
       </c>
       <c r="C3" t="n">
         <v>12</v>
@@ -502,10 +502,10 @@
         <v>45.36</v>
       </c>
       <c r="E3" t="n">
-        <v>1818.759111</v>
+        <v>1674.96034875</v>
       </c>
       <c r="F3" t="n">
-        <v>40.09610033068783</v>
+        <v>36.92593361441798</v>
       </c>
     </row>
   </sheetData>
@@ -551,10 +551,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B2" t="n">
-        <v>96.98999999999999</v>
+        <v>116.35347</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -572,10 +572,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46296.02083333334</v>
+        <v>46297.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>99.05251</v>
+        <v>92.93155</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -593,10 +593,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46296.04166666666</v>
+        <v>46297.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>97.13883</v>
+        <v>91.45762999999999</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -614,10 +614,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46296.0625</v>
+        <v>46297.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>97.63005</v>
+        <v>94.97615</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -635,10 +635,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46296.08333333334</v>
+        <v>46297.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>88.88</v>
+        <v>94.84296000000001</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -656,10 +656,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46296.10416666666</v>
+        <v>46297.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>88.88</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -677,10 +677,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46296.125</v>
+        <v>46297.125</v>
       </c>
       <c r="B8" t="n">
-        <v>88.88</v>
+        <v>90</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -698,10 +698,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46296.14583333334</v>
+        <v>46297.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>86.88</v>
+        <v>90</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -719,10 +719,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46296.16666666666</v>
+        <v>46297.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>86.88</v>
+        <v>90</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -740,10 +740,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46296.1875</v>
+        <v>46297.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>96.98999999999999</v>
+        <v>90</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -761,10 +761,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46296.20833333334</v>
+        <v>46297.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>95.15612</v>
+        <v>94.05391</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -772,7 +772,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -782,10 +782,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46296.22916666666</v>
+        <v>46297.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>92.5778</v>
+        <v>93.29092</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -803,10 +803,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46296.25</v>
+        <v>46297.25</v>
       </c>
       <c r="B14" t="n">
-        <v>96.98999999999999</v>
+        <v>94.99997999999999</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -824,10 +824,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46296.27083333334</v>
+        <v>46297.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>106.25588</v>
+        <v>90</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -845,10 +845,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46296.29166666666</v>
+        <v>46297.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>90.07617999999999</v>
+        <v>75.95014</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -866,10 +866,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46296.3125</v>
+        <v>46297.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>64.95014</v>
+        <v>69.42034</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -887,10 +887,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46296.33333333334</v>
+        <v>46297.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>26.07271</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -908,10 +908,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46296.35416666666</v>
+        <v>46297.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>0.99</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -919,7 +919,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -929,10 +929,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46296.375</v>
+        <v>46297.375</v>
       </c>
       <c r="B20" t="n">
-        <v>11.88</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -950,10 +950,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46296.39583333334</v>
+        <v>46297.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>51.61406</v>
+        <v>76.3</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -971,10 +971,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46296.41666666666</v>
+        <v>46297.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>25.1</v>
+        <v>64.95007</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -992,10 +992,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46296.4375</v>
+        <v>46297.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>11.88</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1013,10 +1013,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46296.45833333334</v>
+        <v>46297.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-5.17</v>
+        <v>75.95014</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1034,10 +1034,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46296.47916666666</v>
+        <v>46297.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>0.99</v>
+        <v>75.95014</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1055,10 +1055,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46296.5</v>
+        <v>46297.5</v>
       </c>
       <c r="B26" t="n">
-        <v>28.8642</v>
+        <v>75.95014</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1076,10 +1076,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46296.52083333334</v>
+        <v>46297.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>11.88</v>
+        <v>64.02</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1097,10 +1097,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46296.54166666666</v>
+        <v>46297.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>16.64713</v>
+        <v>64.95007</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1118,10 +1118,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46296.5625</v>
+        <v>46297.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>45.05655</v>
+        <v>64.95007</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1129,7 +1129,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1139,10 +1139,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46296.58333333334</v>
+        <v>46297.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>45.62481</v>
+        <v>75.95014</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1150,7 +1150,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1160,10 +1160,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46296.60416666666</v>
+        <v>46297.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>61.24946</v>
+        <v>75.96003</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1181,10 +1181,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46296.625</v>
+        <v>46297.625</v>
       </c>
       <c r="B32" t="n">
-        <v>67.18000000000001</v>
+        <v>99.01000000000001</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1202,10 +1202,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46296.64583333334</v>
+        <v>46297.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>64.89</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1223,10 +1223,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46296.66666666666</v>
+        <v>46297.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>67.18000000000001</v>
+        <v>75.95014</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1244,10 +1244,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46296.6875</v>
+        <v>46297.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>96.98999999999999</v>
+        <v>75.95014</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1265,10 +1265,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46296.70833333334</v>
+        <v>46297.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>121.01</v>
+        <v>88.88</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1276,7 +1276,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1286,10 +1286,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46296.72916666666</v>
+        <v>46297.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>299.99</v>
+        <v>119</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1297,7 +1297,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1307,10 +1307,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46296.75</v>
+        <v>46297.75</v>
       </c>
       <c r="B38" t="n">
-        <v>599.60168</v>
+        <v>129.65</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1328,10 +1328,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46296.77083333334</v>
+        <v>46297.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>499.41265</v>
+        <v>129.65</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1349,10 +1349,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46296.79166666666</v>
+        <v>46297.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>499.96</v>
+        <v>129.65</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1370,10 +1370,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46296.8125</v>
+        <v>46297.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>351.07221</v>
+        <v>124.16143</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1391,10 +1391,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46296.83333333334</v>
+        <v>46297.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>299.98</v>
+        <v>122.94671</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1402,7 +1402,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1412,10 +1412,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46296.85416666666</v>
+        <v>46297.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>499.96</v>
+        <v>129.64238</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46296.875</v>
+        <v>46297.875</v>
       </c>
       <c r="B44" t="n">
-        <v>380.26624</v>
+        <v>124.2297</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1454,10 +1454,10 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46296.89583333334</v>
+        <v>46297.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>299.99</v>
+        <v>119.01</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1465,7 +1465,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1475,10 +1475,10 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46296.91666666666</v>
+        <v>46297.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>348.48031</v>
+        <v>119</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1496,10 +1496,10 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46296.9375</v>
+        <v>46297.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>299</v>
+        <v>98.15389999999999</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1507,7 +1507,7 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1517,10 +1517,10 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46296.95833333334</v>
+        <v>46297.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>161.1737</v>
+        <v>99.6602</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1528,7 +1528,7 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1538,18 +1538,18 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46296.97916666666</v>
+        <v>46297.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>299</v>
+        <v>107.82838</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>forecast</t>
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B50" t="n">
-        <v>115.81316</v>
+        <v>108.26163</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1570,7 +1570,7 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1580,10 +1580,10 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46297.02083333334</v>
+        <v>46298.02083333334</v>
       </c>
       <c r="B51" t="n">
-        <v>96.98999999999999</v>
+        <v>108.65019</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1591,7 +1591,7 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1601,10 +1601,10 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46297.04166666666</v>
+        <v>46298.04166666666</v>
       </c>
       <c r="B52" t="n">
-        <v>106.52</v>
+        <v>106.55484</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1622,10 +1622,10 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46297.0625</v>
+        <v>46298.0625</v>
       </c>
       <c r="B53" t="n">
-        <v>95.26188999999999</v>
+        <v>102.18788</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1643,10 +1643,10 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46297.08333333334</v>
+        <v>46298.08333333334</v>
       </c>
       <c r="B54" t="n">
-        <v>93.60917000000001</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1664,7 +1664,7 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46297.10416666666</v>
+        <v>46298.10416666666</v>
       </c>
       <c r="B55" t="n">
         <v>96.98999999999999</v>
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1685,10 +1685,10 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46297.125</v>
+        <v>46298.125</v>
       </c>
       <c r="B56" t="n">
-        <v>97.41298999999999</v>
+        <v>90</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1706,10 +1706,10 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46297.14583333334</v>
+        <v>46298.14583333334</v>
       </c>
       <c r="B57" t="n">
-        <v>96.98999999999999</v>
+        <v>86.80352000000001</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1727,10 +1727,10 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46297.16666666666</v>
+        <v>46298.16666666666</v>
       </c>
       <c r="B58" t="n">
-        <v>96.98999999999999</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1738,20 +1738,20 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46297.1875</v>
+        <v>46298.1875</v>
       </c>
       <c r="B59" t="n">
-        <v>95.31774</v>
+        <v>86.2403</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1759,20 +1759,20 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46297.20833333334</v>
+        <v>46298.20833333334</v>
       </c>
       <c r="B60" t="n">
-        <v>94.00998</v>
+        <v>88.88</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1780,20 +1780,20 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46297.22916666666</v>
+        <v>46298.22916666666</v>
       </c>
       <c r="B61" t="n">
-        <v>93.00270999999999</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1801,20 +1801,20 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46297.25</v>
+        <v>46298.25</v>
       </c>
       <c r="B62" t="n">
-        <v>96.19277</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1822,7 +1822,7 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1832,10 +1832,10 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46297.27083333334</v>
+        <v>46298.27083333334</v>
       </c>
       <c r="B63" t="n">
-        <v>90</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1843,7 +1843,7 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1853,10 +1853,10 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46297.29166666666</v>
+        <v>46298.29166666666</v>
       </c>
       <c r="B64" t="n">
-        <v>75.95014</v>
+        <v>80.12014000000001</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1864,7 +1864,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1874,10 +1874,10 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46297.3125</v>
+        <v>46298.3125</v>
       </c>
       <c r="B65" t="n">
-        <v>67.05934000000001</v>
+        <v>80.12014000000001</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1895,10 +1895,10 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46297.33333333334</v>
+        <v>46298.33333333334</v>
       </c>
       <c r="B66" t="n">
-        <v>75.96017000000001</v>
+        <v>64.02</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1906,7 +1906,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1916,10 +1916,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46297.35416666666</v>
+        <v>46298.35416666666</v>
       </c>
       <c r="B67" t="n">
-        <v>75.95014</v>
+        <v>64.95007</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1937,10 +1937,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46297.375</v>
+        <v>46298.375</v>
       </c>
       <c r="B68" t="n">
-        <v>64.02</v>
+        <v>80.12014000000001</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1958,10 +1958,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46297.39583333334</v>
+        <v>46298.39583333334</v>
       </c>
       <c r="B69" t="n">
-        <v>76.3</v>
+        <v>64.02</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1979,10 +1979,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46297.41666666666</v>
+        <v>46298.41666666666</v>
       </c>
       <c r="B70" t="n">
-        <v>75.95014</v>
+        <v>76.3</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -1990,7 +1990,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2000,7 +2000,7 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46297.4375</v>
+        <v>46298.4375</v>
       </c>
       <c r="B71" t="n">
         <v>64.02</v>
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2021,10 +2021,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46297.45833333334</v>
+        <v>46298.45833333334</v>
       </c>
       <c r="B72" t="n">
-        <v>64.02</v>
+        <v>64.01957</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2032,7 +2032,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2042,10 +2042,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46297.47916666666</v>
+        <v>46298.47916666666</v>
       </c>
       <c r="B73" t="n">
-        <v>75.95014</v>
+        <v>64.02</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2063,10 +2063,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46297.5</v>
+        <v>46298.5</v>
       </c>
       <c r="B74" t="n">
-        <v>75.95014</v>
+        <v>64.02</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2074,7 +2074,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2084,10 +2084,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46297.52083333334</v>
+        <v>46298.52083333334</v>
       </c>
       <c r="B75" t="n">
-        <v>64.02</v>
+        <v>52.58588</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2095,7 +2095,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2105,10 +2105,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46297.54166666666</v>
+        <v>46298.54166666666</v>
       </c>
       <c r="B76" t="n">
-        <v>64.95007</v>
+        <v>57.3901</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2116,7 +2116,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2126,10 +2126,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46297.5625</v>
+        <v>46298.5625</v>
       </c>
       <c r="B77" t="n">
-        <v>75.96003</v>
+        <v>64.02</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2147,10 +2147,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46297.58333333334</v>
+        <v>46298.58333333334</v>
       </c>
       <c r="B78" t="n">
-        <v>75.95014</v>
+        <v>76.3</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2158,7 +2158,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2168,10 +2168,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46297.60416666666</v>
+        <v>46298.60416666666</v>
       </c>
       <c r="B79" t="n">
-        <v>75.95014</v>
+        <v>76.3</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2179,7 +2179,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2189,10 +2189,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46297.625</v>
+        <v>46298.625</v>
       </c>
       <c r="B80" t="n">
-        <v>75.9601</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2200,7 +2200,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2210,10 +2210,10 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46297.64583333334</v>
+        <v>46298.64583333334</v>
       </c>
       <c r="B81" t="n">
-        <v>75.96007</v>
+        <v>64.02</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2231,10 +2231,10 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46297.66666666666</v>
+        <v>46298.66666666666</v>
       </c>
       <c r="B82" t="n">
-        <v>75.95014</v>
+        <v>64.02</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2242,20 +2242,20 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46297.6875</v>
+        <v>46298.6875</v>
       </c>
       <c r="B83" t="n">
-        <v>75.95014</v>
+        <v>64.02</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2263,20 +2263,20 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46297.70833333334</v>
+        <v>46298.70833333334</v>
       </c>
       <c r="B84" t="n">
-        <v>88.88</v>
+        <v>89.30038999999999</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2284,20 +2284,20 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46297.72916666666</v>
+        <v>46298.72916666666</v>
       </c>
       <c r="B85" t="n">
-        <v>119</v>
+        <v>96.06162</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2305,20 +2305,20 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>46297.75</v>
+        <v>46298.75</v>
       </c>
       <c r="B86" t="n">
-        <v>129.65</v>
+        <v>117.80841</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2326,7 +2326,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2336,10 +2336,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>46297.77083333334</v>
+        <v>46298.77083333334</v>
       </c>
       <c r="B87" t="n">
-        <v>121.01</v>
+        <v>119.01</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2347,7 +2347,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2357,10 +2357,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>46297.79166666666</v>
+        <v>46298.79166666666</v>
       </c>
       <c r="B88" t="n">
-        <v>121.01</v>
+        <v>119.01</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2368,7 +2368,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2378,10 +2378,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>46297.8125</v>
+        <v>46298.8125</v>
       </c>
       <c r="B89" t="n">
-        <v>124.1558</v>
+        <v>119</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2389,7 +2389,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2399,10 +2399,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>46297.83333333334</v>
+        <v>46298.83333333334</v>
       </c>
       <c r="B90" t="n">
-        <v>129.65</v>
+        <v>119.01</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2410,7 +2410,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2420,10 +2420,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>46297.85416666666</v>
+        <v>46298.85416666666</v>
       </c>
       <c r="B91" t="n">
-        <v>127.8413</v>
+        <v>119.01</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2431,7 +2431,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2441,10 +2441,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46297.875</v>
+        <v>46298.875</v>
       </c>
       <c r="B92" t="n">
-        <v>119.01</v>
+        <v>126.16382</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2452,7 +2452,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2462,10 +2462,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>46297.89583333334</v>
+        <v>46298.89583333334</v>
       </c>
       <c r="B93" t="n">
-        <v>119.01</v>
+        <v>133.44697</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2483,10 +2483,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>46297.91666666666</v>
+        <v>46298.91666666666</v>
       </c>
       <c r="B94" t="n">
-        <v>119</v>
+        <v>119.01</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2494,7 +2494,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2504,10 +2504,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>46297.9375</v>
+        <v>46298.9375</v>
       </c>
       <c r="B95" t="n">
-        <v>98.14653</v>
+        <v>119.01</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2525,10 +2525,10 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>46297.95833333334</v>
+        <v>46298.95833333334</v>
       </c>
       <c r="B96" t="n">
-        <v>96.99309</v>
+        <v>119.01</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2536,7 +2536,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2546,10 +2546,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>46297.97916666666</v>
+        <v>46298.97916666666</v>
       </c>
       <c r="B97" t="n">
-        <v>97.81703</v>
+        <v>119.01</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2557,7 +2557,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 700)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>1200.537897</v>
+        <v>1448.74320825</v>
       </c>
       <c r="F2" t="n">
-        <v>28.87296529581529</v>
+        <v>34.84230900072149</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46299.27083333334</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46299.72916666666</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>80.004366</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.924106926406927</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -912,11 +932,11 @@
         <v>46298.375</v>
       </c>
       <c r="B20" t="n">
-        <v>64.02</v>
+        <v>75.96003</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -933,11 +953,11 @@
         <v>46298.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>64.02</v>
+        <v>76.3</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +974,11 @@
         <v>46298.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>57.3901</v>
+        <v>64.02</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +995,11 @@
         <v>46298.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>46.99</v>
+        <v>64.02</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46298.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>42.94</v>
+        <v>64.02</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46298.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>42.94</v>
+        <v>64.02</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46298.5</v>
       </c>
       <c r="B26" t="n">
-        <v>42.94</v>
+        <v>64.02</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46298.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>42.80028</v>
+        <v>64.02</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46298.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>52.21</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1121,11 @@
         <v>46298.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>42.94</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46298.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>25.1</v>
+        <v>57.3901</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1163,11 @@
         <v>46298.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>42.08</v>
+        <v>46.99</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46298.625</v>
       </c>
       <c r="B32" t="n">
-        <v>42.08</v>
+        <v>64.95007</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1205,11 @@
         <v>46298.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>57.3901</v>
+        <v>64.95007</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1226,11 @@
         <v>46298.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>57.3901</v>
+        <v>64.02</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1231,7 +1251,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1268,11 @@
         <v>46298.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>80.12014000000001</v>
+        <v>88.88</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1289,11 @@
         <v>46298.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>90</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1310,11 @@
         <v>46298.75</v>
       </c>
       <c r="B38" t="n">
-        <v>97.46984</v>
+        <v>118.65028</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,11 +1331,11 @@
         <v>46298.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>105.67</v>
+        <v>129.65</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1332,7 +1352,7 @@
         <v>46298.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>99.22116</v>
+        <v>129.65</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1353,7 +1373,7 @@
         <v>46298.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>103.61302</v>
+        <v>121.73303</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1374,7 +1394,7 @@
         <v>46298.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>102.51813</v>
+        <v>119.01</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1395,7 +1415,7 @@
         <v>46298.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>95.78762</v>
+        <v>119</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1436,7 @@
         <v>46298.875</v>
       </c>
       <c r="B44" t="n">
-        <v>105.67</v>
+        <v>129.65</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46298.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>119</v>
+        <v>119.01</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46298.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>118.65028</v>
+        <v>112.99085</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46298.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>107.04547</v>
+        <v>98.40696</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1520,7 @@
         <v>46298.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>105.21363</v>
+        <v>97.46102</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46298</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B50" t="n">
+        <v>95.33774</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46299.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46299.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>90.6327</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46299.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>89.18980000000001</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46299.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>89.33371</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46299.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>90</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46299.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>94.16755000000001</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46299.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>88.88153</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46299.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>89.93447</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46299.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46299.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>90</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46299.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>91.70981</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46299.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>93.93267</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46299.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>87.06282</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46299.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46299.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>0.1791</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46299.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>-7.58687</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46299.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>-8.21081</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>-8.14616</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46299.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>-6.62994</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46299.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>-8.01</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46299.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-9.920339999999999</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46299.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-10.01</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46299.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>-11.09656</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46299.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>-9.08</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46299.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>-9.67801</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46299.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>-9.08</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46299.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46299.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-13.58433</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46299.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-8.66527</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46299.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>-8.280950000000001</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46299.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46299.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>-5.20848</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46299.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>4e-05</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46299.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>80.98152</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46299.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>95.17846</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46299.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>127.1626</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46299.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>176.55026</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46299.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46299.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46299.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46299.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46299.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46299.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>235.58817</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46299.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46299.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>299</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46299.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46299.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>122.82939</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 611)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -470,10 +470,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46297</v>
+        <v>46298.08333333334</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46297.66666666666</v>
+        <v>46298.75</v>
       </c>
       <c r="C2" t="n">
         <v>16</v>
@@ -482,18 +482,18 @@
         <v>60.48</v>
       </c>
       <c r="E2" t="n">
-        <v>2613.13440375</v>
+        <v>2307.23846925</v>
       </c>
       <c r="F2" t="n">
-        <v>43.20658736359127</v>
+        <v>38.14878421378968</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46298.25</v>
+        <v>46299.22916666666</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46298.75</v>
+        <v>46299.72916666666</v>
       </c>
       <c r="C3" t="n">
         <v>12</v>
@@ -502,10 +502,10 @@
         <v>45.36</v>
       </c>
       <c r="E3" t="n">
-        <v>1674.96034875</v>
+        <v>325.9209329999999</v>
       </c>
       <c r="F3" t="n">
-        <v>36.92593361441798</v>
+        <v>7.185205753968253</v>
       </c>
     </row>
   </sheetData>
@@ -551,10 +551,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B2" t="n">
-        <v>116.35347</v>
+        <v>106.56351</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -562,20 +562,20 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46297.02083333334</v>
+        <v>46298.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>92.93155</v>
+        <v>98.09988</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -583,20 +583,20 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46297.04166666666</v>
+        <v>46298.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>91.45762999999999</v>
+        <v>98.90249</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -604,20 +604,20 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46297.0625</v>
+        <v>46298.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>94.97615</v>
+        <v>97.63005</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -625,20 +625,20 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46297.08333333334</v>
+        <v>46298.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>94.84296000000001</v>
+        <v>90</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -656,10 +656,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46297.10416666666</v>
+        <v>46298.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>96.98999999999999</v>
+        <v>90</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -677,10 +677,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46297.125</v>
+        <v>46298.125</v>
       </c>
       <c r="B8" t="n">
-        <v>90</v>
+        <v>88.88</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -698,10 +698,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46297.14583333334</v>
+        <v>46298.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>90</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -719,10 +719,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46297.16666666666</v>
+        <v>46298.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>90</v>
+        <v>79.36991999999999</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -740,10 +740,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46297.1875</v>
+        <v>46298.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>90</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -761,10 +761,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46297.20833333334</v>
+        <v>46298.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>94.05391</v>
+        <v>86.48804</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -772,7 +772,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -782,10 +782,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46297.22916666666</v>
+        <v>46298.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>93.29092</v>
+        <v>90</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -803,10 +803,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46297.25</v>
+        <v>46298.25</v>
       </c>
       <c r="B14" t="n">
-        <v>94.99997999999999</v>
+        <v>90</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -824,10 +824,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46297.27083333334</v>
+        <v>46298.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>90</v>
+        <v>83.98999999999999</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -845,10 +845,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46297.29166666666</v>
+        <v>46298.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>75.95014</v>
+        <v>75.9601</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -866,10 +866,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46297.3125</v>
+        <v>46298.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>69.42034</v>
+        <v>75.9601</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -887,10 +887,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46297.33333333334</v>
+        <v>46298.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>84.79000000000001</v>
+        <v>64.02</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -908,10 +908,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46297.35416666666</v>
+        <v>46298.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>84.79000000000001</v>
+        <v>64.02</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -919,7 +919,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -929,10 +929,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46297.375</v>
+        <v>46298.375</v>
       </c>
       <c r="B20" t="n">
-        <v>67.18000000000001</v>
+        <v>75.96003</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -950,7 +950,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46297.39583333334</v>
+        <v>46298.39583333334</v>
       </c>
       <c r="B21" t="n">
         <v>76.3</v>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -971,10 +971,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46297.41666666666</v>
+        <v>46298.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>64.95007</v>
+        <v>64.02</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -992,10 +992,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46297.4375</v>
+        <v>46298.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>67.18000000000001</v>
+        <v>64.02</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1013,10 +1013,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46297.45833333334</v>
+        <v>46298.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>75.95014</v>
+        <v>64.02</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1034,10 +1034,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46297.47916666666</v>
+        <v>46298.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>75.95014</v>
+        <v>64.02</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1055,10 +1055,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46297.5</v>
+        <v>46298.5</v>
       </c>
       <c r="B26" t="n">
-        <v>75.95014</v>
+        <v>64.02</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1076,7 +1076,7 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46297.52083333334</v>
+        <v>46298.52083333334</v>
       </c>
       <c r="B27" t="n">
         <v>64.02</v>
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1097,10 +1097,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46297.54166666666</v>
+        <v>46298.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>64.95007</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1118,10 +1118,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46297.5625</v>
+        <v>46298.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>64.95007</v>
+        <v>67.18000000000001</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1129,7 +1129,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1139,10 +1139,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46297.58333333334</v>
+        <v>46298.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>75.95014</v>
+        <v>57.3901</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1150,7 +1150,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1160,10 +1160,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46297.60416666666</v>
+        <v>46298.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>75.96003</v>
+        <v>46.99</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1181,10 +1181,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46297.625</v>
+        <v>46298.625</v>
       </c>
       <c r="B32" t="n">
-        <v>99.01000000000001</v>
+        <v>64.95007</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1202,10 +1202,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46297.64583333334</v>
+        <v>46298.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>96.98999999999999</v>
+        <v>64.95007</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1223,10 +1223,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46297.66666666666</v>
+        <v>46298.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>75.95014</v>
+        <v>64.02</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1234,20 +1234,20 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46297.6875</v>
+        <v>46298.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>75.95014</v>
+        <v>64.02</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1255,17 +1255,17 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46297.70833333334</v>
+        <v>46298.70833333334</v>
       </c>
       <c r="B36" t="n">
         <v>88.88</v>
@@ -1276,20 +1276,20 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46297.72916666666</v>
+        <v>46298.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>119</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1297,20 +1297,20 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46297.75</v>
+        <v>46298.75</v>
       </c>
       <c r="B38" t="n">
-        <v>129.65</v>
+        <v>118.65028</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1328,7 +1328,7 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46297.77083333334</v>
+        <v>46298.77083333334</v>
       </c>
       <c r="B39" t="n">
         <v>129.65</v>
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1349,10 +1349,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46297.79166666666</v>
+        <v>46298.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>129.65</v>
+        <v>119.01</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1370,10 +1370,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46297.8125</v>
+        <v>46298.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>124.16143</v>
+        <v>119.01</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1391,10 +1391,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46297.83333333334</v>
+        <v>46298.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>122.94671</v>
+        <v>119.01</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1402,7 +1402,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1412,10 +1412,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46297.85416666666</v>
+        <v>46298.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>129.64238</v>
+        <v>119.01</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46297.875</v>
+        <v>46298.875</v>
       </c>
       <c r="B44" t="n">
-        <v>124.2297</v>
+        <v>121.01</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1454,7 +1454,7 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46297.89583333334</v>
+        <v>46298.89583333334</v>
       </c>
       <c r="B45" t="n">
         <v>119.01</v>
@@ -1465,7 +1465,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1475,10 +1475,10 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46297.91666666666</v>
+        <v>46298.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>119</v>
+        <v>119.01</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1496,18 +1496,18 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46297.9375</v>
+        <v>46298.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>98.15389999999999</v>
+        <v>119</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>forecast</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1517,18 +1517,18 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46297.95833333334</v>
+        <v>46298.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>99.6602</v>
+        <v>107.44805</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>forecast</t>
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1538,10 +1538,10 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46297.97916666666</v>
+        <v>46298.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>107.82838</v>
+        <v>102.8908</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1549,7 +1549,7 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="B50" t="n">
-        <v>108.26163</v>
+        <v>100.51697</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1570,7 +1570,7 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1580,10 +1580,10 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46298.02083333334</v>
+        <v>46299.02083333334</v>
       </c>
       <c r="B51" t="n">
-        <v>108.65019</v>
+        <v>97.52566</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1591,7 +1591,7 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1601,10 +1601,10 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46298.04166666666</v>
+        <v>46299.04166666666</v>
       </c>
       <c r="B52" t="n">
-        <v>106.55484</v>
+        <v>98.05883</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1622,10 +1622,10 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46298.0625</v>
+        <v>46299.0625</v>
       </c>
       <c r="B53" t="n">
-        <v>102.18788</v>
+        <v>97.39503999999999</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1643,10 +1643,10 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46298.08333333334</v>
+        <v>46299.08333333334</v>
       </c>
       <c r="B54" t="n">
-        <v>96.98999999999999</v>
+        <v>99.01000000000001</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1664,10 +1664,10 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46298.10416666666</v>
+        <v>46299.10416666666</v>
       </c>
       <c r="B55" t="n">
-        <v>96.98999999999999</v>
+        <v>90.42255</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1685,10 +1685,10 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46298.125</v>
+        <v>46299.125</v>
       </c>
       <c r="B56" t="n">
-        <v>90</v>
+        <v>90.31386000000001</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1706,10 +1706,10 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46298.14583333334</v>
+        <v>46299.14583333334</v>
       </c>
       <c r="B57" t="n">
-        <v>86.80352000000001</v>
+        <v>89.35120999999999</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1727,10 +1727,10 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46298.16666666666</v>
+        <v>46299.16666666666</v>
       </c>
       <c r="B58" t="n">
-        <v>84.79000000000001</v>
+        <v>88.88</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1738,7 +1738,7 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1748,10 +1748,10 @@
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46298.1875</v>
+        <v>46299.1875</v>
       </c>
       <c r="B59" t="n">
-        <v>86.2403</v>
+        <v>90</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1759,7 +1759,7 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1769,10 +1769,10 @@
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46298.20833333334</v>
+        <v>46299.20833333334</v>
       </c>
       <c r="B60" t="n">
-        <v>88.88</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1780,7 +1780,7 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1790,7 +1790,7 @@
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46298.22916666666</v>
+        <v>46299.22916666666</v>
       </c>
       <c r="B61" t="n">
         <v>96.98999999999999</v>
@@ -1801,20 +1801,20 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46298.25</v>
+        <v>46299.25</v>
       </c>
       <c r="B62" t="n">
-        <v>96.98999999999999</v>
+        <v>99.35274</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1822,7 +1822,7 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1832,10 +1832,10 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46298.27083333334</v>
+        <v>46299.27083333334</v>
       </c>
       <c r="B63" t="n">
-        <v>83.98999999999999</v>
+        <v>90</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1843,7 +1843,7 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1853,10 +1853,10 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46298.29166666666</v>
+        <v>46299.29166666666</v>
       </c>
       <c r="B64" t="n">
-        <v>80.12014000000001</v>
+        <v>64.02</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1864,7 +1864,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1874,10 +1874,10 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46298.3125</v>
+        <v>46299.3125</v>
       </c>
       <c r="B65" t="n">
-        <v>80.12014000000001</v>
+        <v>0</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1895,10 +1895,10 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46298.33333333334</v>
+        <v>46299.33333333334</v>
       </c>
       <c r="B66" t="n">
-        <v>64.02</v>
+        <v>-9.08</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1906,7 +1906,7 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1916,10 +1916,10 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46298.35416666666</v>
+        <v>46299.35416666666</v>
       </c>
       <c r="B67" t="n">
-        <v>64.95007</v>
+        <v>-7.15635</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1937,10 +1937,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46298.375</v>
+        <v>46299.375</v>
       </c>
       <c r="B68" t="n">
-        <v>80.12014000000001</v>
+        <v>-6.5</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1958,10 +1958,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46298.39583333334</v>
+        <v>46299.39583333334</v>
       </c>
       <c r="B69" t="n">
-        <v>64.02</v>
+        <v>1.16509</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1979,10 +1979,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46298.41666666666</v>
+        <v>46299.41666666666</v>
       </c>
       <c r="B70" t="n">
-        <v>76.3</v>
+        <v>-9.08</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -1990,7 +1990,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2000,10 +2000,10 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46298.4375</v>
+        <v>46299.4375</v>
       </c>
       <c r="B71" t="n">
-        <v>64.02</v>
+        <v>0.99</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2011,7 +2011,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2021,10 +2021,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46298.45833333334</v>
+        <v>46299.45833333334</v>
       </c>
       <c r="B72" t="n">
-        <v>64.01957</v>
+        <v>-9.43174</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2032,7 +2032,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2042,10 +2042,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46298.47916666666</v>
+        <v>46299.47916666666</v>
       </c>
       <c r="B73" t="n">
-        <v>64.02</v>
+        <v>-12.93476</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2063,10 +2063,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46298.5</v>
+        <v>46299.5</v>
       </c>
       <c r="B74" t="n">
-        <v>64.02</v>
+        <v>-12.51308</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2074,7 +2074,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2084,10 +2084,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46298.52083333334</v>
+        <v>46299.52083333334</v>
       </c>
       <c r="B75" t="n">
-        <v>52.58588</v>
+        <v>-9.79982</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2095,7 +2095,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2105,10 +2105,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46298.54166666666</v>
+        <v>46299.54166666666</v>
       </c>
       <c r="B76" t="n">
-        <v>57.3901</v>
+        <v>-10.5</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2116,7 +2116,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2126,10 +2126,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46298.5625</v>
+        <v>46299.5625</v>
       </c>
       <c r="B77" t="n">
-        <v>64.02</v>
+        <v>-9.272919999999999</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2147,10 +2147,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46298.58333333334</v>
+        <v>46299.58333333334</v>
       </c>
       <c r="B78" t="n">
-        <v>76.3</v>
+        <v>-12.80843</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2158,7 +2158,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2168,10 +2168,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46298.60416666666</v>
+        <v>46299.60416666666</v>
       </c>
       <c r="B79" t="n">
-        <v>76.3</v>
+        <v>-8.29909</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2179,7 +2179,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2189,10 +2189,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46298.625</v>
+        <v>46299.625</v>
       </c>
       <c r="B80" t="n">
-        <v>67.18000000000001</v>
+        <v>-8.293710000000001</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2200,7 +2200,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2210,10 +2210,10 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46298.64583333334</v>
+        <v>46299.64583333334</v>
       </c>
       <c r="B81" t="n">
-        <v>64.02</v>
+        <v>-6.10402</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2221,7 +2221,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2231,10 +2231,10 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46298.66666666666</v>
+        <v>46299.66666666666</v>
       </c>
       <c r="B82" t="n">
-        <v>64.02</v>
+        <v>-3.20366</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2242,7 +2242,7 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2252,10 +2252,10 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46298.6875</v>
+        <v>46299.6875</v>
       </c>
       <c r="B83" t="n">
-        <v>64.02</v>
+        <v>27.69161</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2273,10 +2273,10 @@
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46298.70833333334</v>
+        <v>46299.70833333334</v>
       </c>
       <c r="B84" t="n">
-        <v>89.30038999999999</v>
+        <v>89.04602</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2284,7 +2284,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2294,10 +2294,10 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46298.72916666666</v>
+        <v>46299.72916666666</v>
       </c>
       <c r="B85" t="n">
-        <v>96.06162</v>
+        <v>100.75313</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2305,20 +2305,20 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>46298.75</v>
+        <v>46299.75</v>
       </c>
       <c r="B86" t="n">
-        <v>117.80841</v>
+        <v>167.5</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2326,7 +2326,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2336,10 +2336,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>46298.77083333334</v>
+        <v>46299.77083333334</v>
       </c>
       <c r="B87" t="n">
-        <v>119.01</v>
+        <v>181.90154</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2347,7 +2347,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2357,10 +2357,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>46298.79166666666</v>
+        <v>46299.79166666666</v>
       </c>
       <c r="B88" t="n">
-        <v>119.01</v>
+        <v>199.99</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2368,7 +2368,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2378,10 +2378,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>46298.8125</v>
+        <v>46299.8125</v>
       </c>
       <c r="B89" t="n">
-        <v>119</v>
+        <v>199.99</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2389,7 +2389,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2399,10 +2399,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>46298.83333333334</v>
+        <v>46299.83333333334</v>
       </c>
       <c r="B90" t="n">
-        <v>119.01</v>
+        <v>299.99</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2410,7 +2410,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2420,10 +2420,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>46298.85416666666</v>
+        <v>46299.85416666666</v>
       </c>
       <c r="B91" t="n">
-        <v>119.01</v>
+        <v>299.99</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2431,7 +2431,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2441,10 +2441,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46298.875</v>
+        <v>46299.875</v>
       </c>
       <c r="B92" t="n">
-        <v>126.16382</v>
+        <v>190.44831</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2452,7 +2452,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2462,10 +2462,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>46298.89583333334</v>
+        <v>46299.89583333334</v>
       </c>
       <c r="B93" t="n">
-        <v>133.44697</v>
+        <v>122.01231</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2483,10 +2483,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>46298.91666666666</v>
+        <v>46299.91666666666</v>
       </c>
       <c r="B94" t="n">
-        <v>119.01</v>
+        <v>180.35983</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2494,7 +2494,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2504,10 +2504,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>46298.9375</v>
+        <v>46299.9375</v>
       </c>
       <c r="B95" t="n">
-        <v>119.01</v>
+        <v>199.99</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2515,7 +2515,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2525,10 +2525,10 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>46298.95833333334</v>
+        <v>46299.95833333334</v>
       </c>
       <c r="B96" t="n">
-        <v>119.01</v>
+        <v>130.34938</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2536,7 +2536,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2546,10 +2546,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>46298.97916666666</v>
+        <v>46299.97916666666</v>
       </c>
       <c r="B97" t="n">
-        <v>119.01</v>
+        <v>123.90627</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2557,7 +2557,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 702)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,50 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>167.300211</v>
+        <v>113.6654805</v>
       </c>
       <c r="F2" t="n">
-        <v>4.023574098124098</v>
+        <v>2.73365753968254</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46300.02083333334</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46300.1875</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="E3" t="n">
+        <v>881.95119675</v>
+      </c>
+      <c r="F3" t="n">
+        <v>58.33010560515874</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46300.375</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46300.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>7</v>
+      </c>
+      <c r="D4" t="n">
+        <v>26.46</v>
+      </c>
+      <c r="E4" t="n">
+        <v>468.1241565</v>
+      </c>
+      <c r="F4" t="n">
+        <v>17.69176706349207</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -870,7 +910,7 @@
         <v>46299.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>0.99</v>
+        <v>-8.586119999999999</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -891,7 +931,7 @@
         <v>46299.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>1.16551</v>
+        <v>-8</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -912,11 +952,11 @@
         <v>46299.375</v>
       </c>
       <c r="B20" t="n">
-        <v>-7.79933</v>
+        <v>-8.01</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -933,11 +973,11 @@
         <v>46299.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>-9.99</v>
+        <v>5.08022</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +994,11 @@
         <v>46299.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-10.01</v>
+        <v>-6.5</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +1015,11 @@
         <v>46299.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-10.06093</v>
+        <v>-10.01</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1036,11 @@
         <v>46299.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-10.34</v>
+        <v>-9.4977</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1057,11 @@
         <v>46299.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-9.27187</v>
+        <v>-9.49081</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1078,11 @@
         <v>46299.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-9.821580000000001</v>
+        <v>-12.43166</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1099,11 @@
         <v>46299.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-9.38954</v>
+        <v>-10.01</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1120,11 @@
         <v>46299.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-9.49709</v>
+        <v>-10.01</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1141,11 @@
         <v>46299.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-10.5</v>
+        <v>-8.662409999999999</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1162,11 @@
         <v>46299.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-18.51</v>
+        <v>-9.90681</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1183,11 @@
         <v>46299.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-11.53049</v>
+        <v>-8.35195</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1204,11 @@
         <v>46299.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-9.89889</v>
+        <v>-8</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1225,11 @@
         <v>46299.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>-8.01</v>
+        <v>-6.18763</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1246,11 @@
         <v>46299.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>-3.26808</v>
+        <v>-1.42759</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1267,11 @@
         <v>46299.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>64.02</v>
+        <v>1.24504</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1288,11 @@
         <v>46299.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>96.85491</v>
+        <v>88.88006</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1309,11 @@
         <v>46299.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>117.98772</v>
+        <v>112.49</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1330,11 @@
         <v>46299.75</v>
       </c>
       <c r="B38" t="n">
-        <v>132.38253</v>
+        <v>136.36509</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,11 +1351,11 @@
         <v>46299.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>245.36423</v>
+        <v>167.5</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1332,11 +1372,11 @@
         <v>46299.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>205.87591</v>
+        <v>167.5</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1353,11 +1393,11 @@
         <v>46299.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>278.36817</v>
+        <v>123.77633</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1374,11 +1414,11 @@
         <v>46299.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>166.51531</v>
+        <v>126.28317</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -1395,7 +1435,7 @@
         <v>46299.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>167.5</v>
+        <v>129.65</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1456,7 @@
         <v>46299.875</v>
       </c>
       <c r="B44" t="n">
-        <v>299.99</v>
+        <v>122.65176</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1477,7 @@
         <v>46299.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>167.5</v>
+        <v>121.16272</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1498,7 @@
         <v>46299.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>220.5734</v>
+        <v>119</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1519,7 @@
         <v>46299.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>209.57457</v>
+        <v>119.01</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1540,7 @@
         <v>46299.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>120.09716</v>
+        <v>120.60005</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,17 +1561,1025 @@
         <v>46299.97916666666</v>
       </c>
       <c r="B49" t="n">
+        <v>119</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B50" t="n">
+        <v>126.32746</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46300.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>119</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46300.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>110.34556</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46300.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>110.09849</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46300.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>107.17</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46300.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>113.59724</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46300.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>113.39144</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46300.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>114.54</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46300.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>116.4226</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46300.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>119</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46300.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>119</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46300.22916666666</v>
+      </c>
+      <c r="B61" t="n">
         <v>119.01</v>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>forecast</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="n">
-        <v>46299</v>
-      </c>
-      <c r="E49" t="inlineStr">
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46300.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>125.11812</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46300.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>119</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46300.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>118.67</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46300.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>119</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46300.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>114.15797</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46300.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>104.5699</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46300.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46300.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46300.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46300.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>52.21</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46300.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46300.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>42.08</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46300.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46300.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46300.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46300.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>17.31734</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46300.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>25.01</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46300.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46300.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46300.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>46.99</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46300.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46300.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46300.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>104.86261</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46300.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>127.54427</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46300.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>121.1</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46300.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>128.87481</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46300.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>235.223</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46300.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>289.10782</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46300.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>305.04974</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46300.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>339.28266</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46300.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>559.6804100000001</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46300.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>299</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46300.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>338.33509</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46300.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>339.13085</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46300.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>191.01841</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46300.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>299</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 612)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,10 +470,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46298.08333333334</v>
+        <v>46299.0625</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46298.75</v>
+        <v>46299.72916666666</v>
       </c>
       <c r="C2" t="n">
         <v>16</v>
@@ -482,30 +482,50 @@
         <v>60.48</v>
       </c>
       <c r="E2" t="n">
-        <v>2307.23846925</v>
+        <v>1060.9216215</v>
       </c>
       <c r="F2" t="n">
-        <v>38.14878421378968</v>
+        <v>17.54169347718254</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46299.22916666666</v>
+        <v>46300.125</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46299.72916666666</v>
+        <v>46300.3125</v>
       </c>
       <c r="C3" t="n">
-        <v>12</v>
+        <v>4.5</v>
       </c>
       <c r="D3" t="n">
-        <v>45.36</v>
+        <v>17.01</v>
       </c>
       <c r="E3" t="n">
-        <v>325.9209329999999</v>
+        <v>1011.27309075</v>
       </c>
       <c r="F3" t="n">
-        <v>7.185205753968253</v>
+        <v>59.45168082010583</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46300.35416666666</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46300.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>28.35</v>
+      </c>
+      <c r="E4" t="n">
+        <v>575.5466925000001</v>
+      </c>
+      <c r="F4" t="n">
+        <v>20.30147063492064</v>
       </c>
     </row>
   </sheetData>
@@ -551,10 +571,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="B2" t="n">
-        <v>106.56351</v>
+        <v>103.05074</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -562,7 +582,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -572,10 +592,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46298.02083333334</v>
+        <v>46299.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>98.09988</v>
+        <v>112.86431</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -583,7 +603,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -593,10 +613,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46298.04166666666</v>
+        <v>46299.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>98.90249</v>
+        <v>102.71751</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -604,7 +624,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -614,10 +634,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46298.0625</v>
+        <v>46299.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>97.63005</v>
+        <v>104.80789</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -625,20 +645,20 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46298.08333333334</v>
+        <v>46299.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>90</v>
+        <v>98.28548000000001</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -646,7 +666,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -656,10 +676,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46298.10416666666</v>
+        <v>46299.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>90</v>
+        <v>99.90766000000001</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -667,7 +687,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -677,10 +697,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46298.125</v>
+        <v>46299.125</v>
       </c>
       <c r="B8" t="n">
-        <v>88.88</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -688,7 +708,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -698,10 +718,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46298.14583333334</v>
+        <v>46299.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>83.98999999999999</v>
+        <v>90</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -709,7 +729,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -719,10 +739,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46298.16666666666</v>
+        <v>46299.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>79.36991999999999</v>
+        <v>90</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -730,7 +750,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -740,10 +760,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46298.1875</v>
+        <v>46299.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>84.79000000000001</v>
+        <v>95.49812</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -751,7 +771,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -761,10 +781,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46298.20833333334</v>
+        <v>46299.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>86.48804</v>
+        <v>98.10745</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -772,7 +792,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -782,10 +802,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46298.22916666666</v>
+        <v>46299.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>90</v>
+        <v>97.98032000000001</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -793,7 +813,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -803,10 +823,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46298.25</v>
+        <v>46299.25</v>
       </c>
       <c r="B14" t="n">
-        <v>90</v>
+        <v>99.96784</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -814,7 +834,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -824,10 +844,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46298.27083333334</v>
+        <v>46299.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>83.98999999999999</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -835,7 +855,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -845,10 +865,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46298.29166666666</v>
+        <v>46299.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>75.9601</v>
+        <v>64.02</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -856,7 +876,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -866,10 +886,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46298.3125</v>
+        <v>46299.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>75.9601</v>
+        <v>-4.55266</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -877,7 +897,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -887,10 +907,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46298.33333333334</v>
+        <v>46299.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>64.02</v>
+        <v>-8.586119999999999</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -898,7 +918,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -908,10 +928,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46298.35416666666</v>
+        <v>46299.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>64.02</v>
+        <v>-8</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -919,7 +939,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -929,10 +949,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46298.375</v>
+        <v>46299.375</v>
       </c>
       <c r="B20" t="n">
-        <v>75.96003</v>
+        <v>-8.01</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -940,7 +960,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -950,10 +970,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46298.39583333334</v>
+        <v>46299.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>76.3</v>
+        <v>5.08022</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -961,7 +981,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -971,10 +991,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46298.41666666666</v>
+        <v>46299.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>64.02</v>
+        <v>-6.5</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -982,7 +1002,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -992,10 +1012,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46298.4375</v>
+        <v>46299.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>64.02</v>
+        <v>-10.01</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1003,7 +1023,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1013,10 +1033,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46298.45833333334</v>
+        <v>46299.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>64.02</v>
+        <v>-9.4977</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1024,7 +1044,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1034,10 +1054,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46298.47916666666</v>
+        <v>46299.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>64.02</v>
+        <v>-9.49081</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1045,7 +1065,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1055,10 +1075,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46298.5</v>
+        <v>46299.5</v>
       </c>
       <c r="B26" t="n">
-        <v>64.02</v>
+        <v>-12.43166</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1066,7 +1086,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1076,10 +1096,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46298.52083333334</v>
+        <v>46299.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>64.02</v>
+        <v>-10.01</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1087,7 +1107,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1097,10 +1117,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46298.54166666666</v>
+        <v>46299.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>67.18000000000001</v>
+        <v>-10.01</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1108,7 +1128,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1118,10 +1138,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46298.5625</v>
+        <v>46299.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>67.18000000000001</v>
+        <v>-8.662409999999999</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1129,7 +1149,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1139,10 +1159,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46298.58333333334</v>
+        <v>46299.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>57.3901</v>
+        <v>-9.90681</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1150,7 +1170,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1160,10 +1180,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46298.60416666666</v>
+        <v>46299.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>46.99</v>
+        <v>-8.35195</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1171,7 +1191,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1181,10 +1201,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46298.625</v>
+        <v>46299.625</v>
       </c>
       <c r="B32" t="n">
-        <v>64.95007</v>
+        <v>-8</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1192,7 +1212,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1202,10 +1222,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46298.64583333334</v>
+        <v>46299.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>64.95007</v>
+        <v>-6.18763</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1213,7 +1233,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1223,10 +1243,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46298.66666666666</v>
+        <v>46299.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>64.02</v>
+        <v>-1.42759</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1234,7 +1254,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1244,10 +1264,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46298.6875</v>
+        <v>46299.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>64.02</v>
+        <v>1.24504</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1255,7 +1275,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1265,10 +1285,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46298.70833333334</v>
+        <v>46299.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>88.88</v>
+        <v>88.88006</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1276,7 +1296,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1286,10 +1306,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46298.72916666666</v>
+        <v>46299.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>96.98999999999999</v>
+        <v>112.49</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1297,20 +1317,20 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46298.75</v>
+        <v>46299.75</v>
       </c>
       <c r="B38" t="n">
-        <v>118.65028</v>
+        <v>136.36509</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1318,7 +1338,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1328,10 +1348,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46298.77083333334</v>
+        <v>46299.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>129.65</v>
+        <v>167.5</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1339,7 +1359,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1349,10 +1369,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46298.79166666666</v>
+        <v>46299.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>119.01</v>
+        <v>167.5</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1360,7 +1380,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1370,10 +1390,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46298.8125</v>
+        <v>46299.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>119.01</v>
+        <v>148.26967</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1381,7 +1401,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1391,10 +1411,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46298.83333333334</v>
+        <v>46299.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>119.01</v>
+        <v>206.24895</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1402,7 +1422,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1412,10 +1432,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46298.85416666666</v>
+        <v>46299.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>119.01</v>
+        <v>299.99</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1423,7 +1443,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1433,10 +1453,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46298.875</v>
+        <v>46299.875</v>
       </c>
       <c r="B44" t="n">
-        <v>121.01</v>
+        <v>291.88043</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1444,7 +1464,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1454,10 +1474,10 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46298.89583333334</v>
+        <v>46299.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>119.01</v>
+        <v>199.99</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1465,7 +1485,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1475,10 +1495,10 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46298.91666666666</v>
+        <v>46299.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>119.01</v>
+        <v>114.65826</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1486,7 +1506,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1496,18 +1516,18 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46298.9375</v>
+        <v>46299.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>119</v>
+        <v>114.54</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1517,18 +1537,18 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46298.95833333334</v>
+        <v>46299.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>107.44805</v>
+        <v>119</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1538,18 +1558,18 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46298.97916666666</v>
+        <v>46299.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>102.8908</v>
+        <v>130.8008</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1559,10 +1579,10 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="B50" t="n">
-        <v>100.51697</v>
+        <v>137.89001</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1570,7 +1590,7 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1580,10 +1600,10 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46299.02083333334</v>
+        <v>46300.02083333334</v>
       </c>
       <c r="B51" t="n">
-        <v>97.52566</v>
+        <v>124.47871</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1591,7 +1611,7 @@
         </is>
       </c>
       <c r="D51" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1601,10 +1621,10 @@
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46299.04166666666</v>
+        <v>46300.04166666666</v>
       </c>
       <c r="B52" t="n">
-        <v>98.05883</v>
+        <v>119</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1612,7 +1632,7 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1622,10 +1642,10 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46299.0625</v>
+        <v>46300.0625</v>
       </c>
       <c r="B53" t="n">
-        <v>97.39503999999999</v>
+        <v>119</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1633,7 +1653,7 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1643,10 +1663,10 @@
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46299.08333333334</v>
+        <v>46300.08333333334</v>
       </c>
       <c r="B54" t="n">
-        <v>99.01000000000001</v>
+        <v>119</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1654,7 +1674,7 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1664,10 +1684,10 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46299.10416666666</v>
+        <v>46300.10416666666</v>
       </c>
       <c r="B55" t="n">
-        <v>90.42255</v>
+        <v>118.65028</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1675,7 +1695,7 @@
         </is>
       </c>
       <c r="D55" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1685,10 +1705,10 @@
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46299.125</v>
+        <v>46300.125</v>
       </c>
       <c r="B56" t="n">
-        <v>90.31386000000001</v>
+        <v>118.54983</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1696,20 +1716,20 @@
         </is>
       </c>
       <c r="D56" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46299.14583333334</v>
+        <v>46300.14583333334</v>
       </c>
       <c r="B57" t="n">
-        <v>89.35120999999999</v>
+        <v>116.36301</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1717,20 +1737,20 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46299.16666666666</v>
+        <v>46300.16666666666</v>
       </c>
       <c r="B58" t="n">
-        <v>88.88</v>
+        <v>118.65028</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1738,20 +1758,20 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46299.1875</v>
+        <v>46300.1875</v>
       </c>
       <c r="B59" t="n">
-        <v>90</v>
+        <v>119</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1759,20 +1779,20 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46299.20833333334</v>
+        <v>46300.20833333334</v>
       </c>
       <c r="B60" t="n">
-        <v>96.98999999999999</v>
+        <v>121.01</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1780,20 +1800,20 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46299.22916666666</v>
+        <v>46300.22916666666</v>
       </c>
       <c r="B61" t="n">
-        <v>96.98999999999999</v>
+        <v>113.5</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1801,7 +1821,7 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1811,10 +1831,10 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46299.25</v>
+        <v>46300.25</v>
       </c>
       <c r="B62" t="n">
-        <v>99.35274</v>
+        <v>113.5</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1822,7 +1842,7 @@
         </is>
       </c>
       <c r="D62" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1832,10 +1852,10 @@
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46299.27083333334</v>
+        <v>46300.27083333334</v>
       </c>
       <c r="B63" t="n">
-        <v>90</v>
+        <v>119</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -1843,7 +1863,7 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1853,10 +1873,10 @@
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46299.29166666666</v>
+        <v>46300.29166666666</v>
       </c>
       <c r="B64" t="n">
-        <v>64.02</v>
+        <v>97.63005</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -1864,7 +1884,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1874,10 +1894,10 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46299.3125</v>
+        <v>46300.3125</v>
       </c>
       <c r="B65" t="n">
-        <v>0</v>
+        <v>129.71</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -1885,20 +1905,20 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46299.33333333334</v>
+        <v>46300.33333333334</v>
       </c>
       <c r="B66" t="n">
-        <v>-9.08</v>
+        <v>119.01</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -1906,20 +1926,20 @@
         </is>
       </c>
       <c r="D66" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46299.35416666666</v>
+        <v>46300.35416666666</v>
       </c>
       <c r="B67" t="n">
-        <v>-7.15635</v>
+        <v>110.44436</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -1927,7 +1947,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -1937,10 +1957,10 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46299.375</v>
+        <v>46300.375</v>
       </c>
       <c r="B68" t="n">
-        <v>-6.5</v>
+        <v>87.66081</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -1948,7 +1968,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -1958,10 +1978,10 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46299.39583333334</v>
+        <v>46300.39583333334</v>
       </c>
       <c r="B69" t="n">
-        <v>1.16509</v>
+        <v>64.01963000000001</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -1969,7 +1989,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -1979,10 +1999,10 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46299.41666666666</v>
+        <v>46300.41666666666</v>
       </c>
       <c r="B70" t="n">
-        <v>-9.08</v>
+        <v>52.21</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -1990,7 +2010,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2000,10 +2020,10 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46299.4375</v>
+        <v>46300.4375</v>
       </c>
       <c r="B71" t="n">
-        <v>0.99</v>
+        <v>52.21</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2011,7 +2031,7 @@
         </is>
       </c>
       <c r="D71" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2021,10 +2041,10 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46299.45833333334</v>
+        <v>46300.45833333334</v>
       </c>
       <c r="B72" t="n">
-        <v>-9.43174</v>
+        <v>42.08</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2032,7 +2052,7 @@
         </is>
       </c>
       <c r="D72" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2042,10 +2062,10 @@
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46299.47916666666</v>
+        <v>46300.47916666666</v>
       </c>
       <c r="B73" t="n">
-        <v>-12.93476</v>
+        <v>1.80496</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2053,7 +2073,7 @@
         </is>
       </c>
       <c r="D73" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2063,10 +2083,10 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46299.5</v>
+        <v>46300.5</v>
       </c>
       <c r="B74" t="n">
-        <v>-12.51308</v>
+        <v>0</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2074,7 +2094,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2084,10 +2104,10 @@
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46299.52083333334</v>
+        <v>46300.52083333334</v>
       </c>
       <c r="B75" t="n">
-        <v>-9.79982</v>
+        <v>11.88</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2095,7 +2115,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2105,10 +2125,10 @@
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46299.54166666666</v>
+        <v>46300.54166666666</v>
       </c>
       <c r="B76" t="n">
-        <v>-10.5</v>
+        <v>11.88</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2116,7 +2136,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2126,10 +2146,10 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46299.5625</v>
+        <v>46300.5625</v>
       </c>
       <c r="B77" t="n">
-        <v>-9.272919999999999</v>
+        <v>25.01</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2137,7 +2157,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2147,10 +2167,10 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46299.58333333334</v>
+        <v>46300.58333333334</v>
       </c>
       <c r="B78" t="n">
-        <v>-12.80843</v>
+        <v>29.6375</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2158,7 +2178,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2168,10 +2188,10 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46299.60416666666</v>
+        <v>46300.60416666666</v>
       </c>
       <c r="B79" t="n">
-        <v>-8.29909</v>
+        <v>6.47717</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2179,7 +2199,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2189,10 +2209,10 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46299.625</v>
+        <v>46300.625</v>
       </c>
       <c r="B80" t="n">
-        <v>-8.293710000000001</v>
+        <v>46.99</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2200,7 +2220,7 @@
         </is>
       </c>
       <c r="D80" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2210,10 +2230,10 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46299.64583333334</v>
+        <v>46300.64583333334</v>
       </c>
       <c r="B81" t="n">
-        <v>-6.10402</v>
+        <v>47.99987</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2221,7 +2241,7 @@
         </is>
       </c>
       <c r="D81" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2231,10 +2251,10 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46299.66666666666</v>
+        <v>46300.66666666666</v>
       </c>
       <c r="B82" t="n">
-        <v>-3.20366</v>
+        <v>68.00069000000001</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2242,20 +2262,20 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46299.6875</v>
+        <v>46300.6875</v>
       </c>
       <c r="B83" t="n">
-        <v>27.69161</v>
+        <v>87.62674</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2263,20 +2283,20 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46299.70833333334</v>
+        <v>46300.70833333334</v>
       </c>
       <c r="B84" t="n">
-        <v>89.04602</v>
+        <v>109.05141</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2284,20 +2304,20 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46299.72916666666</v>
+        <v>46300.72916666666</v>
       </c>
       <c r="B85" t="n">
-        <v>100.75313</v>
+        <v>130.23151</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2305,7 +2325,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2315,10 +2335,10 @@
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>46299.75</v>
+        <v>46300.75</v>
       </c>
       <c r="B86" t="n">
-        <v>167.5</v>
+        <v>129.12151</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2326,7 +2346,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2336,10 +2356,10 @@
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>46299.77083333334</v>
+        <v>46300.77083333334</v>
       </c>
       <c r="B87" t="n">
-        <v>181.90154</v>
+        <v>199.99</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2347,7 +2367,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2357,10 +2377,10 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>46299.79166666666</v>
+        <v>46300.79166666666</v>
       </c>
       <c r="B88" t="n">
-        <v>199.99</v>
+        <v>280.04092</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2368,7 +2388,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2378,10 +2398,10 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>46299.8125</v>
+        <v>46300.8125</v>
       </c>
       <c r="B89" t="n">
-        <v>199.99</v>
+        <v>276.2289</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -2389,7 +2409,7 @@
         </is>
       </c>
       <c r="D89" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2399,10 +2419,10 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>46299.83333333334</v>
+        <v>46300.83333333334</v>
       </c>
       <c r="B90" t="n">
-        <v>299.99</v>
+        <v>170.97036</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2410,7 +2430,7 @@
         </is>
       </c>
       <c r="D90" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2420,10 +2440,10 @@
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>46299.85416666666</v>
+        <v>46300.85416666666</v>
       </c>
       <c r="B91" t="n">
-        <v>299.99</v>
+        <v>284.51425</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2431,7 +2451,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2441,10 +2461,10 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>46299.875</v>
+        <v>46300.875</v>
       </c>
       <c r="B92" t="n">
-        <v>190.44831</v>
+        <v>322.5488</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2452,7 +2472,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2462,10 +2482,10 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>46299.89583333334</v>
+        <v>46300.89583333334</v>
       </c>
       <c r="B93" t="n">
-        <v>122.01231</v>
+        <v>299</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2473,7 +2493,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2483,10 +2503,10 @@
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>46299.91666666666</v>
+        <v>46300.91666666666</v>
       </c>
       <c r="B94" t="n">
-        <v>180.35983</v>
+        <v>331.88084</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2494,7 +2514,7 @@
         </is>
       </c>
       <c r="D94" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2504,10 +2524,10 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>46299.9375</v>
+        <v>46300.9375</v>
       </c>
       <c r="B95" t="n">
-        <v>199.99</v>
+        <v>216.73836</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2515,7 +2535,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2525,10 +2545,10 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>46299.95833333334</v>
+        <v>46300.95833333334</v>
       </c>
       <c r="B96" t="n">
-        <v>130.34938</v>
+        <v>132.66495</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2536,7 +2556,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2546,10 +2566,10 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>46299.97916666666</v>
+        <v>46300.97916666666</v>
       </c>
       <c r="B97" t="n">
-        <v>123.90627</v>
+        <v>199.99</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2557,7 +2577,7 @@
         </is>
       </c>
       <c r="D97" s="3" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 704)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,42 +470,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46300.14583333334</v>
+        <v>46300.29166666666</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46300.3125</v>
+        <v>46300.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>15.12</v>
+        <v>34.02</v>
       </c>
       <c r="E2" t="n">
-        <v>885.7996485</v>
+        <v>966.5846775</v>
       </c>
       <c r="F2" t="n">
-        <v>58.58463283730159</v>
+        <v>28.41224801587302</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46300.375</v>
+        <v>46300.91666666666</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46300.66666666666</v>
+        <v>46301.08333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>26.46</v>
+        <v>15.12</v>
       </c>
       <c r="E3" t="n">
-        <v>748.9637999999999</v>
+        <v>1054.13377875</v>
       </c>
       <c r="F3" t="n">
-        <v>28.30551020408163</v>
+        <v>69.71784250992063</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46301.29166666666</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46301.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D4" t="n">
+        <v>34.02</v>
+      </c>
+      <c r="E4" t="n">
+        <v>266.203041</v>
+      </c>
+      <c r="F4" t="n">
+        <v>7.824898324514992</v>
       </c>
     </row>
   </sheetData>
@@ -519,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -713,7 +733,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -734,7 +754,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -755,7 +775,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -776,7 +796,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -797,7 +817,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -818,7 +838,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -839,7 +859,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -881,7 +901,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -902,7 +922,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -911,7 +931,7 @@
         <v>46300.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>118.67</v>
+        <v>110.30642</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -923,7 +943,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -932,7 +952,7 @@
         <v>46300.375</v>
       </c>
       <c r="B20" t="n">
-        <v>118.65035</v>
+        <v>87.05283</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -953,11 +973,11 @@
         <v>46300.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>101.22385</v>
+        <v>64.02</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -974,11 +994,11 @@
         <v>46300.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>64.02</v>
+        <v>42.94</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -995,11 +1015,11 @@
         <v>46300.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>42.94</v>
+        <v>25.01</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -1016,11 +1036,11 @@
         <v>46300.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>46.99</v>
+        <v>11.88</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1037,11 +1057,11 @@
         <v>46300.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>52.21</v>
+        <v>11.88</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1058,11 +1078,11 @@
         <v>46300.5</v>
       </c>
       <c r="B26" t="n">
-        <v>27.31728</v>
+        <v>25.01</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1079,11 +1099,11 @@
         <v>46300.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>46.99</v>
+        <v>40.44566</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1104,7 +1124,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1121,11 +1141,11 @@
         <v>46300.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>41.87652</v>
+        <v>25.01</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1142,11 +1162,11 @@
         <v>46300.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>46.99</v>
+        <v>41.88</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1163,11 +1183,11 @@
         <v>46300.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>42.94</v>
+        <v>25.01</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1184,11 +1204,11 @@
         <v>46300.625</v>
       </c>
       <c r="B32" t="n">
-        <v>46.99</v>
+        <v>56.90399</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1209,7 +1229,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1230,7 +1250,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1247,11 +1267,11 @@
         <v>46300.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>96.98999999999999</v>
+        <v>90</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1272,7 +1292,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1289,11 +1309,11 @@
         <v>46300.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>130.99922</v>
+        <v>134.28717</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1310,11 +1330,11 @@
         <v>46300.75</v>
       </c>
       <c r="B38" t="n">
-        <v>121.80286</v>
+        <v>121.93099</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1331,11 +1351,11 @@
         <v>46300.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>137.89</v>
+        <v>143.00071</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1352,11 +1372,11 @@
         <v>46300.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>135.62184</v>
+        <v>279.66701</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1373,11 +1393,11 @@
         <v>46300.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>184.91968</v>
+        <v>274.51635</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1394,11 +1414,11 @@
         <v>46300.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>225.75255</v>
+        <v>137.42255</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -1415,11 +1435,11 @@
         <v>46300.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>299</v>
+        <v>143.0001</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
@@ -1436,7 +1456,7 @@
         <v>46300.875</v>
       </c>
       <c r="B44" t="n">
-        <v>161.20111</v>
+        <v>158.1249</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1457,7 +1477,7 @@
         <v>46300.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>166.69336</v>
+        <v>156.27402</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1478,7 +1498,7 @@
         <v>46300.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>237.85</v>
+        <v>137.89</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1490,7 +1510,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1519,7 @@
         <v>46300.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>146.48971</v>
+        <v>134.79082</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1511,7 +1531,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1540,7 @@
         <v>46300.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>121.1</v>
+        <v>124.47483</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1532,7 +1552,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1561,7 @@
         <v>46300.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>130.01</v>
+        <v>126.43612</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1552,6 +1572,1014 @@
         <v>46300</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B50" t="n">
+        <v>148.25667</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46301.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>134.91008</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46301.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>137.89</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46301.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>136.51433</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46301.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>124.17877</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46301.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>133.22392</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46301.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>133.72391</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46301.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>132.67568</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46301.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>119.01</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46301.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>130.64019</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46301.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>138.63333</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46301.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>148.37917</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46301.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>299</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46301.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>299</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46301.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>95.55871</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46301.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>65.51000000000001</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46301.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>51.95709</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46301.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46301.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>0.01076</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46301.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>0</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46301.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>0.0108</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46301.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46301.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-5.11529</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46301.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>-2.67428</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46301.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>-5.06548</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46301.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>-1.20776</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46301.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>-5.35786</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46301.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-4.87538</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46301.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-4.4667</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46301.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46301.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>-2.92189</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46301.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>67.90604</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46301.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>87.17019000000001</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46301.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>90.20999999999999</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46301.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>118.90946</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46301.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>119</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46301.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>143.37588</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46301.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>129.65</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46301.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>127.84051</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46301.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>125.70356</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46301.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>234.32784</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46301.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>268.36093</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46301.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>241.59473</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46301.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46301.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46301.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46301.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>200.75</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46301.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 706)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,42 +470,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46301.0625</v>
+        <v>46301.29166666666</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46301.22916666666</v>
+        <v>46301.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>15.12</v>
+        <v>34.02</v>
       </c>
       <c r="E2" t="n">
-        <v>1070.925999</v>
+        <v>289.7281139999999</v>
       </c>
       <c r="F2" t="n">
-        <v>70.82843908730158</v>
+        <v>8.516405467372133</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46301.35416666666</v>
+        <v>46301.91666666666</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46301.64583333334</v>
+        <v>46302.08333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>26.46</v>
+        <v>15.12</v>
       </c>
       <c r="E3" t="n">
-        <v>209.078883</v>
+        <v>904.4711520000001</v>
       </c>
       <c r="F3" t="n">
-        <v>7.901696258503403</v>
+        <v>59.81952063492064</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46302.29166666666</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46302.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D4" t="n">
+        <v>34.02</v>
+      </c>
+      <c r="E4" t="n">
+        <v>221.444925</v>
+      </c>
+      <c r="F4" t="n">
+        <v>6.509257054673721</v>
       </c>
     </row>
   </sheetData>
@@ -519,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -629,7 +649,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -650,7 +670,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -671,7 +691,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -692,7 +712,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -713,7 +733,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -734,7 +754,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -755,7 +775,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -776,7 +796,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -860,7 +880,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -881,7 +901,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -902,7 +922,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -995,7 +1015,7 @@
         <v>46301.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>64.95</v>
+        <v>0</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1016,7 +1036,7 @@
         <v>46301.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>52.21</v>
+        <v>-2.79745</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1037,7 +1057,7 @@
         <v>46301.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>25.1</v>
+        <v>-6.5</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1058,11 +1078,11 @@
         <v>46301.5</v>
       </c>
       <c r="B26" t="n">
-        <v>24.96487</v>
+        <v>-5.03516</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1079,11 +1099,11 @@
         <v>46301.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>24.94</v>
+        <v>0.00984</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1100,11 +1120,11 @@
         <v>46301.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>5.48126</v>
+        <v>-5.12583</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1121,11 +1141,11 @@
         <v>46301.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-2.71539</v>
+        <v>-4.91155</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1142,11 +1162,11 @@
         <v>46301.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-6.54575</v>
+        <v>-4.93285</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1163,11 +1183,11 @@
         <v>46301.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-7.28463</v>
+        <v>-4.37285</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1184,11 +1204,11 @@
         <v>46301.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-4.70405</v>
+        <v>18.53144</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1205,11 +1225,11 @@
         <v>46301.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>40.34488</v>
+        <v>41.60183</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1217,7 +1237,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1226,11 +1246,11 @@
         <v>46301.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>86.78682000000001</v>
+        <v>84.79000000000001</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1247,11 +1267,11 @@
         <v>46301.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>86.94862999999999</v>
+        <v>90.55507</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1268,11 +1288,11 @@
         <v>46301.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>121.01</v>
+        <v>118.65028</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1289,11 +1309,11 @@
         <v>46301.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>199.97905</v>
+        <v>120.894</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1310,11 +1330,11 @@
         <v>46301.75</v>
       </c>
       <c r="B38" t="n">
-        <v>145.02</v>
+        <v>151.49176</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1331,11 +1351,11 @@
         <v>46301.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>137.67</v>
+        <v>146.11</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1352,11 +1372,11 @@
         <v>46301.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>136.06037</v>
+        <v>146.11</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1373,11 +1393,11 @@
         <v>46301.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>125.30898</v>
+        <v>146.11</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1394,11 +1414,11 @@
         <v>46301.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>137.67</v>
+        <v>112.09641</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -1415,11 +1435,11 @@
         <v>46301.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>137.89006</v>
+        <v>116.23617</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
@@ -1436,7 +1456,7 @@
         <v>46301.875</v>
       </c>
       <c r="B44" t="n">
-        <v>119.01</v>
+        <v>115.84164</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1457,7 +1477,7 @@
         <v>46301.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>126.32459</v>
+        <v>115.08059</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1478,7 +1498,7 @@
         <v>46301.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>179.48449</v>
+        <v>110.98</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1490,7 +1510,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1519,7 @@
         <v>46301.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>128.66056</v>
+        <v>110.98</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1511,7 +1531,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1540,7 @@
         <v>46301.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>199.99</v>
+        <v>111.38216</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1532,7 +1552,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1561,7 @@
         <v>46301.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>199.99</v>
+        <v>119.01</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1552,6 +1572,1014 @@
         <v>46301</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B50" t="n">
+        <v>119.01</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46302.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>119</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46302.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>118.65028</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46302.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>118.65028</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46302.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>117.12066</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46302.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>113.5</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46302.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>102.93449</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46302.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>103.59778</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46302.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>100.56095</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46302.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>122.40548</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46302.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>121.1</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46302.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>121.1</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46302.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>131.36937</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46302.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>128.65337</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46302.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>80.12035</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46302.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46302.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>43.01</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46302.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>25.15</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46302.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>6.00716</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46302.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>-6e-05</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46302.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>-5.17</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46302.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-5.84321</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46302.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-5.17</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46302.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46302.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46302.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>-4.72918</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>0</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46302.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-5.49605</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46302.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46302.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-5.57546</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46302.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>-2.90055</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46302.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>0</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46302.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>51.77496</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46302.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46302.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>80.12014000000001</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46302.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>93.32324</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46302.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>121.04871</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46302.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>129.69</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46302.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>129.65</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46302.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>129.65</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46302.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>137.89</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46302.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>129.65</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46302.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>129.69</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46302.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>121.01</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46302.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>121.01</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46302.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>126.59086</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46302.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>129.65</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46302.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>129.65</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 614)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -470,10 +470,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46301.66666666666</v>
+        <v>46302.66666666666</v>
       </c>
       <c r="C2" t="n">
         <v>16</v>
@@ -482,10 +482,10 @@
         <v>60.48</v>
       </c>
       <c r="E2" t="n">
-        <v>2653.8667545</v>
+        <v>2061.57922425</v>
       </c>
       <c r="F2" t="n">
-        <v>43.88007199900795</v>
+        <v>34.08695807291667</v>
       </c>
     </row>
   </sheetData>
@@ -531,10 +531,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B2" t="n">
-        <v>177.82296</v>
+        <v>119</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -552,10 +552,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46301.02083333334</v>
+        <v>46302.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>143.0001</v>
+        <v>113.06068</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -573,18 +573,18 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46301.04166666666</v>
+        <v>46302.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>150.85824</v>
+        <v>119</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>forecast</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -594,18 +594,18 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46301.0625</v>
+        <v>46302.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>157.11104</v>
+        <v>121.01</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>forecast</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -615,18 +615,18 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46301.08333333334</v>
+        <v>46302.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>143.22923</v>
+        <v>115.59353</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>forecast</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -636,10 +636,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46301.10416666666</v>
+        <v>46302.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>122.84595</v>
+        <v>114.92596</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -657,10 +657,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46301.125</v>
+        <v>46302.125</v>
       </c>
       <c r="B8" t="n">
-        <v>130.23</v>
+        <v>110.29051</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -678,10 +678,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46301.14583333334</v>
+        <v>46302.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>140.67457</v>
+        <v>114.54</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -699,10 +699,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46301.16666666666</v>
+        <v>46302.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>130.23</v>
+        <v>113.5</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -720,10 +720,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46301.1875</v>
+        <v>46302.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>152.78611</v>
+        <v>121.1</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -741,10 +741,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46301.20833333334</v>
+        <v>46302.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>199.99</v>
+        <v>121.1</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -762,10 +762,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46301.22916666666</v>
+        <v>46302.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>166.27121</v>
+        <v>130.10878</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -783,10 +783,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46301.25</v>
+        <v>46302.25</v>
       </c>
       <c r="B14" t="n">
-        <v>299</v>
+        <v>132.15265</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -804,10 +804,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46301.27083333334</v>
+        <v>46302.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>299.99</v>
+        <v>120.17772</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -825,10 +825,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46301.29166666666</v>
+        <v>46302.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>99.01000000000001</v>
+        <v>81.38142000000001</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -836,7 +836,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -846,10 +846,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46301.3125</v>
+        <v>46302.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>71.00576</v>
+        <v>69.02645</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -867,10 +867,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46301.33333333334</v>
+        <v>46302.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>64.02</v>
+        <v>43.01</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -888,10 +888,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46301.35416666666</v>
+        <v>46302.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>24.15254</v>
+        <v>25.15</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -909,10 +909,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46301.375</v>
+        <v>46302.375</v>
       </c>
       <c r="B20" t="n">
-        <v>7.55273</v>
+        <v>17.83433</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -920,7 +920,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -930,10 +930,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46301.39583333334</v>
+        <v>46302.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>5.98501</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -951,10 +951,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46301.41666666666</v>
+        <v>46302.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-2.99803</v>
+        <v>42.08</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -972,10 +972,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46301.4375</v>
+        <v>46302.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-1.32105</v>
+        <v>25.1</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -983,7 +983,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -993,10 +993,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46301.45833333334</v>
+        <v>46302.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-2.95255</v>
+        <v>25.1</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1014,10 +1014,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46301.47916666666</v>
+        <v>46302.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-4.55172</v>
+        <v>25.1</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1035,10 +1035,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46301.5</v>
+        <v>46302.5</v>
       </c>
       <c r="B26" t="n">
-        <v>0</v>
+        <v>-5.17</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1046,7 +1046,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1056,10 +1056,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46301.52083333334</v>
+        <v>46302.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-3.02848</v>
+        <v>2e-05</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1077,10 +1077,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46301.54166666666</v>
+        <v>46302.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>5.1297</v>
+        <v>7.56696</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1088,7 +1088,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1098,10 +1098,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46301.5625</v>
+        <v>46302.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-5.14304</v>
+        <v>-5.02</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1109,7 +1109,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1119,10 +1119,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46301.58333333334</v>
+        <v>46302.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-5.08966</v>
+        <v>0</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1140,10 +1140,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46301.60416666666</v>
+        <v>46302.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-4.95292</v>
+        <v>-1.23</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1161,10 +1161,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46301.625</v>
+        <v>46302.625</v>
       </c>
       <c r="B32" t="n">
-        <v>24.64184</v>
+        <v>45.98094</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1172,7 +1172,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1182,10 +1182,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46301.64583333334</v>
+        <v>46302.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>42.40009</v>
+        <v>46.98527</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1203,10 +1203,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46301.66666666666</v>
+        <v>46302.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>83.98999999999999</v>
+        <v>64.02</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1224,10 +1224,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46301.6875</v>
+        <v>46302.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>92.22475</v>
+        <v>64.02</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1245,10 +1245,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46301.70833333334</v>
+        <v>46302.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>110.98</v>
+        <v>88.38278</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1256,7 +1256,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1266,10 +1266,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46301.72916666666</v>
+        <v>46302.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>123.20069</v>
+        <v>103.97678</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1277,7 +1277,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1287,10 +1287,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46301.75</v>
+        <v>46302.75</v>
       </c>
       <c r="B38" t="n">
-        <v>335.80268</v>
+        <v>123.61107</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1308,10 +1308,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46301.77083333334</v>
+        <v>46302.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>320.89608</v>
+        <v>144.36007</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1329,10 +1329,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46301.79166666666</v>
+        <v>46302.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>146.11</v>
+        <v>129.65</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1340,7 +1340,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1350,10 +1350,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46301.8125</v>
+        <v>46302.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>198.53884</v>
+        <v>129.69805</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1361,7 +1361,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1371,10 +1371,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46301.83333333334</v>
+        <v>46302.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>203.01493</v>
+        <v>129.69</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1392,10 +1392,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46301.85416666666</v>
+        <v>46302.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>311.06862</v>
+        <v>129.69</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1413,10 +1413,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46301.875</v>
+        <v>46302.875</v>
       </c>
       <c r="B44" t="n">
-        <v>146.11</v>
+        <v>129.69</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1424,7 +1424,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1434,10 +1434,10 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46301.89583333334</v>
+        <v>46302.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>311.44664</v>
+        <v>121.01</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1445,7 +1445,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1455,10 +1455,10 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46301.91666666666</v>
+        <v>46302.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>299.99</v>
+        <v>121.01</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1466,7 +1466,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1476,10 +1476,10 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46301.9375</v>
+        <v>46302.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>299</v>
+        <v>121.01</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1497,10 +1497,10 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46301.95833333334</v>
+        <v>46302.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>299</v>
+        <v>129.54189</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1508,7 +1508,7 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1518,10 +1518,10 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46301.97916666666</v>
+        <v>46302.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>199.99</v>
+        <v>130.66537</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 708)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,22 +470,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46302.20833333334</v>
+        <v>46302.29166666666</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46302.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>41.58</v>
+        <v>34.02</v>
       </c>
       <c r="E2" t="n">
-        <v>1647.408282</v>
+        <v>399.5117295000001</v>
       </c>
       <c r="F2" t="n">
-        <v>39.62020880230881</v>
+        <v>11.74343708112875</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46302.91666666666</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46303.08333333334</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="E3" t="n">
+        <v>764.35664175</v>
+      </c>
+      <c r="F3" t="n">
+        <v>50.55268794642858</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46303.29166666666</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46303.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D4" t="n">
+        <v>34.02</v>
+      </c>
+      <c r="E4" t="n">
+        <v>772.470582</v>
+      </c>
+      <c r="F4" t="n">
+        <v>22.70636631393299</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -756,7 +796,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -777,7 +817,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -798,7 +838,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -819,7 +859,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -912,7 +952,7 @@
         <v>46302.375</v>
       </c>
       <c r="B20" t="n">
-        <v>76.3</v>
+        <v>25.85235</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -933,7 +973,7 @@
         <v>46302.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>76.3</v>
+        <v>25.1</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -954,11 +994,11 @@
         <v>46302.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>76.3</v>
+        <v>25.1</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +1015,11 @@
         <v>46302.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>76.3</v>
+        <v>0</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1036,11 @@
         <v>46302.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>67.44</v>
+        <v>1.16484</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1057,11 @@
         <v>46302.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>67.44</v>
+        <v>-6.43898</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1078,11 @@
         <v>46302.5</v>
       </c>
       <c r="B26" t="n">
-        <v>66.32958000000001</v>
+        <v>-5.7075</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1099,11 @@
         <v>46302.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>62.24716</v>
+        <v>4e-05</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1120,11 @@
         <v>46302.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>63.72</v>
+        <v>23.95</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1141,11 @@
         <v>46302.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>62.47547</v>
+        <v>-5.29361</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1162,11 @@
         <v>46302.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>59.15034</v>
+        <v>-2.84352</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1183,11 @@
         <v>46302.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>63.72</v>
+        <v>0</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1204,11 @@
         <v>46302.625</v>
       </c>
       <c r="B32" t="n">
-        <v>64.02</v>
+        <v>47.48929</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1225,11 @@
         <v>46302.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>67.18000000000001</v>
+        <v>51.69509</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1246,11 @@
         <v>46302.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>67.44</v>
+        <v>64.02</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1267,11 @@
         <v>46302.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>67.44</v>
+        <v>64.02</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1288,11 @@
         <v>46302.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>81.19974000000001</v>
+        <v>91.75014</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1309,11 @@
         <v>46302.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>111.57539</v>
+        <v>118.6503</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1330,11 @@
         <v>46302.75</v>
       </c>
       <c r="B38" t="n">
-        <v>121.01</v>
+        <v>129.65</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,11 +1351,11 @@
         <v>46302.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>129.69</v>
+        <v>169.28399</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1332,11 +1372,11 @@
         <v>46302.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>121.47102</v>
+        <v>129.65</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1353,11 +1393,11 @@
         <v>46302.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>123.28912</v>
+        <v>121.01</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1374,11 +1414,11 @@
         <v>46302.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>129.69</v>
+        <v>97.81807000000001</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -1395,11 +1435,11 @@
         <v>46302.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>124.15383</v>
+        <v>98.59357</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
@@ -1416,7 +1456,7 @@
         <v>46302.875</v>
       </c>
       <c r="B44" t="n">
-        <v>121.87945</v>
+        <v>105.38478</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1477,7 @@
         <v>46302.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>121.01</v>
+        <v>99.46668</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1498,7 @@
         <v>46302.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>121.01</v>
+        <v>98.66186999999999</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1470,7 +1510,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1519,7 @@
         <v>46302.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>121.01</v>
+        <v>101.75713</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1491,7 +1531,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1540,7 @@
         <v>46302.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>121.01</v>
+        <v>97.94665000000001</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1512,7 +1552,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1561,7 @@
         <v>46302.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>130.72191</v>
+        <v>97.63005</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1572,1014 @@
         <v>46302</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B50" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46303.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>96.98983</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46303.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46303.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46303.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>100</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46303.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>97.63005</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46303.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>100</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46303.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>97.63005</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46303.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>97.63005</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46303.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>114.54</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46303.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>121.1</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46303.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>127.2569</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46303.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>130.71626</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46303.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>129.69</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46303.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46303.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46303.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46303.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>50.93592</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46303.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46303.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46303.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>25.15</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46303.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>39.07647</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46303.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>43.01</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46303.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>52.21</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46303.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>26.38924</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46303.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>15.80677</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>24.54032</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46303.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>29.9888</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46303.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>42.08</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46303.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>25.15</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46303.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>43.01</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46303.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46303.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46303.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>88.89</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46303.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>121.01</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46303.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>167.5</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46303.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>327.05492</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46303.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>325.5366</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46303.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>258.94132</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46303.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>201.22125</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46303.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>990</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46303.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>297.99</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46303.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>212.6727</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46303.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>209.35145</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46303.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>200.76115</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46303.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46303.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46303.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 615)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -470,10 +470,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46302.66666666666</v>
+        <v>46303.66666666666</v>
       </c>
       <c r="C2" t="n">
         <v>16</v>
@@ -482,10 +482,10 @@
         <v>60.48</v>
       </c>
       <c r="E2" t="n">
-        <v>2061.57922425</v>
+        <v>2368.1720595</v>
       </c>
       <c r="F2" t="n">
-        <v>34.08695807291667</v>
+        <v>39.15628405257936</v>
       </c>
     </row>
   </sheetData>
@@ -531,10 +531,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B2" t="n">
-        <v>119</v>
+        <v>108.27201</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -552,10 +552,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46302.02083333334</v>
+        <v>46303.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>113.06068</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -573,18 +573,18 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46302.04166666666</v>
+        <v>46303.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>119</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -594,10 +594,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46302.0625</v>
+        <v>46303.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>121.01</v>
+        <v>100</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -615,10 +615,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46302.08333333334</v>
+        <v>46303.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>115.59353</v>
+        <v>103.10411</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -636,10 +636,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46302.10416666666</v>
+        <v>46303.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>114.92596</v>
+        <v>106.32054</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -657,10 +657,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46302.125</v>
+        <v>46303.125</v>
       </c>
       <c r="B8" t="n">
-        <v>110.29051</v>
+        <v>100</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -678,10 +678,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46302.14583333334</v>
+        <v>46303.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>114.54</v>
+        <v>116.0543</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -699,10 +699,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46302.16666666666</v>
+        <v>46303.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>113.5</v>
+        <v>107.64305</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -720,10 +720,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46302.1875</v>
+        <v>46303.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>121.1</v>
+        <v>116.92766</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -741,10 +741,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46302.20833333334</v>
+        <v>46303.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>121.1</v>
+        <v>123.35994</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -762,10 +762,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46302.22916666666</v>
+        <v>46303.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>130.10878</v>
+        <v>129.69</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -783,10 +783,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46302.25</v>
+        <v>46303.25</v>
       </c>
       <c r="B14" t="n">
-        <v>132.15265</v>
+        <v>129.69</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -804,10 +804,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46302.27083333334</v>
+        <v>46303.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>120.17772</v>
+        <v>133.04165</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -825,10 +825,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46302.29166666666</v>
+        <v>46303.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>81.38142000000001</v>
+        <v>97.63005</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -836,7 +836,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -846,10 +846,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46302.3125</v>
+        <v>46303.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>69.02645</v>
+        <v>64.97</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -867,10 +867,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46302.33333333334</v>
+        <v>46303.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>43.01</v>
+        <v>64.02</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -888,10 +888,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46302.35416666666</v>
+        <v>46303.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>25.15</v>
+        <v>64.95</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -909,10 +909,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46302.375</v>
+        <v>46303.375</v>
       </c>
       <c r="B20" t="n">
-        <v>17.83433</v>
+        <v>64.95</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -920,7 +920,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -930,10 +930,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46302.39583333334</v>
+        <v>46303.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>5.98501</v>
+        <v>42.94</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -951,10 +951,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46302.41666666666</v>
+        <v>46303.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>42.08</v>
+        <v>42.94</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -972,10 +972,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46302.4375</v>
+        <v>46303.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>25.1</v>
+        <v>43.01</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -983,7 +983,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -993,10 +993,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46302.45833333334</v>
+        <v>46303.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>25.1</v>
+        <v>25.15</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1014,10 +1014,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46302.47916666666</v>
+        <v>46303.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>25.1</v>
+        <v>42.94</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1035,10 +1035,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46302.5</v>
+        <v>46303.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-5.17</v>
+        <v>43.01</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1046,7 +1046,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1056,10 +1056,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46302.52083333334</v>
+        <v>46303.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>2e-05</v>
+        <v>42.94</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1077,10 +1077,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46302.54166666666</v>
+        <v>46303.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>7.56696</v>
+        <v>25.15</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1088,7 +1088,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1098,10 +1098,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46302.5625</v>
+        <v>46303.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-5.02</v>
+        <v>27.01638</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1109,7 +1109,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1119,10 +1119,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46302.58333333334</v>
+        <v>46303.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>0</v>
+        <v>27.61864</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1140,10 +1140,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46302.60416666666</v>
+        <v>46303.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-1.23</v>
+        <v>43.01</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1161,10 +1161,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46302.625</v>
+        <v>46303.625</v>
       </c>
       <c r="B32" t="n">
-        <v>45.98094</v>
+        <v>43.01</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1172,7 +1172,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1182,10 +1182,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46302.64583333334</v>
+        <v>46303.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>46.98527</v>
+        <v>55.55609</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1203,10 +1203,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46302.66666666666</v>
+        <v>46303.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>64.02</v>
+        <v>80.12009</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1224,10 +1224,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46302.6875</v>
+        <v>46303.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>64.02</v>
+        <v>100.88865</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1245,10 +1245,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46302.70833333334</v>
+        <v>46303.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>88.38278</v>
+        <v>121.01</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1256,7 +1256,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1266,10 +1266,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46302.72916666666</v>
+        <v>46303.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>103.97678</v>
+        <v>187.66778</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1277,7 +1277,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1287,10 +1287,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46302.75</v>
+        <v>46303.75</v>
       </c>
       <c r="B38" t="n">
-        <v>123.61107</v>
+        <v>327.21793</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1308,10 +1308,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46302.77083333334</v>
+        <v>46303.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>144.36007</v>
+        <v>332.94077</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1329,10 +1329,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46302.79166666666</v>
+        <v>46303.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>129.65</v>
+        <v>299.8</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1340,7 +1340,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1350,10 +1350,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46302.8125</v>
+        <v>46303.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>129.69805</v>
+        <v>205.28645</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1361,7 +1361,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1371,10 +1371,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46302.83333333334</v>
+        <v>46303.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>129.69</v>
+        <v>359.01268</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1392,10 +1392,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46302.85416666666</v>
+        <v>46303.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>129.69</v>
+        <v>299.81</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1413,10 +1413,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46302.875</v>
+        <v>46303.875</v>
       </c>
       <c r="B44" t="n">
-        <v>129.69</v>
+        <v>299.81</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1424,7 +1424,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1434,10 +1434,10 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46302.89583333334</v>
+        <v>46303.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>121.01</v>
+        <v>299.81</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1445,7 +1445,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1455,10 +1455,10 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46302.91666666666</v>
+        <v>46303.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>121.01</v>
+        <v>271.21082</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1466,7 +1466,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1476,10 +1476,10 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46302.9375</v>
+        <v>46303.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>121.01</v>
+        <v>299.81</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1497,10 +1497,10 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46302.95833333334</v>
+        <v>46303.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>129.54189</v>
+        <v>299.81</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1508,7 +1508,7 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1518,10 +1518,10 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46302.97916666666</v>
+        <v>46303.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>130.66537</v>
+        <v>299.81</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 710)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,22 +470,62 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46303.20833333334</v>
+        <v>46303.29166666666</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46303.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>41.58</v>
+        <v>34.02</v>
       </c>
       <c r="E2" t="n">
-        <v>1487.036421</v>
+        <v>837.20173875</v>
       </c>
       <c r="F2" t="n">
-        <v>35.76326168831168</v>
+        <v>24.60910460758378</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46303.91666666666</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46304.08333333334</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1338.507222</v>
+      </c>
+      <c r="F3" t="n">
+        <v>88.52560992063492</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46304.29166666666</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46304.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D4" t="n">
+        <v>34.02</v>
+      </c>
+      <c r="E4" t="n">
+        <v>101.9905185</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.997957627865961</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -756,7 +796,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -777,7 +817,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -798,7 +838,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -819,7 +859,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -933,7 +973,7 @@
         <v>46303.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>53.15</v>
+        <v>43.01</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -954,7 +994,7 @@
         <v>46303.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>53.15</v>
+        <v>41.88</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -975,11 +1015,11 @@
         <v>46303.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>53.15</v>
+        <v>42.94</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1036,11 @@
         <v>46303.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>53.15</v>
+        <v>43.01</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1057,11 @@
         <v>46303.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>53.15</v>
+        <v>52.21</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1078,11 @@
         <v>46303.5</v>
       </c>
       <c r="B26" t="n">
-        <v>53.15</v>
+        <v>43.01</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1099,11 @@
         <v>46303.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>53.15</v>
+        <v>25.15</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1120,11 @@
         <v>46303.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>53.15</v>
+        <v>43.01</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1141,11 @@
         <v>46303.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>51.60212</v>
+        <v>27.32304</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1162,11 @@
         <v>46303.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>53.15</v>
+        <v>42.94</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1183,11 @@
         <v>46303.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>53.15</v>
+        <v>43.01</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1204,11 @@
         <v>46303.625</v>
       </c>
       <c r="B32" t="n">
-        <v>53.15</v>
+        <v>43.01</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1225,11 @@
         <v>46303.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>63.32585</v>
+        <v>61.70542</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1246,11 @@
         <v>46303.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>95.15133</v>
+        <v>80.12009</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1267,11 @@
         <v>46303.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>113.76443</v>
+        <v>98.25327</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1288,11 @@
         <v>46303.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>128.10566</v>
+        <v>121.01</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1309,11 @@
         <v>46303.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>167.5</v>
+        <v>266.13194</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1330,11 @@
         <v>46303.75</v>
       </c>
       <c r="B38" t="n">
-        <v>275.75616</v>
+        <v>329.59911</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,11 +1351,11 @@
         <v>46303.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>280.44074</v>
+        <v>319.70997</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1332,11 +1372,11 @@
         <v>46303.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>273.46496</v>
+        <v>350.69798</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1353,11 +1393,11 @@
         <v>46303.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>338.0111</v>
+        <v>339.24419</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1374,11 +1414,11 @@
         <v>46303.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>299.81</v>
+        <v>168.96</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -1395,11 +1435,11 @@
         <v>46303.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>359.24057</v>
+        <v>200.75</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
@@ -1416,7 +1456,7 @@
         <v>46303.875</v>
       </c>
       <c r="B44" t="n">
-        <v>340.49308</v>
+        <v>200.75</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1477,7 @@
         <v>46303.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>299.81</v>
+        <v>200.75</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1498,7 @@
         <v>46303.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>299.8</v>
+        <v>129.65</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1470,7 +1510,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1519,7 @@
         <v>46303.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>299</v>
+        <v>200.75</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1491,7 +1531,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1540,7 @@
         <v>46303.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>293.52837</v>
+        <v>167.49</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1512,7 +1552,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -1521,17 +1561,1025 @@
         <v>46303.97916666666</v>
       </c>
       <c r="B49" t="n">
+        <v>237.85</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B50" t="n">
+        <v>247.74577</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46304.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>129.7</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46304.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>129.7</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46304.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>129.94215</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46304.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>130.04284</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46304.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>137.38695</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46304.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>157.0232</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46304.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>130.14551</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46304.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>146.11</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46304.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>146.11</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46304.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46304.22916666666</v>
+      </c>
+      <c r="B61" t="n">
         <v>299.81</v>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>forecast</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="n">
-        <v>46303</v>
-      </c>
-      <c r="E49" t="inlineStr">
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46304.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>299.81</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46304.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>129.69</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46304.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>86.35982</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46304.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>64.95</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46304.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46304.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46304.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46304.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46304.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46304.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46304.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46304.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46304.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46304.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>-5.54</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>-8</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46304.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-8.07634</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46304.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-8</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46304.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-8.51296</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46304.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>-8.41183</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46304.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>-8.263030000000001</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46304.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46304.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>69.93843</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46304.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>98.83965999999999</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46304.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>131.17423</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46304.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46304.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>136.34103</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46304.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>194.64231</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46304.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>130.01</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46304.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>518.24572</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46304.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>321.35817</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46304.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>299.98</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46304.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>262.94715</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46304.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>139.0413</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46304.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>129.69</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46304.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>100.84815</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46304.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 616)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,22 +470,42 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46303</v>
+        <v>46304.16666666666</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46303.66666666666</v>
+        <v>46304.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D2" t="n">
-        <v>60.48</v>
+        <v>45.36</v>
       </c>
       <c r="E2" t="n">
-        <v>2368.1720595</v>
+        <v>1767.35517075</v>
       </c>
       <c r="F2" t="n">
-        <v>39.15628405257936</v>
+        <v>38.96285649801588</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46304.83333333334</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1418.1257805</v>
+      </c>
+      <c r="F3" t="n">
+        <v>93.79138759920636</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,10 +551,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46303</v>
+        <v>46304.02083333334</v>
       </c>
       <c r="B2" t="n">
-        <v>108.27201</v>
+        <v>297.56</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -542,20 +562,20 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46303.02083333334</v>
+        <v>46304.04166666666</v>
       </c>
       <c r="B3" t="n">
-        <v>96.98999999999999</v>
+        <v>234.6502</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -563,41 +583,41 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46303.04166666666</v>
+        <v>46304.0625</v>
       </c>
       <c r="B4" t="n">
-        <v>96.98999999999999</v>
+        <v>234.65025</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>forecast</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46303.0625</v>
+        <v>46304.08333333334</v>
       </c>
       <c r="B5" t="n">
-        <v>100</v>
+        <v>234.65025</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -605,20 +625,20 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46303.08333333334</v>
+        <v>46304.10416666666</v>
       </c>
       <c r="B6" t="n">
-        <v>103.10411</v>
+        <v>242.58099</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -626,20 +646,20 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46303.10416666666</v>
+        <v>46304.125</v>
       </c>
       <c r="B7" t="n">
-        <v>106.32054</v>
+        <v>241.12334</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -647,20 +667,20 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46303.125</v>
+        <v>46304.14583333334</v>
       </c>
       <c r="B8" t="n">
-        <v>100</v>
+        <v>244.22853</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -668,20 +688,20 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46303.14583333334</v>
+        <v>46304.16666666666</v>
       </c>
       <c r="B9" t="n">
-        <v>116.0543</v>
+        <v>264.74756</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -689,7 +709,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -699,10 +719,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46303.16666666666</v>
+        <v>46304.1875</v>
       </c>
       <c r="B10" t="n">
-        <v>107.64305</v>
+        <v>264.59866</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -710,7 +730,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -720,10 +740,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46303.1875</v>
+        <v>46304.20833333334</v>
       </c>
       <c r="B11" t="n">
-        <v>116.92766</v>
+        <v>299</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -731,7 +751,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -741,10 +761,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46303.20833333334</v>
+        <v>46304.22916666666</v>
       </c>
       <c r="B12" t="n">
-        <v>123.35994</v>
+        <v>299.81</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -752,7 +772,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -762,10 +782,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46303.22916666666</v>
+        <v>46304.25</v>
       </c>
       <c r="B13" t="n">
-        <v>129.69</v>
+        <v>299.99</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -773,7 +793,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -783,10 +803,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46303.25</v>
+        <v>46304.27083333334</v>
       </c>
       <c r="B14" t="n">
-        <v>129.69</v>
+        <v>260.65423</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -794,7 +814,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -804,10 +824,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46303.27083333334</v>
+        <v>46304.29166666666</v>
       </c>
       <c r="B15" t="n">
-        <v>133.04165</v>
+        <v>101.44493</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -815,7 +835,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -825,10 +845,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46303.29166666666</v>
+        <v>46304.3125</v>
       </c>
       <c r="B16" t="n">
-        <v>97.63005</v>
+        <v>75.9601</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -836,7 +856,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -846,10 +866,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46303.3125</v>
+        <v>46304.33333333334</v>
       </c>
       <c r="B17" t="n">
-        <v>64.97</v>
+        <v>0.9</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -857,7 +877,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -867,10 +887,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46303.33333333334</v>
+        <v>46304.35416666666</v>
       </c>
       <c r="B18" t="n">
-        <v>64.02</v>
+        <v>0.9</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -878,7 +898,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -888,10 +908,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46303.35416666666</v>
+        <v>46304.375</v>
       </c>
       <c r="B19" t="n">
-        <v>64.95</v>
+        <v>0.9</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -899,7 +919,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -909,10 +929,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46303.375</v>
+        <v>46304.39583333334</v>
       </c>
       <c r="B20" t="n">
-        <v>64.95</v>
+        <v>0.9</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -920,7 +940,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -930,10 +950,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46303.39583333334</v>
+        <v>46304.41666666666</v>
       </c>
       <c r="B21" t="n">
-        <v>42.94</v>
+        <v>0.9</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -941,7 +961,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -951,10 +971,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46303.41666666666</v>
+        <v>46304.4375</v>
       </c>
       <c r="B22" t="n">
-        <v>42.94</v>
+        <v>0.9</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -962,7 +982,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -972,10 +992,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46303.4375</v>
+        <v>46304.45833333334</v>
       </c>
       <c r="B23" t="n">
-        <v>43.01</v>
+        <v>0.9</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -983,7 +1003,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -993,10 +1013,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46303.45833333334</v>
+        <v>46304.47916666666</v>
       </c>
       <c r="B24" t="n">
-        <v>25.15</v>
+        <v>0.9</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1004,7 +1024,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1014,10 +1034,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46303.47916666666</v>
+        <v>46304.5</v>
       </c>
       <c r="B25" t="n">
-        <v>42.94</v>
+        <v>0.9</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1025,7 +1045,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1035,10 +1055,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46303.5</v>
+        <v>46304.52083333334</v>
       </c>
       <c r="B26" t="n">
-        <v>43.01</v>
+        <v>-7.69435</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1046,7 +1066,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1056,10 +1076,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46303.52083333334</v>
+        <v>46304.54166666666</v>
       </c>
       <c r="B27" t="n">
-        <v>42.94</v>
+        <v>-10.5</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1067,7 +1087,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1077,10 +1097,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46303.54166666666</v>
+        <v>46304.5625</v>
       </c>
       <c r="B28" t="n">
-        <v>25.15</v>
+        <v>-10.5</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1088,7 +1108,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1098,10 +1118,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46303.5625</v>
+        <v>46304.58333333334</v>
       </c>
       <c r="B29" t="n">
-        <v>27.01638</v>
+        <v>-8.380000000000001</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1109,7 +1129,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1119,10 +1139,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46303.58333333334</v>
+        <v>46304.60416666666</v>
       </c>
       <c r="B30" t="n">
-        <v>27.61864</v>
+        <v>-8.09989</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1130,7 +1150,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1140,10 +1160,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46303.60416666666</v>
+        <v>46304.625</v>
       </c>
       <c r="B31" t="n">
-        <v>43.01</v>
+        <v>-8.45927</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1151,7 +1171,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1161,10 +1181,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46303.625</v>
+        <v>46304.64583333334</v>
       </c>
       <c r="B32" t="n">
-        <v>43.01</v>
+        <v>-8</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1172,7 +1192,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1182,10 +1202,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46303.64583333334</v>
+        <v>46304.66666666666</v>
       </c>
       <c r="B33" t="n">
-        <v>55.55609</v>
+        <v>17.72946</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1193,20 +1213,20 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46303.66666666666</v>
+        <v>46304.6875</v>
       </c>
       <c r="B34" t="n">
-        <v>80.12009</v>
+        <v>75.9601</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1214,7 +1234,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1224,10 +1244,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46303.6875</v>
+        <v>46304.70833333334</v>
       </c>
       <c r="B35" t="n">
-        <v>100.88865</v>
+        <v>114.16818</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1235,7 +1255,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1245,10 +1265,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46303.70833333334</v>
+        <v>46304.72916666666</v>
       </c>
       <c r="B36" t="n">
-        <v>121.01</v>
+        <v>138.19332</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1256,7 +1276,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1266,10 +1286,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46303.72916666666</v>
+        <v>46304.75</v>
       </c>
       <c r="B37" t="n">
-        <v>187.66778</v>
+        <v>199.99</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1277,7 +1297,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1287,10 +1307,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46303.75</v>
+        <v>46304.77083333334</v>
       </c>
       <c r="B38" t="n">
-        <v>327.21793</v>
+        <v>195.37102</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1298,7 +1318,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1308,10 +1328,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46303.77083333334</v>
+        <v>46304.79166666666</v>
       </c>
       <c r="B39" t="n">
-        <v>332.94077</v>
+        <v>146.11</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1319,7 +1339,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1329,10 +1349,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46303.79166666666</v>
+        <v>46304.8125</v>
       </c>
       <c r="B40" t="n">
-        <v>299.8</v>
+        <v>146.11</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1340,7 +1360,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1350,10 +1370,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46303.8125</v>
+        <v>46304.83333333334</v>
       </c>
       <c r="B41" t="n">
-        <v>205.28645</v>
+        <v>198.77062</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1361,20 +1381,20 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46303.83333333334</v>
+        <v>46304.85416666666</v>
       </c>
       <c r="B42" t="n">
-        <v>359.01268</v>
+        <v>206.85458</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1382,20 +1402,20 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46303.85416666666</v>
+        <v>46304.875</v>
       </c>
       <c r="B43" t="n">
-        <v>299.81</v>
+        <v>299.8</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1403,20 +1423,20 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46303.875</v>
+        <v>46304.89583333334</v>
       </c>
       <c r="B44" t="n">
-        <v>299.81</v>
+        <v>213.53357</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1424,20 +1444,20 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46303.89583333334</v>
+        <v>46304.91666666666</v>
       </c>
       <c r="B45" t="n">
-        <v>299.81</v>
+        <v>160.71605</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1445,20 +1465,20 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46303.91666666666</v>
+        <v>46304.9375</v>
       </c>
       <c r="B46" t="n">
-        <v>271.21082</v>
+        <v>141.50528</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1466,20 +1486,20 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46303.9375</v>
+        <v>46304.95833333334</v>
       </c>
       <c r="B47" t="n">
-        <v>299.81</v>
+        <v>123.69402</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1487,20 +1507,20 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46303.95833333334</v>
+        <v>46304.97916666666</v>
       </c>
       <c r="B48" t="n">
-        <v>299.81</v>
+        <v>109.61386</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1508,32 +1528,11 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>OFF</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="n">
-        <v>46303.97916666666</v>
-      </c>
-      <c r="B49" t="n">
-        <v>299.81</v>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>forecast</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="n">
-        <v>46303</v>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update latest output (run 712)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,30 +470,30 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46304.375</v>
+        <v>46304.29166666666</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>46304.66666666666</v>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
-        <v>26.46</v>
+        <v>34.02</v>
       </c>
       <c r="E2" t="n">
-        <v>33.98082675000001</v>
+        <v>126.35669475</v>
       </c>
       <c r="F2" t="n">
-        <v>1.284233815192744</v>
+        <v>3.714188558201057</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46304.83333333334</v>
+        <v>46304.91666666666</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46305</v>
+        <v>46305.08333333334</v>
       </c>
       <c r="C3" t="n">
         <v>4</v>
@@ -502,10 +502,30 @@
         <v>15.12</v>
       </c>
       <c r="E3" t="n">
-        <v>1047.381816</v>
+        <v>812.38722825</v>
       </c>
       <c r="F3" t="n">
-        <v>69.27128412698414</v>
+        <v>53.72931403769842</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46305.29166666666</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D4" t="n">
+        <v>34.02</v>
+      </c>
+      <c r="E4" t="n">
+        <v>336.268023</v>
+      </c>
+      <c r="F4" t="n">
+        <v>9.884421604938272</v>
       </c>
     </row>
   </sheetData>
@@ -519,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -860,7 +880,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -881,7 +901,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -902,7 +922,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -923,7 +943,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -974,7 +994,7 @@
         <v>46304.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>42.94</v>
+        <v>0.9</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -995,7 +1015,7 @@
         <v>46304.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>40.3126</v>
+        <v>0.9</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1020,7 +1040,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1037,11 +1057,11 @@
         <v>46304.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>0.9</v>
+        <v>-5.17</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1062,7 +1082,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1083,7 +1103,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1100,11 +1120,11 @@
         <v>46304.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-9.1563</v>
+        <v>-7.89901</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1121,11 +1141,11 @@
         <v>46304.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-9.08</v>
+        <v>-6.51</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1142,11 +1162,11 @@
         <v>46304.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-9.30073</v>
+        <v>-7.82536</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1163,11 +1183,11 @@
         <v>46304.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-9.08</v>
+        <v>-8.03912</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1184,11 +1204,11 @@
         <v>46304.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-9.32344</v>
+        <v>-8</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1205,11 +1225,11 @@
         <v>46304.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>-7.86</v>
+        <v>-8.01</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1226,11 +1246,11 @@
         <v>46304.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>2e-05</v>
+        <v>4e-05</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1247,11 +1267,11 @@
         <v>46304.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>83.06013</v>
+        <v>75.9601</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1268,11 +1288,11 @@
         <v>46304.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>110.98</v>
+        <v>114.17673</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1289,11 +1309,11 @@
         <v>46304.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>119</v>
+        <v>135.84878</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1310,11 +1330,11 @@
         <v>46304.75</v>
       </c>
       <c r="B38" t="n">
-        <v>132.36287</v>
+        <v>297.99</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1331,11 +1351,11 @@
         <v>46304.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>127.28044</v>
+        <v>199.30695</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1352,11 +1372,11 @@
         <v>46304.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>142.9802</v>
+        <v>154.36123</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1373,11 +1393,11 @@
         <v>46304.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>137.54752</v>
+        <v>146.11</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1394,11 +1414,11 @@
         <v>46304.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>199.99005</v>
+        <v>167.48</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -1406,7 +1426,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -1415,11 +1435,11 @@
         <v>46304.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>153.21977</v>
+        <v>130.01</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
@@ -1427,7 +1447,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1456,7 @@
         <v>46304.875</v>
       </c>
       <c r="B44" t="n">
-        <v>133.38548</v>
+        <v>272.93895</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1448,7 +1468,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1477,7 @@
         <v>46304.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>133.87475</v>
+        <v>167.48</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1469,7 +1489,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1498,7 @@
         <v>46304.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>135.82223</v>
+        <v>129.69</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1499,7 +1519,7 @@
         <v>46304.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>120.95548</v>
+        <v>129.69</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1520,7 +1540,7 @@
         <v>46304.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1541,19 +1561,1027 @@
         <v>46304.97916666666</v>
       </c>
       <c r="B49" t="n">
+        <v>97.07293</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B50" t="n">
         <v>96.98999999999999</v>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>forecast</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="n">
-        <v>46304</v>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>ON</t>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46305.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46305.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>82.71997</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46305.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>81.06477</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46305.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>73.90243</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46305.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>75.37671</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46305.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>74.92214</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46305.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>87.60751</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46305.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>72.27958</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46305.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>74.93462</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46305.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>85.38386</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46305.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>96.99014</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46305.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>99.18199</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46305.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>87.23354999999999</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46305.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46305.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46305.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>46.50031</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46305.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46305.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>25.15</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46305.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46305.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46305.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46305.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>0</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46305.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>3e-05</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46305.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46305.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46305.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>0</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46305.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-5.0402</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46305.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-4.50494</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46305.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-5.29467</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46305.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>56.67403</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46305.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>66.02572000000001</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>114.99576</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46305.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>121.1</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46305.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>192.35062</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46305.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>323.13718</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46305.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>340.46862</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46305.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>329.20062</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46305.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46305.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>297.99</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46305.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46305.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>343.27594</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46305.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46305.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46305.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46305.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46305.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46305.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update latest output (run 617)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -470,42 +470,42 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46304.16666666666</v>
+        <v>46305</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46304.66666666666</v>
+        <v>46305.1875</v>
       </c>
       <c r="C2" t="n">
-        <v>12</v>
+        <v>4.5</v>
       </c>
       <c r="D2" t="n">
-        <v>45.36</v>
+        <v>17.01</v>
       </c>
       <c r="E2" t="n">
-        <v>1767.35517075</v>
+        <v>866.4046852499999</v>
       </c>
       <c r="F2" t="n">
-        <v>38.96285649801588</v>
+        <v>50.93501970899471</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46304.83333333334</v>
+        <v>46305.20833333334</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46305</v>
+        <v>46305.6875</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>11.5</v>
       </c>
       <c r="D3" t="n">
-        <v>15.12</v>
+        <v>43.47</v>
       </c>
       <c r="E3" t="n">
-        <v>1418.1257805</v>
+        <v>865.7002282499999</v>
       </c>
       <c r="F3" t="n">
-        <v>93.79138759920636</v>
+        <v>19.91488907867495</v>
       </c>
     </row>
   </sheetData>
@@ -519,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,10 +551,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46304.02083333334</v>
+        <v>46305</v>
       </c>
       <c r="B2" t="n">
-        <v>297.56</v>
+        <v>119</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -562,20 +562,20 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46304.04166666666</v>
+        <v>46305.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>234.6502</v>
+        <v>100</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -583,20 +583,20 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46304.0625</v>
+        <v>46305.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>234.65025</v>
+        <v>96.99014</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -604,20 +604,20 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46304.08333333334</v>
+        <v>46305.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>234.65025</v>
+        <v>97.63005</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -625,20 +625,20 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46304.10416666666</v>
+        <v>46305.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>242.58099</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -646,20 +646,20 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46304.125</v>
+        <v>46305.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>241.12334</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -667,20 +667,20 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46304.14583333334</v>
+        <v>46305.125</v>
       </c>
       <c r="B8" t="n">
-        <v>244.22853</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -688,20 +688,20 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46304.16666666666</v>
+        <v>46305.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>264.74756</v>
+        <v>87.04000000000001</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -719,10 +719,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46304.1875</v>
+        <v>46305.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>264.59866</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -740,10 +740,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46304.20833333334</v>
+        <v>46305.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>299</v>
+        <v>120.00007</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -751,20 +751,20 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46304.22916666666</v>
+        <v>46305.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>299.81</v>
+        <v>96.99014</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -772,7 +772,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -782,10 +782,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46304.25</v>
+        <v>46305.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>299.99</v>
+        <v>100</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -803,10 +803,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46304.27083333334</v>
+        <v>46305.25</v>
       </c>
       <c r="B14" t="n">
-        <v>260.65423</v>
+        <v>109.77624</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -824,10 +824,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46304.29166666666</v>
+        <v>46305.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>101.44493</v>
+        <v>86.07635000000001</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -845,10 +845,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46304.3125</v>
+        <v>46305.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>75.9601</v>
+        <v>64.02</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -866,10 +866,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46304.33333333334</v>
+        <v>46305.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>0.9</v>
+        <v>25.15</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -887,10 +887,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46304.35416666666</v>
+        <v>46305.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>0.9</v>
+        <v>42.94</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -908,10 +908,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46304.375</v>
+        <v>46305.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>0.9</v>
+        <v>29.66726</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -919,7 +919,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -929,10 +929,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46304.39583333334</v>
+        <v>46305.375</v>
       </c>
       <c r="B20" t="n">
-        <v>0.9</v>
+        <v>29.55907</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -950,10 +950,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46304.41666666666</v>
+        <v>46305.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>0.9</v>
+        <v>11.88</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -971,10 +971,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46304.4375</v>
+        <v>46305.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>0.9</v>
+        <v>2.38664</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -982,7 +982,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -992,10 +992,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46304.45833333334</v>
+        <v>46305.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>0.9</v>
+        <v>25.1</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46304.47916666666</v>
+        <v>46305.45833333334</v>
       </c>
       <c r="B24" t="n">
         <v>0.9</v>
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1034,10 +1034,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46304.5</v>
+        <v>46305.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>0.9</v>
+        <v>3e-05</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1055,10 +1055,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46304.52083333334</v>
+        <v>46305.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-7.69435</v>
+        <v>0.9</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1076,10 +1076,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46304.54166666666</v>
+        <v>46305.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-10.5</v>
+        <v>24.52702</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1097,10 +1097,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46304.5625</v>
+        <v>46305.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-10.5</v>
+        <v>23.88063</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1118,10 +1118,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46304.58333333334</v>
+        <v>46305.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-8.380000000000001</v>
+        <v>-4.69495</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1129,7 +1129,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1139,10 +1139,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46304.60416666666</v>
+        <v>46305.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-8.09989</v>
+        <v>-1.15573</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1150,7 +1150,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1160,10 +1160,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46304.625</v>
+        <v>46305.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-8.45927</v>
+        <v>22.85928</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1181,10 +1181,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46304.64583333334</v>
+        <v>46305.625</v>
       </c>
       <c r="B32" t="n">
-        <v>-8</v>
+        <v>23.65049</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1202,10 +1202,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46304.66666666666</v>
+        <v>46305.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>17.72946</v>
+        <v>64.02</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1213,20 +1213,20 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46304.6875</v>
+        <v>46305.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>75.9601</v>
+        <v>109.4652</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1234,20 +1234,20 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46304.70833333334</v>
+        <v>46305.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>114.16818</v>
+        <v>125.77579</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1265,10 +1265,10 @@
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46304.72916666666</v>
+        <v>46305.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>138.19332</v>
+        <v>261.43281</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1276,7 +1276,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1286,10 +1286,10 @@
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46304.75</v>
+        <v>46305.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>199.99</v>
+        <v>332.2569</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1297,7 +1297,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1307,10 +1307,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46304.77083333334</v>
+        <v>46305.75</v>
       </c>
       <c r="B38" t="n">
-        <v>195.37102</v>
+        <v>349.52506</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1328,10 +1328,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46304.79166666666</v>
+        <v>46305.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>146.11</v>
+        <v>333.37805</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1349,10 +1349,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46304.8125</v>
+        <v>46305.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>146.11</v>
+        <v>346.84938</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1370,10 +1370,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46304.83333333334</v>
+        <v>46305.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>198.77062</v>
+        <v>299.99</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1381,20 +1381,20 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46304.85416666666</v>
+        <v>46305.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>206.85458</v>
+        <v>299.99</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1402,20 +1402,20 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46304.875</v>
+        <v>46305.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>299.8</v>
+        <v>341.01874</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1423,20 +1423,20 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46304.89583333334</v>
+        <v>46305.875</v>
       </c>
       <c r="B44" t="n">
-        <v>213.53357</v>
+        <v>338.69059</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1444,20 +1444,20 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46304.91666666666</v>
+        <v>46305.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>160.71605</v>
+        <v>299.99</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1465,20 +1465,20 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46304.9375</v>
+        <v>46305.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>141.50528</v>
+        <v>299.99</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1486,20 +1486,20 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46304.95833333334</v>
+        <v>46305.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>123.69402</v>
+        <v>318.74561</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1507,20 +1507,20 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46304.97916666666</v>
+        <v>46305.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>109.61386</v>
+        <v>296.07756</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1528,11 +1528,32 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>46305.97916666666</v>
+      </c>
+      <c r="B49" t="n">
+        <v>212.56945</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update latest output (run 714)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,10 +470,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46305.22916666666</v>
+        <v>46305.20833333334</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46305.6875</v>
+        <v>46305.66666666666</v>
       </c>
       <c r="C2" t="n">
         <v>11</v>
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>1241.24029575</v>
+        <v>740.4488325</v>
       </c>
       <c r="F2" t="n">
-        <v>29.85185896464646</v>
+        <v>17.80781222943723</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46306.25</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46306.70833333334</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>444.5170177500001</v>
+      </c>
+      <c r="F3" t="n">
+        <v>10.69064496753247</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -756,7 +776,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
@@ -912,7 +932,7 @@
         <v>46305.375</v>
       </c>
       <c r="B20" t="n">
-        <v>90.65000000000001</v>
+        <v>29.55895</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -933,7 +953,7 @@
         <v>46305.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>90.65000000000001</v>
+        <v>25.15</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -954,11 +974,11 @@
         <v>46305.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>90.65000000000001</v>
+        <v>25.1</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +995,11 @@
         <v>46305.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>88.89</v>
+        <v>2.29761</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46305.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>64.02</v>
+        <v>0.9</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46305.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>42.93</v>
+        <v>3e-05</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46305.5</v>
       </c>
       <c r="B26" t="n">
-        <v>52.21</v>
+        <v>0.9</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46305.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>26.05459</v>
+        <v>6.85907</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46305.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>25.34222</v>
+        <v>10.09365</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1121,11 @@
         <v>46305.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>26.12</v>
+        <v>-4.8196</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46305.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>40.95196</v>
+        <v>-4.51511</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1163,11 @@
         <v>46305.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>1.83823</v>
+        <v>0.00065</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46305.625</v>
       </c>
       <c r="B32" t="n">
-        <v>42.6827</v>
+        <v>57.03183</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1205,11 @@
         <v>46305.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>56.3464</v>
+        <v>66.01524999999999</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1226,11 @@
         <v>46305.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>85.85850000000001</v>
+        <v>109.45351</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1218,7 +1238,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
@@ -1227,11 +1247,11 @@
         <v>46305.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>119</v>
+        <v>126.7109</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1268,11 @@
         <v>46305.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>143.78288</v>
+        <v>289.88</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1289,11 @@
         <v>46305.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>200.82471</v>
+        <v>332.20741</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1310,11 @@
         <v>46305.75</v>
       </c>
       <c r="B38" t="n">
-        <v>280.89589</v>
+        <v>349.49329</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,11 +1331,11 @@
         <v>46305.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>297.99</v>
+        <v>335.46219</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1332,11 +1352,11 @@
         <v>46305.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>293.78701</v>
+        <v>324.38957</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1353,11 +1373,11 @@
         <v>46305.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>299.81</v>
+        <v>164.11</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1374,11 +1394,11 @@
         <v>46305.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>299.8</v>
+        <v>146.11</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -1395,7 +1415,7 @@
         <v>46305.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>299.81</v>
+        <v>126.91</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1416,7 +1436,7 @@
         <v>46305.875</v>
       </c>
       <c r="B44" t="n">
-        <v>299.81</v>
+        <v>140.88696</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46305.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>299.8</v>
+        <v>210</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46305.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>299.81</v>
+        <v>163.58526</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46305.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>297.99</v>
+        <v>150.59625</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1520,7 @@
         <v>46305.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>297.99</v>
+        <v>166.67005</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,7 +1541,7 @@
         <v>46305.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>289.88</v>
+        <v>163.64</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46305</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B50" t="n">
+        <v>156.82565</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46306.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>145.60684</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46306.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>148.67407</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46306.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>145.11487</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46306.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>143.43631</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46306.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>142.62</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46306.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>130.22</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46306.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>137.67</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46306.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>130.22</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46306.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>154.96981</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46306.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>152.97545</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46306.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>154.01077</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46306.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>130.33236</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46306.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>87.70359000000001</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46306.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46306.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46306.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>25.15</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46306.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46306.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>-6.5</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46306.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>-6.51</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46306.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>-9.42498</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46306.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-9.2547</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46306.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-9.174189999999999</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46306.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>-23.5</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46306.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>-10.5</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46306.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>-9.666119999999999</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46306.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>-18.51</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46306.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>-23.5</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46306.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>-9.08</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46306.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>-7.6879</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46306.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>-5.07397</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46306.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46306.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>108.9708</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46306.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>96.98999999999999</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46306.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>133.99249</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46306.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>137.67</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46306.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>353.91622</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46306.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>517.04731</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46306.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>342.22145</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46306.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>361.49029</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46306.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>360.17299</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46306.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>499</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46306.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46306.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46306.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46306.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46306.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46306.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>299.99</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 618)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,42 +470,22 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46305</v>
+        <v>46306.0625</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46305.1875</v>
+        <v>46306.72916666666</v>
       </c>
       <c r="C2" t="n">
-        <v>4.5</v>
+        <v>16</v>
       </c>
       <c r="D2" t="n">
-        <v>17.01</v>
+        <v>60.48</v>
       </c>
       <c r="E2" t="n">
-        <v>866.4046852499999</v>
+        <v>1857.663209999999</v>
       </c>
       <c r="F2" t="n">
-        <v>50.93501970899471</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>46305.20833333334</v>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>46305.6875</v>
-      </c>
-      <c r="C3" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="D3" t="n">
-        <v>43.47</v>
-      </c>
-      <c r="E3" t="n">
-        <v>865.7002282499999</v>
-      </c>
-      <c r="F3" t="n">
-        <v>19.91488907867495</v>
+        <v>30.7153308531746</v>
       </c>
     </row>
   </sheetData>
@@ -551,10 +531,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="B2" t="n">
-        <v>119</v>
+        <v>137.05622</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -562,41 +542,41 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46305.02083333334</v>
+        <v>46306.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>100</v>
+        <v>152.89228</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>historical</t>
+          <t>forecast</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46305.04166666666</v>
+        <v>46306.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>96.99014</v>
+        <v>156.08731</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -604,20 +584,20 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>OFF</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46305.0625</v>
+        <v>46306.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>97.63005</v>
+        <v>149.49336</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -625,7 +605,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -635,10 +615,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46305.08333333334</v>
+        <v>46306.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>96.98999999999999</v>
+        <v>152.52671</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -646,7 +626,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -656,10 +636,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46305.10416666666</v>
+        <v>46306.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>96.98999999999999</v>
+        <v>123.39695</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -667,7 +647,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -677,10 +657,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46305.125</v>
+        <v>46306.125</v>
       </c>
       <c r="B8" t="n">
-        <v>96.98999999999999</v>
+        <v>152.73703</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -688,7 +668,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -698,10 +678,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46305.14583333334</v>
+        <v>46306.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>87.04000000000001</v>
+        <v>153.76487</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -709,7 +689,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -719,10 +699,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46305.16666666666</v>
+        <v>46306.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>96.98999999999999</v>
+        <v>152.84596</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -730,7 +710,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -740,10 +720,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46305.1875</v>
+        <v>46306.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>120.00007</v>
+        <v>152.86632</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -751,20 +731,20 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46305.20833333334</v>
+        <v>46306.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>96.99014</v>
+        <v>130.01</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -772,7 +752,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -782,10 +762,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46305.22916666666</v>
+        <v>46306.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>100</v>
+        <v>151.98421</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -793,7 +773,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -803,10 +783,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46305.25</v>
+        <v>46306.25</v>
       </c>
       <c r="B14" t="n">
-        <v>109.77624</v>
+        <v>137.94391</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -814,7 +794,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -824,10 +804,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46305.27083333334</v>
+        <v>46306.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>86.07635000000001</v>
+        <v>80.12009</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -835,7 +815,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -845,10 +825,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46305.29166666666</v>
+        <v>46306.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>64.02</v>
+        <v>63.74113</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -856,7 +836,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -866,10 +846,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46305.3125</v>
+        <v>46306.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>25.15</v>
+        <v>51.86838</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -877,7 +857,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -887,10 +867,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46305.33333333334</v>
+        <v>46306.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>42.94</v>
+        <v>33.8616</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -898,7 +878,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -908,10 +888,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46305.35416666666</v>
+        <v>46306.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>29.66726</v>
+        <v>11.88</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -919,7 +899,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -929,10 +909,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46305.375</v>
+        <v>46306.375</v>
       </c>
       <c r="B20" t="n">
-        <v>29.55907</v>
+        <v>-2.28805</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -940,7 +920,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -950,10 +930,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46305.39583333334</v>
+        <v>46306.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>11.88</v>
+        <v>5.75782</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -961,7 +941,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -971,10 +951,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46305.41666666666</v>
+        <v>46306.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>2.38664</v>
+        <v>-9.413399999999999</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -982,7 +962,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -992,10 +972,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46305.4375</v>
+        <v>46306.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>25.1</v>
+        <v>-10.01</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1003,7 +983,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1013,10 +993,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46305.45833333334</v>
+        <v>46306.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>0.9</v>
+        <v>-9.45725</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1024,7 +1004,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1034,10 +1014,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46305.47916666666</v>
+        <v>46306.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>3e-05</v>
+        <v>-18.51</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1045,7 +1025,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1055,10 +1035,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46305.5</v>
+        <v>46306.5</v>
       </c>
       <c r="B26" t="n">
-        <v>0.9</v>
+        <v>-24.99064</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1066,7 +1046,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1076,10 +1056,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46305.52083333334</v>
+        <v>46306.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>24.52702</v>
+        <v>-18.51</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1087,7 +1067,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1097,10 +1077,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46305.54166666666</v>
+        <v>46306.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>23.88063</v>
+        <v>-18.48</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1108,7 +1088,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1118,10 +1098,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46305.5625</v>
+        <v>46306.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-4.69495</v>
+        <v>-12.19929</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1129,7 +1109,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1139,10 +1119,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46305.58333333334</v>
+        <v>46306.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-1.15573</v>
+        <v>-9.78486</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1150,7 +1130,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1160,10 +1140,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46305.60416666666</v>
+        <v>46306.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>22.85928</v>
+        <v>-7.65584</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1171,7 +1151,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1181,10 +1161,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46305.625</v>
+        <v>46306.625</v>
       </c>
       <c r="B32" t="n">
-        <v>23.65049</v>
+        <v>0</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1192,7 +1172,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1202,10 +1182,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46305.64583333334</v>
+        <v>46306.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>64.02</v>
+        <v>27.01652</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1213,7 +1193,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1223,10 +1203,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46305.66666666666</v>
+        <v>46306.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>109.4652</v>
+        <v>80.12007</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1234,7 +1214,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1244,10 +1224,10 @@
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>46305.6875</v>
+        <v>46306.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>125.77579</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1255,20 +1235,20 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>46305.70833333334</v>
+        <v>46306.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>261.43281</v>
+        <v>137.67</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1276,20 +1256,20 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46305.72916666666</v>
+        <v>46306.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>332.2569</v>
+        <v>301.4723</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1297,7 +1277,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1307,10 +1287,10 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>46305.75</v>
+        <v>46306.75</v>
       </c>
       <c r="B38" t="n">
-        <v>349.52506</v>
+        <v>1133.16202</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1318,7 +1298,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1328,10 +1308,10 @@
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>46305.77083333334</v>
+        <v>46306.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>333.37805</v>
+        <v>351.4565</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1339,7 +1319,7 @@
         </is>
       </c>
       <c r="D39" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1349,10 +1329,10 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46305.79166666666</v>
+        <v>46306.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>346.84938</v>
+        <v>514.591</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1360,7 +1340,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1370,10 +1350,10 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46305.8125</v>
+        <v>46306.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>299.99</v>
+        <v>343.22431</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1381,7 +1361,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1391,10 +1371,10 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46305.83333333334</v>
+        <v>46306.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>299.99</v>
+        <v>493.46883</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1402,7 +1382,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1412,10 +1392,10 @@
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46305.85416666666</v>
+        <v>46306.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>341.01874</v>
+        <v>20111.11</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1423,7 +1403,7 @@
         </is>
       </c>
       <c r="D43" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1433,10 +1413,10 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46305.875</v>
+        <v>46306.875</v>
       </c>
       <c r="B44" t="n">
-        <v>338.69059</v>
+        <v>499.96</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1444,7 +1424,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1454,10 +1434,10 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46305.89583333334</v>
+        <v>46306.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>299.99</v>
+        <v>361.17453</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1465,7 +1445,7 @@
         </is>
       </c>
       <c r="D45" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1475,7 +1455,7 @@
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46305.91666666666</v>
+        <v>46306.91666666666</v>
       </c>
       <c r="B46" t="n">
         <v>299.99</v>
@@ -1486,7 +1466,7 @@
         </is>
       </c>
       <c r="D46" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1496,10 +1476,10 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46305.9375</v>
+        <v>46306.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>318.74561</v>
+        <v>299.99</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1507,7 +1487,7 @@
         </is>
       </c>
       <c r="D47" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1517,10 +1497,10 @@
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46305.95833333334</v>
+        <v>46306.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>296.07756</v>
+        <v>299.99</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1528,7 +1508,7 @@
         </is>
       </c>
       <c r="D48" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1538,10 +1518,10 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46305.97916666666</v>
+        <v>46306.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>212.56945</v>
+        <v>299.99</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1549,7 +1529,7 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest output (run 716)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,10 +482,30 @@
         <v>41.58</v>
       </c>
       <c r="E2" t="n">
-        <v>503.3737605</v>
+        <v>328.1669430000001</v>
       </c>
       <c r="F2" t="n">
-        <v>12.10615104617605</v>
+        <v>7.892422871572873</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46307.10416666666</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>46307.5625</v>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1475.751303</v>
+      </c>
+      <c r="F3" t="n">
+        <v>35.49185432900433</v>
       </c>
     </row>
   </sheetData>
@@ -499,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -891,7 +911,7 @@
         <v>46306.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>42.94</v>
+        <v>11.88</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -912,7 +932,7 @@
         <v>46306.375</v>
       </c>
       <c r="B20" t="n">
-        <v>0.99</v>
+        <v>-6.51</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -933,11 +953,11 @@
         <v>46306.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>0.99</v>
+        <v>-9.583769999999999</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -954,11 +974,11 @@
         <v>46306.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>0</v>
+        <v>-6.51</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -975,11 +995,11 @@
         <v>46306.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-6.51</v>
+        <v>-9.29766</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -996,11 +1016,11 @@
         <v>46306.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-9.12692</v>
+        <v>-18.51</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -1017,11 +1037,11 @@
         <v>46306.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-8.53078</v>
+        <v>-28.34427</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -1038,11 +1058,11 @@
         <v>46306.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-7.86</v>
+        <v>-18.51</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -1059,11 +1079,11 @@
         <v>46306.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-8.278510000000001</v>
+        <v>-10.5</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -1080,11 +1100,11 @@
         <v>46306.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-18.51</v>
+        <v>-23.5</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1101,11 +1121,11 @@
         <v>46306.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-11.82537</v>
+        <v>-18.51</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1122,11 +1142,11 @@
         <v>46306.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-8.3941</v>
+        <v>-10.5</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1143,11 +1163,11 @@
         <v>46306.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-7.58135</v>
+        <v>-7.54454</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1164,11 +1184,11 @@
         <v>46306.625</v>
       </c>
       <c r="B32" t="n">
-        <v>0</v>
+        <v>-6.5</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
@@ -1185,11 +1205,11 @@
         <v>46306.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>57.39</v>
+        <v>3e-05</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D33" s="3" t="n">
@@ -1206,11 +1226,11 @@
         <v>46306.66666666666</v>
       </c>
       <c r="B34" t="n">
-        <v>80.12007</v>
+        <v>81.19159999999999</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
@@ -1227,11 +1247,11 @@
         <v>46306.6875</v>
       </c>
       <c r="B35" t="n">
-        <v>99.62765</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D35" s="3" t="n">
@@ -1248,11 +1268,11 @@
         <v>46306.70833333334</v>
       </c>
       <c r="B36" t="n">
-        <v>137.67</v>
+        <v>130.01</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D36" s="3" t="n">
@@ -1269,11 +1289,11 @@
         <v>46306.72916666666</v>
       </c>
       <c r="B37" t="n">
-        <v>185.38711</v>
+        <v>248.06411</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D37" s="3" t="n">
@@ -1290,11 +1310,11 @@
         <v>46306.75</v>
       </c>
       <c r="B38" t="n">
-        <v>353.44825</v>
+        <v>1110.04483</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
@@ -1311,11 +1331,11 @@
         <v>46306.77083333334</v>
       </c>
       <c r="B39" t="n">
-        <v>299.99</v>
+        <v>513.9490500000001</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D39" s="3" t="n">
@@ -1332,11 +1352,11 @@
         <v>46306.79166666666</v>
       </c>
       <c r="B40" t="n">
-        <v>311.91</v>
+        <v>514.591</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -1353,11 +1373,11 @@
         <v>46306.8125</v>
       </c>
       <c r="B41" t="n">
-        <v>366.35072</v>
+        <v>289.88005</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -1374,11 +1394,11 @@
         <v>46306.83333333334</v>
       </c>
       <c r="B42" t="n">
-        <v>502.79364</v>
+        <v>266.41892</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -1395,11 +1415,11 @@
         <v>46306.85416666666</v>
       </c>
       <c r="B43" t="n">
-        <v>585.79788</v>
+        <v>194.80143</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D43" s="3" t="n">
@@ -1416,7 +1436,7 @@
         <v>46306.875</v>
       </c>
       <c r="B44" t="n">
-        <v>299.99</v>
+        <v>167.48</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1437,7 +1457,7 @@
         <v>46306.89583333334</v>
       </c>
       <c r="B45" t="n">
-        <v>299.99</v>
+        <v>166.6701</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1458,7 +1478,7 @@
         <v>46306.91666666666</v>
       </c>
       <c r="B46" t="n">
-        <v>299.99</v>
+        <v>132.222</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1479,7 +1499,7 @@
         <v>46306.9375</v>
       </c>
       <c r="B47" t="n">
-        <v>299.99</v>
+        <v>167.48</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1500,7 +1520,7 @@
         <v>46306.95833333334</v>
       </c>
       <c r="B48" t="n">
-        <v>299.99</v>
+        <v>145.86894</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1521,7 +1541,7 @@
         <v>46306.97916666666</v>
       </c>
       <c r="B49" t="n">
-        <v>299.99</v>
+        <v>129.69</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1532,6 +1552,1014 @@
         <v>46306</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B50" t="n">
+        <v>126.91</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46307.02083333334</v>
+      </c>
+      <c r="B51" t="n">
+        <v>121.51154</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46307.04166666666</v>
+      </c>
+      <c r="B52" t="n">
+        <v>127.6796</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46307.0625</v>
+      </c>
+      <c r="B53" t="n">
+        <v>120.00012</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46307.08333333334</v>
+      </c>
+      <c r="B54" t="n">
+        <v>119</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46307.10416666666</v>
+      </c>
+      <c r="B55" t="n">
+        <v>112.81966</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46307.125</v>
+      </c>
+      <c r="B56" t="n">
+        <v>118.6503</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46307.14583333334</v>
+      </c>
+      <c r="B57" t="n">
+        <v>119</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46307.16666666666</v>
+      </c>
+      <c r="B58" t="n">
+        <v>119</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46307.1875</v>
+      </c>
+      <c r="B59" t="n">
+        <v>107.87589</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46307.20833333334</v>
+      </c>
+      <c r="B60" t="n">
+        <v>106.52003</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46307.22916666666</v>
+      </c>
+      <c r="B61" t="n">
+        <v>106.6</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46307.25</v>
+      </c>
+      <c r="B62" t="n">
+        <v>102.29942</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46307.27083333334</v>
+      </c>
+      <c r="B63" t="n">
+        <v>97.36544000000001</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46307.29166666666</v>
+      </c>
+      <c r="B64" t="n">
+        <v>85.65257</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46307.3125</v>
+      </c>
+      <c r="B65" t="n">
+        <v>80.12035</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46307.33333333334</v>
+      </c>
+      <c r="B66" t="n">
+        <v>61.02</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46307.35416666666</v>
+      </c>
+      <c r="B67" t="n">
+        <v>2.14119</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46307.375</v>
+      </c>
+      <c r="B68" t="n">
+        <v>42.08</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46307.39583333334</v>
+      </c>
+      <c r="B69" t="n">
+        <v>-1.12006</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>46307.41666666666</v>
+      </c>
+      <c r="B70" t="n">
+        <v>-3.9093</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>46307.4375</v>
+      </c>
+      <c r="B71" t="n">
+        <v>-3.29273</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>46307.45833333334</v>
+      </c>
+      <c r="B72" t="n">
+        <v>-5.72006</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>46307.47916666666</v>
+      </c>
+      <c r="B73" t="n">
+        <v>6.13828</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>46307.5</v>
+      </c>
+      <c r="B74" t="n">
+        <v>64.95010000000001</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>46307.52083333334</v>
+      </c>
+      <c r="B75" t="n">
+        <v>88.88</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>46307.54166666666</v>
+      </c>
+      <c r="B76" t="n">
+        <v>106.52</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>46307.5625</v>
+      </c>
+      <c r="B77" t="n">
+        <v>119</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>46307.58333333334</v>
+      </c>
+      <c r="B78" t="n">
+        <v>129.71</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>46307.60416666666</v>
+      </c>
+      <c r="B79" t="n">
+        <v>121.01</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>46307.625</v>
+      </c>
+      <c r="B80" t="n">
+        <v>121.01</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>46307.64583333334</v>
+      </c>
+      <c r="B81" t="n">
+        <v>23107</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>46307.66666666666</v>
+      </c>
+      <c r="B82" t="n">
+        <v>23151.0001</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>46307.6875</v>
+      </c>
+      <c r="B83" t="n">
+        <v>23151.0001</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>46307.70833333334</v>
+      </c>
+      <c r="B84" t="n">
+        <v>23151.00034</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>46307.72916666666</v>
+      </c>
+      <c r="B85" t="n">
+        <v>23107</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46307.75</v>
+      </c>
+      <c r="B86" t="n">
+        <v>23151.0001</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46307.77083333334</v>
+      </c>
+      <c r="B87" t="n">
+        <v>23151.00046</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46307.79166666666</v>
+      </c>
+      <c r="B88" t="n">
+        <v>23151.0001</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46307.8125</v>
+      </c>
+      <c r="B89" t="n">
+        <v>23151.0001</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46307.83333333334</v>
+      </c>
+      <c r="B90" t="n">
+        <v>23151.0001</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46307.85416666666</v>
+      </c>
+      <c r="B91" t="n">
+        <v>10940.62523</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>46307.875</v>
+      </c>
+      <c r="B92" t="n">
+        <v>342.99958</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>46307.89583333334</v>
+      </c>
+      <c r="B93" t="n">
+        <v>192.70855</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>46307.91666666666</v>
+      </c>
+      <c r="B94" t="n">
+        <v>133.18318</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>46307.9375</v>
+      </c>
+      <c r="B95" t="n">
+        <v>189.00331</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>46307.95833333334</v>
+      </c>
+      <c r="B96" t="n">
+        <v>281.12481</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>46307.97916666666</v>
+      </c>
+      <c r="B97" t="n">
+        <v>166.67005</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>

<commit_message>
Update latest output (run 619)
</commit_message>
<xml_diff>
--- a/data/latest/optimisation_result.xlsx
+++ b/data/latest/optimisation_result.xlsx
@@ -470,10 +470,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46306.0625</v>
+        <v>46307</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46306.72916666666</v>
+        <v>46307.66666666666</v>
       </c>
       <c r="C2" t="n">
         <v>16</v>
@@ -482,10 +482,10 @@
         <v>60.48</v>
       </c>
       <c r="E2" t="n">
-        <v>1857.663209999999</v>
+        <v>25795.83235125</v>
       </c>
       <c r="F2" t="n">
-        <v>30.7153308531746</v>
+        <v>426.5183920510913</v>
       </c>
     </row>
   </sheetData>
@@ -531,10 +531,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="B2" t="n">
-        <v>137.05622</v>
+        <v>248.28</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -542,41 +542,41 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46306.02083333334</v>
+        <v>46307.02083333334</v>
       </c>
       <c r="B3" t="n">
-        <v>152.89228</v>
+        <v>210.19774</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>forecast</t>
+          <t>historical</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46306.04166666666</v>
+        <v>46307.04166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>156.08731</v>
+        <v>129.69</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -584,20 +584,20 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>OFF</t>
+          <t>ON</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46306.0625</v>
+        <v>46307.0625</v>
       </c>
       <c r="B5" t="n">
-        <v>149.49336</v>
+        <v>129.69</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -615,10 +615,10 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46306.08333333334</v>
+        <v>46307.08333333334</v>
       </c>
       <c r="B6" t="n">
-        <v>152.52671</v>
+        <v>128.72428</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -636,10 +636,10 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46306.10416666666</v>
+        <v>46307.10416666666</v>
       </c>
       <c r="B7" t="n">
-        <v>123.39695</v>
+        <v>129.69</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -657,10 +657,10 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46306.125</v>
+        <v>46307.125</v>
       </c>
       <c r="B8" t="n">
-        <v>152.73703</v>
+        <v>130.22</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -678,10 +678,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46306.14583333334</v>
+        <v>46307.14583333334</v>
       </c>
       <c r="B9" t="n">
-        <v>153.76487</v>
+        <v>127.25477</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -699,10 +699,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46306.16666666666</v>
+        <v>46307.16666666666</v>
       </c>
       <c r="B10" t="n">
-        <v>152.84596</v>
+        <v>124.29</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -720,10 +720,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46306.1875</v>
+        <v>46307.1875</v>
       </c>
       <c r="B11" t="n">
-        <v>152.86632</v>
+        <v>119</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -741,10 +741,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46306.20833333334</v>
+        <v>46307.20833333334</v>
       </c>
       <c r="B12" t="n">
-        <v>130.01</v>
+        <v>106.6</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -762,10 +762,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46306.22916666666</v>
+        <v>46307.22916666666</v>
       </c>
       <c r="B13" t="n">
-        <v>151.98421</v>
+        <v>119</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -783,10 +783,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46306.25</v>
+        <v>46307.25</v>
       </c>
       <c r="B14" t="n">
-        <v>137.94391</v>
+        <v>106.6</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -804,10 +804,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46306.27083333334</v>
+        <v>46307.27083333334</v>
       </c>
       <c r="B15" t="n">
-        <v>80.12009</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -825,10 +825,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46306.29166666666</v>
+        <v>46307.29166666666</v>
       </c>
       <c r="B16" t="n">
-        <v>63.74113</v>
+        <v>80.13</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -836,7 +836,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -846,10 +846,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46306.3125</v>
+        <v>46307.3125</v>
       </c>
       <c r="B17" t="n">
-        <v>51.86838</v>
+        <v>63.81834</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -867,10 +867,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46306.33333333334</v>
+        <v>46307.33333333334</v>
       </c>
       <c r="B18" t="n">
-        <v>33.8616</v>
+        <v>40.28718</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -888,10 +888,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46306.35416666666</v>
+        <v>46307.35416666666</v>
       </c>
       <c r="B19" t="n">
-        <v>11.88</v>
+        <v>27.9337</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -899,7 +899,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -909,10 +909,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46306.375</v>
+        <v>46307.375</v>
       </c>
       <c r="B20" t="n">
-        <v>-2.28805</v>
+        <v>42.08</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -920,7 +920,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -930,10 +930,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46306.39583333334</v>
+        <v>46307.39583333334</v>
       </c>
       <c r="B21" t="n">
-        <v>5.75782</v>
+        <v>26.4</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -951,10 +951,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46306.41666666666</v>
+        <v>46307.41666666666</v>
       </c>
       <c r="B22" t="n">
-        <v>-9.413399999999999</v>
+        <v>26.4</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -972,10 +972,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46306.4375</v>
+        <v>46307.4375</v>
       </c>
       <c r="B23" t="n">
-        <v>-10.01</v>
+        <v>26.4</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -983,7 +983,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -993,10 +993,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46306.45833333334</v>
+        <v>46307.45833333334</v>
       </c>
       <c r="B24" t="n">
-        <v>-9.45725</v>
+        <v>42.67</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -1014,10 +1014,10 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46306.47916666666</v>
+        <v>46307.47916666666</v>
       </c>
       <c r="B25" t="n">
-        <v>-18.51</v>
+        <v>3.89744</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1035,10 +1035,10 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46306.5</v>
+        <v>46307.5</v>
       </c>
       <c r="B26" t="n">
-        <v>-24.99064</v>
+        <v>80.12035</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1046,7 +1046,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1056,10 +1056,10 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46306.52083333334</v>
+        <v>46307.52083333334</v>
       </c>
       <c r="B27" t="n">
-        <v>-18.51</v>
+        <v>106.52</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1077,10 +1077,10 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>46306.54166666666</v>
+        <v>46307.54166666666</v>
       </c>
       <c r="B28" t="n">
-        <v>-18.48</v>
+        <v>119</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1088,7 +1088,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1098,10 +1098,10 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46306.5625</v>
+        <v>46307.5625</v>
       </c>
       <c r="B29" t="n">
-        <v>-12.19929</v>
+        <v>119</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1109,7 +1109,7 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1119,10 +1119,10 @@
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46306.58333333334</v>
+        <v>46307.58333333334</v>
       </c>
       <c r="B30" t="n">
-        <v>-9.78486</v>
+        <v>299</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1140,10 +1140,10 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46306.60416666666</v>
+        <v>46307.60416666666</v>
       </c>
       <c r="B31" t="n">
-        <v>-7.65584</v>
+        <v>129.71</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1161,10 +1161,10 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46306.625</v>
+        <v>46307.625</v>
       </c>
       <c r="B32" t="n">
-        <v>0</v>
+        <v>166.67005</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1172,7 +1172,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1182,10 +1182,10 @@
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46306.64583333334</v>
+        <v>46307.64583333334</v>
       </c>
       <c r="B33" t="n">
-        <v>27.01652</v>
+        <v>23151.0001</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1203,10 +1203,10 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46306.66666666666</v>
+        <v>46307.66666666666</v>
       </c>
  